<commit_message>
plan: PB-15 zamkniete; braki z makiety po stronie wezla jako PB-19 (sprint 19) i tryb agencji jako PB-20 (sprint 18)
- PB-15: ekran-wzorzec zaakceptowany, tokeny i klocki w components/panel, ciemny i jasny motyw, kontrast AA
- PB-19: ruch/TTFB/5xx, technologia strony i zakladka Logi — wymagaja dzialajacego wezla
- PB-20: przelacznik klienta w trybie agencji — nie wymaga wezla, wymaga decyzji o modelu Resellera

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$13</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$99)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$101)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$99,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$99,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$101,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$101,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$99,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$101,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$99,"zrobione",'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$101,"zrobione",'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P99"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7659,12 +7659,12 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-20</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>Tryb agencji: przełącznik klienta w menu bocznym</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
@@ -7679,14 +7679,14 @@
       </c>
       <c r="E89" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F89" s="10" t="n">
         <v>16</v>
       </c>
       <c r="G89" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H89" s="10" t="inlineStr">
         <is>
@@ -7695,12 +7695,12 @@
       </c>
       <c r="I89" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J89" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K89" s="10" t="inlineStr">
@@ -7715,17 +7715,17 @@
       </c>
       <c r="M89" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Decyzja o modelu zapisana w docs/VERRIS.md; przełącznik widoczny tylko dla kont z klientami; przełączenie zmienia kontekst usług, domen i płatności; guard uprawnień obejmuje nowe trasy (Z-04); testy w CI.</t>
         </is>
       </c>
       <c r="O89" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
+          <t>Element makiety („Piekarnia Zdrój · klient · 3 usługi” nad menu): konto agencji/resellera przełącza się między swoimi klientami bez wylogowania. Wymaga decyzji, jak Reseller (white-label) mapuje klientów na konta i uprawnienia (IAM).</t>
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr">
@@ -7737,12 +7737,12 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
@@ -7793,17 +7793,17 @@
       </c>
       <c r="M90" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N90" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7815,12 +7815,12 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
@@ -7839,20 +7839,24 @@
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G91" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H91" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H91" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I91" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J91" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K91" s="10" t="inlineStr">
@@ -7867,17 +7871,17 @@
       </c>
       <c r="M91" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury.</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7889,54 +7893,58 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="H92" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H92" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I92" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J92" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K92" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L92" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M92" s="11" t="inlineStr">
@@ -7946,12 +7954,12 @@
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7963,69 +7971,69 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G93" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H93" s="10" t="inlineStr"/>
       <c r="I93" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J93" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K93" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L93" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M93" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8037,12 +8045,12 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8052,16 +8060,16 @@
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>21</v>
@@ -8079,12 +8087,12 @@
       </c>
       <c r="K94" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M94" s="11" t="inlineStr">
@@ -8094,12 +8102,12 @@
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
+          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8111,12 +8119,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8126,12 +8134,12 @@
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F95" s="10" t="n">
@@ -8153,12 +8161,12 @@
       </c>
       <c r="K95" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L95" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M95" s="11" t="inlineStr">
@@ -8168,12 +8176,12 @@
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8185,12 +8193,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8200,7 +8208,7 @@
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E96" s="10" t="inlineStr">
@@ -8227,12 +8235,12 @@
       </c>
       <c r="K96" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L96" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M96" s="11" t="inlineStr">
@@ -8242,12 +8250,12 @@
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8259,31 +8267,31 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>21</v>
@@ -8301,27 +8309,27 @@
       </c>
       <c r="K97" s="10" t="inlineStr">
         <is>
+          <t>b.d.</t>
+        </is>
+      </c>
+      <c r="L97" s="11" t="inlineStr">
+        <is>
+          <t>poza kodem panelu</t>
+        </is>
+      </c>
+      <c r="M97" s="11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L97" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M97" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8333,69 +8341,69 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E98" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G98" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H98" s="10" t="inlineStr"/>
       <c r="I98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K98" s="10" t="inlineStr">
         <is>
+          <t>CZĘŚCIOWE</t>
+        </is>
+      </c>
+      <c r="L98" s="11" t="inlineStr">
+        <is>
+          <t>services.controller.ts:125</t>
+        </is>
+      </c>
+      <c r="M98" s="11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L98" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M98" s="11" t="inlineStr">
-        <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
-        </is>
-      </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8407,12 +8415,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8427,60 +8435,208 @@
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G99" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H99" s="10" t="inlineStr"/>
       <c r="I99" s="10" t="inlineStr">
         <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="J99" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-22</t>
+        </is>
+      </c>
+      <c r="K99" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L99" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M99" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N99" s="11" t="inlineStr">
+        <is>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+        </is>
+      </c>
+      <c r="O99" s="11" t="inlineStr">
+        <is>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+        </is>
+      </c>
+      <c r="P99" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t>PB-05</t>
+        </is>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>Test end-to-end „pierwszy klient”</t>
+        </is>
+      </c>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F100" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="G100" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H100" s="10" t="inlineStr"/>
+      <c r="I100" s="10" t="inlineStr">
+        <is>
           <t>2027-01-25</t>
         </is>
       </c>
-      <c r="J99" s="10" t="inlineStr">
+      <c r="J100" s="10" t="inlineStr">
         <is>
           <t>2027-01-29</t>
         </is>
       </c>
-      <c r="K99" s="10" t="inlineStr">
+      <c r="K100" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L99" s="11" t="inlineStr">
+      <c r="L100" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M99" s="11" t="inlineStr">
+      <c r="M100" s="11" t="inlineStr">
+        <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N100" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O100" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P100" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E101" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F101" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G101" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H101" s="10" t="inlineStr"/>
+      <c r="I101" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J101" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K101" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L101" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M101" s="11" t="inlineStr">
         <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N99" s="11" t="inlineStr">
+      <c r="N101" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O99" s="11" t="inlineStr">
+      <c r="O101" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P99" s="10" t="inlineStr">
+      <c r="P101" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P99"/>
-  <conditionalFormatting sqref="E2:E99">
+  <autoFilter ref="A1:P101"/>
+  <conditionalFormatting sqref="E2:E101">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -8500,7 +8656,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P99">
+  <conditionalFormatting sqref="P2:P101">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -8610,11 +8766,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A2,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A2,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -8655,11 +8811,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A3,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A3,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -8700,11 +8856,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A4,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A4,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -8745,11 +8901,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A5,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A5,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -8790,11 +8946,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A6,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A6,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -8835,11 +8991,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A7,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A7,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -8880,11 +9036,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A8,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A8,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -8925,11 +9081,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A9,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A9,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -8970,11 +9126,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A10,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A10,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -9015,11 +9171,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A11,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A11,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -9060,11 +9216,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A12,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A12,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -9105,11 +9261,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A13,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A13,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -9150,11 +9306,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A14,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A14,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -9195,11 +9351,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A15,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A15,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -9240,11 +9396,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A16,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A16,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -9285,11 +9441,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A17,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A17,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -9330,11 +9486,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A18,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A18,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -9375,11 +9531,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A19,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A19,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -9420,11 +9576,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A20,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A20,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -9461,11 +9617,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A21,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A21,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -9502,11 +9658,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A22,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A22,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -9543,11 +9699,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$99,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$99,A23,'Backlog do startu'!$F$2:$F$99)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A23,'Backlog do startu'!$F$2:$F$101)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">

</xml_diff>

<commit_message>
plan: PB-21 — DNS platformy i D3 edytora DNS/poczty w sprincie 18 (serwer testowy)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$102</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$13</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$101)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$102)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$101,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$101,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$102,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$102,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$101,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$102,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$101,"zrobione",'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$102,"zrobione",'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:P102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7737,12 +7737,12 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -7761,10 +7761,10 @@
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G90" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H90" s="10" t="inlineStr">
         <is>
@@ -7773,12 +7773,12 @@
       </c>
       <c r="I90" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J90" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K90" s="10" t="inlineStr">
@@ -7793,17 +7793,17 @@
       </c>
       <c r="M90" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N90" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM.</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7815,12 +7815,12 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
@@ -7835,7 +7835,7 @@
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
@@ -7871,17 +7871,17 @@
       </c>
       <c r="M91" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7893,12 +7893,12 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -7917,7 +7917,7 @@
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>19</v>
@@ -7954,12 +7954,12 @@
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury.</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7971,12 +7971,12 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -7995,20 +7995,24 @@
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G93" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H93" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H93" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I93" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J93" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K93" s="10" t="inlineStr">
@@ -8023,17 +8027,17 @@
       </c>
       <c r="M93" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8045,69 +8049,69 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G94" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H94" s="10" t="inlineStr"/>
       <c r="I94" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J94" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K94" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M94" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8119,12 +8123,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8134,16 +8138,16 @@
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G95" s="10" t="n">
         <v>21</v>
@@ -8166,7 +8170,7 @@
       </c>
       <c r="L95" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M95" s="11" t="inlineStr">
@@ -8181,7 +8185,7 @@
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8193,12 +8197,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8208,7 +8212,7 @@
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E96" s="10" t="inlineStr">
@@ -8235,12 +8239,12 @@
       </c>
       <c r="K96" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L96" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M96" s="11" t="inlineStr">
@@ -8250,12 +8254,12 @@
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8267,12 +8271,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8287,7 +8291,7 @@
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F97" s="10" t="n">
@@ -8314,7 +8318,7 @@
       </c>
       <c r="L97" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M97" s="11" t="inlineStr">
@@ -8329,7 +8333,7 @@
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8341,12 +8345,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8356,12 +8360,12 @@
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E98" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F98" s="10" t="n">
@@ -8383,12 +8387,12 @@
       </c>
       <c r="K98" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L98" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M98" s="11" t="inlineStr">
@@ -8398,12 +8402,12 @@
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8415,31 +8419,31 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G99" s="10" t="n">
         <v>21</v>
@@ -8457,27 +8461,27 @@
       </c>
       <c r="K99" s="10" t="inlineStr">
         <is>
+          <t>CZĘŚCIOWE</t>
+        </is>
+      </c>
+      <c r="L99" s="11" t="inlineStr">
+        <is>
+          <t>services.controller.ts:125</t>
+        </is>
+      </c>
+      <c r="M99" s="11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L99" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M99" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8489,12 +8493,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8509,24 +8513,24 @@
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F100" s="10" t="n">
         <v>16</v>
       </c>
       <c r="G100" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H100" s="10" t="inlineStr"/>
       <c r="I100" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K100" s="10" t="inlineStr">
@@ -8541,17 +8545,17 @@
       </c>
       <c r="M100" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8563,12 +8567,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8587,7 +8591,7 @@
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G101" s="10" t="n">
         <v>22</v>
@@ -8615,28 +8619,102 @@
       </c>
       <c r="M101" s="11" t="inlineStr">
         <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N101" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O101" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P101" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F102" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G102" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H102" s="10" t="inlineStr"/>
+      <c r="I102" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J102" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K102" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L102" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M102" s="11" t="inlineStr">
+        <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N101" s="11" t="inlineStr">
+      <c r="N102" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O101" s="11" t="inlineStr">
+      <c r="O102" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P101" s="10" t="inlineStr">
+      <c r="P102" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P101"/>
-  <conditionalFormatting sqref="E2:E101">
+  <autoFilter ref="A1:P102"/>
+  <conditionalFormatting sqref="E2:E102">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -8656,7 +8734,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P101">
+  <conditionalFormatting sqref="P2:P102">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -8766,11 +8844,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A2,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A2,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -8811,11 +8889,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A3,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A3,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -8856,11 +8934,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A4,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A4,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -8901,11 +8979,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A5,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A5,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -8946,11 +9024,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A6,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A6,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -8991,11 +9069,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A7,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A7,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -9036,11 +9114,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A8,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A8,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -9081,11 +9159,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A9,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A9,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -9126,11 +9204,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A10,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A10,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -9171,11 +9249,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A11,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A11,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -9216,11 +9294,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A12,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A12,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -9261,11 +9339,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A13,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A13,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -9306,11 +9384,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A14,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A14,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -9351,11 +9429,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A15,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A15,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -9396,11 +9474,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A16,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A16,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -9441,11 +9519,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A17,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A17,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -9486,11 +9564,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A18,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A18,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -9531,11 +9609,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A19,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A19,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -9547,7 +9625,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>BLOK DOKUMENTOW — przesuniety na koniec decyzja wlasciciela 2026-09-22: najpierw kod i infrastruktura, dokumenty na sam koniec, przed pierwszym klientem. Kolejnosc wewnatrz bloku wymuszona zaleznosciami: regulamin (PB-03) przed kredytami SLA (N-16), cennik (PB-07) przed landingiem (PB-06), landing przed kampania (PB-10), wszystko przed sciezka pierwszego klienta (PB-05). N-16 (kredyty SLA) po PB-03, bo regulamin obiecuje kredyty — najpierw przeliczyc je na realnych danych z probe-ow. Cennik zgodny z PB-01 (45 zl/mies brutto, 399 zl/rok).</t>
+          <t>BLOK DOKUMENTOW — przesuniety na koniec decyzja wlasciciela 2026-09-22: najpierw kod i infrastruktura, dokumenty na sam koniec, przed pierwszym klientem. Kolejnosc wewnatrz bloku wymuszona zaleznosciami: regulamin (PB-03) przed kredytami SLA (N-16), cennik (PB-07) przed landingiem (PB-06), landing przed kampania (PB-10), wszystko przed sciezka pierwszego klienta (PB-05). N-16 (kredyty SLA) po PB-03, bo regulamin obiecuje kredyty — najpierw przeliczyc je na realnych danych z probe-ow. Cennik zgodny z PB-01 (45 zl/mies brutto, 399 zl/rok). | 2026-09-23: PB-21 (DNS platformy i D3 edytora DNS/poczty) tutaj, bo w tym sprincie pojawia się serwer testowy.</t>
         </is>
       </c>
     </row>
@@ -9576,11 +9654,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A20,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A20,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -9617,11 +9695,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A21,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A21,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -9658,11 +9736,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A22,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A22,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -9699,11 +9777,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$101,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$102,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$101,A23,'Backlog do startu'!$F$2:$F$101)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$102,A23,'Backlog do startu'!$F$2:$F$102)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">

</xml_diff>

<commit_message>
plan: PB-23 — każdy widok osiągalny z menu (zasada właściciela), sprint 16
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$13</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$103)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$104)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$103,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$103,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$104,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$104,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$103,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$104,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$103,"zrobione",'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$104,"zrobione",'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P103"/>
+  <dimension ref="A1:P104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7269,34 +7269,34 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>PB-23</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Podpisane DPA z subprocesorami (część)</t>
+          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F84" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H84" s="10" t="inlineStr">
         <is>
@@ -7305,22 +7305,22 @@
       </c>
       <c r="I84" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="J84" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="K84" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
@@ -7330,12 +7330,12 @@
       </c>
       <c r="N84" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
         </is>
       </c>
       <c r="O84" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile.</t>
+          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem.</t>
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr">
@@ -7347,31 +7347,31 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>PB-03</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Finalizacja dokumentów prawnych 1.0.0</t>
+          <t>Podpisane DPA z subprocesorami (część)</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F85" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G85" s="10" t="n">
         <v>17</v>
@@ -7393,27 +7393,27 @@
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
+          <t>BRAK</t>
+        </is>
+      </c>
+      <c r="L85" s="11" t="inlineStr">
+        <is>
+          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
+        </is>
+      </c>
+      <c r="M85" s="11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L85" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M85" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O85" s="11" t="inlineStr">
         <is>
-          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu.</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile.</t>
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr">
@@ -7425,12 +7425,12 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>PB-04</t>
+          <t>PB-03</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
+          <t>Finalizacja dokumentów prawnych 1.0.0</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -7445,11 +7445,11 @@
       </c>
       <c r="E86" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F86" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G86" s="10" t="n">
         <v>17</v>
@@ -7486,12 +7486,12 @@
       </c>
       <c r="N86" s="11" t="inlineStr">
         <is>
-          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
+          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
         </is>
       </c>
       <c r="O86" s="11" t="inlineStr">
         <is>
-          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów.</t>
+          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu.</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr">
@@ -7503,34 +7503,34 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>N-16</t>
+          <t>PB-04</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>SLA z zapisanymi kredytami</t>
+          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F87" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G87" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H87" s="10" t="inlineStr">
         <is>
@@ -7539,37 +7539,37 @@
       </c>
       <c r="I87" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-21</t>
         </is>
       </c>
       <c r="J87" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="K87" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L87" s="11" t="inlineStr">
         <is>
-          <t>sla-credit.scheduler.ts:79 — if (!policy.enabled) return; SLA_CREDITS_ENABLED default '0' (platform-settings.keys.ts:116)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M87" s="11" t="inlineStr">
         <is>
-          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N87" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
         </is>
       </c>
       <c r="O87" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza.</t>
+          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów.</t>
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr">
@@ -7581,31 +7581,31 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>PB-07</t>
+          <t>N-16</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Treści i cennik na verris.pl</t>
+          <t>SLA z zapisanymi kredytami</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>18</v>
@@ -7627,27 +7627,27 @@
       </c>
       <c r="K88" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>sla-credit.scheduler.ts:79 — if (!policy.enabled) return; SLA_CREDITS_ENABLED default '0' (platform-settings.keys.ts:116)</t>
         </is>
       </c>
       <c r="M88" s="11" t="inlineStr">
         <is>
-          <t>PB-01 (cennik zależy od unit economics)</t>
+          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
         </is>
       </c>
       <c r="N88" s="11" t="inlineStr">
         <is>
-          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O88" s="11" t="inlineStr">
         <is>
-          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku.</t>
+          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza.</t>
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>PB-11</t>
+          <t>PB-07</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
+          <t>Treści i cennik na verris.pl</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
@@ -7683,7 +7683,7 @@
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G89" s="10" t="n">
         <v>18</v>
@@ -7715,17 +7715,17 @@
       </c>
       <c r="M89" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-01 (cennik zależy od unit economics)</t>
         </is>
       </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
+          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
         </is>
       </c>
       <c r="O89" s="11" t="inlineStr">
         <is>
-          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień.</t>
+          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku.</t>
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr">
@@ -7737,12 +7737,12 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>PB-20</t>
+          <t>PB-11</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Tryb agencji: przełącznik klienta w menu bocznym</t>
+          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -7757,11 +7757,11 @@
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>18</v>
@@ -7798,12 +7798,12 @@
       </c>
       <c r="N90" s="11" t="inlineStr">
         <is>
-          <t>Decyzja o modelu zapisana w docs/VERRIS.md; przełącznik widoczny tylko dla kont z klientami; przełączenie zmienia kontekst usług, domen i płatności; guard uprawnień obejmuje nowe trasy (Z-04); testy w CI.</t>
+          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
         </is>
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>Element makiety („Piekarnia Zdrój · klient · 3 usługi” nad menu): konto agencji/resellera przełącza się między swoimi klientami bez wylogowania. Wymaga decyzji, jak Reseller (white-label) mapuje klientów na konta i uprawnienia (IAM).</t>
+          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień.</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7815,12 +7815,12 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>PB-21</t>
+          <t>PB-20</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>DNS platformy i poczty na serwerze testowym</t>
+          <t>Tryb agencji: przełącznik klienta w menu bocznym</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
@@ -7835,11 +7835,11 @@
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G91" s="10" t="n">
         <v>18</v>
@@ -7876,12 +7876,12 @@
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
+          <t>Decyzja o modelu zapisana w docs/VERRIS.md; przełącznik widoczny tylko dla kont z klientami; przełączenie zmienia kontekst usług, domen i płatności; guard uprawnień obejmuje nowe trasy (Z-04); testy w CI.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
+          <t>Element makiety („Piekarnia Zdrój · klient · 3 usługi” nad menu): konto agencji/resellera przełącza się między swoimi klientami bez wylogowania. Wymaga decyzji, jak Reseller (white-label) mapuje klientów na konta i uprawnienia (IAM).</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7893,12 +7893,12 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -7917,10 +7917,10 @@
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H92" s="10" t="inlineStr">
         <is>
@@ -7929,12 +7929,12 @@
       </c>
       <c r="I92" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J92" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K92" s="10" t="inlineStr">
@@ -7949,17 +7949,17 @@
       </c>
       <c r="M92" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7971,12 +7971,12 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -7991,7 +7991,7 @@
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
@@ -8027,17 +8027,17 @@
       </c>
       <c r="M93" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8049,12 +8049,12 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8073,7 +8073,7 @@
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>19</v>
@@ -8110,12 +8110,12 @@
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury.</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8127,12 +8127,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8151,20 +8151,24 @@
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G95" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H95" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H95" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I95" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J95" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K95" s="10" t="inlineStr">
@@ -8179,17 +8183,17 @@
       </c>
       <c r="M95" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8201,69 +8205,69 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E96" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F96" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G96" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H96" s="10" t="inlineStr"/>
       <c r="I96" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J96" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K96" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L96" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M96" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8275,12 +8279,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8290,16 +8294,16 @@
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>21</v>
@@ -8322,7 +8326,7 @@
       </c>
       <c r="L97" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M97" s="11" t="inlineStr">
@@ -8337,7 +8341,7 @@
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8349,12 +8353,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8364,7 +8368,7 @@
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E98" s="10" t="inlineStr">
@@ -8391,12 +8395,12 @@
       </c>
       <c r="K98" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L98" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M98" s="11" t="inlineStr">
@@ -8406,12 +8410,12 @@
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8423,12 +8427,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8443,7 +8447,7 @@
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
@@ -8470,7 +8474,7 @@
       </c>
       <c r="L99" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M99" s="11" t="inlineStr">
@@ -8485,7 +8489,7 @@
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8497,12 +8501,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8512,12 +8516,12 @@
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F100" s="10" t="n">
@@ -8539,12 +8543,12 @@
       </c>
       <c r="K100" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L100" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M100" s="11" t="inlineStr">
@@ -8554,12 +8558,12 @@
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8571,31 +8575,31 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G101" s="10" t="n">
         <v>21</v>
@@ -8613,27 +8617,27 @@
       </c>
       <c r="K101" s="10" t="inlineStr">
         <is>
+          <t>CZĘŚCIOWE</t>
+        </is>
+      </c>
+      <c r="L101" s="11" t="inlineStr">
+        <is>
+          <t>services.controller.ts:125</t>
+        </is>
+      </c>
+      <c r="M101" s="11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L101" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M101" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8645,12 +8649,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8665,24 +8669,24 @@
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
         <v>16</v>
       </c>
       <c r="G102" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H102" s="10" t="inlineStr"/>
       <c r="I102" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J102" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K102" s="10" t="inlineStr">
@@ -8697,17 +8701,17 @@
       </c>
       <c r="M102" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8719,12 +8723,12 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8743,7 +8747,7 @@
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G103" s="10" t="n">
         <v>22</v>
@@ -8771,28 +8775,102 @@
       </c>
       <c r="M103" s="11" t="inlineStr">
         <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N103" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O103" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P103" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B104" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F104" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G104" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H104" s="10" t="inlineStr"/>
+      <c r="I104" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J104" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K104" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L104" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M104" s="11" t="inlineStr">
+        <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N103" s="11" t="inlineStr">
+      <c r="N104" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O103" s="11" t="inlineStr">
+      <c r="O104" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P103" s="10" t="inlineStr">
+      <c r="P104" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P103"/>
-  <conditionalFormatting sqref="E2:E103">
+  <autoFilter ref="A1:P104"/>
+  <conditionalFormatting sqref="E2:E104">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -8812,7 +8890,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P103">
+  <conditionalFormatting sqref="P2:P104">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -8922,11 +9000,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A2,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A2,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -8967,11 +9045,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A3,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A3,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -9012,11 +9090,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A4,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A4,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -9057,11 +9135,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A5,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A5,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -9102,11 +9180,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A6,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A6,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -9147,11 +9225,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A7,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A7,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -9192,11 +9270,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A8,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A8,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -9237,11 +9315,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A9,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A9,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -9282,11 +9360,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A10,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A10,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -9327,11 +9405,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A11,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A11,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -9372,11 +9450,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A12,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A12,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -9417,11 +9495,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A13,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A13,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -9462,11 +9540,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A14,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A14,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -9507,11 +9585,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A15,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A15,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -9552,11 +9630,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A16,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A16,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -9597,11 +9675,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A17,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A17,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -9642,11 +9720,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A18,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A18,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -9687,11 +9765,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A19,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A19,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -9732,11 +9810,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A20,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A20,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -9773,11 +9851,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A21,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A21,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -9814,11 +9892,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A22,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A22,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -9855,11 +9933,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$103,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$104,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$103,A23,'Backlog do startu'!$F$2:$F$103)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$104,A23,'Backlog do startu'!$F$2:$F$104)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">

</xml_diff>

<commit_message>
docs: sprint 17 — dokumenty prawne do stanu faktycznego, decyzje KSC/AI/kontakt
Regulamin 1.2.0 (§9 ust. 4: faktury VAT z programu księgowego, dokument
rozliczeniowy do czasu faktury), polityka 1.0.2 (Streamsoft Firmino),
lista podwykonawców i tracker DPA (Firmino, ClouDNS, AI wyłączone),
LEGAL_LIVE_INPUTS na @verris.pl, skrypt publikacji bez fałszywego
„po akceptacji prawnika”. Decyzje w docs/VERRIS.md; PB-24 (KSC) w sprincie 18.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$106</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$13</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$105)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$106)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$105,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$105,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$106,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$106,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$105,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$106,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$105,"zrobione",'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$106,"zrobione",'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P105"/>
+  <dimension ref="A1:P106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7421,7 +7421,7 @@
       </c>
       <c r="O85" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile.</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18.</t>
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr">
@@ -7499,7 +7499,7 @@
       </c>
       <c r="O86" s="11" t="inlineStr">
         <is>
-          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu.</t>
+          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@.</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr">
@@ -8057,12 +8057,12 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-24</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8081,10 +8081,10 @@
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G94" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H94" s="10" t="inlineStr">
         <is>
@@ -8093,12 +8093,12 @@
       </c>
       <c r="I94" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J94" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K94" s="10" t="inlineStr">
@@ -8113,17 +8113,17 @@
       </c>
       <c r="M94" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
+          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h).</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8135,12 +8135,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="E95" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F95" s="10" t="n">
@@ -8191,17 +8191,17 @@
       </c>
       <c r="M95" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,12 +8213,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8237,7 +8237,7 @@
         </is>
       </c>
       <c r="F96" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G96" s="10" t="n">
         <v>19</v>
@@ -8274,12 +8274,12 @@
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury.</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,12 +8291,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8315,20 +8315,24 @@
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G97" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H97" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H97" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I97" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J97" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K97" s="10" t="inlineStr">
@@ -8343,17 +8347,17 @@
       </c>
       <c r="M97" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8365,69 +8369,69 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E98" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G98" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H98" s="10" t="inlineStr"/>
       <c r="I98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K98" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L98" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M98" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8439,12 +8443,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8454,16 +8458,16 @@
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G99" s="10" t="n">
         <v>21</v>
@@ -8486,7 +8490,7 @@
       </c>
       <c r="L99" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M99" s="11" t="inlineStr">
@@ -8501,7 +8505,7 @@
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8513,12 +8517,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8528,7 +8532,7 @@
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
@@ -8555,12 +8559,12 @@
       </c>
       <c r="K100" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L100" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M100" s="11" t="inlineStr">
@@ -8570,12 +8574,12 @@
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8587,12 +8591,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8607,7 +8611,7 @@
       </c>
       <c r="E101" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F101" s="10" t="n">
@@ -8634,7 +8638,7 @@
       </c>
       <c r="L101" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M101" s="11" t="inlineStr">
@@ -8649,7 +8653,7 @@
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8661,12 +8665,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8676,12 +8680,12 @@
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
@@ -8703,12 +8707,12 @@
       </c>
       <c r="K102" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L102" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M102" s="11" t="inlineStr">
@@ -8718,12 +8722,12 @@
       </c>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8735,31 +8739,31 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G103" s="10" t="n">
         <v>21</v>
@@ -8777,27 +8781,27 @@
       </c>
       <c r="K103" s="10" t="inlineStr">
         <is>
+          <t>CZĘŚCIOWE</t>
+        </is>
+      </c>
+      <c r="L103" s="11" t="inlineStr">
+        <is>
+          <t>services.controller.ts:125</t>
+        </is>
+      </c>
+      <c r="M103" s="11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L103" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M103" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="N103" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8809,12 +8813,12 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
@@ -8829,24 +8833,24 @@
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F104" s="10" t="n">
         <v>16</v>
       </c>
       <c r="G104" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H104" s="10" t="inlineStr"/>
       <c r="I104" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J104" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K104" s="10" t="inlineStr">
@@ -8861,17 +8865,17 @@
       </c>
       <c r="M104" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8883,12 +8887,12 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -8907,7 +8911,7 @@
         </is>
       </c>
       <c r="F105" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G105" s="10" t="n">
         <v>22</v>
@@ -8935,28 +8939,102 @@
       </c>
       <c r="M105" s="11" t="inlineStr">
         <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N105" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O105" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P105" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E106" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F106" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G106" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H106" s="10" t="inlineStr"/>
+      <c r="I106" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J106" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K106" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L106" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M106" s="11" t="inlineStr">
+        <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N105" s="11" t="inlineStr">
+      <c r="N106" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O105" s="11" t="inlineStr">
+      <c r="O106" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P105" s="10" t="inlineStr">
+      <c r="P106" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P105"/>
-  <conditionalFormatting sqref="E2:E105">
+  <autoFilter ref="A1:P106"/>
+  <conditionalFormatting sqref="E2:E106">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -8976,7 +9054,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P105">
+  <conditionalFormatting sqref="P2:P106">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -9086,11 +9164,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A2,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A2,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -9131,11 +9209,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A3,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A3,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -9176,11 +9254,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A4,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A4,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -9221,11 +9299,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A5,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A5,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -9266,11 +9344,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A6,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A6,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -9311,11 +9389,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A7,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A7,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -9356,11 +9434,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A8,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A8,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -9401,11 +9479,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A9,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A9,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -9446,11 +9524,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A10,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A10,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -9491,11 +9569,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A11,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A11,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -9536,11 +9614,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A12,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A12,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -9581,11 +9659,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A13,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A13,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -9626,11 +9704,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A14,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A14,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -9671,11 +9749,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A15,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A15,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -9716,11 +9794,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A16,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A16,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -9761,11 +9839,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A17,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A17,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -9806,11 +9884,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A18,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A18,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -9851,11 +9929,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A19,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A19,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -9896,11 +9974,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A20,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A20,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -9937,11 +10015,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A21,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A21,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -9978,11 +10056,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A22,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A22,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -10019,11 +10097,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$105,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$105,A23,'Backlog do startu'!$F$2:$F$105)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A23,'Backlog do startu'!$F$2:$F$106)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">

</xml_diff>

<commit_message>
audyt: PB-25 — white label na węźle (sprint 18)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$107</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$21</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$106)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$107)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$106,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$106,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$107,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$107,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$106,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$107,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$106,"zrobione",'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$107,"zrobione",'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P106"/>
+  <dimension ref="A1:P107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8135,12 +8135,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-25</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>White label na węźle — klient nie widzi DirectAdmina</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8159,10 +8159,10 @@
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G95" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H95" s="10" t="inlineStr">
         <is>
@@ -8171,12 +8171,12 @@
       </c>
       <c r="I95" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J95" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K95" s="10" t="inlineStr">
@@ -8191,17 +8191,17 @@
       </c>
       <c r="M95" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
+          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,12 +8213,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="E96" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F96" s="10" t="n">
@@ -8269,17 +8269,17 @@
       </c>
       <c r="M96" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,12 +8291,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8315,7 +8315,7 @@
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>19</v>
@@ -8352,12 +8352,12 @@
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8369,12 +8369,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8393,20 +8393,24 @@
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G98" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H98" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H98" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K98" s="10" t="inlineStr">
@@ -8421,17 +8425,17 @@
       </c>
       <c r="M98" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8443,69 +8447,69 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G99" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H99" s="10" t="inlineStr"/>
       <c r="I99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K99" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L99" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M99" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8517,12 +8521,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8532,16 +8536,16 @@
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G100" s="10" t="n">
         <v>21</v>
@@ -8564,7 +8568,7 @@
       </c>
       <c r="L100" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M100" s="11" t="inlineStr">
@@ -8579,7 +8583,7 @@
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8591,12 +8595,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8606,7 +8610,7 @@
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
@@ -8633,12 +8637,12 @@
       </c>
       <c r="K101" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L101" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M101" s="11" t="inlineStr">
@@ -8648,12 +8652,12 @@
       </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8665,12 +8669,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8685,7 +8689,7 @@
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
@@ -8712,7 +8716,7 @@
       </c>
       <c r="L102" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M102" s="11" t="inlineStr">
@@ -8727,7 +8731,7 @@
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1.</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8739,12 +8743,12 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8754,12 +8758,12 @@
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
@@ -8781,12 +8785,12 @@
       </c>
       <c r="K103" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L103" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M103" s="11" t="inlineStr">
@@ -8796,12 +8800,12 @@
       </c>
       <c r="N103" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8813,31 +8817,31 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F104" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G104" s="10" t="n">
         <v>21</v>
@@ -8855,12 +8859,12 @@
       </c>
       <c r="K104" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L104" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>services.controller.ts:125</t>
         </is>
       </c>
       <c r="M104" s="11" t="inlineStr">
@@ -8870,12 +8874,12 @@
       </c>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8887,12 +8891,12 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -8907,24 +8911,24 @@
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F105" s="10" t="n">
         <v>16</v>
       </c>
       <c r="G105" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H105" s="10" t="inlineStr"/>
       <c r="I105" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J105" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K105" s="10" t="inlineStr">
@@ -8939,17 +8943,17 @@
       </c>
       <c r="M105" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N105" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O105" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr">
@@ -8961,12 +8965,12 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -8985,7 +8989,7 @@
         </is>
       </c>
       <c r="F106" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G106" s="10" t="n">
         <v>22</v>
@@ -9013,28 +9017,102 @@
       </c>
       <c r="M106" s="11" t="inlineStr">
         <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N106" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O106" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P106" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D107" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E107" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F107" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G107" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H107" s="10" t="inlineStr"/>
+      <c r="I107" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J107" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K107" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L107" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M107" s="11" t="inlineStr">
+        <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N106" s="11" t="inlineStr">
+      <c r="N107" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O106" s="11" t="inlineStr">
+      <c r="O107" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P106" s="10" t="inlineStr">
+      <c r="P107" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P106"/>
-  <conditionalFormatting sqref="E2:E106">
+  <autoFilter ref="A1:P107"/>
+  <conditionalFormatting sqref="E2:E107">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -9054,7 +9132,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P106">
+  <conditionalFormatting sqref="P2:P107">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -9164,11 +9242,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A2,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A2,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -9209,11 +9287,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A3,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A3,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -9254,11 +9332,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A4,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A4,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -9299,11 +9377,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A5,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A5,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -9344,11 +9422,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A6,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A6,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -9389,11 +9467,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A7,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A7,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -9434,11 +9512,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A8,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A8,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -9479,11 +9557,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A9,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A9,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -9524,11 +9602,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A10,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A10,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -9569,11 +9647,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A11,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A11,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -9614,11 +9692,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A12,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A12,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -9659,11 +9737,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A13,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A13,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -9704,11 +9782,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A14,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A14,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -9749,11 +9827,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A15,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A15,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -9794,11 +9872,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A16,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A16,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -9839,11 +9917,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A17,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A17,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -9884,11 +9962,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A18,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A18,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -9929,11 +10007,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A19,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A19,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -9974,11 +10052,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A20,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A20,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -10015,11 +10093,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A21,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A21,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -10056,11 +10134,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A22,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A22,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -10097,11 +10175,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$106,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$106,A23,'Backlog do startu'!$F$2:$F$106)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A23,'Backlog do startu'!$F$2:$F$107)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">

</xml_diff>

<commit_message>
plan: PB-26 — otwarte testy (beta) przed decyzją GO, plan w docs/ops/BETA_TESTY.md
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$108</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$21</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$107)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$108)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$107,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$107,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$108,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$108,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$107,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$108,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$107,"zrobione",'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$108,"zrobione",'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P107"/>
+  <dimension ref="A1:P108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8965,12 +8965,12 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-26</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -8985,11 +8985,11 @@
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F106" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G106" s="10" t="n">
         <v>22</v>
@@ -9017,17 +9017,17 @@
       </c>
       <c r="M106" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N106" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
         </is>
       </c>
       <c r="O106" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina.</t>
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr">
@@ -9039,12 +9039,12 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -9063,7 +9063,7 @@
         </is>
       </c>
       <c r="F107" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G107" s="10" t="n">
         <v>22</v>
@@ -9091,28 +9091,102 @@
       </c>
       <c r="M107" s="11" t="inlineStr">
         <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N107" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O107" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P107" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C108" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D108" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E108" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F108" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G108" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H108" s="10" t="inlineStr"/>
+      <c r="I108" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J108" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K108" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L108" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M108" s="11" t="inlineStr">
+        <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N107" s="11" t="inlineStr">
+      <c r="N108" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O107" s="11" t="inlineStr">
+      <c r="O108" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P107" s="10" t="inlineStr">
+      <c r="P108" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P107"/>
-  <conditionalFormatting sqref="E2:E107">
+  <autoFilter ref="A1:P108"/>
+  <conditionalFormatting sqref="E2:E108">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -9132,7 +9206,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P107">
+  <conditionalFormatting sqref="P2:P108">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -9242,11 +9316,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A2,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A2,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -9287,11 +9361,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A3,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A3,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -9332,11 +9406,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A4,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A4,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -9377,11 +9451,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A5,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A5,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -9422,11 +9496,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A6,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A6,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -9467,11 +9541,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A7,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A7,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -9512,11 +9586,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A8,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A8,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -9557,11 +9631,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A9,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A9,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -9602,11 +9676,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A10,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A10,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -9647,11 +9721,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A11,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A11,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -9692,11 +9766,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A12,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A12,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -9737,11 +9811,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A13,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A13,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -9782,11 +9856,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A14,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A14,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -9827,11 +9901,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A15,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A15,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -9872,11 +9946,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A16,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A16,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -9917,11 +9991,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A17,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A17,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -9962,11 +10036,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A18,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A18,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -10007,11 +10081,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A19,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A19,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -10052,11 +10126,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A20,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A20,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -10093,11 +10167,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A21,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A21,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -10134,11 +10208,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A22,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A22,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -10175,11 +10249,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$107,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$107,A23,'Backlog do startu'!$F$2:$F$107)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A23,'Backlog do startu'!$F$2:$F$108)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">
@@ -10191,7 +10265,7 @@
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>BLOK DOKUMENTOW — przesuniety na koniec decyzja wlasciciela 2026-09-22: najpierw kod i infrastruktura, dokumenty na sam koniec, przed pierwszym klientem. Kolejnosc wewnatrz bloku wymuszona zaleznosciami: regulamin (PB-03) przed kredytami SLA (N-16), cennik (PB-07) przed landingiem (PB-06), landing przed kampania (PB-10), wszystko przed sciezka pierwszego klienta (PB-05). Kampania powstaje wstrzymana. PB-05 to jedyny moment w planie, w ktorym powstaje dowod D3 calej sciezki — kazdy nieudany krok wraca do backlogu jako bloker i przesuwa start. PB-05 wymaga wezla, dlatego stoi zaraz po sprincie 18.</t>
+          <t>BLOK DOKUMENTOW — przesuniety na koniec decyzja wlasciciela 2026-09-22: najpierw kod i infrastruktura, dokumenty na sam koniec, przed pierwszym klientem. Kolejnosc wewnatrz bloku wymuszona zaleznosciami: regulamin (PB-03) przed kredytami SLA (N-16), cennik (PB-07) przed landingiem (PB-06), landing przed kampania (PB-10), wszystko przed sciezka pierwszego klienta (PB-05). Kampania powstaje wstrzymana. PB-05 to jedyny moment w planie, w ktorym powstaje dowod D3 calej sciezki — kazdy nieudany krok wraca do backlogu jako bloker i przesuwa start. PB-05 wymaga wezla, dlatego stoi zaraz po sprincie 18. | 2026-09-24: PB-26 (otwarte testy z zaproszonymi osobami) przed PB-05/PB-12 — decyzja GO dopiero po spełnieniu kryteriów końca bety (docs/ops/BETA_TESTY.md).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
decyzja(PB-20): tryb agencji po starcie — sprint 23 „Po starcie”, notka w VERRIS.md
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$108</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$21</definedName>
   </definedNames>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>22 sprintów · 30 h netto na sprint · wygenerowane 2026-09-25 z audyt/dane/</t>
+          <t>23 sprintów · 30 h netto na sprint · wygenerowane 2026-09-25 z audyt/dane/</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>660</v>
+        <v>690</v>
       </c>
     </row>
     <row r="9">
@@ -7901,12 +7901,12 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>PB-20</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Tryb agencji: przełącznik klienta w menu bocznym</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -7921,11 +7921,11 @@
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>18</v>
@@ -7962,12 +7962,12 @@
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Decyzja o modelu zapisana w docs/VERRIS.md; przełącznik widoczny tylko dla kont z klientami; przełączenie zmienia kontekst usług, domen i płatności; guard uprawnień obejmuje nowe trasy (Z-04); testy w CI.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>Element makiety („Piekarnia Zdrój · klient · 3 usługi” nad menu): konto agencji/resellera przełącza się między swoimi klientami bez wylogowania. Wymaga decyzji, jak Reseller (white-label) mapuje klientów na konta i uprawnienia (IAM).</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>PB-21</t>
+          <t>PB-24</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>DNS platformy i poczty na serwerze testowym</t>
+          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -8003,7 +8003,7 @@
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G93" s="10" t="n">
         <v>18</v>
@@ -8040,12 +8040,12 @@
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
+          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
+          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h).</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8057,12 +8057,12 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>PB-24</t>
+          <t>PB-25</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
+          <t>White label na węźle — klient nie widzi DirectAdmina</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8081,7 +8081,7 @@
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>18</v>
@@ -8118,12 +8118,12 @@
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
+          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h).</t>
+          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8135,12 +8135,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>PB-25</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>White label na węźle — klient nie widzi DirectAdmina</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8159,10 +8159,10 @@
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G95" s="10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H95" s="10" t="inlineStr">
         <is>
@@ -8171,12 +8171,12 @@
       </c>
       <c r="I95" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J95" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K95" s="10" t="inlineStr">
@@ -8191,17 +8191,17 @@
       </c>
       <c r="M95" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,12 +8213,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="E96" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F96" s="10" t="n">
@@ -8269,17 +8269,17 @@
       </c>
       <c r="M96" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach.</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,12 +8291,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8315,7 +8315,7 @@
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>19</v>
@@ -8352,12 +8352,12 @@
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8369,12 +8369,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8393,24 +8393,20 @@
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="G98" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="H98" s="10" t="inlineStr">
-        <is>
-          <t>Faza 3 — Wejście na rynek</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="H98" s="10" t="inlineStr"/>
       <c r="I98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K98" s="10" t="inlineStr">
@@ -8425,17 +8421,17 @@
       </c>
       <c r="M98" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”).</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8447,69 +8443,69 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G99" s="10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H99" s="10" t="inlineStr"/>
       <c r="I99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K99" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L99" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M99" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8521,12 +8517,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8536,16 +8532,16 @@
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G100" s="10" t="n">
         <v>21</v>
@@ -8568,7 +8564,7 @@
       </c>
       <c r="L100" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M100" s="11" t="inlineStr">
@@ -8583,7 +8579,7 @@
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8595,12 +8591,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8610,7 +8606,7 @@
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
@@ -8637,12 +8633,12 @@
       </c>
       <c r="K101" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L101" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M101" s="11" t="inlineStr">
@@ -8652,12 +8648,12 @@
       </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8669,12 +8665,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8689,7 +8685,7 @@
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
@@ -8716,7 +8712,7 @@
       </c>
       <c r="L102" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M102" s="11" t="inlineStr">
@@ -8731,7 +8727,7 @@
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8743,12 +8739,12 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8758,12 +8754,12 @@
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
@@ -8785,12 +8781,12 @@
       </c>
       <c r="K103" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L103" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>services.controller.ts:125</t>
         </is>
       </c>
       <c r="M103" s="11" t="inlineStr">
@@ -8800,12 +8796,12 @@
       </c>
       <c r="N103" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8817,31 +8813,31 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F104" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G104" s="10" t="n">
         <v>21</v>
@@ -8859,12 +8855,12 @@
       </c>
       <c r="K104" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L104" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M104" s="11" t="inlineStr">
@@ -8874,12 +8870,12 @@
       </c>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8891,12 +8887,12 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>PB-26</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -8915,20 +8911,20 @@
         </is>
       </c>
       <c r="F105" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G105" s="10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H105" s="10" t="inlineStr"/>
       <c r="I105" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-25</t>
         </is>
       </c>
       <c r="J105" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-29</t>
         </is>
       </c>
       <c r="K105" s="10" t="inlineStr">
@@ -8948,12 +8944,12 @@
       </c>
       <c r="N105" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
         </is>
       </c>
       <c r="O105" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr">
@@ -8965,12 +8961,12 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>PB-26</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -8985,11 +8981,11 @@
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F106" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G106" s="10" t="n">
         <v>22</v>
@@ -9017,17 +9013,17 @@
       </c>
       <c r="M106" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
         </is>
       </c>
       <c r="N106" s="11" t="inlineStr">
         <is>
-          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
         </is>
       </c>
       <c r="O106" s="11" t="inlineStr">
         <is>
-          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr">
@@ -9039,12 +9035,12 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-12</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Runbook startu i decyzja GO</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -9063,7 +9059,7 @@
         </is>
       </c>
       <c r="F107" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G107" s="10" t="n">
         <v>22</v>
@@ -9091,17 +9087,17 @@
       </c>
       <c r="M107" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
       <c r="N107" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
       <c r="O107" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr">
@@ -9113,12 +9109,12 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-20</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Tryb agencji: przełącznik klienta w menu bocznym</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -9133,24 +9129,24 @@
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F108" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G108" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H108" s="10" t="inlineStr"/>
       <c r="I108" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-02-01</t>
         </is>
       </c>
       <c r="J108" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="K108" s="10" t="inlineStr">
@@ -9165,17 +9161,17 @@
       </c>
       <c r="M108" s="11" t="inlineStr">
         <is>
-          <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N108" s="11" t="inlineStr">
         <is>
-          <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
+          <t>Decyzja o modelu zapisana w docs/VERRIS.md; przełącznik widoczny tylko dla kont z klientami; przełączenie zmienia kontekst usług, domen i płatności; guard uprawnień obejmuje nowe trasy (Z-04); testy w CI.</t>
         </is>
       </c>
       <c r="O108" s="11" t="inlineStr">
         <is>
-          <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
+          <t>Element makiety („Piekarnia Zdrój · klient · 3 usługi” nad menu): konto agencji/resellera przełącza się między swoimi klientami bez wylogowania. Wymaga decyzji, jak Reseller (white-label) mapuje klientów na konta i uprawnienia (IAM). | DECYZJA WŁAŚCICIELA 2026-09-25: PO STARCIE. Dziś reseller ma listę swoich klientów i narzut; przełącznik klienta wraca przy pierwszych agencjach, gdy będzie wiadomo, jak z niego korzystają (mniej ryzyka przy dostępie do cudzych kont). Model do wyboru wtedy: przełączenie na konto klienta (jak impersonacja, tylko własni klienci, dziennik obu stron) albo klienci w koncie agencji.</t>
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr">
@@ -9224,7 +9220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10269,9 +10265,50 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>2027-02-01</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>2027-02-05</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr"/>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Po starcie — odłożone decyzją właściciela</t>
+        </is>
+      </c>
+      <c r="F24" s="10">
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A24)</f>
+        <v/>
+      </c>
+      <c r="G24" s="10">
+        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A24,'Backlog do startu'!$F$2:$F$108)</f>
+        <v/>
+      </c>
+      <c r="H24" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" s="12">
+        <f>IFERROR(G24/H24,0)</f>
+        <v/>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>Poza ścieżką do startu (2027-01-01): pozycje, które właściciel świadomie przesunął na czas po pierwszych klientach. PB-20 (tryb agencji) — decyzja 2026-09-25.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J23"/>
-  <conditionalFormatting sqref="G2:G23">
+  <autoFilter ref="A1:J24"/>
+  <conditionalFormatting sqref="G2:G24">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>

</xml_diff>

<commit_message>
chore(audyt): decyzje właściciela 26.09 — PB-27 indywidualne warunki usługi, PB-28 rozliczenie poza Verris, PB-29..32 węzły (blokery, manifest wersji, automatyzacja kreatora, aktualizacje falami)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$114</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$22</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$108)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$114)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$108,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$108,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$114,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$114,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$108,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$114,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$108,"zrobione",'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$114,"zrobione",'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P108"/>
+  <dimension ref="A1:P114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6731,58 +6731,58 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>X-41</t>
+          <t>PB-27</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
+          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F77" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G77" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H77" s="10" t="inlineStr">
         <is>
-          <t>Faza 3 — Wejście na rynek</t>
+          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
         </is>
       </c>
       <c r="I77" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J77" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K77" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L77" s="11" t="inlineStr">
         <is>
-          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M77" s="11" t="inlineStr">
@@ -6792,12 +6792,12 @@
       </c>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
         </is>
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
+          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157).</t>
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr">
@@ -6809,58 +6809,58 @@
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>PB-28</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
+          <t>Rozliczenie poza Verris (całe konto)</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G78" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H78" s="10" t="inlineStr">
         <is>
-          <t>Faza 3 — Wejście na rynek</t>
+          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
         </is>
       </c>
       <c r="I78" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J78" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K78" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L78" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M78" s="11" t="inlineStr">
@@ -6870,12 +6870,12 @@
       </c>
       <c r="N78" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
         </is>
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
+          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego.</t>
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr">
@@ -6887,31 +6887,31 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>PB-22</t>
+          <t>X-41</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
+          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G79" s="10" t="n">
         <v>15</v>
@@ -6933,12 +6933,12 @@
       </c>
       <c r="K79" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L79" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
         </is>
       </c>
       <c r="M79" s="11" t="inlineStr">
@@ -6948,12 +6948,12 @@
       </c>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O79" s="11" t="inlineStr">
         <is>
-          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
         </is>
       </c>
       <c r="P79" s="10" t="inlineStr">
@@ -6965,12 +6965,12 @@
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Log egressu jest próbką, nie zapisem</t>
+          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -6989,10 +6989,10 @@
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H80" s="10" t="inlineStr">
         <is>
@@ -7001,22 +7001,22 @@
       </c>
       <c r="I80" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="J80" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="K80" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L80" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
         </is>
       </c>
       <c r="M80" s="11" t="inlineStr">
@@ -7026,12 +7026,12 @@
       </c>
       <c r="N80" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr">
@@ -7043,34 +7043,34 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>PB-22</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
+          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G81" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H81" s="10" t="inlineStr">
         <is>
@@ -7079,22 +7079,22 @@
       </c>
       <c r="I81" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="K81" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L81" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M81" s="11" t="inlineStr">
@@ -7104,12 +7104,12 @@
       </c>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
         </is>
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
+          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr">
@@ -7121,12 +7121,12 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Tryb `--strict` jest atrapą</t>
+          <t>Log egressu jest próbką, nie zapisem</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
@@ -7145,7 +7145,7 @@
         </is>
       </c>
       <c r="F82" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G82" s="10" t="n">
         <v>16</v>
@@ -7167,12 +7167,12 @@
       </c>
       <c r="K82" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
+          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M82" s="11" t="inlineStr">
@@ -7182,12 +7182,12 @@
       </c>
       <c r="N82" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O82" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr">
@@ -7199,12 +7199,12 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
+          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
@@ -7223,7 +7223,7 @@
         </is>
       </c>
       <c r="F83" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G83" s="10" t="n">
         <v>16</v>
@@ -7245,12 +7245,12 @@
       </c>
       <c r="K83" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
-          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
+          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M83" s="11" t="inlineStr">
@@ -7260,12 +7260,12 @@
       </c>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O83" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr">
@@ -7277,12 +7277,12 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
+          <t>Tryb `--strict` jest atrapą</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -7297,11 +7297,11 @@
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F84" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G84" s="10" t="n">
         <v>16</v>
@@ -7323,12 +7323,12 @@
       </c>
       <c r="K84" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
+          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
@@ -7338,12 +7338,12 @@
       </c>
       <c r="N84" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O84" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr">
@@ -7355,31 +7355,31 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>PB-23</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
+          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F85" s="10" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G85" s="10" t="n">
         <v>16</v>
@@ -7401,12 +7401,12 @@
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
         </is>
       </c>
       <c r="M85" s="11" t="inlineStr">
@@ -7416,12 +7416,12 @@
       </c>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O85" s="11" t="inlineStr">
         <is>
-          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr">
@@ -7433,12 +7433,12 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>Podpisane DPA z subprocesorami (część)</t>
+          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -7448,19 +7448,19 @@
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E86" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F86" s="10" t="n">
         <v>6</v>
       </c>
       <c r="G86" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H86" s="10" t="inlineStr">
         <is>
@@ -7469,12 +7469,12 @@
       </c>
       <c r="I86" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="J86" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="K86" s="10" t="inlineStr">
@@ -7484,7 +7484,7 @@
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
+          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr">
@@ -7499,7 +7499,7 @@
       </c>
       <c r="O86" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr">
@@ -7511,12 +7511,12 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>PB-03</t>
+          <t>PB-23</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Finalizacja dokumentów prawnych 1.0.0</t>
+          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -7531,15 +7531,15 @@
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F87" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G87" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="G87" s="10" t="n">
-        <v>17</v>
-      </c>
       <c r="H87" s="10" t="inlineStr">
         <is>
           <t>Faza 3 — Wejście na rynek</t>
@@ -7547,12 +7547,12 @@
       </c>
       <c r="I87" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="J87" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="K87" s="10" t="inlineStr">
@@ -7572,12 +7572,12 @@
       </c>
       <c r="N87" s="11" t="inlineStr">
         <is>
-          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
+          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
         </is>
       </c>
       <c r="O87" s="11" t="inlineStr">
         <is>
-          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr">
@@ -7589,31 +7589,31 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>PB-04</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
+          <t>Podpisane DPA z subprocesorami (część)</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>17</v>
@@ -7635,12 +7635,12 @@
       </c>
       <c r="K88" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
         </is>
       </c>
       <c r="M88" s="11" t="inlineStr">
@@ -7650,12 +7650,12 @@
       </c>
       <c r="N88" s="11" t="inlineStr">
         <is>
-          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O88" s="11" t="inlineStr">
         <is>
-          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr">
@@ -7667,34 +7667,34 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>N-16</t>
+          <t>PB-03</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>SLA z zapisanymi kredytami</t>
+          <t>Finalizacja dokumentów prawnych 1.0.0</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G89" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H89" s="10" t="inlineStr">
         <is>
@@ -7703,37 +7703,37 @@
       </c>
       <c r="I89" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-21</t>
         </is>
       </c>
       <c r="J89" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="K89" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L89" s="11" t="inlineStr">
         <is>
-          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M89" s="11" t="inlineStr">
         <is>
-          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
         </is>
       </c>
       <c r="O89" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
+          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr">
@@ -7745,34 +7745,34 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>PB-04</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G90" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H90" s="10" t="inlineStr">
         <is>
@@ -7781,22 +7781,22 @@
       </c>
       <c r="I90" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-21</t>
         </is>
       </c>
       <c r="J90" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="K90" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L90" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M90" s="11" t="inlineStr">
@@ -7806,12 +7806,12 @@
       </c>
       <c r="N90" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
         </is>
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7823,31 +7823,31 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>PB-07</t>
+          <t>N-16</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Treści i cennik na verris.pl</t>
+          <t>SLA z zapisanymi kredytami</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G91" s="10" t="n">
         <v>18</v>
@@ -7869,27 +7869,27 @@
       </c>
       <c r="K91" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L91" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
         </is>
       </c>
       <c r="M91" s="11" t="inlineStr">
         <is>
-          <t>PB-01 (cennik zależy od unit economics)</t>
+          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
         </is>
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
+          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7901,31 +7901,31 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>PB-11</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>18</v>
@@ -7947,12 +7947,12 @@
       </c>
       <c r="K92" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L92" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M92" s="11" t="inlineStr">
@@ -7962,12 +7962,12 @@
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>PB-21</t>
+          <t>PB-07</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>DNS platformy i poczty na serwerze testowym</t>
+          <t>Treści i cennik na verris.pl</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -8003,7 +8003,7 @@
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G93" s="10" t="n">
         <v>18</v>
@@ -8035,17 +8035,17 @@
       </c>
       <c r="M93" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-01 (cennik zależy od unit economics)</t>
         </is>
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
+          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
+          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8057,12 +8057,12 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>PB-24</t>
+          <t>PB-11</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
+          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8081,7 +8081,7 @@
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>18</v>
@@ -8118,12 +8118,12 @@
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
+          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8135,12 +8135,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>PB-25</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>White label na węźle — klient nie widzi DirectAdmina</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8159,7 +8159,7 @@
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G95" s="10" t="n">
         <v>18</v>
@@ -8196,12 +8196,12 @@
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,12 +8213,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-24</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8237,10 +8237,10 @@
         </is>
       </c>
       <c r="F96" s="10" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G96" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H96" s="10" t="inlineStr">
         <is>
@@ -8249,12 +8249,12 @@
       </c>
       <c r="I96" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J96" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K96" s="10" t="inlineStr">
@@ -8269,17 +8269,17 @@
       </c>
       <c r="M96" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
+          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,12 +8291,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-25</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>White label na węźle — klient nie widzi DirectAdmina</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8311,14 +8311,14 @@
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G97" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H97" s="10" t="inlineStr">
         <is>
@@ -8327,12 +8327,12 @@
       </c>
       <c r="I97" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J97" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K97" s="10" t="inlineStr">
@@ -8352,12 +8352,12 @@
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
+          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8369,12 +8369,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8389,11 +8389,11 @@
       </c>
       <c r="E98" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G98" s="10" t="n">
         <v>19</v>
@@ -8425,17 +8425,17 @@
       </c>
       <c r="M98" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8447,12 +8447,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8471,20 +8471,24 @@
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G99" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H99" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H99" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K99" s="10" t="inlineStr">
@@ -8499,17 +8503,17 @@
       </c>
       <c r="M99" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8521,54 +8525,58 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G100" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="H100" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H100" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I100" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K100" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L100" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M100" s="11" t="inlineStr">
@@ -8578,12 +8586,12 @@
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8595,69 +8603,69 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G101" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H101" s="10" t="inlineStr"/>
       <c r="I101" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J101" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K101" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L101" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M101" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8669,12 +8677,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8684,16 +8692,16 @@
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G102" s="10" t="n">
         <v>21</v>
@@ -8711,12 +8719,12 @@
       </c>
       <c r="K102" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L102" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M102" s="11" t="inlineStr">
@@ -8726,12 +8734,12 @@
       </c>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
+          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8743,12 +8751,12 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8758,12 +8766,12 @@
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
@@ -8785,12 +8793,12 @@
       </c>
       <c r="K103" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L103" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M103" s="11" t="inlineStr">
@@ -8800,12 +8808,12 @@
       </c>
       <c r="N103" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8817,12 +8825,12 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
@@ -8832,7 +8840,7 @@
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E104" s="10" t="inlineStr">
@@ -8859,12 +8867,12 @@
       </c>
       <c r="K104" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L104" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M104" s="11" t="inlineStr">
@@ -8874,12 +8882,12 @@
       </c>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8891,31 +8899,31 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F105" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G105" s="10" t="n">
         <v>21</v>
@@ -8933,12 +8941,12 @@
       </c>
       <c r="K105" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L105" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M105" s="11" t="inlineStr">
@@ -8948,12 +8956,12 @@
       </c>
       <c r="N105" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O105" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr">
@@ -8965,54 +8973,54 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>PB-26</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F106" s="10" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G106" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H106" s="10" t="inlineStr"/>
       <c r="I106" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J106" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K106" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L106" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>services.controller.ts:125</t>
         </is>
       </c>
       <c r="M106" s="11" t="inlineStr">
@@ -9022,12 +9030,12 @@
       </c>
       <c r="N106" s="11" t="inlineStr">
         <is>
-          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O106" s="11" t="inlineStr">
         <is>
-          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr">
@@ -9039,12 +9047,12 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -9059,24 +9067,24 @@
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F107" s="10" t="n">
         <v>16</v>
       </c>
       <c r="G107" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H107" s="10" t="inlineStr"/>
       <c r="I107" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J107" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K107" s="10" t="inlineStr">
@@ -9091,17 +9099,17 @@
       </c>
       <c r="M107" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N107" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O107" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr">
@@ -9113,12 +9121,12 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-29</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -9133,60 +9141,504 @@
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F108" s="10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G108" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H108" s="10" t="inlineStr"/>
       <c r="I108" s="10" t="inlineStr">
         <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="J108" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-22</t>
+        </is>
+      </c>
+      <c r="K108" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L108" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M108" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N108" s="11" t="inlineStr">
+        <is>
+          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
+        </is>
+      </c>
+      <c r="O108" s="11" t="inlineStr">
+        <is>
+          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API.</t>
+        </is>
+      </c>
+      <c r="P108" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>PB-30</t>
+        </is>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>Jeden plik wersji dla floty + test zgodności</t>
+        </is>
+      </c>
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E109" s="10" t="inlineStr">
+        <is>
+          <t>WYSOKI</t>
+        </is>
+      </c>
+      <c r="F109" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="G109" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="H109" s="10" t="inlineStr"/>
+      <c r="I109" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="J109" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-22</t>
+        </is>
+      </c>
+      <c r="K109" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L109" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M109" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N109" s="11" t="inlineStr">
+        <is>
+          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
+        </is>
+      </c>
+      <c r="O109" s="11" t="inlineStr">
+        <is>
+          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami.</t>
+        </is>
+      </c>
+      <c r="P109" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="inlineStr">
+        <is>
+          <t>PB-31</t>
+        </is>
+      </c>
+      <c r="B110" s="11" t="inlineStr">
+        <is>
+          <t>Pełna automatyzacja kreatora węzła</t>
+        </is>
+      </c>
+      <c r="C110" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
+        <is>
+          <t>WYSOKI</t>
+        </is>
+      </c>
+      <c r="F110" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="G110" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="H110" s="10" t="inlineStr"/>
+      <c r="I110" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="J110" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-22</t>
+        </is>
+      </c>
+      <c r="K110" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L110" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M110" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N110" s="11" t="inlineStr">
+        <is>
+          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
+        </is>
+      </c>
+      <c r="O110" s="11" t="inlineStr">
+        <is>
+          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…).</t>
+        </is>
+      </c>
+      <c r="P110" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>PB-32</t>
+        </is>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
+          <t>Aktualizacje węzłów falami</t>
+        </is>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E111" s="10" t="inlineStr">
+        <is>
+          <t>ŚREDNI</t>
+        </is>
+      </c>
+      <c r="F111" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G111" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="H111" s="10" t="inlineStr"/>
+      <c r="I111" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="J111" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-22</t>
+        </is>
+      </c>
+      <c r="K111" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L111" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M111" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N111" s="11" t="inlineStr">
+        <is>
+          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
+        </is>
+      </c>
+      <c r="O111" s="11" t="inlineStr">
+        <is>
+          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic.</t>
+        </is>
+      </c>
+      <c r="P111" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>PB-26</t>
+        </is>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
+        </is>
+      </c>
+      <c r="C112" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D112" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E112" s="10" t="inlineStr">
+        <is>
+          <t>WYSOKI</t>
+        </is>
+      </c>
+      <c r="F112" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="G112" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H112" s="10" t="inlineStr"/>
+      <c r="I112" s="10" t="inlineStr">
+        <is>
           <t>2027-01-25</t>
         </is>
       </c>
-      <c r="J108" s="10" t="inlineStr">
+      <c r="J112" s="10" t="inlineStr">
         <is>
           <t>2027-01-29</t>
         </is>
       </c>
-      <c r="K108" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L108" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M108" s="11" t="inlineStr">
+      <c r="K112" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L112" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M112" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N112" s="11" t="inlineStr">
+        <is>
+          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
+        </is>
+      </c>
+      <c r="O112" s="11" t="inlineStr">
+        <is>
+          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
+        </is>
+      </c>
+      <c r="P112" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>PB-05</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>Test end-to-end „pierwszy klient”</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D113" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E113" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F113" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="G113" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H113" s="10" t="inlineStr"/>
+      <c r="I113" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J113" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K113" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L113" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M113" s="11" t="inlineStr">
+        <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N113" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O113" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P113" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B114" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E114" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F114" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G114" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H114" s="10" t="inlineStr"/>
+      <c r="I114" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J114" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K114" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L114" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M114" s="11" t="inlineStr">
         <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N108" s="11" t="inlineStr">
+      <c r="N114" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O108" s="11" t="inlineStr">
+      <c r="O114" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P108" s="10" t="inlineStr">
+      <c r="P114" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P108"/>
-  <conditionalFormatting sqref="E2:E108">
+  <autoFilter ref="A1:P114"/>
+  <conditionalFormatting sqref="E2:E114">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -9206,7 +9658,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P108">
+  <conditionalFormatting sqref="P2:P114">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -9316,11 +9768,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A2,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A2,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -9361,11 +9813,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A3,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A3,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -9406,11 +9858,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A4,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A4,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -9451,11 +9903,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A5,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A5,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -9496,11 +9948,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A6,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A6,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -9541,11 +9993,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A7,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A7,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -9586,11 +10038,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A8,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A8,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -9631,11 +10083,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A9,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A9,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -9676,11 +10128,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A10,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A10,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -9721,11 +10173,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A11,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A11,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -9766,11 +10218,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A12,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A12,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -9811,11 +10263,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A13,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A13,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -9856,11 +10308,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A14,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A14,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -9901,11 +10353,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A15,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A15,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -9946,11 +10398,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A16,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A16,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -9991,11 +10443,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A17,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A17,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -10036,11 +10488,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A18,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A18,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -10081,11 +10533,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A19,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A19,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -10126,11 +10578,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A20,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A20,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -10167,11 +10619,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A21,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A21,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -10208,11 +10660,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A22,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A22,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -10249,11 +10701,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A23,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A23,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">
@@ -10290,11 +10742,11 @@
         </is>
       </c>
       <c r="F24" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$108,A24)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A24)</f>
         <v/>
       </c>
       <c r="G24" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$108,A24,'Backlog do startu'!$F$2:$F$108)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A24,'Backlog do startu'!$F$2:$F$114)</f>
         <v/>
       </c>
       <c r="H24" s="10" t="n">

</xml_diff>

<commit_message>
chore(audyt): tablice po PB-27..PB-32
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -6797,7 +6797,7 @@
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157).</t>
+          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego.</t>
+          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="O108" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API.</t>
+          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr">
@@ -9257,7 +9257,7 @@
       </c>
       <c r="O109" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami.</t>
+          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr">
@@ -9331,7 +9331,7 @@
       </c>
       <c r="O110" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…).</t>
+          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr">
@@ -9405,7 +9405,7 @@
       </c>
       <c r="O111" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic.</t>
+          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr">

</xml_diff>

<commit_message>
chore(audyt): tablice po PB-33/35/36
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$22</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$114)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$118)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$114,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$114,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$118,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$118,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$114,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$118,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$114,"zrobione",'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$118,"zrobione",'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P114"/>
+  <dimension ref="A1:P118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4781,34 +4781,34 @@
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>PB-34</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>Rekordy SPF — kreator</t>
+          <t>Panele admina i obsługi na poziomie panelu klienta</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F52" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="G52" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
@@ -4817,22 +4817,22 @@
       </c>
       <c r="I52" s="10" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J52" s="10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L52" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: deliverability/mail-auth.ts (buildMailAuthChecks) + deliverability.service.ts (strefa DA + delegacja NS); UI app/dashboard/email/deliverability-panel.tsx podpięty w MailTab (zakładka Poczta); test mail-auth.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M52" s="11" t="inlineStr">
@@ -4842,12 +4842,12 @@
       </c>
       <c r="N52" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Makieta zaakceptowana; wszystkie ekrany admina i obsługi na v2, bramka a11y zielona.</t>
         </is>
       </c>
       <c r="O52" s="11" t="inlineStr">
         <is>
-          <t>deliverability-panel.tsx:26 to komponent osierocony — nikt go nie importuje | KOD: kreator pokazuje stan z publicznego DNS i gotowy rekord — „Dodaj/Zamień rekord w DNS” gdy domena na NS Verris, inaczej do skopiowania u dostawcy DNS. Zalecany SPF to `v=spf1 a mx ip4:&lt;IP węzła&gt; ~all`. ZNALEZISKO: dotychczasowa podpowiedź include:_spf.verris.pl odwołuje się do nieistniejącego rekordu (NXDOMAIN) → SPF permerror; usunięta z podpowiedzi, presetu DNS i artykułów KB, a kreator wykrywa ją u klientów. OTWARTE do D3 (węzeł): zapis rekordu przez CMD_API_DNS_CONTROL.</t>
+          <t>Decyzja właściciela 2026-09-26: najpierw makieta 3–4 kluczowych ekranów (pulpit, węzły/węzeł, karta klienta, zgłoszenie) do akceptacji, potem przeniesienie wszystkich ekranów 1:1 na tokeny i komponenty v2 (jasny i ciemny motyw). DEV_HANDOFF.md przewidywał „ten sam zestaw tokenów, później”.</t>
         </is>
       </c>
       <c r="P52" s="10" t="inlineStr">
@@ -4859,12 +4859,12 @@
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>E-16</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Rekordy DKIM — konfiguracja</t>
+          <t>Rekordy SPF — kreator</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -4910,12 +4910,12 @@
       </c>
       <c r="L53" s="11" t="inlineStr">
         <is>
-          <t>deliverability/mail-auth.ts (akcja enable-dkim); servers/directadmin.service.ts enableHostingDkim; POST /services/:id/hosting-email/dkim; email/deliverability-panel.tsx; testy mail-auth.spec.ts, directadmin.narzedzia.spec.ts</t>
+          <t>2026-09-23 D1: deliverability/mail-auth.ts (buildMailAuthChecks) + deliverability.service.ts (strefa DA + delegacja NS); UI app/dashboard/email/deliverability-panel.tsx podpięty w MailTab (zakładka Poczta); test mail-auth.spec.ts</t>
         </is>
       </c>
       <c r="M53" s="11" t="inlineStr">
         <is>
-          <t>E-15 (ten sam panel dostarczalności)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N53" s="11" t="inlineStr">
@@ -4925,7 +4925,7 @@
       </c>
       <c r="O53" s="11" t="inlineStr">
         <is>
-          <t>j.w. | KOD: DKIM odczytywany ze strefy DA (DA dopisuje klucz sam przy włączonym DKIM). Brak klucza = link do zgłoszenia. OTWARTE: włączanie DKIM z panelu (komenda DA niepotwierdzona bez węzła) — D3 w sprincie 18. | 2026-09-25: KOD (D2) — „Włącz DKIM dla &lt;domena&gt;” w sekcji Dostarczalność zamiast „napisz zgłoszenie”. Komenda DA potwierdzona w dokumentacji (changelog 1.57.2): CMD_API_EMAIL_POP action=set_dkim&amp;domain=…&amp;enable=… — DA tworzy klucze i dopisuje rekord TXT do strefy. Tylko domena z konta usługi, konto zawieszone bez zmian, wpis w dzienniku (HOSTING_DKIM_ENABLED). Wyłączenia celowo brak: ponowne włączenie generuje nowe klucze i rekord u zewnętrznego DNS przestałby pasować. Przy DNS u innego dostawcy panel po włączeniu pokazuje rekord do skopiowania (istniejąca ścieżka „klucz w strefie”). D3: pierwsze włączenie na węźle. | 2026-09-25 (dokumentacja DirectAdmin „Exim → DKIM”): dkim=2 udostępnia włączanie DKIM użytkownikom per domena, dkim=1 generuje klucze automatycznie przy tworzeniu domeny (tylko gdy DNS jest lokalny). Profil węzła ustawia dkim=1 — przycisk w panelu pojawia się tylko dla domen bez klucza. D3 ma potwierdzić, że set_dkim działa przy dkim=1; jeśli nie — alternatywa z dokumentacji: scripts/dkim_create.sh &lt;domena&gt; po stronie węzła (zadanie agenta).</t>
+          <t>deliverability-panel.tsx:26 to komponent osierocony — nikt go nie importuje | KOD: kreator pokazuje stan z publicznego DNS i gotowy rekord — „Dodaj/Zamień rekord w DNS” gdy domena na NS Verris, inaczej do skopiowania u dostawcy DNS. Zalecany SPF to `v=spf1 a mx ip4:&lt;IP węzła&gt; ~all`. ZNALEZISKO: dotychczasowa podpowiedź include:_spf.verris.pl odwołuje się do nieistniejącego rekordu (NXDOMAIN) → SPF permerror; usunięta z podpowiedzi, presetu DNS i artykułów KB, a kreator wykrywa ją u klientów. OTWARTE do D3 (węzeł): zapis rekordu przez CMD_API_DNS_CONTROL.</t>
         </is>
       </c>
       <c r="P53" s="10" t="inlineStr">
@@ -4937,12 +4937,12 @@
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>E-17</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>Rekord DMARC — konfiguracja</t>
+          <t>Rekordy DKIM — konfiguracja</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -4988,12 +4988,12 @@
       </c>
       <c r="L54" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: mail-auth.ts dmarcCheck (brak / p=none / kilka rekordów) + lib/dmarc.ts tuneDmarc (polityka + adres raportów) w deliverability-panel.tsx; testy mail-auth.spec.ts, dmarc.spec.ts</t>
+          <t>deliverability/mail-auth.ts (akcja enable-dkim); servers/directadmin.service.ts enableHostingDkim; POST /services/:id/hosting-email/dkim; email/deliverability-panel.tsx; testy mail-auth.spec.ts, directadmin.narzedzia.spec.ts</t>
         </is>
       </c>
       <c r="M54" s="11" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>E-15 (ten sam panel dostarczalności)</t>
         </is>
       </c>
       <c r="N54" s="11" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="O54" s="11" t="inlineStr">
         <is>
-          <t>j.w. | KOD: kreator DMARC — wybór polityki i opcjonalny adres raportów, zachowuje pozostałe tagi. Sugestia bez rua na verris.pl (raporty do obcej domeny wymagają rekordu autoryzacji). OTWARTE do D3: zapis do strefy DA.</t>
+          <t>j.w. | KOD: DKIM odczytywany ze strefy DA (DA dopisuje klucz sam przy włączonym DKIM). Brak klucza = link do zgłoszenia. OTWARTE: włączanie DKIM z panelu (komenda DA niepotwierdzona bez węzła) — D3 w sprincie 18. | 2026-09-25: KOD (D2) — „Włącz DKIM dla &lt;domena&gt;” w sekcji Dostarczalność zamiast „napisz zgłoszenie”. Komenda DA potwierdzona w dokumentacji (changelog 1.57.2): CMD_API_EMAIL_POP action=set_dkim&amp;domain=…&amp;enable=… — DA tworzy klucze i dopisuje rekord TXT do strefy. Tylko domena z konta usługi, konto zawieszone bez zmian, wpis w dzienniku (HOSTING_DKIM_ENABLED). Wyłączenia celowo brak: ponowne włączenie generuje nowe klucze i rekord u zewnętrznego DNS przestałby pasować. Przy DNS u innego dostawcy panel po włączeniu pokazuje rekord do skopiowania (istniejąca ścieżka „klucz w strefie”). D3: pierwsze włączenie na węźle. | 2026-09-25 (dokumentacja DirectAdmin „Exim → DKIM”): dkim=2 udostępnia włączanie DKIM użytkownikom per domena, dkim=1 generuje klucze automatycznie przy tworzeniu domeny (tylko gdy DNS jest lokalny). Profil węzła ustawia dkim=1 — przycisk w panelu pojawia się tylko dla domen bez klucza. D3 ma potwierdzić, że set_dkim działa przy dkim=1; jeśli nie — alternatywa z dokumentacji: scripts/dkim_create.sh &lt;domena&gt; po stronie węzła (zadanie agenta).</t>
         </is>
       </c>
       <c r="P54" s="10" t="inlineStr">
@@ -5015,12 +5015,12 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>E-05</t>
+          <t>E-17</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Zmiana quoty ISTNIEJĄCEJ skrzynki</t>
+          <t>Rekord DMARC — konfiguracja</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -5066,12 +5066,12 @@
       </c>
       <c r="L55" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/hosting-email/quota (ZmienRozmiarSkrzynkiDto 10–102400 MB) → directadmin.service changeHostingEmailQuota (CMD_API_POP action=modify bez passwd) + audyt HOSTING_EMAIL_QUOTA_CHANGED; UI MailTab — klik w rozmiar skrzynki</t>
+          <t>2026-09-23 D1: mail-auth.ts dmarcCheck (brak / p=none / kilka rekordów) + lib/dmarc.ts tuneDmarc (polityka + adres raportów) w deliverability-panel.tsx; testy mail-auth.spec.ts, dmarc.spec.ts</t>
         </is>
       </c>
       <c r="M55" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="N55" s="11" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O55" s="11" t="inlineStr">
         <is>
-          <t>brak jakiejkolwiek ścieżki edycji — klient musi usunąć i odtworzyć skrzynkę | KOD: zmiana rozmiaru bez usuwania skrzynki. Przy okazji body tworzenia skrzynki i zmiany hasła dostały klasy DTO (wcześniej interfejs = zero walidacji na granicy zaufania). OTWARTE do D3: czy DA przy modify bez passwd zostawia hasło (komentarz ponytail).</t>
+          <t>j.w. | KOD: kreator DMARC — wybór polityki i opcjonalny adres raportów, zachowuje pozostałe tagi. Sugestia bez rua na verris.pl (raporty do obcej domeny wymagają rekordu autoryzacji). OTWARTE do D3: zapis do strefy DA.</t>
         </is>
       </c>
       <c r="P55" s="10" t="inlineStr">
@@ -5093,12 +5093,12 @@
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>M-26</t>
+          <t>E-05</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>Usunięcie zapisanej karty przez klienta</t>
+          <t>Zmiana quoty ISTNIEJĄCEJ skrzynki</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="E56" s="10" t="inlineStr">
@@ -5139,12 +5139,12 @@
       </c>
       <c r="K56" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: DELETE /billing/payment-methods/:id (ParseUUIDPipe) → billing.service deleteMyPaymentMethod: Stripe detach, usunięcie wiersza, zerowanie karty domyślnej i auto-doładowania, audyt PAYMENT_METHOD_REMOVED; UI billing-extras-forms „Zapisane karty”; test usun-karte.spec.ts | 2026-09-23: zapis kart — billing.service handlePaymentMethodAttached/Detached (webhooki payment_method.attached/.detached, upsert po provider+providerRef, pierwsza karta domyślna); test D2 zapis-karty.spec.ts</t>
+          <t>2026-09-23 D1: POST /services/:id/hosting-email/quota (ZmienRozmiarSkrzynkiDto 10–102400 MB) → directadmin.service changeHostingEmailQuota (CMD_API_POP action=modify bez passwd) + audyt HOSTING_EMAIL_QUOTA_CHANGED; UI MailTab — klik w rozmiar skrzynki</t>
         </is>
       </c>
       <c r="M56" s="11" t="inlineStr">
@@ -5154,12 +5154,12 @@
       </c>
       <c r="N56" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O56" s="11" t="inlineStr">
         <is>
-          <t>wymóg konsumencki | KOD gotowy i przetestowany na atrapach. UWAGA: nic w API nie zapisuje dziś wierszy PaymentMethod (brak create/upsert) — lista kart jest zawsze pusta, więc usuwanie da się sprawdzić dopiero, gdy zapis kart zostanie podpięty (webhook Stripe po płatności kartą). | 2026-09-23: domknięty brakujący zapis — karta zapisana w Stripe (np. przy subskrypcji kartą) pojawia się w panelu, odpięta (także z dashboardu Stripe) znika i odpina się od auto-doładowania. WYMAGA OD WŁAŚCICIELA: dopisać zdarzenia payment_method.attached i payment_method.detached do endpointu webhooka w Stripe (DEPLOY.md, OPERATIONAL_CHECKLIST). Karty zapisane przed tą zmianą nie pojawią się wstecz. D3 przy pierwszej płatności kartą.</t>
+          <t>brak jakiejkolwiek ścieżki edycji — klient musi usunąć i odtworzyć skrzynkę | KOD: zmiana rozmiaru bez usuwania skrzynki. Przy okazji body tworzenia skrzynki i zmiany hasła dostały klasy DTO (wcześniej interfejs = zero walidacji na granicy zaufania). OTWARTE do D3: czy DA przy modify bez passwd zostawia hasło (komentarz ponytail).</t>
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr">
@@ -5171,58 +5171,58 @@
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>PB-17</t>
+          <t>M-26</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Asystent v1: dymki, naprawy jednym kliknięciem, czat z danymi konta</t>
+          <t>Usunięcie zapisanej karty przez klienta</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F57" s="10" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G57" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
+          <t>Faza 1 — Rozliczenia i dowód odtworzenia</t>
         </is>
       </c>
       <c r="I57" s="10" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J57" s="10" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K57" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L57" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-09-23 D1: DELETE /billing/payment-methods/:id (ParseUUIDPipe) → billing.service deleteMyPaymentMethod: Stripe detach, usunięcie wiersza, zerowanie karty domyślnej i auto-doładowania, audyt PAYMENT_METHOD_REMOVED; UI billing-extras-forms „Zapisane karty”; test usun-karte.spec.ts | 2026-09-23: zapis kart — billing.service handlePaymentMethodAttached/Detached (webhooki payment_method.attached/.detached, upsert po provider+providerRef, pierwsza karta domyślna); test D2 zapis-karty.spec.ts</t>
         </is>
       </c>
       <c r="M57" s="11" t="inlineStr">
@@ -5232,12 +5232,12 @@
       </c>
       <c r="N57" s="11" t="inlineStr">
         <is>
-          <t>Co najmniej 5 reguł dymków z testami; każda naprawa ma cofnięcie i wpis audytu; czat odpowiada z kontekstem usługi; brak akcji destrukcyjnych w v1.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O57" s="11" t="inlineStr">
         <is>
-          <t>Dymki kontekstowe na regułach (bez kosztu AI): dysk, domena nie wskazuje na nas, SPF/DKIM, SSL wygasa, backup nieświeży — najwyżej jeden na ekran, „nie pokazuj więcej”. Naprawy jednym kliknięciem tylko dla akcji odwracalnych, z kartą podglądu skutku i „Cofnij”. Obecny czat (HostingAssistant, RAG) dostaje odczyt danych konta. Każda akcja w audycie. Diagnoza i naprawy po naszej stronie za darmo.</t>
+          <t>wymóg konsumencki | KOD gotowy i przetestowany na atrapach. UWAGA: nic w API nie zapisuje dziś wierszy PaymentMethod (brak create/upsert) — lista kart jest zawsze pusta, więc usuwanie da się sprawdzić dopiero, gdy zapis kart zostanie podpięty (webhook Stripe po płatności kartą). | 2026-09-23: domknięty brakujący zapis — karta zapisana w Stripe (np. przy subskrypcji kartą) pojawia się w panelu, odpięta (także z dashboardu Stripe) znika i odpina się od auto-doładowania. WYMAGA OD WŁAŚCICIELA: dopisać zdarzenia payment_method.attached i payment_method.detached do endpointu webhooka w Stripe (DEPLOY.md, OPERATIONAL_CHECKLIST). Karty zapisane przed tą zmianą nie pojawią się wstecz. D3 przy pierwszej płatności kartą.</t>
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr">
@@ -5249,12 +5249,12 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>PB-18</t>
+          <t>PB-17</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Tickety v2: podgląd klienta, szablony ze zmiennymi, szkice odpowiedzi</t>
+          <t>Asystent v1: dymki, naprawy jednym kliknięciem, czat z danymi konta</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -5273,10 +5273,10 @@
         </is>
       </c>
       <c r="F58" s="10" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
@@ -5285,12 +5285,12 @@
       </c>
       <c r="I58" s="10" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="J58" s="10" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K58" s="10" t="inlineStr">
@@ -5310,12 +5310,12 @@
       </c>
       <c r="N58" s="11" t="inlineStr">
         <is>
-          <t>Podgląd klienta bez przechodzenia między ekranami; szablony podstawiają zmienne z testem; szkic odpowiedzi dla 6 kategorii (DNS, SSL, poczta, płatność, migracja, awaria).</t>
+          <t>Co najmniej 5 reguł dymków z testami; każda naprawa ma cofnięcie i wpis audytu; czat odpowiada z kontekstem usługi; brak akcji destrukcyjnych w v1.</t>
         </is>
       </c>
       <c r="O58" s="11" t="inlineStr">
         <is>
-          <t>Panel staff: boczny podgląd klienta w tickecie (usługi, saldo, faktury/dokumenty, zdarzenia, historia zgłoszeń, health score); szablony odpowiedzi ze zmiennymi (imię, domena, usługa, termin) i kategoriami — rozbudowa canned responses; klasyfikacja zgłoszenia i szkic odpowiedzi z bazy wiedzy i danych konta (do akceptacji, bez auto-wysyłki w v2); akcje z ticketu z audytem; licznik SLA.</t>
+          <t>Dymki kontekstowe na regułach (bez kosztu AI): dysk, domena nie wskazuje na nas, SPF/DKIM, SSL wygasa, backup nieświeży — najwyżej jeden na ekran, „nie pokazuj więcej”. Naprawy jednym kliknięciem tylko dla akcji odwracalnych, z kartą podglądu skutku i „Cofnij”. Obecny czat (HostingAssistant, RAG) dostaje odczyt danych konta. Każda akcja w audycie. Diagnoza i naprawy po naszej stronie za darmo.</t>
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr">
@@ -5327,34 +5327,34 @@
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>A-25</t>
+          <t>PB-18</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>Ręczne zawieszenie usługi przez operatora</t>
+          <t>Tickety v2: podgląd klienta, szablony ze zmiennymi, szkice odpowiedzi</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="G59" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
@@ -5363,22 +5363,22 @@
       </c>
       <c r="I59" s="10" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="J59" s="10" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="K59" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L59" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: admin-panel subscriptions/[id]/suspend-form.tsx + suspend-actions.ts → POST /admin/subscriptions/:id/suspend (powód, notatka, potwierdzenie)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M59" s="11" t="inlineStr">
@@ -5388,12 +5388,12 @@
       </c>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Podgląd klienta bez przechodzenia między ekranami; szablony podstawiają zmienne z testem; szkic odpowiedzi dla 6 kategorii (DNS, SSL, poczta, płatność, migracja, awaria).</t>
         </is>
       </c>
       <c r="O59" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: endpoint działa i jest osiągalny (curl + DirectAdmin), auto-suspend za brak płatności działa. Brakuje UI, nie możliwości zatrzymania szkody. | UI zrobione. OTWARTE do D3 (PB-21, serwer testowy): zawieszenie konta w DirectAdminie na żywym węźle.</t>
+          <t>Panel staff: boczny podgląd klienta w tickecie (usługi, saldo, faktury/dokumenty, zdarzenia, historia zgłoszeń, health score); szablony odpowiedzi ze zmiennymi (imię, domena, usługa, termin) i kategoriami — rozbudowa canned responses; klasyfikacja zgłoszenia i szkic odpowiedzi z bazy wiedzy i danych konta (do akceptacji, bez auto-wysyłki w v2); akcje z ticketu z audytem; licznik SLA.</t>
         </is>
       </c>
       <c r="P59" s="10" t="inlineStr">
@@ -5405,12 +5405,12 @@
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>A-26</t>
+          <t>A-25</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>Ręczne odwieszenie usługi przez operatora</t>
+          <t>Ręczne zawieszenie usługi przez operatora</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
@@ -5456,12 +5456,12 @@
       </c>
       <c r="L60" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: ten sam formularz — odwieszenie z opcją obciążenia za odnowienie (chargeRenewal)</t>
+          <t>2026-09-23 D1: admin-panel subscriptions/[id]/suspend-form.tsx + suspend-actions.ts → POST /admin/subscriptions/:id/suspend (powód, notatka, potwierdzenie)</t>
         </is>
       </c>
       <c r="M60" s="11" t="inlineStr">
         <is>
-          <t>A-25 (ten sam widok)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N60" s="11" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="O60" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: jak A-25, endpoint subscriptions.admin.controller.ts:210 działa z chargeRenewal. | UI zrobione. OTWARTE do D3 (PB-21): odwieszenie konta w DA na żywym węźle.</t>
+          <t>Skorygowane: endpoint działa i jest osiągalny (curl + DirectAdmin), auto-suspend za brak płatności działa. Brakuje UI, nie możliwości zatrzymania szkody. | UI zrobione. OTWARTE do D3 (PB-21, serwer testowy): zawieszenie konta w DirectAdminie na żywym węźle.</t>
         </is>
       </c>
       <c r="P60" s="10" t="inlineStr">
@@ -5483,12 +5483,12 @@
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>N-07</t>
+          <t>A-26</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Ręczne tworzenie incydentu na status page</t>
+          <t>Ręczne odwieszenie usługi przez operatora</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
@@ -5529,27 +5529,27 @@
       </c>
       <c r="K61" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L61" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D2: admin-panel status/incidents/incident-compose.tsx → POST /admin/product-ops/incidents; przycisk „Rozwiąż” (PATCH incidents/:id status=RESOLVED); probe-ingest.service.ts isManualIncident; test status/incydent-reczny.spec.ts</t>
+          <t>2026-09-23 D1: ten sam formularz — odwieszenie z opcją obciążenia za odnowienie (chargeRenewal)</t>
         </is>
       </c>
       <c r="M61" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A-25 (ten sam widok)</t>
         </is>
       </c>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O61" s="11" t="inlineStr">
         <is>
-          <t>w kryzysie nie ma jak zakomunikować awarii | ZNALEZISKO: incydent ogłoszony ręcznie zamykał się sam przy pierwszej udanej próbie monitora (w ciągu minut), więc komunikat o awarii, której monitor nie widzi, znikał ze status page. Teraz zamyka go tylko operator; zamknięcie wysyła webhook INCIDENT_RESOLVED i trafia do audytu.</t>
+          <t>Skorygowane: jak A-25, endpoint subscriptions.admin.controller.ts:210 działa z chargeRenewal. | UI zrobione. OTWARTE do D3 (PB-21): odwieszenie konta w DA na żywym węźle.</t>
         </is>
       </c>
       <c r="P61" s="10" t="inlineStr">
@@ -5561,12 +5561,12 @@
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>N-14</t>
+          <t>N-07</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Cordon wysyłki poczty (auto-blokada spamu)</t>
+          <t>Ręczne tworzenie incydentu na status page</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="L62" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: admin-panel /deliverability (Blokady wysyłki poczty, link w menu) → GET/POST /admin/deliverability/cordons; lista z e-mailem i nazwą klienta</t>
+          <t>2026-09-23 D2: admin-panel status/incidents/incident-compose.tsx → POST /admin/product-ops/incidents; przycisk „Rozwiąż” (PATCH incidents/:id status=RESOLVED); probe-ingest.service.ts isManualIncident; test status/incydent-reczny.spec.ts</t>
         </is>
       </c>
       <c r="M62" s="11" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="O62" s="11" t="inlineStr">
         <is>
-          <t>mechanizm działa, operator nie może go zobaczyć ani zdjąć | Operator widzi kogo i dlaczego zablokowano oraz zdejmuje blokadę (ADMIN, z potwierdzeniem, audyt po stronie API).</t>
+          <t>w kryzysie nie ma jak zakomunikować awarii | ZNALEZISKO: incydent ogłoszony ręcznie zamykał się sam przy pierwszej udanej próbie monitora (w ciągu minut), więc komunikat o awarii, której monitor nie widzi, znikał ze status page. Teraz zamyka go tylko operator; zamknięcie wysyła webhook INCIDENT_RESOLVED i trafia do audytu.</t>
         </is>
       </c>
       <c r="P62" s="10" t="inlineStr">
@@ -5639,12 +5639,12 @@
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>H-22</t>
+          <t>N-14</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Panel odtwarzania w widocznym miejscu</t>
+          <t>Cordon wysyłki poczty (auto-blokada spamu)</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -5654,7 +5654,7 @@
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E63" s="10" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="L63" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: client-panel BackupsTab.tsx — sekcja „Kopie poza serwerem” (HostingOffsitePanel) w zakładce Kopie zapasowe; zdublowany panel przywracania usunięty z Zużycia zasobów (hosting-backup-restore-panel.tsx)</t>
+          <t>2026-09-23: admin-panel /deliverability (Blokady wysyłki poczty, link w menu) → GET/POST /admin/deliverability/cordons; lista z e-mailem i nazwą klienta</t>
         </is>
       </c>
       <c r="M63" s="11" t="inlineStr">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="O63" s="11" t="inlineStr">
         <is>
-          <t>klient w kryzysie tego nie znajdzie | Kopie off-site są tam, gdzie klient ich szuka w kryzysie; przywracanie jest w jednym miejscu, z potwierdzeniem domeną.</t>
+          <t>mechanizm działa, operator nie może go zobaczyć ani zdjąć | Operator widzi kogo i dlaczego zablokowano oraz zdejmuje blokadę (ADMIN, z potwierdzeniem, audyt po stronie API).</t>
         </is>
       </c>
       <c r="P63" s="10" t="inlineStr">
@@ -5717,12 +5717,12 @@
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>H-09</t>
+          <t>H-22</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>Kopia bezpieczeństwa przed odtworzeniem</t>
+          <t>Panel odtwarzania w widocznym miejscu</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -5744,7 +5744,7 @@
         <v>6</v>
       </c>
       <c r="G64" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
@@ -5753,22 +5753,22 @@
       </c>
       <c r="I64" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J64" s="10" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K64" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L64" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
+          <t>2026-09-23: client-panel BackupsTab.tsx — sekcja „Kopie poza serwerem” (HostingOffsitePanel) w zakładce Kopie zapasowe; zdublowany panel przywracania usunięty z Zużycia zasobów (hosting-backup-restore-panel.tsx)</t>
         </is>
       </c>
       <c r="M64" s="11" t="inlineStr">
@@ -5778,12 +5778,12 @@
       </c>
       <c r="N64" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O64" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: hosting-restore.service.ts:167 tylko KOLEJKUJE backup w DA i nie czeka na wynik — destrukcyjne odtworzenie rusza mimo nieudanej kopii. Job dostaje COMPLETED (:182) w chwili przyjęcia zadania, nie po odtworzeniu. | Naprawione: nadpisywanie danych bez siatki. Status COMPLETED w panelu klienta opisany uczciwie („Odtwarzanie zlecone — serwer odtwarza dane w tle”), bo DA przyjmuje odtworzenie asynchronicznie. OTWARTE do D3 (PB-21): pełny przebieg na żywym DA i wykrycie końca odtwarzania.</t>
+          <t>klient w kryzysie tego nie znajdzie | Kopie off-site są tam, gdzie klient ich szuka w kryzysie; przywracanie jest w jednym miejscu, z potwierdzeniem domeną.</t>
         </is>
       </c>
       <c r="P64" s="10" t="inlineStr">
@@ -5795,12 +5795,12 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>H-17</t>
+          <t>H-09</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>Tryb restore skryptu odtwarzającego osiągalny z produktu</t>
+          <t>Kopia bezpieczeństwa przed odtworzeniem</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -5841,27 +5841,27 @@
       </c>
       <c r="K65" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L65" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: produktowa ścieżka odtwarzania z off-site = „Pobierz na serwer” (fetch, agent) + przywrócenie z listy kopii z kopią bezpieczeństwa (H-09) i potwierdzeniem domeną; tryb `restore` skryptu (DA type=admin, bez kopii bezpieczeństwa) celowo zostaje tylko w CLI/runbooku DR</t>
+          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
         </is>
       </c>
       <c r="M65" s="11" t="inlineStr">
         <is>
-          <t>H-20 (najpierw potwierdzone odtworzenie, potem wystawienie trybu w produkcie)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N65" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O65" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: tryb restore jest martwy z poziomu produktu, ale żywy z CLI (node-account-restore.sh:120-124) i udokumentowany w runbooku. | DO DECYZJI WŁAŚCICIELA: proponuję zamknąć jako PARYTET przez równoważną ścieżkę produktową — wystawienie trybu `restore` ominęłoby kopię bezpieczeństwa z H-09. Tryb restore działa też tylko przy istniejącym koncie na węźle, czyli dokładnie tam, gdzie wystarcza fetch + przywrócenie. | DECYZJA WŁAŚCICIELA 2026-09-23: zamknięte jako PARYTET — ścieżka produktowa (pobierz na serwer + przywrócenie z kopią bezpieczeństwa i potwierdzeniem domeną) daje ten sam efekt bezpieczniej; tryb restore skryptu zostaje wyłącznie w CLI/runbooku DR.</t>
+          <t>OSŁABIONE: hosting-restore.service.ts:167 tylko KOLEJKUJE backup w DA i nie czeka na wynik — destrukcyjne odtworzenie rusza mimo nieudanej kopii. Job dostaje COMPLETED (:182) w chwili przyjęcia zadania, nie po odtworzeniu. | Naprawione: nadpisywanie danych bez siatki. Status COMPLETED w panelu klienta opisany uczciwie („Odtwarzanie zlecone — serwer odtwarza dane w tle”), bo DA przyjmuje odtworzenie asynchronicznie. OTWARTE do D3 (PB-21): pełny przebieg na żywym DA i wykrycie końca odtwarzania.</t>
         </is>
       </c>
       <c r="P65" s="10" t="inlineStr">
@@ -5873,12 +5873,12 @@
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>G-20</t>
+          <t>H-17</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Ochrona przed atakiem słownikowym na panel</t>
+          <t>Tryb restore skryptu odtwarzającego osiągalny z produktu</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="E66" s="10" t="inlineStr">
@@ -5924,12 +5924,12 @@
       </c>
       <c r="L66" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D2: common/guards/rate-limit.guard.spec.ts (6 testów: limit per IP, per e-mail z wielu IP, reset okna, zakresy i @SkipRateLimit, przepełnienie mapy, awaria Redisa)</t>
+          <t>2026-09-23: produktowa ścieżka odtwarzania z off-site = „Pobierz na serwer” (fetch, agent) + przywrócenie z listy kopii z kopią bezpieczeństwa (H-09) i potwierdzeniem domeną; tryb `restore` skryptu (DA type=admin, bez kopii bezpieczeństwa) celowo zostaje tylko w CLI/runbooku DR</t>
         </is>
       </c>
       <c r="M66" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>H-20 (najpierw potwierdzone odtworzenie, potem wystawienie trybu w produkcie)</t>
         </is>
       </c>
       <c r="N66" s="11" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="O66" s="11" t="inlineStr">
         <is>
-          <t>brak dowodu D2 na krytycznym guardzie | ZNALEZISKO przy pisaniu testów: w trybie pamięciowym przepełnienie mapy (50 tys. kluczy) czyściło WSZYSTKIE liczniki — losowe e-maile zerowały licznik prób logowania do atakowanego konta (fail-open). Teraz usuwane są tylko wygasłe, a przy pełnej mapie nowe klucze dostają 429 (fail-closed).</t>
+          <t>Skorygowane: tryb restore jest martwy z poziomu produktu, ale żywy z CLI (node-account-restore.sh:120-124) i udokumentowany w runbooku. | DO DECYZJI WŁAŚCICIELA: proponuję zamknąć jako PARYTET przez równoważną ścieżkę produktową — wystawienie trybu `restore` ominęłoby kopię bezpieczeństwa z H-09. Tryb restore działa też tylko przy istniejącym koncie na węźle, czyli dokładnie tam, gdzie wystarcza fetch + przywrócenie. | DECYZJA WŁAŚCICIELA 2026-09-23: zamknięte jako PARYTET — ścieżka produktowa (pobierz na serwer + przywrócenie z kopią bezpieczeństwa i potwierdzeniem domeną) daje ten sam efekt bezpieczniej; tryb restore skryptu zostaje wyłącznie w CLI/runbooku DR.</t>
         </is>
       </c>
       <c r="P66" s="10" t="inlineStr">
@@ -5951,12 +5951,12 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>I-11</t>
+          <t>G-20</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>Staging — publikacja na produkcję</t>
+          <t>Ochrona przed atakiem słownikowym na panel</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E67" s="10" t="inlineStr">
@@ -5997,12 +5997,12 @@
       </c>
       <c r="K67" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L67" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
+          <t>2026-09-23 D2: common/guards/rate-limit.guard.spec.ts (6 testów: limit per IP, per e-mail z wielu IP, reset okna, zakresy i @SkipRateLimit, przepełnienie mapy, awaria Redisa)</t>
         </is>
       </c>
       <c r="M67" s="11" t="inlineStr">
@@ -6012,12 +6012,12 @@
       </c>
       <c r="N67" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O67" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: node-staging-sync.sh:141-142 backup plików jest twardą bramką, ale :152-153 backup bazy LIVE jest best-effort — linia 158 robi wp db import na produkcji mimo braku kopii. | Naprawione: import bazy staging na produkcję mimo braku kopii bazy LIVE. OTWARTE do D3 (PB-21): publikacja stagingu na żywym węźle.</t>
+          <t>brak dowodu D2 na krytycznym guardzie | ZNALEZISKO przy pisaniu testów: w trybie pamięciowym przepełnienie mapy (50 tys. kluczy) czyściło WSZYSTKIE liczniki — losowe e-maile zerowały licznik prób logowania do atakowanego konta (fail-open). Teraz usuwane są tylko wygasłe, a przy pełnej mapie nowe klucze dostają 429 (fail-closed).</t>
         </is>
       </c>
       <c r="P67" s="10" t="inlineStr">
@@ -6029,12 +6029,12 @@
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>X-31</t>
+          <t>I-11</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>Kanał alertów daje znak życia (dead man's switch)</t>
+          <t>Staging — publikacja na produkcję</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -6044,19 +6044,19 @@
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F68" s="10" t="n">
         <v>6</v>
       </c>
       <c r="G68" s="10" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
@@ -6065,22 +6065,22 @@
       </c>
       <c r="I68" s="10" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="J68" s="10" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="K68" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L68" s="11" t="inlineStr">
         <is>
-          <t>ops/observability/grafana/provisioning/alerting/rules.yaml — grupa verris_kanal_alertow, reguła VerrisKanalAlertowZyje (vector(1), for: 0s, oba stany awaryjne na Alerting, etykieta kanal: heartbeat); policies.yaml — gałąź object_matchers kanal=heartbeat, repeat_interval 24h; apps/api/src/test/routing-alertow.spec.ts (5 asercji X-31); docs/ops/GRAFANA_ALERTING.md §4. BRAK: pierwszego maila [FIRING:1] VerrisKanalAlertowZyje — dowód D3 jeszcze nie powstał.</t>
+          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
         </is>
       </c>
       <c r="M68" s="11" t="inlineStr">
@@ -6090,12 +6090,12 @@
       </c>
       <c r="N68" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 powstanie przy pierwszym mailu. Decyzja właściciela produktu: wariant „jeden mail na dobę". | PROBLEM: po naprawie X-30 alerty ucichną, a cisza będzie znaczyła „nic się nie pali" — i będzie wyglądała IDENTYCZNIE jak: Grafana padła, Postfix przestał przyjmować, mail.hvln.pl zaczął odrzucać albo wrzucać do spamu, ktoś zmienił adres w punkcie kontaktowym, polityka przestała pasować do etykiet. To dokładnie ta sama cisza, która przez miesiąc znaczyła „kopia bazy jest w porządku" (H-23) i kosztowała wszystkie kopie zapasowe. | ROZWIĄZANIE: VerrisKanalAlertowZyje — reguła vector(1), pali się ZAWSZE, jej BRAK jest sygnałem. for: 0s, noDataState: Alerting, execErrState: Alerting — nie da się jej „nie zapalić": normalnie warunek jest spełniony, a gdyby źródło danych przestało odpowiadać, oba stany awaryjne też prowadzą do Alerting. Milczenie ma znaczyć awarię, nigdy spokój. | JEDEN MAIL NA DOBĘ, NIE SZEŚĆ: osobna gałąź polityki na etykiecie kanal: heartbeat z repeat_interval 24h. Na domyślnej (4h) byłoby sześć dziennie, a alert przychodzący sześć razy dziennie przestaje być czytany po tygodniu — wtedy przestaje cokolwiek dawać, bo jego BRAK jest jedyną informacją, jaką niesie. Strażnik pilnuje osobno, że polityka domyślna NIE została przy okazji przestawiona na dobę: prawdziwy alarm ma się przypominać co cztery godziny. | HACZYK, KTÓRY TRZEBA NAZWAĆ: mail, którego się nie czyta, wraca do punktu wyjścia. Jeśli po tygodniu przestanie być zauważany, reguła przestaje działać — nie dlatego, że jest zepsuta, tylko dlatego, że przestała być czytana. Tego nie da się naprawić kodem. | CZEGO NIE OBEJMUJE: awarii całego serwera (heartbeat mieszka na tej samej maszynie co Grafana i milczy razem z nią — odporny byłby watchdog SPOZA naszej infrastruktury, pukany cronem; nie ma go i to świadoma decyzja, nie przeoczenie) ani poprawności pozostałych reguł (tego pilnuje bramka z X-30). | Czerwieni się na starym kodzie: 5 z 36. | Doszła lista DOPISANE_POZNIEJ, trzymana osobno od ALERTY: tamta odpowiada na pytanie „czy migracja czegoś nie zgubiła" i ma zostać zamrożona, ta na „czy ktoś czegoś po cichu nie dołożył". Dokumentacja: docs/archiwum/zadania/X-31-znak-zycia-kanalu-alertow.md | 2026-09-22 D3: wlasciciel potwierdza, ze mail [FIRING:1] VerrisKanalAlertowZyje przychodzi codziennie. Kanal alertow dziala koniec-do-konca.</t>
+          <t>OSŁABIONE: node-staging-sync.sh:141-142 backup plików jest twardą bramką, ale :152-153 backup bazy LIVE jest best-effort — linia 158 robi wp db import na produkcji mimo braku kopii. | Naprawione: import bazy staging na produkcję mimo braku kopii bazy LIVE. OTWARTE do D3 (PB-21): publikacja stagingu na żywym węźle.</t>
         </is>
       </c>
       <c r="P68" s="10" t="inlineStr">
@@ -6107,12 +6107,12 @@
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>X-32</t>
+          <t>X-31</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Martwy job da się odrzucić z panelu, ze śladem w audycie</t>
+          <t>Kanał alertów daje znak życia (dead man's switch)</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="L69" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/common/audit/audit.actions.ts — PROVISIONING_JOB_DISCARDED_BY_ADMIN; provisioning-queue.service.ts — odrzucJob (getState() === failed, ślad przed job.remove(), audyt z subskrypcją, typem, liczbą prób, failedReason i powodem); provisioning-queue.admin.controller.ts — POST :id/odrzuc za @StaffPerm('PROVISIONING_MANAGE'); apps/admin-panel/.../provisioning-queue/ — actions.ts, odrzuc-button.tsx (dwa kliknięcia, powód ≥5 znaków, zdanie o nietkniętej subskrypcji), page.tsx; apps/api/src/test/odrzucenie-martwego-joba.spec.ts (13). BRAK: pierwszego odrzucenia na produkcji — dowód D3 jeszcze nie powstał.</t>
+          <t>ops/observability/grafana/provisioning/alerting/rules.yaml — grupa verris_kanal_alertow, reguła VerrisKanalAlertowZyje (vector(1), for: 0s, oba stany awaryjne na Alerting, etykieta kanal: heartbeat); policies.yaml — gałąź object_matchers kanal=heartbeat, repeat_interval 24h; apps/api/src/test/routing-alertow.spec.ts (5 asercji X-31); docs/ops/GRAFANA_ALERTING.md §4. BRAK: pierwszego maila [FIRING:1] VerrisKanalAlertowZyje — dowód D3 jeszcze nie powstał.</t>
         </is>
       </c>
       <c r="M69" s="11" t="inlineStr">
@@ -6173,7 +6173,7 @@
       </c>
       <c r="O69" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 przy pierwszym odrzuceniu na produkcji — a to da się zrobić od razu po wdrożeniu, w odróżnieniu od Z-18, który czeka na węzeł. Decyzja właściciela produktu: dorobić akcję w panelu zamiast jednorazowego czyszczenia Redisa. | JAK TO WYSZŁO: X-30 naprawiło alerting, VerrisProvisioningQueueFailed zapalił się z prawdziwego powodu i wskazał cztery martwe joby (to z nich wyszło Z-18). Naturalny następny ruch — usunąć je — okazał się NIEWYKONALNY: panel ma przy nich wyłącznie „Retry", a kontroler administracyjny dokładnie dwa endpointy, listowanie i ponowienie. Retry nic nie daje, bo węzła nie ma: job padnie ponownie, podbije licznik prób i dołoży wpisy do audytu — cztery martwe joby zamieniają się w cztery martwe joby z dłuższą historią. Zostawało grzebanie w Redisie ręcznie, czyli zmiana stanu produkcyjnego dotyczącego subskrypcji klientów BEZ ŚLADU W AUDYCIE. | TO NIE JEST USTERKA TYCH CZTERECH JOBÓW, tylko luka w warstwie operatorskiej, która ujawni się ponownie przy pierwszym prawdziwym niepowodzeniu provisioningu — z tą różnicą, że wtedy po drugiej stronie będzie klient. | ROZWIĄZANIE: POST /admin/provisioning-queue/:id/odrzuc + przycisk „Odrzuć" obok Retry. TRZY REGUŁY: (1) TYLKO STAN failed — usunięcie joba aktywnego albo czekającego osierociłoby provisioning w trakcie, konto na węźle mogłoby powstać, a system przestałby o nim wiedzieć; ograniczenie siedzi w usłudze, nie w kontrolerze, bo to reguła o kolejce, nie o HTTP; (2) POWÓD WYMAGANY, tak samo jak przy retry — operacja bez powodu to operacja, której za pół roku nikt nie wyjaśni; (3) NAJPIERW ODCZYT, POTEM USUNIĘCIE — ślad zbierany PRZED job.remove(), bo po usunięciu nie ma już czego odczytać; zapisujemy subskrypcję, joba, typ, liczbę prób, ostatni błąd i powód. Po Z-18 ten ostatni błąd niesie PRAWDZIWĄ przyczynę, więc wpis ma realną wartość dowodową — jeszcze wczoraj zapisałby zdanie o brakującym pakiecie DirectAdmina, którego nigdy nie brakowało. | OSOBNA AKCJA AUDYTU (PROVISIONING_JOB_DISCARDED_BY_ADMIN), nie wariant retry: w raportach odrzucenie i ponowienie to dwie różne decyzje i nie wolno im się zlewać. | DWA KLIKNIĘCIA, NIE JEDNO: retry można cofnąć następnym retry, odrzucenia nie da się cofnąć wcale. Potwierdzenie jest po to, żeby ta różnica była wyczuwalna w palcach. | ZDANIE PRZY PRZYCISKU: „Usuwa wpis z kolejki bez możliwości cofnięcia. Subskrypcja zostaje nietknięta." Operator ma prawo założyć, że „odrzuć" anuluje zamówienie — nie anuluje. Musi to być napisane tam, gdzie się klika, a nie w dokumentacji, której nikt nie otworzy w trakcie incydentu. | Czerwieni się na starym kodzie: 11 z 13. | DWIE UWAGI O SAMYCH TESTACH: odczyty plików panelu są LENIWE, bo odczyt na poziomie describe wywalał cały plik testowy, zanim cokolwiek się policzyło — a wtedy nie wiadomo, ILE asercji się czerwieni, tylko że „nie skompilowało się"; asercja o warunku row.failedReason nie mierzy odległości w znakach, tylko relację między warunkiem a przyciskiem, bo wersja licząca znaki zepsuła się od dopisania komentarza i kusiło, żeby poszerzyć okno zamiast poprawić asercję — to byłoby naprawianie testu zamiast kodu. | CZEGO NIE OBEJMUJE: losu czterech subskrypcji, które dostały zwrot i status PENDING_PAYMENT (odrzucenie joba ich nie dotyka — osobne sprzątanie po stronie bazy); odrzucania hurtem — świadomie, bo przycisk „odrzuć wszystkie" jest wygodny dokładnie do momentu, w którym ktoś kliknie go na kolejce z prawdziwym zamówieniem. | JAK ZAMKNĄĆ: odrzucić jeden z czterech martwych jobów, obejrzeć wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie i sprawdzić, że verris_provisioning_queue_depth{state="failed"} spadło o jeden. Dokumentacja: docs/archiwum/zadania/X-32-odrzucenie-martwego-joba.md | 2026-09-22 D3: wlasciciel odrzucil martwy job przyciskiem 'Odrzuc' w panelu admina na produkcji (potwierdzenie wlasciciela; wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie).</t>
+          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 powstanie przy pierwszym mailu. Decyzja właściciela produktu: wariant „jeden mail na dobę". | PROBLEM: po naprawie X-30 alerty ucichną, a cisza będzie znaczyła „nic się nie pali" — i będzie wyglądała IDENTYCZNIE jak: Grafana padła, Postfix przestał przyjmować, mail.hvln.pl zaczął odrzucać albo wrzucać do spamu, ktoś zmienił adres w punkcie kontaktowym, polityka przestała pasować do etykiet. To dokładnie ta sama cisza, która przez miesiąc znaczyła „kopia bazy jest w porządku" (H-23) i kosztowała wszystkie kopie zapasowe. | ROZWIĄZANIE: VerrisKanalAlertowZyje — reguła vector(1), pali się ZAWSZE, jej BRAK jest sygnałem. for: 0s, noDataState: Alerting, execErrState: Alerting — nie da się jej „nie zapalić": normalnie warunek jest spełniony, a gdyby źródło danych przestało odpowiadać, oba stany awaryjne też prowadzą do Alerting. Milczenie ma znaczyć awarię, nigdy spokój. | JEDEN MAIL NA DOBĘ, NIE SZEŚĆ: osobna gałąź polityki na etykiecie kanal: heartbeat z repeat_interval 24h. Na domyślnej (4h) byłoby sześć dziennie, a alert przychodzący sześć razy dziennie przestaje być czytany po tygodniu — wtedy przestaje cokolwiek dawać, bo jego BRAK jest jedyną informacją, jaką niesie. Strażnik pilnuje osobno, że polityka domyślna NIE została przy okazji przestawiona na dobę: prawdziwy alarm ma się przypominać co cztery godziny. | HACZYK, KTÓRY TRZEBA NAZWAĆ: mail, którego się nie czyta, wraca do punktu wyjścia. Jeśli po tygodniu przestanie być zauważany, reguła przestaje działać — nie dlatego, że jest zepsuta, tylko dlatego, że przestała być czytana. Tego nie da się naprawić kodem. | CZEGO NIE OBEJMUJE: awarii całego serwera (heartbeat mieszka na tej samej maszynie co Grafana i milczy razem z nią — odporny byłby watchdog SPOZA naszej infrastruktury, pukany cronem; nie ma go i to świadoma decyzja, nie przeoczenie) ani poprawności pozostałych reguł (tego pilnuje bramka z X-30). | Czerwieni się na starym kodzie: 5 z 36. | Doszła lista DOPISANE_POZNIEJ, trzymana osobno od ALERTY: tamta odpowiada na pytanie „czy migracja czegoś nie zgubiła" i ma zostać zamrożona, ta na „czy ktoś czegoś po cichu nie dołożył". Dokumentacja: docs/archiwum/zadania/X-31-znak-zycia-kanalu-alertow.md | 2026-09-22 D3: wlasciciel potwierdza, ze mail [FIRING:1] VerrisKanalAlertowZyje przychodzi codziennie. Kanal alertow dziala koniec-do-konca.</t>
         </is>
       </c>
       <c r="P69" s="10" t="inlineStr">
@@ -6185,12 +6185,12 @@
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>X-32</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>W drzewie stoją dwa majory ESLinta naraz</t>
+          <t>Martwy job da się odrzucić z panelu, ze śladem w audycie</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -6205,7 +6205,7 @@
       </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F70" s="10" t="n">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="L70" s="11" t="inlineStr">
         <is>
-          <t>package.json (korzeń) — @eslint/js ^10.0.1 przy braku jakiegokolwiek eslint.config.* w korzeniu; libs/eslint-config/node_modules: eslint 10.9.0 obok @eslint/js 9.39.5; apps/api, apps/www, apps/client-panel, apps/status-page, libs/directadmin-sdk — eslint 9.39.5 | 2026-09-23: z korzenia zdjęte nieużywane @eslint/js ^10 i typescript-eslint; libs/eslint-config peer eslint ^9.39.5 (było &gt;=9 → auto-install dociągał 10.9.0); lockfile bez eslint 10; strażnik apps/api/src/test/eslint-jeden-major.spec.ts (deklaracje + peer + lockfile)</t>
+          <t>apps/api/src/common/audit/audit.actions.ts — PROVISIONING_JOB_DISCARDED_BY_ADMIN; provisioning-queue.service.ts — odrzucJob (getState() === failed, ślad przed job.remove(), audyt z subskrypcją, typem, liczbą prób, failedReason i powodem); provisioning-queue.admin.controller.ts — POST :id/odrzuc za @StaffPerm('PROVISIONING_MANAGE'); apps/admin-panel/.../provisioning-queue/ — actions.ts, odrzuc-button.tsx (dwa kliknięcia, powód ≥5 znaków, zdanie o nietkniętej subskrypcji), page.tsx; apps/api/src/test/odrzucenie-martwego-joba.spec.ts (13). BRAK: pierwszego odrzucenia na produkcji — dowód D3 jeszcze nie powstał.</t>
         </is>
       </c>
       <c r="M70" s="11" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="O70" s="11" t="inlineStr">
         <is>
-          <t>Odkryte 2026-08-28 przy DEP-01. Korzeń deklaruje @eslint/js ^10.0.1, którego peer to eslint ^10.0.0 — i to on wciąga eslint@10.9.0 do drzewa. Tymczasem KAŻDY pakiet, który realnie lintuje, ma 9.39.5. Najostrzej widać to wewnątrz libs/eslint-config, czyli wspólnej konfiguracji: node_modules/eslint = 10.9.0, node_modules/@eslint/js = 9.39.5 — dwie połowy jednego narzędzia z różnych majorów w jednym katalogu. | Korzeń NIE MA żadnego eslint.config.* i nie odpala lintera (pnpm lint = turbo run lint), więc te zależności nie robią nic poza wciąganiem majora, którego nikt nie używa. | To nie awaria — bramka jest zielona, 0 błędów. To BRAK KONTROLI: żaden strażnik nie sprawdza, czy major ESLinta jest jeden, tak jak do ENV-01 nic nie sprawdzało wersji Node. | DO ZROBIENIA: zdjąć z korzenia nieużywane @eslint/js i typescript-eslint albo cofnąć je do dziewiątki (rusza lockfile — osobny commit z pełną bramką), plus strażnik spójności majora na wzór wersja-node.spec.ts. | 2026-09-23: zrobione zgodnie z DO ZROBIENIA; lockfile zmieniony wyłącznie o usunięcie gałęzi eslint 10 (pnpm 9.5.0 --lockfile-only). Przed bramką lokalną: pnpm install.</t>
+          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 przy pierwszym odrzuceniu na produkcji — a to da się zrobić od razu po wdrożeniu, w odróżnieniu od Z-18, który czeka na węzeł. Decyzja właściciela produktu: dorobić akcję w panelu zamiast jednorazowego czyszczenia Redisa. | JAK TO WYSZŁO: X-30 naprawiło alerting, VerrisProvisioningQueueFailed zapalił się z prawdziwego powodu i wskazał cztery martwe joby (to z nich wyszło Z-18). Naturalny następny ruch — usunąć je — okazał się NIEWYKONALNY: panel ma przy nich wyłącznie „Retry", a kontroler administracyjny dokładnie dwa endpointy, listowanie i ponowienie. Retry nic nie daje, bo węzła nie ma: job padnie ponownie, podbije licznik prób i dołoży wpisy do audytu — cztery martwe joby zamieniają się w cztery martwe joby z dłuższą historią. Zostawało grzebanie w Redisie ręcznie, czyli zmiana stanu produkcyjnego dotyczącego subskrypcji klientów BEZ ŚLADU W AUDYCIE. | TO NIE JEST USTERKA TYCH CZTERECH JOBÓW, tylko luka w warstwie operatorskiej, która ujawni się ponownie przy pierwszym prawdziwym niepowodzeniu provisioningu — z tą różnicą, że wtedy po drugiej stronie będzie klient. | ROZWIĄZANIE: POST /admin/provisioning-queue/:id/odrzuc + przycisk „Odrzuć" obok Retry. TRZY REGUŁY: (1) TYLKO STAN failed — usunięcie joba aktywnego albo czekającego osierociłoby provisioning w trakcie, konto na węźle mogłoby powstać, a system przestałby o nim wiedzieć; ograniczenie siedzi w usłudze, nie w kontrolerze, bo to reguła o kolejce, nie o HTTP; (2) POWÓD WYMAGANY, tak samo jak przy retry — operacja bez powodu to operacja, której za pół roku nikt nie wyjaśni; (3) NAJPIERW ODCZYT, POTEM USUNIĘCIE — ślad zbierany PRZED job.remove(), bo po usunięciu nie ma już czego odczytać; zapisujemy subskrypcję, joba, typ, liczbę prób, ostatni błąd i powód. Po Z-18 ten ostatni błąd niesie PRAWDZIWĄ przyczynę, więc wpis ma realną wartość dowodową — jeszcze wczoraj zapisałby zdanie o brakującym pakiecie DirectAdmina, którego nigdy nie brakowało. | OSOBNA AKCJA AUDYTU (PROVISIONING_JOB_DISCARDED_BY_ADMIN), nie wariant retry: w raportach odrzucenie i ponowienie to dwie różne decyzje i nie wolno im się zlewać. | DWA KLIKNIĘCIA, NIE JEDNO: retry można cofnąć następnym retry, odrzucenia nie da się cofnąć wcale. Potwierdzenie jest po to, żeby ta różnica była wyczuwalna w palcach. | ZDANIE PRZY PRZYCISKU: „Usuwa wpis z kolejki bez możliwości cofnięcia. Subskrypcja zostaje nietknięta." Operator ma prawo założyć, że „odrzuć" anuluje zamówienie — nie anuluje. Musi to być napisane tam, gdzie się klika, a nie w dokumentacji, której nikt nie otworzy w trakcie incydentu. | Czerwieni się na starym kodzie: 11 z 13. | DWIE UWAGI O SAMYCH TESTACH: odczyty plików panelu są LENIWE, bo odczyt na poziomie describe wywalał cały plik testowy, zanim cokolwiek się policzyło — a wtedy nie wiadomo, ILE asercji się czerwieni, tylko że „nie skompilowało się"; asercja o warunku row.failedReason nie mierzy odległości w znakach, tylko relację między warunkiem a przyciskiem, bo wersja licząca znaki zepsuła się od dopisania komentarza i kusiło, żeby poszerzyć okno zamiast poprawić asercję — to byłoby naprawianie testu zamiast kodu. | CZEGO NIE OBEJMUJE: losu czterech subskrypcji, które dostały zwrot i status PENDING_PAYMENT (odrzucenie joba ich nie dotyka — osobne sprzątanie po stronie bazy); odrzucania hurtem — świadomie, bo przycisk „odrzuć wszystkie" jest wygodny dokładnie do momentu, w którym ktoś kliknie go na kolejce z prawdziwym zamówieniem. | JAK ZAMKNĄĆ: odrzucić jeden z czterech martwych jobów, obejrzeć wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie i sprawdzić, że verris_provisioning_queue_depth{state="failed"} spadło o jeden. Dokumentacja: docs/archiwum/zadania/X-32-odrzucenie-martwego-joba.md | 2026-09-22 D3: wlasciciel odrzucil martwy job przyciskiem 'Odrzuc' w panelu admina na produkcji (potwierdzenie wlasciciela; wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie).</t>
         </is>
       </c>
       <c r="P70" s="10" t="inlineStr">
@@ -6263,12 +6263,12 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>M-08</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>Anulowanie faktury (VOID) z panelu</t>
+          <t>W drzewie stoją dwa majory ESLinta naraz</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -6278,12 +6278,12 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F71" s="10" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="L71" s="11" t="inlineStr">
         <is>
-          <t>billing/anulowanie.service.ts (POST /admin/invoices/:id/anuluj, BILLING_MANAGE); admin: invoices/void-button.tsx; test D2 anulowanie.service.spec.ts</t>
+          <t>package.json (korzeń) — @eslint/js ^10.0.1 przy braku jakiegokolwiek eslint.config.* w korzeniu; libs/eslint-config/node_modules: eslint 10.9.0 obok @eslint/js 9.39.5; apps/api, apps/www, apps/client-panel, apps/status-page, libs/directadmin-sdk — eslint 9.39.5 | 2026-09-23: z korzenia zdjęte nieużywane @eslint/js ^10 i typescript-eslint; libs/eslint-config peer eslint ^9.39.5 (było &gt;=9 → auto-install dociągał 10.9.0); lockfile bez eslint 10; strażnik apps/api/src/test/eslint-jeden-major.spec.ts (deklaracje + peer + lockfile)</t>
         </is>
       </c>
       <c r="M71" s="11" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="O71" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: anulować wolno tylko dokument nieopłacony (DRAFT/OPEN); opłacony, także z portfela, zmienia się korektą (M-06). Faktura Stripe unieważniana najpierw w Stripe, błąd = brak zmiany lokalnej. Numer zostaje (ciągłość), powód w audycie INVOICE_VOIDED.</t>
+          <t>Odkryte 2026-08-28 przy DEP-01. Korzeń deklaruje @eslint/js ^10.0.1, którego peer to eslint ^10.0.0 — i to on wciąga eslint@10.9.0 do drzewa. Tymczasem KAŻDY pakiet, który realnie lintuje, ma 9.39.5. Najostrzej widać to wewnątrz libs/eslint-config, czyli wspólnej konfiguracji: node_modules/eslint = 10.9.0, node_modules/@eslint/js = 9.39.5 — dwie połowy jednego narzędzia z różnych majorów w jednym katalogu. | Korzeń NIE MA żadnego eslint.config.* i nie odpala lintera (pnpm lint = turbo run lint), więc te zależności nie robią nic poza wciąganiem majora, którego nikt nie używa. | To nie awaria — bramka jest zielona, 0 błędów. To BRAK KONTROLI: żaden strażnik nie sprawdza, czy major ESLinta jest jeden, tak jak do ENV-01 nic nie sprawdzało wersji Node. | DO ZROBIENIA: zdjąć z korzenia nieużywane @eslint/js i typescript-eslint albo cofnąć je do dziewiątki (rusza lockfile — osobny commit z pełną bramką), plus strażnik spójności majora na wzór wersja-node.spec.ts. | 2026-09-23: zrobione zgodnie z DO ZROBIENIA; lockfile zmieniony wyłącznie o usunięcie gałęzi eslint 10 (pnpm 9.5.0 --lockfile-only). Przed bramką lokalną: pnpm install.</t>
         </is>
       </c>
       <c r="P71" s="10" t="inlineStr">
@@ -6341,12 +6341,12 @@
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>C-18</t>
+          <t>M-08</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Konto FTP — zmiana hasła</t>
+          <t>Anulowanie faktury (VOID) z panelu</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="E72" s="10" t="inlineStr">
@@ -6387,12 +6387,12 @@
       </c>
       <c r="K72" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L72" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/hosting-ftp/:username/password (ZmienHasloFtpDto) → directadmin.service changeHostingFtpPassword (action=modify, katalog zachowany) + audyt HOSTING_FTP_PASSWORD_CHANGED; UI FtpTab — kluczyk przy koncie; test servers/zmiana-hasla-ftp.spec.ts</t>
+          <t>billing/anulowanie.service.ts (POST /admin/invoices/:id/anuluj, BILLING_MANAGE); admin: invoices/void-button.tsx; test D2 anulowanie.service.spec.ts</t>
         </is>
       </c>
       <c r="M72" s="11" t="inlineStr">
@@ -6402,12 +6402,12 @@
       </c>
       <c r="N72" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O72" s="11" t="inlineStr">
         <is>
-          <t>brak jakiejkolwiek ścieżki edycji istniejącego konta | Przy okazji body tworzenia konta FTP dostało klasę DTO (login, hasło, katalog bez „..”). OTWARTE do D3 (PB-21): format action=modify na żywym DA.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: anulować wolno tylko dokument nieopłacony (DRAFT/OPEN); opłacony, także z portfela, zmienia się korektą (M-06). Faktura Stripe unieważniana najpierw w Stripe, błąd = brak zmiany lokalnej. Numer zostaje (ciągłość), powód w audycie INVOICE_VOIDED.</t>
         </is>
       </c>
       <c r="P72" s="10" t="inlineStr">
@@ -6419,12 +6419,12 @@
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>C-18</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>Konto FTP — zmiana hasła</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -6434,7 +6434,7 @@
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
@@ -6446,7 +6446,7 @@
         <v>6</v>
       </c>
       <c r="G73" s="10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H73" s="10" t="inlineStr">
         <is>
@@ -6455,22 +6455,22 @@
       </c>
       <c r="I73" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="J73" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="K73" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L73" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>2026-09-23 D1: POST /services/:id/hosting-ftp/:username/password (ZmienHasloFtpDto) → directadmin.service changeHostingFtpPassword (action=modify, katalog zachowany) + audyt HOSTING_FTP_PASSWORD_CHANGED; UI FtpTab — kluczyk przy koncie; test servers/zmiana-hasla-ftp.spec.ts</t>
         </is>
       </c>
       <c r="M73" s="11" t="inlineStr">
@@ -6480,12 +6480,12 @@
       </c>
       <c r="N73" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O73" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>brak jakiejkolwiek ścieżki edycji istniejącego konta | Przy okazji body tworzenia konta FTP dostało klasę DTO (login, hasło, katalog bez „..”). OTWARTE do D3 (PB-21): format action=modify na żywym DA.</t>
         </is>
       </c>
       <c r="P73" s="10" t="inlineStr">
@@ -6497,12 +6497,12 @@
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>C-11</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>Spakowanie do archiwum</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -6512,12 +6512,12 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E74" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F74" s="10" t="n">
@@ -6543,12 +6543,12 @@
       </c>
       <c r="K74" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L74" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M74" s="11" t="inlineStr">
@@ -6558,12 +6558,12 @@
       </c>
       <c r="N74" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O74" s="11" t="inlineStr">
         <is>
-          <t>standard we wszystkich panelach | OTWARTE do D3 (PB-21): format action=compress na żywym DA.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P74" s="10" t="inlineStr">
@@ -6575,12 +6575,12 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>NODE-03</t>
+          <t>C-11</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>Pojemność węzła nigdy się nie odświeża</t>
+          <t>Spakowanie do archiwum</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
@@ -6626,7 +6626,7 @@
       </c>
       <c r="L75" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: verris-lve.sh node_capacity (nproc, MemTotal, df /) w każdym raporcie, lve-agent/1.1; telemetry.dto NodeStatusDto.totalCpuCores/totalMemoryMb/totalDiskMb; telemetry.service aktualizuje Server; test telemetry/pojemnosc-wezla.spec.ts</t>
+          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych</t>
         </is>
       </c>
       <c r="M75" s="11" t="inlineStr">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="O75" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Pojemność węzła nigdy się nie odświeża. `totalCpuCores`/`totalMemoryMb`/`totalDiskMb` ustawiane wyłącznie w handshake; telemetria ich nie aktualizuje — mimo komentarza w schemacie „reported via handshake / heartbeat”. Rozbudowa węzła nie dociera do `NodeSelector`. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Telemetria aktualizuje totalCpuCores/totalMemoryMb/totalDiskMb, nie tylko handshake. | Stary agent bez pól niczego nie zeruje. OTWARTE do D3 (PB-21): raport z agenta na żywym węźle i odświeżona pojemność w panelu admina. | 2026-09-25: pojemność z agenta trafia też do planera pojemności (admin → Product Ops): ryzyko liczone względem rdzeni i RAM węzła (CPU 2×/4× rdzeni, RAM 1×/1,5×; test ryzyko-pojemnosci.spec.ts), a opis „CPU 250%” zastąpiony „przydzielone limity: CPU 2,5 rdz. z N · RAM x z y GB” — wcześniej wyglądało jak zużycie ponad 100%.</t>
+          <t>standard we wszystkich panelach | OTWARTE do D3 (PB-21): format action=compress na żywym DA.</t>
         </is>
       </c>
       <c r="P75" s="10" t="inlineStr">
@@ -6653,31 +6653,31 @@
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>PB-08</t>
+          <t>NODE-03</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
+          <t>Pojemność węzła nigdy się nie odświeża</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E76" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F76" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G76" s="10" t="n">
         <v>14</v>
@@ -6699,12 +6699,12 @@
       </c>
       <c r="K76" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L76" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-09-23 D1: verris-lve.sh node_capacity (nproc, MemTotal, df /) w każdym raporcie, lve-agent/1.1; telemetry.dto NodeStatusDto.totalCpuCores/totalMemoryMb/totalDiskMb; telemetry.service aktualizuje Server; test telemetry/pojemnosc-wezla.spec.ts</t>
         </is>
       </c>
       <c r="M76" s="11" t="inlineStr">
@@ -6714,12 +6714,12 @@
       </c>
       <c r="N76" s="11" t="inlineStr">
         <is>
-          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O76" s="11" t="inlineStr">
         <is>
-          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Pojemność węzła nigdy się nie odświeża. `totalCpuCores`/`totalMemoryMb`/`totalDiskMb` ustawiane wyłącznie w handshake; telemetria ich nie aktualizuje — mimo komentarza w schemacie „reported via handshake / heartbeat”. Rozbudowa węzła nie dociera do `NodeSelector`. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Telemetria aktualizuje totalCpuCores/totalMemoryMb/totalDiskMb, nie tylko handshake. | Stary agent bez pól niczego nie zeruje. OTWARTE do D3 (PB-21): raport z agenta na żywym węźle i odświeżona pojemność w panelu admina. | 2026-09-25: pojemność z agenta trafia też do planera pojemności (admin → Product Ops): ryzyko liczone względem rdzeni i RAM węzła (CPU 2×/4× rdzeni, RAM 1×/1,5×; test ryzyko-pojemnosci.spec.ts), a opis „CPU 250%” zastąpiony „przydzielone limity: CPU 2,5 rdz. z N · RAM x z y GB” — wcześniej wyglądało jak zużycie ponad 100%.</t>
         </is>
       </c>
       <c r="P76" s="10" t="inlineStr">
@@ -6731,12 +6731,12 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>PB-27</t>
+          <t>PB-08</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
+          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -6751,11 +6751,11 @@
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F77" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G77" s="10" t="n">
         <v>14</v>
@@ -6792,12 +6792,12 @@
       </c>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
+          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
         </is>
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr">
@@ -6809,12 +6809,12 @@
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>PB-28</t>
+          <t>PB-27</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>Rozliczenie poza Verris (całe konto)</t>
+          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
@@ -6833,7 +6833,7 @@
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G78" s="10" t="n">
         <v>14</v>
@@ -6870,12 +6870,12 @@
       </c>
       <c r="N78" s="11" t="inlineStr">
         <is>
-          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
+          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
         </is>
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr">
@@ -6887,58 +6887,58 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>X-41</t>
+          <t>PB-28</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
+          <t>Rozliczenie poza Verris (całe konto)</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G79" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H79" s="10" t="inlineStr">
         <is>
-          <t>Faza 3 — Wejście na rynek</t>
+          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
         </is>
       </c>
       <c r="I79" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J79" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K79" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L79" s="11" t="inlineStr">
         <is>
-          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M79" s="11" t="inlineStr">
@@ -6948,12 +6948,12 @@
       </c>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
         </is>
       </c>
       <c r="O79" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
+          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P79" s="10" t="inlineStr">
@@ -6965,12 +6965,12 @@
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>X-41</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
+          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E80" s="10" t="inlineStr">
@@ -7016,7 +7016,7 @@
       </c>
       <c r="L80" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
+          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
         </is>
       </c>
       <c r="M80" s="11" t="inlineStr">
@@ -7031,7 +7031,7 @@
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr">
@@ -7043,31 +7043,31 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>PB-22</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
+          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G81" s="10" t="n">
         <v>15</v>
@@ -7089,12 +7089,12 @@
       </c>
       <c r="K81" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L81" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
         </is>
       </c>
       <c r="M81" s="11" t="inlineStr">
@@ -7104,12 +7104,12 @@
       </c>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr">
@@ -7121,34 +7121,34 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>PB-22</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Log egressu jest próbką, nie zapisem</t>
+          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E82" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F82" s="10" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H82" s="10" t="inlineStr">
         <is>
@@ -7157,22 +7157,22 @@
       </c>
       <c r="I82" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="J82" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="K82" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M82" s="11" t="inlineStr">
@@ -7182,12 +7182,12 @@
       </c>
       <c r="N82" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
         </is>
       </c>
       <c r="O82" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
+          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr">
@@ -7199,12 +7199,12 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
+          <t>Log egressu jest próbką, nie zapisem</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
@@ -7245,12 +7245,12 @@
       </c>
       <c r="K83" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M83" s="11" t="inlineStr">
@@ -7260,12 +7260,12 @@
       </c>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O83" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr">
@@ -7277,12 +7277,12 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Tryb `--strict` jest atrapą</t>
+          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -7301,7 +7301,7 @@
         </is>
       </c>
       <c r="F84" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G84" s="10" t="n">
         <v>16</v>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
+          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="O84" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr">
@@ -7355,12 +7355,12 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
+          <t>Tryb `--strict` jest atrapą</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -7401,12 +7401,12 @@
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
-          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
+          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
         </is>
       </c>
       <c r="M85" s="11" t="inlineStr">
@@ -7416,12 +7416,12 @@
       </c>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O85" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr">
@@ -7433,12 +7433,12 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
+          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -7453,11 +7453,11 @@
       </c>
       <c r="E86" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F86" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G86" s="10" t="n">
         <v>16</v>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
+          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr">
@@ -7499,7 +7499,7 @@
       </c>
       <c r="O86" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr">
@@ -7511,31 +7511,31 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>PB-23</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
+          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F87" s="10" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G87" s="10" t="n">
         <v>16</v>
@@ -7557,12 +7557,12 @@
       </c>
       <c r="K87" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L87" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
         </is>
       </c>
       <c r="M87" s="11" t="inlineStr">
@@ -7572,12 +7572,12 @@
       </c>
       <c r="N87" s="11" t="inlineStr">
         <is>
-          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O87" s="11" t="inlineStr">
         <is>
-          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr">
@@ -7589,34 +7589,34 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>PB-23</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Podpisane DPA z subprocesorami (część)</t>
+          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G88" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H88" s="10" t="inlineStr">
         <is>
@@ -7625,22 +7625,22 @@
       </c>
       <c r="I88" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="J88" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="K88" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M88" s="11" t="inlineStr">
@@ -7650,12 +7650,12 @@
       </c>
       <c r="N88" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
         </is>
       </c>
       <c r="O88" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
+          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr">
@@ -7667,31 +7667,31 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>PB-03</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Finalizacja dokumentów prawnych 1.0.0</t>
+          <t>Podpisane DPA z subprocesorami (część)</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G89" s="10" t="n">
         <v>17</v>
@@ -7713,12 +7713,12 @@
       </c>
       <c r="K89" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L89" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
         </is>
       </c>
       <c r="M89" s="11" t="inlineStr">
@@ -7728,12 +7728,12 @@
       </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O89" s="11" t="inlineStr">
         <is>
-          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr">
@@ -7745,12 +7745,12 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>PB-04</t>
+          <t>PB-03</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
+          <t>Finalizacja dokumentów prawnych 1.0.0</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -7765,11 +7765,11 @@
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>17</v>
@@ -7806,12 +7806,12 @@
       </c>
       <c r="N90" s="11" t="inlineStr">
         <is>
-          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
+          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
         </is>
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
+          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7823,34 +7823,34 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>N-16</t>
+          <t>PB-04</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>SLA z zapisanymi kredytami</t>
+          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G91" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H91" s="10" t="inlineStr">
         <is>
@@ -7859,37 +7859,37 @@
       </c>
       <c r="I91" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-21</t>
         </is>
       </c>
       <c r="J91" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="K91" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L91" s="11" t="inlineStr">
         <is>
-          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M91" s="11" t="inlineStr">
         <is>
-          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
+          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7901,12 +7901,12 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>N-16</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>SLA z zapisanymi kredytami</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
@@ -7947,27 +7947,27 @@
       </c>
       <c r="K92" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L92" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
         </is>
       </c>
       <c r="M92" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
         </is>
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7979,31 +7979,31 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>PB-07</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>Treści i cennik na verris.pl</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G93" s="10" t="n">
         <v>18</v>
@@ -8025,27 +8025,27 @@
       </c>
       <c r="K93" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L93" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M93" s="11" t="inlineStr">
         <is>
-          <t>PB-01 (cennik zależy od unit economics)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8057,12 +8057,12 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>PB-11</t>
+          <t>PB-07</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
+          <t>Treści i cennik na verris.pl</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8081,7 +8081,7 @@
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>18</v>
@@ -8113,17 +8113,17 @@
       </c>
       <c r="M94" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-01 (cennik zależy od unit economics)</t>
         </is>
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
+          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
+          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8135,12 +8135,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>PB-21</t>
+          <t>PB-11</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>DNS platformy i poczty na serwerze testowym</t>
+          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8159,7 +8159,7 @@
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G95" s="10" t="n">
         <v>18</v>
@@ -8196,12 +8196,12 @@
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
+          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
+          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,12 +8213,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>PB-24</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8237,7 +8237,7 @@
         </is>
       </c>
       <c r="F96" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G96" s="10" t="n">
         <v>18</v>
@@ -8274,12 +8274,12 @@
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,12 +8291,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-25</t>
+          <t>PB-24</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>White label na węźle — klient nie widzi DirectAdmina</t>
+          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8315,7 +8315,7 @@
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>18</v>
@@ -8352,12 +8352,12 @@
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
+          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
+          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8369,12 +8369,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-25</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>White label na węźle — klient nie widzi DirectAdmina</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8393,10 +8393,10 @@
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G98" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H98" s="10" t="inlineStr">
         <is>
@@ -8405,12 +8405,12 @@
       </c>
       <c r="I98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K98" s="10" t="inlineStr">
@@ -8425,17 +8425,17 @@
       </c>
       <c r="M98" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
+          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8447,12 +8447,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
@@ -8503,17 +8503,17 @@
       </c>
       <c r="M99" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8525,12 +8525,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8549,7 +8549,7 @@
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G100" s="10" t="n">
         <v>19</v>
@@ -8586,12 +8586,12 @@
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8603,12 +8603,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8627,20 +8627,24 @@
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G101" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H101" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H101" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I101" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J101" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K101" s="10" t="inlineStr">
@@ -8655,17 +8659,17 @@
       </c>
       <c r="M101" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8677,69 +8681,69 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G102" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H102" s="10" t="inlineStr"/>
       <c r="I102" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J102" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K102" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L102" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M102" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8751,12 +8755,12 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8766,16 +8770,16 @@
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G103" s="10" t="n">
         <v>21</v>
@@ -8798,7 +8802,7 @@
       </c>
       <c r="L103" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M103" s="11" t="inlineStr">
@@ -8813,7 +8817,7 @@
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8825,12 +8829,12 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
@@ -8840,7 +8844,7 @@
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E104" s="10" t="inlineStr">
@@ -8867,12 +8871,12 @@
       </c>
       <c r="K104" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L104" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M104" s="11" t="inlineStr">
@@ -8882,12 +8886,12 @@
       </c>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8899,12 +8903,12 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -8919,7 +8923,7 @@
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F105" s="10" t="n">
@@ -8946,7 +8950,7 @@
       </c>
       <c r="L105" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M105" s="11" t="inlineStr">
@@ -8961,7 +8965,7 @@
       </c>
       <c r="O105" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr">
@@ -8973,12 +8977,12 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -8988,12 +8992,12 @@
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F106" s="10" t="n">
@@ -9015,12 +9019,12 @@
       </c>
       <c r="K106" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L106" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M106" s="11" t="inlineStr">
@@ -9030,12 +9034,12 @@
       </c>
       <c r="N106" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O106" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr">
@@ -9047,31 +9051,31 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F107" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G107" s="10" t="n">
         <v>21</v>
@@ -9089,12 +9093,12 @@
       </c>
       <c r="K107" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L107" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>services.controller.ts:125</t>
         </is>
       </c>
       <c r="M107" s="11" t="inlineStr">
@@ -9104,12 +9108,12 @@
       </c>
       <c r="N107" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O107" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr">
@@ -9121,12 +9125,12 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>PB-29</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -9141,11 +9145,11 @@
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>KRYTYCZNY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F108" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G108" s="10" t="n">
         <v>21</v>
@@ -9178,12 +9182,12 @@
       </c>
       <c r="N108" s="11" t="inlineStr">
         <is>
-          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O108" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr">
@@ -9195,12 +9199,12 @@
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>PB-30</t>
+          <t>PB-29</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>Jeden plik wersji dla floty + test zgodności</t>
+          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
         </is>
       </c>
       <c r="C109" s="10" t="inlineStr">
@@ -9215,7 +9219,7 @@
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F109" s="10" t="n">
@@ -9252,12 +9256,12 @@
       </c>
       <c r="N109" s="11" t="inlineStr">
         <is>
-          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
+          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="O109" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
+          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr">
@@ -9269,12 +9273,12 @@
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>PB-31</t>
+          <t>PB-30</t>
         </is>
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>Pełna automatyzacja kreatora węzła</t>
+          <t>Jeden plik wersji dla floty + test zgodności</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
@@ -9293,7 +9297,7 @@
         </is>
       </c>
       <c r="F110" s="10" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G110" s="10" t="n">
         <v>21</v>
@@ -9326,12 +9330,12 @@
       </c>
       <c r="N110" s="11" t="inlineStr">
         <is>
-          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
+          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
         </is>
       </c>
       <c r="O110" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
+          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr">
@@ -9343,12 +9347,12 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>PB-32</t>
+          <t>PB-31</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Aktualizacje węzłów falami</t>
+          <t>Pełna automatyzacja kreatora węzła</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
@@ -9363,11 +9367,11 @@
       </c>
       <c r="E111" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F111" s="10" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G111" s="10" t="n">
         <v>21</v>
@@ -9400,12 +9404,12 @@
       </c>
       <c r="N111" s="11" t="inlineStr">
         <is>
-          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
+          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
         </is>
       </c>
       <c r="O111" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
+          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr">
@@ -9417,12 +9421,12 @@
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>PB-26</t>
+          <t>PB-32</t>
         </is>
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
-          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
+          <t>Aktualizacje węzłów falami</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -9437,24 +9441,24 @@
       </c>
       <c r="E112" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F112" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G112" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H112" s="10" t="inlineStr"/>
       <c r="I112" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J112" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K112" s="10" t="inlineStr">
@@ -9474,12 +9478,12 @@
       </c>
       <c r="N112" s="11" t="inlineStr">
         <is>
-          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
+          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
         </is>
       </c>
       <c r="O112" s="11" t="inlineStr">
         <is>
-          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
+          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
         </is>
       </c>
       <c r="P112" s="10" t="inlineStr">
@@ -9491,12 +9495,12 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-33</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Wersje stosu floty w panelu + wyrównanie falą</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
@@ -9511,24 +9515,24 @@
       </c>
       <c r="E113" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F113" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G113" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H113" s="10" t="inlineStr"/>
       <c r="I113" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J113" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K113" s="10" t="inlineStr">
@@ -9543,17 +9547,17 @@
       </c>
       <c r="M113" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N113" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Zmiana wersji w panelu → nowy węzeł instaluje ją, istniejące wyrównane falą; audyt zgodności zielony.</t>
         </is>
       </c>
       <c r="O113" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Decyzja właściciela 2026-09-26: strona „Wersje stosu floty” w panelu admina (DB, PHP, LiteSpeed, DirectAdmin) z dozwolonymi wartościami z oficjalnych list; zmiana obowiązuje nowe węzły od razu, „Wyrównaj flotę” aktualizuje istniejące falą (PHP/LiteSpeed przez CustomBuild, MariaDB po jednej wersji z kopią bazy — wymóg CloudLinux Governor). | 2026-09-26 ZROBIONE W KODZIE: manifest w bazie (StosWezlaService), strona Admin → Wersje stosu floty (dozwolone wartości z oficjalnych list, tabela zgodności), „Wyrównaj flotę” = fala z php1_release + łańcuch DB_UPGRADE krok po kroku z kopią; bootstrap i agent biorą manifest z bazy. Testy na PostgreSQL. Zostało: wyrównanie na węzłach (D3).</t>
         </is>
       </c>
       <c r="P113" s="10" t="inlineStr">
@@ -9565,12 +9569,12 @@
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-35</t>
         </is>
       </c>
       <c r="B114" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Automatyczna fala aktualizacji węzłów co tydzień</t>
         </is>
       </c>
       <c r="C114" s="10" t="inlineStr">
@@ -9585,60 +9589,356 @@
       </c>
       <c r="E114" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F114" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G114" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H114" s="10" t="inlineStr"/>
       <c r="I114" s="10" t="inlineStr">
         <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="J114" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-22</t>
+        </is>
+      </c>
+      <c r="K114" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L114" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M114" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N114" s="11" t="inlineStr">
+        <is>
+          <t>Fala startuje sama w oknie; zatrzymanie widoczne w powiadomieniach admina.</t>
+        </is>
+      </c>
+      <c r="O114" s="11" t="inlineStr">
+        <is>
+          <t>Decyzja właściciela 2026-09-26: fala rusza sama we wtorki o 4:00 (kanarek → reszta po jednym, błąd zatrzymuje, powiadomienie). Węzły same już niczego nie instalują (dnf-automatic tylko pobiera). | 2026-09-26 ZROBIONE W KODZIE: FalaTygodniowaScheduler (wtorek 4:00 Europe/Warsaw), zatrzymanie fali → powiadomienie adminów. Test na PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="P114" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>PB-36</t>
+        </is>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>Podpisane skrypty węzła i klucz SSH ograniczony do control-plane</t>
+        </is>
+      </c>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D115" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E115" s="10" t="inlineStr">
+        <is>
+          <t>KRYTYCZNY</t>
+        </is>
+      </c>
+      <c r="F115" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G115" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="H115" s="10" t="inlineStr"/>
+      <c r="I115" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="J115" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-22</t>
+        </is>
+      </c>
+      <c r="K115" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L115" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M115" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N115" s="11" t="inlineStr">
+        <is>
+          <t>Niepodpisany/zmieniony skrypt odrzucony przez węzeł; authorized_keys zawiera tylko aktualny klucz z ograniczeniem IP.</t>
+        </is>
+      </c>
+      <c r="O115" s="11" t="inlineStr">
+        <is>
+          <t>Decyzja właściciela 2026-09-26: przed startem. Węzeł uruchamia tylko skrypty podpisane kluczem Verris (przejęte API nie daje roota na flocie); klucz SSH z from= na IP control-plane, stare klucze usuwane (dziś agent co minutę tylko dopisuje klucz). | 2026-09-26 ZROBIONE W KODZIE: podpis Ed25519 każdej odpowiedzi GET /agent/tasks/* (skrypty zadań, pakiety onboardu i strony domyślnej, manifest stosu, konfiguracja kopii, zlecenia, klucz deploy) — podpis obejmuje ścieżkę, id węzła, czas i SHA-256 treści (bez podmiany, przeniesienia na inną ścieżkę/węzeł, powtórki po 5 min). Węzeł pobiera wyłącznie przez /usr/local/bin/verris-fetch (openssl pkeyutl -verify), klucz publiczny przywozi bootstrap / instalacja agenta. Klucz deploy: jeden wpis from="VERRIS_CONTROL_PLANE_IPS" bez przekierowań, poprzedni usuwany (rotacja). API w produkcji nie wystartuje bez VERRIS_SCRIPT_SIGNING_KEY albo z kluczem deploy bez adresów control-plane. Test: prawdziwy verris-fetch vs serwer podpisujący (zmieniona treść / inna ścieżka / inny węzeł / stary podpis / brak podpisu → odrzucone) + smoke na lokalnym API. Do sprawdzenia na D3: openssl na CloudLinux 9, rotacja klucza deploy.</t>
+        </is>
+      </c>
+      <c r="P115" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t>PB-26</t>
+        </is>
+      </c>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
+        </is>
+      </c>
+      <c r="C116" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E116" s="10" t="inlineStr">
+        <is>
+          <t>WYSOKI</t>
+        </is>
+      </c>
+      <c r="F116" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="G116" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H116" s="10" t="inlineStr"/>
+      <c r="I116" s="10" t="inlineStr">
+        <is>
           <t>2027-01-25</t>
         </is>
       </c>
-      <c r="J114" s="10" t="inlineStr">
+      <c r="J116" s="10" t="inlineStr">
         <is>
           <t>2027-01-29</t>
         </is>
       </c>
-      <c r="K114" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L114" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M114" s="11" t="inlineStr">
+      <c r="K116" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L116" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M116" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N116" s="11" t="inlineStr">
+        <is>
+          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
+        </is>
+      </c>
+      <c r="O116" s="11" t="inlineStr">
+        <is>
+          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
+        </is>
+      </c>
+      <c r="P116" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t>PB-05</t>
+        </is>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>Test end-to-end „pierwszy klient”</t>
+        </is>
+      </c>
+      <c r="C117" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E117" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F117" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="G117" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H117" s="10" t="inlineStr"/>
+      <c r="I117" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J117" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K117" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L117" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M117" s="11" t="inlineStr">
+        <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N117" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O117" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P117" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B118" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G118" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H118" s="10" t="inlineStr"/>
+      <c r="I118" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J118" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K118" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L118" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M118" s="11" t="inlineStr">
         <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N114" s="11" t="inlineStr">
+      <c r="N118" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O114" s="11" t="inlineStr">
+      <c r="O118" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P114" s="10" t="inlineStr">
+      <c r="P118" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P114"/>
-  <conditionalFormatting sqref="E2:E114">
+  <autoFilter ref="A1:P118"/>
+  <conditionalFormatting sqref="E2:E118">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -9658,7 +9958,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P114">
+  <conditionalFormatting sqref="P2:P118">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -9768,11 +10068,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A2,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A2,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -9813,11 +10113,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A3,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A3,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -9858,11 +10158,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A4,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A4,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -9903,11 +10203,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A5,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A5,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -9948,11 +10248,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A6,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A6,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -9993,11 +10293,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A7,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A7,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -10038,11 +10338,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A8,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A8,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -10083,11 +10383,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A9,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A9,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -10128,11 +10428,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A10,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A10,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -10173,11 +10473,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A11,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A11,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -10218,11 +10518,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A12,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A12,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -10263,11 +10563,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A13,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A13,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -10308,11 +10608,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A14,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A14,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -10353,11 +10653,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A15,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A15,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -10398,11 +10698,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A16,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A16,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -10443,11 +10743,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A17,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A17,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -10488,11 +10788,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A18,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A18,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -10533,11 +10833,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A19,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A19,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -10578,11 +10878,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A20,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A20,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -10619,11 +10919,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A21,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A21,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -10660,11 +10960,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A22,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A22,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -10701,11 +11001,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A23,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A23,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">
@@ -10742,11 +11042,11 @@
         </is>
       </c>
       <c r="F24" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$114,A24)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A24)</f>
         <v/>
       </c>
       <c r="G24" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$114,A24,'Backlog do startu'!$F$2:$F$114)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A24,'Backlog do startu'!$F$2:$F$118)</f>
         <v/>
       </c>
       <c r="H24" s="10" t="n">

</xml_diff>

<commit_message>
chore(audyt): tablice po PB-37
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$119</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$22</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$118)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$119)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$118,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$118,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$119,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$119,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$118,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$119,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$118,"zrobione",'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$119,"zrobione",'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P118"/>
+  <dimension ref="A1:P119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4847,7 +4847,7 @@
       </c>
       <c r="O52" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: najpierw makieta 3–4 kluczowych ekranów (pulpit, węzły/węzeł, karta klienta, zgłoszenie) do akceptacji, potem przeniesienie wszystkich ekranów 1:1 na tokeny i komponenty v2 (jasny i ciemny motyw). DEV_HANDOFF.md przewidywał „ten sam zestaw tokenów, później”.</t>
+          <t>Decyzja właściciela 2026-09-26: najpierw makieta 3–4 kluczowych ekranów (pulpit, węzły/węzeł, karta klienta, zgłoszenie) do akceptacji, potem przeniesienie wszystkich ekranów 1:1 na tokeny i komponenty v2 (jasny i ciemny motyw). DEV_HANDOFF.md przewidywał „ten sam zestaw tokenów, później”. | 2026-09-26: makieta zaakceptowana (właściciel: „wyglądają super”, dodać podpowiedzi na zgłoszeniu — zrobione jako PB-37). PANEL OBSŁUGI PRZENIESIONY: menu i pasek 1:1 z makietą (ciemne menu, jasna treść, przełącznik motywu, menu na telefonie), skrzynka od nowa (Moje, Czeka na klienta, terminy), zgłoszenie 1:1 z makietą; pozostałe ekrany obsługi na tokenach v2 przez warstwę .v2-skin (jak PB-16). ZOSTAJE: panel admina (pulpit, węzeł, karta klienta 1:1 z makietą + reszta ekranów).</t>
         </is>
       </c>
       <c r="P52" s="10" t="inlineStr">
@@ -4859,34 +4859,34 @@
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>PB-37</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Rekordy SPF — kreator</t>
+          <t>Opieka nad zgłoszeniem: podpowiedzi dla obsługi, automatyczne wiadomości, oceny opiekuna</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F53" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G53" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
@@ -4895,22 +4895,22 @@
       </c>
       <c r="I53" s="10" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J53" s="10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K53" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L53" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: deliverability/mail-auth.ts (buildMailAuthChecks) + deliverability.service.ts (strefa DA + delegacja NS); UI app/dashboard/email/deliverability-panel.tsx podpięty w MailTab (zakładka Poczta); test mail-auth.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M53" s="11" t="inlineStr">
@@ -4920,12 +4920,12 @@
       </c>
       <c r="N53" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Klient dostaje potwierdzenie z opiekunem i terminem, widzi „przeczytane” i postęp; po zamknięciu ocenia opiekuna i obsługę; obsługa ma szkic i szablony w jednym bloku.</t>
         </is>
       </c>
       <c r="O53" s="11" t="inlineStr">
         <is>
-          <t>deliverability-panel.tsx:26 to komponent osierocony — nikt go nie importuje | KOD: kreator pokazuje stan z publicznego DNS i gotowy rekord — „Dodaj/Zamień rekord w DNS” gdy domena na NS Verris, inaczej do skopiowania u dostawcy DNS. Zalecany SPF to `v=spf1 a mx ip4:&lt;IP węzła&gt; ~all`. ZNALEZISKO: dotychczasowa podpowiedź include:_spf.verris.pl odwołuje się do nieistniejącego rekordu (NXDOMAIN) → SPF permerror; usunięta z podpowiedzi, presetu DNS i artykułów KB, a kreator wykrywa ją u klientów. OTWARTE do D3 (węzeł): zapis rekordu przez CMD_API_DNS_CONTROL.</t>
+          <t>Decyzja właściciela 2026-09-26 (formularz): cztery automatyczne wiadomości (potwierdzenie z opiekunem i terminem, „opiekun się tym zajmuje”, „wciąż nad tym pracujemy” po połowie czasu odpowiedzi najwyżej raz na dobę, podziękowanie z oceną), ocena opiekuna + obsługi ogólnie + „czy rozwiązane”, szkic asystenta gotowy sam przy otwarciu. | 2026-09-26 ZROBIONE W KODZIE: OpiekaZgloszenService (treści w platform_settings, edycja: Admin → Opieka nad zgłoszeniami), wiadomości jako wpis w wątku + e-mail, NIE liczą się jako odpowiedź (SLA, stan, metryki czasu odpowiedzi bez zmian); „przeczytane” (otwarcie przez opiekuna), ponowne otwarcie do 7 dni, szkic asystenta w tle po każdej wiadomości klienta; obsługa: blok Podpowiedzi (szkic / szablony wg sytuacji / baza wiedzy, /skrót w polu odpowiedzi), „Co widzi klient”, „Twoje oceny”, „Wyślij” vs „Wyślij i czekaj na klienta”; klient: postęp (przyjęte → opiekun → przeczytane → odpowiedź → rozwiązane), opiekun z imienia, ocena i ponowne otwarcie; szablony z kategorią i skrótem (seed + formularz admina). Testy na PostgreSQL (5). Panel klienta nie widzi już notatek wewnętrznych obsługi (ryzyko, eskalacja, szkic, id pracowników).</t>
         </is>
       </c>
       <c r="P53" s="10" t="inlineStr">
@@ -4937,12 +4937,12 @@
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>E-16</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>Rekordy DKIM — konfiguracja</t>
+          <t>Rekordy SPF — kreator</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -4988,12 +4988,12 @@
       </c>
       <c r="L54" s="11" t="inlineStr">
         <is>
-          <t>deliverability/mail-auth.ts (akcja enable-dkim); servers/directadmin.service.ts enableHostingDkim; POST /services/:id/hosting-email/dkim; email/deliverability-panel.tsx; testy mail-auth.spec.ts, directadmin.narzedzia.spec.ts</t>
+          <t>2026-09-23 D1: deliverability/mail-auth.ts (buildMailAuthChecks) + deliverability.service.ts (strefa DA + delegacja NS); UI app/dashboard/email/deliverability-panel.tsx podpięty w MailTab (zakładka Poczta); test mail-auth.spec.ts</t>
         </is>
       </c>
       <c r="M54" s="11" t="inlineStr">
         <is>
-          <t>E-15 (ten sam panel dostarczalności)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N54" s="11" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="O54" s="11" t="inlineStr">
         <is>
-          <t>j.w. | KOD: DKIM odczytywany ze strefy DA (DA dopisuje klucz sam przy włączonym DKIM). Brak klucza = link do zgłoszenia. OTWARTE: włączanie DKIM z panelu (komenda DA niepotwierdzona bez węzła) — D3 w sprincie 18. | 2026-09-25: KOD (D2) — „Włącz DKIM dla &lt;domena&gt;” w sekcji Dostarczalność zamiast „napisz zgłoszenie”. Komenda DA potwierdzona w dokumentacji (changelog 1.57.2): CMD_API_EMAIL_POP action=set_dkim&amp;domain=…&amp;enable=… — DA tworzy klucze i dopisuje rekord TXT do strefy. Tylko domena z konta usługi, konto zawieszone bez zmian, wpis w dzienniku (HOSTING_DKIM_ENABLED). Wyłączenia celowo brak: ponowne włączenie generuje nowe klucze i rekord u zewnętrznego DNS przestałby pasować. Przy DNS u innego dostawcy panel po włączeniu pokazuje rekord do skopiowania (istniejąca ścieżka „klucz w strefie”). D3: pierwsze włączenie na węźle. | 2026-09-25 (dokumentacja DirectAdmin „Exim → DKIM”): dkim=2 udostępnia włączanie DKIM użytkownikom per domena, dkim=1 generuje klucze automatycznie przy tworzeniu domeny (tylko gdy DNS jest lokalny). Profil węzła ustawia dkim=1 — przycisk w panelu pojawia się tylko dla domen bez klucza. D3 ma potwierdzić, że set_dkim działa przy dkim=1; jeśli nie — alternatywa z dokumentacji: scripts/dkim_create.sh &lt;domena&gt; po stronie węzła (zadanie agenta).</t>
+          <t>deliverability-panel.tsx:26 to komponent osierocony — nikt go nie importuje | KOD: kreator pokazuje stan z publicznego DNS i gotowy rekord — „Dodaj/Zamień rekord w DNS” gdy domena na NS Verris, inaczej do skopiowania u dostawcy DNS. Zalecany SPF to `v=spf1 a mx ip4:&lt;IP węzła&gt; ~all`. ZNALEZISKO: dotychczasowa podpowiedź include:_spf.verris.pl odwołuje się do nieistniejącego rekordu (NXDOMAIN) → SPF permerror; usunięta z podpowiedzi, presetu DNS i artykułów KB, a kreator wykrywa ją u klientów. OTWARTE do D3 (węzeł): zapis rekordu przez CMD_API_DNS_CONTROL.</t>
         </is>
       </c>
       <c r="P54" s="10" t="inlineStr">
@@ -5015,12 +5015,12 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>E-17</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Rekord DMARC — konfiguracja</t>
+          <t>Rekordy DKIM — konfiguracja</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -5066,12 +5066,12 @@
       </c>
       <c r="L55" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: mail-auth.ts dmarcCheck (brak / p=none / kilka rekordów) + lib/dmarc.ts tuneDmarc (polityka + adres raportów) w deliverability-panel.tsx; testy mail-auth.spec.ts, dmarc.spec.ts</t>
+          <t>deliverability/mail-auth.ts (akcja enable-dkim); servers/directadmin.service.ts enableHostingDkim; POST /services/:id/hosting-email/dkim; email/deliverability-panel.tsx; testy mail-auth.spec.ts, directadmin.narzedzia.spec.ts</t>
         </is>
       </c>
       <c r="M55" s="11" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>E-15 (ten sam panel dostarczalności)</t>
         </is>
       </c>
       <c r="N55" s="11" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O55" s="11" t="inlineStr">
         <is>
-          <t>j.w. | KOD: kreator DMARC — wybór polityki i opcjonalny adres raportów, zachowuje pozostałe tagi. Sugestia bez rua na verris.pl (raporty do obcej domeny wymagają rekordu autoryzacji). OTWARTE do D3: zapis do strefy DA.</t>
+          <t>j.w. | KOD: DKIM odczytywany ze strefy DA (DA dopisuje klucz sam przy włączonym DKIM). Brak klucza = link do zgłoszenia. OTWARTE: włączanie DKIM z panelu (komenda DA niepotwierdzona bez węzła) — D3 w sprincie 18. | 2026-09-25: KOD (D2) — „Włącz DKIM dla &lt;domena&gt;” w sekcji Dostarczalność zamiast „napisz zgłoszenie”. Komenda DA potwierdzona w dokumentacji (changelog 1.57.2): CMD_API_EMAIL_POP action=set_dkim&amp;domain=…&amp;enable=… — DA tworzy klucze i dopisuje rekord TXT do strefy. Tylko domena z konta usługi, konto zawieszone bez zmian, wpis w dzienniku (HOSTING_DKIM_ENABLED). Wyłączenia celowo brak: ponowne włączenie generuje nowe klucze i rekord u zewnętrznego DNS przestałby pasować. Przy DNS u innego dostawcy panel po włączeniu pokazuje rekord do skopiowania (istniejąca ścieżka „klucz w strefie”). D3: pierwsze włączenie na węźle. | 2026-09-25 (dokumentacja DirectAdmin „Exim → DKIM”): dkim=2 udostępnia włączanie DKIM użytkownikom per domena, dkim=1 generuje klucze automatycznie przy tworzeniu domeny (tylko gdy DNS jest lokalny). Profil węzła ustawia dkim=1 — przycisk w panelu pojawia się tylko dla domen bez klucza. D3 ma potwierdzić, że set_dkim działa przy dkim=1; jeśli nie — alternatywa z dokumentacji: scripts/dkim_create.sh &lt;domena&gt; po stronie węzła (zadanie agenta).</t>
         </is>
       </c>
       <c r="P55" s="10" t="inlineStr">
@@ -5093,12 +5093,12 @@
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>E-05</t>
+          <t>E-17</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>Zmiana quoty ISTNIEJĄCEJ skrzynki</t>
+          <t>Rekord DMARC — konfiguracja</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -5144,12 +5144,12 @@
       </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/hosting-email/quota (ZmienRozmiarSkrzynkiDto 10–102400 MB) → directadmin.service changeHostingEmailQuota (CMD_API_POP action=modify bez passwd) + audyt HOSTING_EMAIL_QUOTA_CHANGED; UI MailTab — klik w rozmiar skrzynki</t>
+          <t>2026-09-23 D1: mail-auth.ts dmarcCheck (brak / p=none / kilka rekordów) + lib/dmarc.ts tuneDmarc (polityka + adres raportów) w deliverability-panel.tsx; testy mail-auth.spec.ts, dmarc.spec.ts</t>
         </is>
       </c>
       <c r="M56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="N56" s="11" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="O56" s="11" t="inlineStr">
         <is>
-          <t>brak jakiejkolwiek ścieżki edycji — klient musi usunąć i odtworzyć skrzynkę | KOD: zmiana rozmiaru bez usuwania skrzynki. Przy okazji body tworzenia skrzynki i zmiany hasła dostały klasy DTO (wcześniej interfejs = zero walidacji na granicy zaufania). OTWARTE do D3: czy DA przy modify bez passwd zostawia hasło (komentarz ponytail).</t>
+          <t>j.w. | KOD: kreator DMARC — wybór polityki i opcjonalny adres raportów, zachowuje pozostałe tagi. Sugestia bez rua na verris.pl (raporty do obcej domeny wymagają rekordu autoryzacji). OTWARTE do D3: zapis do strefy DA.</t>
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr">
@@ -5171,12 +5171,12 @@
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>M-26</t>
+          <t>E-05</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Usunięcie zapisanej karty przez klienta</t>
+          <t>Zmiana quoty ISTNIEJĄCEJ skrzynki</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
@@ -5217,12 +5217,12 @@
       </c>
       <c r="K57" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L57" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: DELETE /billing/payment-methods/:id (ParseUUIDPipe) → billing.service deleteMyPaymentMethod: Stripe detach, usunięcie wiersza, zerowanie karty domyślnej i auto-doładowania, audyt PAYMENT_METHOD_REMOVED; UI billing-extras-forms „Zapisane karty”; test usun-karte.spec.ts | 2026-09-23: zapis kart — billing.service handlePaymentMethodAttached/Detached (webhooki payment_method.attached/.detached, upsert po provider+providerRef, pierwsza karta domyślna); test D2 zapis-karty.spec.ts</t>
+          <t>2026-09-23 D1: POST /services/:id/hosting-email/quota (ZmienRozmiarSkrzynkiDto 10–102400 MB) → directadmin.service changeHostingEmailQuota (CMD_API_POP action=modify bez passwd) + audyt HOSTING_EMAIL_QUOTA_CHANGED; UI MailTab — klik w rozmiar skrzynki</t>
         </is>
       </c>
       <c r="M57" s="11" t="inlineStr">
@@ -5232,12 +5232,12 @@
       </c>
       <c r="N57" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O57" s="11" t="inlineStr">
         <is>
-          <t>wymóg konsumencki | KOD gotowy i przetestowany na atrapach. UWAGA: nic w API nie zapisuje dziś wierszy PaymentMethod (brak create/upsert) — lista kart jest zawsze pusta, więc usuwanie da się sprawdzić dopiero, gdy zapis kart zostanie podpięty (webhook Stripe po płatności kartą). | 2026-09-23: domknięty brakujący zapis — karta zapisana w Stripe (np. przy subskrypcji kartą) pojawia się w panelu, odpięta (także z dashboardu Stripe) znika i odpina się od auto-doładowania. WYMAGA OD WŁAŚCICIELA: dopisać zdarzenia payment_method.attached i payment_method.detached do endpointu webhooka w Stripe (DEPLOY.md, OPERATIONAL_CHECKLIST). Karty zapisane przed tą zmianą nie pojawią się wstecz. D3 przy pierwszej płatności kartą.</t>
+          <t>brak jakiejkolwiek ścieżki edycji — klient musi usunąć i odtworzyć skrzynkę | KOD: zmiana rozmiaru bez usuwania skrzynki. Przy okazji body tworzenia skrzynki i zmiany hasła dostały klasy DTO (wcześniej interfejs = zero walidacji na granicy zaufania). OTWARTE do D3: czy DA przy modify bez passwd zostawia hasło (komentarz ponytail).</t>
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr">
@@ -5249,58 +5249,58 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>PB-17</t>
+          <t>M-26</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Asystent v1: dymki, naprawy jednym kliknięciem, czat z danymi konta</t>
+          <t>Usunięcie zapisanej karty przez klienta</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F58" s="10" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
+          <t>Faza 1 — Rozliczenia i dowód odtworzenia</t>
         </is>
       </c>
       <c r="I58" s="10" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J58" s="10" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K58" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-09-23 D1: DELETE /billing/payment-methods/:id (ParseUUIDPipe) → billing.service deleteMyPaymentMethod: Stripe detach, usunięcie wiersza, zerowanie karty domyślnej i auto-doładowania, audyt PAYMENT_METHOD_REMOVED; UI billing-extras-forms „Zapisane karty”; test usun-karte.spec.ts | 2026-09-23: zapis kart — billing.service handlePaymentMethodAttached/Detached (webhooki payment_method.attached/.detached, upsert po provider+providerRef, pierwsza karta domyślna); test D2 zapis-karty.spec.ts</t>
         </is>
       </c>
       <c r="M58" s="11" t="inlineStr">
@@ -5310,12 +5310,12 @@
       </c>
       <c r="N58" s="11" t="inlineStr">
         <is>
-          <t>Co najmniej 5 reguł dymków z testami; każda naprawa ma cofnięcie i wpis audytu; czat odpowiada z kontekstem usługi; brak akcji destrukcyjnych w v1.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O58" s="11" t="inlineStr">
         <is>
-          <t>Dymki kontekstowe na regułach (bez kosztu AI): dysk, domena nie wskazuje na nas, SPF/DKIM, SSL wygasa, backup nieświeży — najwyżej jeden na ekran, „nie pokazuj więcej”. Naprawy jednym kliknięciem tylko dla akcji odwracalnych, z kartą podglądu skutku i „Cofnij”. Obecny czat (HostingAssistant, RAG) dostaje odczyt danych konta. Każda akcja w audycie. Diagnoza i naprawy po naszej stronie za darmo.</t>
+          <t>wymóg konsumencki | KOD gotowy i przetestowany na atrapach. UWAGA: nic w API nie zapisuje dziś wierszy PaymentMethod (brak create/upsert) — lista kart jest zawsze pusta, więc usuwanie da się sprawdzić dopiero, gdy zapis kart zostanie podpięty (webhook Stripe po płatności kartą). | 2026-09-23: domknięty brakujący zapis — karta zapisana w Stripe (np. przy subskrypcji kartą) pojawia się w panelu, odpięta (także z dashboardu Stripe) znika i odpina się od auto-doładowania. WYMAGA OD WŁAŚCICIELA: dopisać zdarzenia payment_method.attached i payment_method.detached do endpointu webhooka w Stripe (DEPLOY.md, OPERATIONAL_CHECKLIST). Karty zapisane przed tą zmianą nie pojawią się wstecz. D3 przy pierwszej płatności kartą.</t>
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr">
@@ -5327,12 +5327,12 @@
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>PB-18</t>
+          <t>PB-17</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>Tickety v2: podgląd klienta, szablony ze zmiennymi, szkice odpowiedzi</t>
+          <t>Asystent v1: dymki, naprawy jednym kliknięciem, czat z danymi konta</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -5351,10 +5351,10 @@
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G59" s="10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
@@ -5363,12 +5363,12 @@
       </c>
       <c r="I59" s="10" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="J59" s="10" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K59" s="10" t="inlineStr">
@@ -5388,12 +5388,12 @@
       </c>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>Podgląd klienta bez przechodzenia między ekranami; szablony podstawiają zmienne z testem; szkic odpowiedzi dla 6 kategorii (DNS, SSL, poczta, płatność, migracja, awaria).</t>
+          <t>Co najmniej 5 reguł dymków z testami; każda naprawa ma cofnięcie i wpis audytu; czat odpowiada z kontekstem usługi; brak akcji destrukcyjnych w v1.</t>
         </is>
       </c>
       <c r="O59" s="11" t="inlineStr">
         <is>
-          <t>Panel staff: boczny podgląd klienta w tickecie (usługi, saldo, faktury/dokumenty, zdarzenia, historia zgłoszeń, health score); szablony odpowiedzi ze zmiennymi (imię, domena, usługa, termin) i kategoriami — rozbudowa canned responses; klasyfikacja zgłoszenia i szkic odpowiedzi z bazy wiedzy i danych konta (do akceptacji, bez auto-wysyłki w v2); akcje z ticketu z audytem; licznik SLA.</t>
+          <t>Dymki kontekstowe na regułach (bez kosztu AI): dysk, domena nie wskazuje na nas, SPF/DKIM, SSL wygasa, backup nieświeży — najwyżej jeden na ekran, „nie pokazuj więcej”. Naprawy jednym kliknięciem tylko dla akcji odwracalnych, z kartą podglądu skutku i „Cofnij”. Obecny czat (HostingAssistant, RAG) dostaje odczyt danych konta. Każda akcja w audycie. Diagnoza i naprawy po naszej stronie za darmo.</t>
         </is>
       </c>
       <c r="P59" s="10" t="inlineStr">
@@ -5405,34 +5405,34 @@
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>A-25</t>
+          <t>PB-18</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>Ręczne zawieszenie usługi przez operatora</t>
+          <t>Tickety v2: podgląd klienta, szablony ze zmiennymi, szkice odpowiedzi</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F60" s="10" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="G60" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
@@ -5441,22 +5441,22 @@
       </c>
       <c r="I60" s="10" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="J60" s="10" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="K60" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L60" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: admin-panel subscriptions/[id]/suspend-form.tsx + suspend-actions.ts → POST /admin/subscriptions/:id/suspend (powód, notatka, potwierdzenie)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M60" s="11" t="inlineStr">
@@ -5466,12 +5466,12 @@
       </c>
       <c r="N60" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Podgląd klienta bez przechodzenia między ekranami; szablony podstawiają zmienne z testem; szkic odpowiedzi dla 6 kategorii (DNS, SSL, poczta, płatność, migracja, awaria).</t>
         </is>
       </c>
       <c r="O60" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: endpoint działa i jest osiągalny (curl + DirectAdmin), auto-suspend za brak płatności działa. Brakuje UI, nie możliwości zatrzymania szkody. | UI zrobione. OTWARTE do D3 (PB-21, serwer testowy): zawieszenie konta w DirectAdminie na żywym węźle.</t>
+          <t>Panel staff: boczny podgląd klienta w tickecie (usługi, saldo, faktury/dokumenty, zdarzenia, historia zgłoszeń, health score); szablony odpowiedzi ze zmiennymi (imię, domena, usługa, termin) i kategoriami — rozbudowa canned responses; klasyfikacja zgłoszenia i szkic odpowiedzi z bazy wiedzy i danych konta (do akceptacji, bez auto-wysyłki w v2); akcje z ticketu z audytem; licznik SLA.</t>
         </is>
       </c>
       <c r="P60" s="10" t="inlineStr">
@@ -5483,12 +5483,12 @@
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>A-26</t>
+          <t>A-25</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Ręczne odwieszenie usługi przez operatora</t>
+          <t>Ręczne zawieszenie usługi przez operatora</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -5534,12 +5534,12 @@
       </c>
       <c r="L61" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: ten sam formularz — odwieszenie z opcją obciążenia za odnowienie (chargeRenewal)</t>
+          <t>2026-09-23 D1: admin-panel subscriptions/[id]/suspend-form.tsx + suspend-actions.ts → POST /admin/subscriptions/:id/suspend (powód, notatka, potwierdzenie)</t>
         </is>
       </c>
       <c r="M61" s="11" t="inlineStr">
         <is>
-          <t>A-25 (ten sam widok)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N61" s="11" t="inlineStr">
@@ -5549,7 +5549,7 @@
       </c>
       <c r="O61" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: jak A-25, endpoint subscriptions.admin.controller.ts:210 działa z chargeRenewal. | UI zrobione. OTWARTE do D3 (PB-21): odwieszenie konta w DA na żywym węźle.</t>
+          <t>Skorygowane: endpoint działa i jest osiągalny (curl + DirectAdmin), auto-suspend za brak płatności działa. Brakuje UI, nie możliwości zatrzymania szkody. | UI zrobione. OTWARTE do D3 (PB-21, serwer testowy): zawieszenie konta w DirectAdminie na żywym węźle.</t>
         </is>
       </c>
       <c r="P61" s="10" t="inlineStr">
@@ -5561,12 +5561,12 @@
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>N-07</t>
+          <t>A-26</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Ręczne tworzenie incydentu na status page</t>
+          <t>Ręczne odwieszenie usługi przez operatora</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
@@ -5607,27 +5607,27 @@
       </c>
       <c r="K62" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L62" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D2: admin-panel status/incidents/incident-compose.tsx → POST /admin/product-ops/incidents; przycisk „Rozwiąż” (PATCH incidents/:id status=RESOLVED); probe-ingest.service.ts isManualIncident; test status/incydent-reczny.spec.ts</t>
+          <t>2026-09-23 D1: ten sam formularz — odwieszenie z opcją obciążenia za odnowienie (chargeRenewal)</t>
         </is>
       </c>
       <c r="M62" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A-25 (ten sam widok)</t>
         </is>
       </c>
       <c r="N62" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O62" s="11" t="inlineStr">
         <is>
-          <t>w kryzysie nie ma jak zakomunikować awarii | ZNALEZISKO: incydent ogłoszony ręcznie zamykał się sam przy pierwszej udanej próbie monitora (w ciągu minut), więc komunikat o awarii, której monitor nie widzi, znikał ze status page. Teraz zamyka go tylko operator; zamknięcie wysyła webhook INCIDENT_RESOLVED i trafia do audytu.</t>
+          <t>Skorygowane: jak A-25, endpoint subscriptions.admin.controller.ts:210 działa z chargeRenewal. | UI zrobione. OTWARTE do D3 (PB-21): odwieszenie konta w DA na żywym węźle.</t>
         </is>
       </c>
       <c r="P62" s="10" t="inlineStr">
@@ -5639,12 +5639,12 @@
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>N-14</t>
+          <t>N-07</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Cordon wysyłki poczty (auto-blokada spamu)</t>
+          <t>Ręczne tworzenie incydentu na status page</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="L63" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: admin-panel /deliverability (Blokady wysyłki poczty, link w menu) → GET/POST /admin/deliverability/cordons; lista z e-mailem i nazwą klienta</t>
+          <t>2026-09-23 D2: admin-panel status/incidents/incident-compose.tsx → POST /admin/product-ops/incidents; przycisk „Rozwiąż” (PATCH incidents/:id status=RESOLVED); probe-ingest.service.ts isManualIncident; test status/incydent-reczny.spec.ts</t>
         </is>
       </c>
       <c r="M63" s="11" t="inlineStr">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="O63" s="11" t="inlineStr">
         <is>
-          <t>mechanizm działa, operator nie może go zobaczyć ani zdjąć | Operator widzi kogo i dlaczego zablokowano oraz zdejmuje blokadę (ADMIN, z potwierdzeniem, audyt po stronie API).</t>
+          <t>w kryzysie nie ma jak zakomunikować awarii | ZNALEZISKO: incydent ogłoszony ręcznie zamykał się sam przy pierwszej udanej próbie monitora (w ciągu minut), więc komunikat o awarii, której monitor nie widzi, znikał ze status page. Teraz zamyka go tylko operator; zamknięcie wysyła webhook INCIDENT_RESOLVED i trafia do audytu.</t>
         </is>
       </c>
       <c r="P63" s="10" t="inlineStr">
@@ -5717,12 +5717,12 @@
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>H-22</t>
+          <t>N-14</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>Panel odtwarzania w widocznym miejscu</t>
+          <t>Cordon wysyłki poczty (auto-blokada spamu)</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E64" s="10" t="inlineStr">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="L64" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: client-panel BackupsTab.tsx — sekcja „Kopie poza serwerem” (HostingOffsitePanel) w zakładce Kopie zapasowe; zdublowany panel przywracania usunięty z Zużycia zasobów (hosting-backup-restore-panel.tsx)</t>
+          <t>2026-09-23: admin-panel /deliverability (Blokady wysyłki poczty, link w menu) → GET/POST /admin/deliverability/cordons; lista z e-mailem i nazwą klienta</t>
         </is>
       </c>
       <c r="M64" s="11" t="inlineStr">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="O64" s="11" t="inlineStr">
         <is>
-          <t>klient w kryzysie tego nie znajdzie | Kopie off-site są tam, gdzie klient ich szuka w kryzysie; przywracanie jest w jednym miejscu, z potwierdzeniem domeną.</t>
+          <t>mechanizm działa, operator nie może go zobaczyć ani zdjąć | Operator widzi kogo i dlaczego zablokowano oraz zdejmuje blokadę (ADMIN, z potwierdzeniem, audyt po stronie API).</t>
         </is>
       </c>
       <c r="P64" s="10" t="inlineStr">
@@ -5795,12 +5795,12 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>H-09</t>
+          <t>H-22</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>Kopia bezpieczeństwa przed odtworzeniem</t>
+          <t>Panel odtwarzania w widocznym miejscu</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -5822,7 +5822,7 @@
         <v>6</v>
       </c>
       <c r="G65" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H65" s="10" t="inlineStr">
         <is>
@@ -5831,22 +5831,22 @@
       </c>
       <c r="I65" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J65" s="10" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K65" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L65" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
+          <t>2026-09-23: client-panel BackupsTab.tsx — sekcja „Kopie poza serwerem” (HostingOffsitePanel) w zakładce Kopie zapasowe; zdublowany panel przywracania usunięty z Zużycia zasobów (hosting-backup-restore-panel.tsx)</t>
         </is>
       </c>
       <c r="M65" s="11" t="inlineStr">
@@ -5856,12 +5856,12 @@
       </c>
       <c r="N65" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O65" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: hosting-restore.service.ts:167 tylko KOLEJKUJE backup w DA i nie czeka na wynik — destrukcyjne odtworzenie rusza mimo nieudanej kopii. Job dostaje COMPLETED (:182) w chwili przyjęcia zadania, nie po odtworzeniu. | Naprawione: nadpisywanie danych bez siatki. Status COMPLETED w panelu klienta opisany uczciwie („Odtwarzanie zlecone — serwer odtwarza dane w tle”), bo DA przyjmuje odtworzenie asynchronicznie. OTWARTE do D3 (PB-21): pełny przebieg na żywym DA i wykrycie końca odtwarzania.</t>
+          <t>klient w kryzysie tego nie znajdzie | Kopie off-site są tam, gdzie klient ich szuka w kryzysie; przywracanie jest w jednym miejscu, z potwierdzeniem domeną.</t>
         </is>
       </c>
       <c r="P65" s="10" t="inlineStr">
@@ -5873,12 +5873,12 @@
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>H-17</t>
+          <t>H-09</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Tryb restore skryptu odtwarzającego osiągalny z produktu</t>
+          <t>Kopia bezpieczeństwa przed odtworzeniem</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -5919,27 +5919,27 @@
       </c>
       <c r="K66" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L66" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: produktowa ścieżka odtwarzania z off-site = „Pobierz na serwer” (fetch, agent) + przywrócenie z listy kopii z kopią bezpieczeństwa (H-09) i potwierdzeniem domeną; tryb `restore` skryptu (DA type=admin, bez kopii bezpieczeństwa) celowo zostaje tylko w CLI/runbooku DR</t>
+          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
         </is>
       </c>
       <c r="M66" s="11" t="inlineStr">
         <is>
-          <t>H-20 (najpierw potwierdzone odtworzenie, potem wystawienie trybu w produkcie)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N66" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O66" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: tryb restore jest martwy z poziomu produktu, ale żywy z CLI (node-account-restore.sh:120-124) i udokumentowany w runbooku. | DO DECYZJI WŁAŚCICIELA: proponuję zamknąć jako PARYTET przez równoważną ścieżkę produktową — wystawienie trybu `restore` ominęłoby kopię bezpieczeństwa z H-09. Tryb restore działa też tylko przy istniejącym koncie na węźle, czyli dokładnie tam, gdzie wystarcza fetch + przywrócenie. | DECYZJA WŁAŚCICIELA 2026-09-23: zamknięte jako PARYTET — ścieżka produktowa (pobierz na serwer + przywrócenie z kopią bezpieczeństwa i potwierdzeniem domeną) daje ten sam efekt bezpieczniej; tryb restore skryptu zostaje wyłącznie w CLI/runbooku DR.</t>
+          <t>OSŁABIONE: hosting-restore.service.ts:167 tylko KOLEJKUJE backup w DA i nie czeka na wynik — destrukcyjne odtworzenie rusza mimo nieudanej kopii. Job dostaje COMPLETED (:182) w chwili przyjęcia zadania, nie po odtworzeniu. | Naprawione: nadpisywanie danych bez siatki. Status COMPLETED w panelu klienta opisany uczciwie („Odtwarzanie zlecone — serwer odtwarza dane w tle”), bo DA przyjmuje odtworzenie asynchronicznie. OTWARTE do D3 (PB-21): pełny przebieg na żywym DA i wykrycie końca odtwarzania.</t>
         </is>
       </c>
       <c r="P66" s="10" t="inlineStr">
@@ -5951,12 +5951,12 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>G-20</t>
+          <t>H-17</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>Ochrona przed atakiem słownikowym na panel</t>
+          <t>Tryb restore skryptu odtwarzającego osiągalny z produktu</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="E67" s="10" t="inlineStr">
@@ -6002,12 +6002,12 @@
       </c>
       <c r="L67" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D2: common/guards/rate-limit.guard.spec.ts (6 testów: limit per IP, per e-mail z wielu IP, reset okna, zakresy i @SkipRateLimit, przepełnienie mapy, awaria Redisa)</t>
+          <t>2026-09-23: produktowa ścieżka odtwarzania z off-site = „Pobierz na serwer” (fetch, agent) + przywrócenie z listy kopii z kopią bezpieczeństwa (H-09) i potwierdzeniem domeną; tryb `restore` skryptu (DA type=admin, bez kopii bezpieczeństwa) celowo zostaje tylko w CLI/runbooku DR</t>
         </is>
       </c>
       <c r="M67" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>H-20 (najpierw potwierdzone odtworzenie, potem wystawienie trybu w produkcie)</t>
         </is>
       </c>
       <c r="N67" s="11" t="inlineStr">
@@ -6017,7 +6017,7 @@
       </c>
       <c r="O67" s="11" t="inlineStr">
         <is>
-          <t>brak dowodu D2 na krytycznym guardzie | ZNALEZISKO przy pisaniu testów: w trybie pamięciowym przepełnienie mapy (50 tys. kluczy) czyściło WSZYSTKIE liczniki — losowe e-maile zerowały licznik prób logowania do atakowanego konta (fail-open). Teraz usuwane są tylko wygasłe, a przy pełnej mapie nowe klucze dostają 429 (fail-closed).</t>
+          <t>Skorygowane: tryb restore jest martwy z poziomu produktu, ale żywy z CLI (node-account-restore.sh:120-124) i udokumentowany w runbooku. | DO DECYZJI WŁAŚCICIELA: proponuję zamknąć jako PARYTET przez równoważną ścieżkę produktową — wystawienie trybu `restore` ominęłoby kopię bezpieczeństwa z H-09. Tryb restore działa też tylko przy istniejącym koncie na węźle, czyli dokładnie tam, gdzie wystarcza fetch + przywrócenie. | DECYZJA WŁAŚCICIELA 2026-09-23: zamknięte jako PARYTET — ścieżka produktowa (pobierz na serwer + przywrócenie z kopią bezpieczeństwa i potwierdzeniem domeną) daje ten sam efekt bezpieczniej; tryb restore skryptu zostaje wyłącznie w CLI/runbooku DR.</t>
         </is>
       </c>
       <c r="P67" s="10" t="inlineStr">
@@ -6029,12 +6029,12 @@
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>I-11</t>
+          <t>G-20</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>Staging — publikacja na produkcję</t>
+          <t>Ochrona przed atakiem słownikowym na panel</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E68" s="10" t="inlineStr">
@@ -6075,12 +6075,12 @@
       </c>
       <c r="K68" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L68" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
+          <t>2026-09-23 D2: common/guards/rate-limit.guard.spec.ts (6 testów: limit per IP, per e-mail z wielu IP, reset okna, zakresy i @SkipRateLimit, przepełnienie mapy, awaria Redisa)</t>
         </is>
       </c>
       <c r="M68" s="11" t="inlineStr">
@@ -6090,12 +6090,12 @@
       </c>
       <c r="N68" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: node-staging-sync.sh:141-142 backup plików jest twardą bramką, ale :152-153 backup bazy LIVE jest best-effort — linia 158 robi wp db import na produkcji mimo braku kopii. | Naprawione: import bazy staging na produkcję mimo braku kopii bazy LIVE. OTWARTE do D3 (PB-21): publikacja stagingu na żywym węźle.</t>
+          <t>brak dowodu D2 na krytycznym guardzie | ZNALEZISKO przy pisaniu testów: w trybie pamięciowym przepełnienie mapy (50 tys. kluczy) czyściło WSZYSTKIE liczniki — losowe e-maile zerowały licznik prób logowania do atakowanego konta (fail-open). Teraz usuwane są tylko wygasłe, a przy pełnej mapie nowe klucze dostają 429 (fail-closed).</t>
         </is>
       </c>
       <c r="P68" s="10" t="inlineStr">
@@ -6107,12 +6107,12 @@
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>X-31</t>
+          <t>I-11</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Kanał alertów daje znak życia (dead man's switch)</t>
+          <t>Staging — publikacja na produkcję</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -6122,19 +6122,19 @@
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="E69" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F69" s="10" t="n">
         <v>6</v>
       </c>
       <c r="G69" s="10" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H69" s="10" t="inlineStr">
         <is>
@@ -6143,22 +6143,22 @@
       </c>
       <c r="I69" s="10" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="J69" s="10" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="K69" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L69" s="11" t="inlineStr">
         <is>
-          <t>ops/observability/grafana/provisioning/alerting/rules.yaml — grupa verris_kanal_alertow, reguła VerrisKanalAlertowZyje (vector(1), for: 0s, oba stany awaryjne na Alerting, etykieta kanal: heartbeat); policies.yaml — gałąź object_matchers kanal=heartbeat, repeat_interval 24h; apps/api/src/test/routing-alertow.spec.ts (5 asercji X-31); docs/ops/GRAFANA_ALERTING.md §4. BRAK: pierwszego maila [FIRING:1] VerrisKanalAlertowZyje — dowód D3 jeszcze nie powstał.</t>
+          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
         </is>
       </c>
       <c r="M69" s="11" t="inlineStr">
@@ -6168,12 +6168,12 @@
       </c>
       <c r="N69" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O69" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 powstanie przy pierwszym mailu. Decyzja właściciela produktu: wariant „jeden mail na dobę". | PROBLEM: po naprawie X-30 alerty ucichną, a cisza będzie znaczyła „nic się nie pali" — i będzie wyglądała IDENTYCZNIE jak: Grafana padła, Postfix przestał przyjmować, mail.hvln.pl zaczął odrzucać albo wrzucać do spamu, ktoś zmienił adres w punkcie kontaktowym, polityka przestała pasować do etykiet. To dokładnie ta sama cisza, która przez miesiąc znaczyła „kopia bazy jest w porządku" (H-23) i kosztowała wszystkie kopie zapasowe. | ROZWIĄZANIE: VerrisKanalAlertowZyje — reguła vector(1), pali się ZAWSZE, jej BRAK jest sygnałem. for: 0s, noDataState: Alerting, execErrState: Alerting — nie da się jej „nie zapalić": normalnie warunek jest spełniony, a gdyby źródło danych przestało odpowiadać, oba stany awaryjne też prowadzą do Alerting. Milczenie ma znaczyć awarię, nigdy spokój. | JEDEN MAIL NA DOBĘ, NIE SZEŚĆ: osobna gałąź polityki na etykiecie kanal: heartbeat z repeat_interval 24h. Na domyślnej (4h) byłoby sześć dziennie, a alert przychodzący sześć razy dziennie przestaje być czytany po tygodniu — wtedy przestaje cokolwiek dawać, bo jego BRAK jest jedyną informacją, jaką niesie. Strażnik pilnuje osobno, że polityka domyślna NIE została przy okazji przestawiona na dobę: prawdziwy alarm ma się przypominać co cztery godziny. | HACZYK, KTÓRY TRZEBA NAZWAĆ: mail, którego się nie czyta, wraca do punktu wyjścia. Jeśli po tygodniu przestanie być zauważany, reguła przestaje działać — nie dlatego, że jest zepsuta, tylko dlatego, że przestała być czytana. Tego nie da się naprawić kodem. | CZEGO NIE OBEJMUJE: awarii całego serwera (heartbeat mieszka na tej samej maszynie co Grafana i milczy razem z nią — odporny byłby watchdog SPOZA naszej infrastruktury, pukany cronem; nie ma go i to świadoma decyzja, nie przeoczenie) ani poprawności pozostałych reguł (tego pilnuje bramka z X-30). | Czerwieni się na starym kodzie: 5 z 36. | Doszła lista DOPISANE_POZNIEJ, trzymana osobno od ALERTY: tamta odpowiada na pytanie „czy migracja czegoś nie zgubiła" i ma zostać zamrożona, ta na „czy ktoś czegoś po cichu nie dołożył". Dokumentacja: docs/archiwum/zadania/X-31-znak-zycia-kanalu-alertow.md | 2026-09-22 D3: wlasciciel potwierdza, ze mail [FIRING:1] VerrisKanalAlertowZyje przychodzi codziennie. Kanal alertow dziala koniec-do-konca.</t>
+          <t>OSŁABIONE: node-staging-sync.sh:141-142 backup plików jest twardą bramką, ale :152-153 backup bazy LIVE jest best-effort — linia 158 robi wp db import na produkcji mimo braku kopii. | Naprawione: import bazy staging na produkcję mimo braku kopii bazy LIVE. OTWARTE do D3 (PB-21): publikacja stagingu na żywym węźle.</t>
         </is>
       </c>
       <c r="P69" s="10" t="inlineStr">
@@ -6185,12 +6185,12 @@
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>X-32</t>
+          <t>X-31</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>Martwy job da się odrzucić z panelu, ze śladem w audycie</t>
+          <t>Kanał alertów daje znak życia (dead man's switch)</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="L70" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/common/audit/audit.actions.ts — PROVISIONING_JOB_DISCARDED_BY_ADMIN; provisioning-queue.service.ts — odrzucJob (getState() === failed, ślad przed job.remove(), audyt z subskrypcją, typem, liczbą prób, failedReason i powodem); provisioning-queue.admin.controller.ts — POST :id/odrzuc za @StaffPerm('PROVISIONING_MANAGE'); apps/admin-panel/.../provisioning-queue/ — actions.ts, odrzuc-button.tsx (dwa kliknięcia, powód ≥5 znaków, zdanie o nietkniętej subskrypcji), page.tsx; apps/api/src/test/odrzucenie-martwego-joba.spec.ts (13). BRAK: pierwszego odrzucenia na produkcji — dowód D3 jeszcze nie powstał.</t>
+          <t>ops/observability/grafana/provisioning/alerting/rules.yaml — grupa verris_kanal_alertow, reguła VerrisKanalAlertowZyje (vector(1), for: 0s, oba stany awaryjne na Alerting, etykieta kanal: heartbeat); policies.yaml — gałąź object_matchers kanal=heartbeat, repeat_interval 24h; apps/api/src/test/routing-alertow.spec.ts (5 asercji X-31); docs/ops/GRAFANA_ALERTING.md §4. BRAK: pierwszego maila [FIRING:1] VerrisKanalAlertowZyje — dowód D3 jeszcze nie powstał.</t>
         </is>
       </c>
       <c r="M70" s="11" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="O70" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 przy pierwszym odrzuceniu na produkcji — a to da się zrobić od razu po wdrożeniu, w odróżnieniu od Z-18, który czeka na węzeł. Decyzja właściciela produktu: dorobić akcję w panelu zamiast jednorazowego czyszczenia Redisa. | JAK TO WYSZŁO: X-30 naprawiło alerting, VerrisProvisioningQueueFailed zapalił się z prawdziwego powodu i wskazał cztery martwe joby (to z nich wyszło Z-18). Naturalny następny ruch — usunąć je — okazał się NIEWYKONALNY: panel ma przy nich wyłącznie „Retry", a kontroler administracyjny dokładnie dwa endpointy, listowanie i ponowienie. Retry nic nie daje, bo węzła nie ma: job padnie ponownie, podbije licznik prób i dołoży wpisy do audytu — cztery martwe joby zamieniają się w cztery martwe joby z dłuższą historią. Zostawało grzebanie w Redisie ręcznie, czyli zmiana stanu produkcyjnego dotyczącego subskrypcji klientów BEZ ŚLADU W AUDYCIE. | TO NIE JEST USTERKA TYCH CZTERECH JOBÓW, tylko luka w warstwie operatorskiej, która ujawni się ponownie przy pierwszym prawdziwym niepowodzeniu provisioningu — z tą różnicą, że wtedy po drugiej stronie będzie klient. | ROZWIĄZANIE: POST /admin/provisioning-queue/:id/odrzuc + przycisk „Odrzuć" obok Retry. TRZY REGUŁY: (1) TYLKO STAN failed — usunięcie joba aktywnego albo czekającego osierociłoby provisioning w trakcie, konto na węźle mogłoby powstać, a system przestałby o nim wiedzieć; ograniczenie siedzi w usłudze, nie w kontrolerze, bo to reguła o kolejce, nie o HTTP; (2) POWÓD WYMAGANY, tak samo jak przy retry — operacja bez powodu to operacja, której za pół roku nikt nie wyjaśni; (3) NAJPIERW ODCZYT, POTEM USUNIĘCIE — ślad zbierany PRZED job.remove(), bo po usunięciu nie ma już czego odczytać; zapisujemy subskrypcję, joba, typ, liczbę prób, ostatni błąd i powód. Po Z-18 ten ostatni błąd niesie PRAWDZIWĄ przyczynę, więc wpis ma realną wartość dowodową — jeszcze wczoraj zapisałby zdanie o brakującym pakiecie DirectAdmina, którego nigdy nie brakowało. | OSOBNA AKCJA AUDYTU (PROVISIONING_JOB_DISCARDED_BY_ADMIN), nie wariant retry: w raportach odrzucenie i ponowienie to dwie różne decyzje i nie wolno im się zlewać. | DWA KLIKNIĘCIA, NIE JEDNO: retry można cofnąć następnym retry, odrzucenia nie da się cofnąć wcale. Potwierdzenie jest po to, żeby ta różnica była wyczuwalna w palcach. | ZDANIE PRZY PRZYCISKU: „Usuwa wpis z kolejki bez możliwości cofnięcia. Subskrypcja zostaje nietknięta." Operator ma prawo założyć, że „odrzuć" anuluje zamówienie — nie anuluje. Musi to być napisane tam, gdzie się klika, a nie w dokumentacji, której nikt nie otworzy w trakcie incydentu. | Czerwieni się na starym kodzie: 11 z 13. | DWIE UWAGI O SAMYCH TESTACH: odczyty plików panelu są LENIWE, bo odczyt na poziomie describe wywalał cały plik testowy, zanim cokolwiek się policzyło — a wtedy nie wiadomo, ILE asercji się czerwieni, tylko że „nie skompilowało się"; asercja o warunku row.failedReason nie mierzy odległości w znakach, tylko relację między warunkiem a przyciskiem, bo wersja licząca znaki zepsuła się od dopisania komentarza i kusiło, żeby poszerzyć okno zamiast poprawić asercję — to byłoby naprawianie testu zamiast kodu. | CZEGO NIE OBEJMUJE: losu czterech subskrypcji, które dostały zwrot i status PENDING_PAYMENT (odrzucenie joba ich nie dotyka — osobne sprzątanie po stronie bazy); odrzucania hurtem — świadomie, bo przycisk „odrzuć wszystkie" jest wygodny dokładnie do momentu, w którym ktoś kliknie go na kolejce z prawdziwym zamówieniem. | JAK ZAMKNĄĆ: odrzucić jeden z czterech martwych jobów, obejrzeć wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie i sprawdzić, że verris_provisioning_queue_depth{state="failed"} spadło o jeden. Dokumentacja: docs/archiwum/zadania/X-32-odrzucenie-martwego-joba.md | 2026-09-22 D3: wlasciciel odrzucil martwy job przyciskiem 'Odrzuc' w panelu admina na produkcji (potwierdzenie wlasciciela; wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie).</t>
+          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 powstanie przy pierwszym mailu. Decyzja właściciela produktu: wariant „jeden mail na dobę". | PROBLEM: po naprawie X-30 alerty ucichną, a cisza będzie znaczyła „nic się nie pali" — i będzie wyglądała IDENTYCZNIE jak: Grafana padła, Postfix przestał przyjmować, mail.hvln.pl zaczął odrzucać albo wrzucać do spamu, ktoś zmienił adres w punkcie kontaktowym, polityka przestała pasować do etykiet. To dokładnie ta sama cisza, która przez miesiąc znaczyła „kopia bazy jest w porządku" (H-23) i kosztowała wszystkie kopie zapasowe. | ROZWIĄZANIE: VerrisKanalAlertowZyje — reguła vector(1), pali się ZAWSZE, jej BRAK jest sygnałem. for: 0s, noDataState: Alerting, execErrState: Alerting — nie da się jej „nie zapalić": normalnie warunek jest spełniony, a gdyby źródło danych przestało odpowiadać, oba stany awaryjne też prowadzą do Alerting. Milczenie ma znaczyć awarię, nigdy spokój. | JEDEN MAIL NA DOBĘ, NIE SZEŚĆ: osobna gałąź polityki na etykiecie kanal: heartbeat z repeat_interval 24h. Na domyślnej (4h) byłoby sześć dziennie, a alert przychodzący sześć razy dziennie przestaje być czytany po tygodniu — wtedy przestaje cokolwiek dawać, bo jego BRAK jest jedyną informacją, jaką niesie. Strażnik pilnuje osobno, że polityka domyślna NIE została przy okazji przestawiona na dobę: prawdziwy alarm ma się przypominać co cztery godziny. | HACZYK, KTÓRY TRZEBA NAZWAĆ: mail, którego się nie czyta, wraca do punktu wyjścia. Jeśli po tygodniu przestanie być zauważany, reguła przestaje działać — nie dlatego, że jest zepsuta, tylko dlatego, że przestała być czytana. Tego nie da się naprawić kodem. | CZEGO NIE OBEJMUJE: awarii całego serwera (heartbeat mieszka na tej samej maszynie co Grafana i milczy razem z nią — odporny byłby watchdog SPOZA naszej infrastruktury, pukany cronem; nie ma go i to świadoma decyzja, nie przeoczenie) ani poprawności pozostałych reguł (tego pilnuje bramka z X-30). | Czerwieni się na starym kodzie: 5 z 36. | Doszła lista DOPISANE_POZNIEJ, trzymana osobno od ALERTY: tamta odpowiada na pytanie „czy migracja czegoś nie zgubiła" i ma zostać zamrożona, ta na „czy ktoś czegoś po cichu nie dołożył". Dokumentacja: docs/archiwum/zadania/X-31-znak-zycia-kanalu-alertow.md | 2026-09-22 D3: wlasciciel potwierdza, ze mail [FIRING:1] VerrisKanalAlertowZyje przychodzi codziennie. Kanal alertow dziala koniec-do-konca.</t>
         </is>
       </c>
       <c r="P70" s="10" t="inlineStr">
@@ -6263,12 +6263,12 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>X-32</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>W drzewie stoją dwa majory ESLinta naraz</t>
+          <t>Martwy job da się odrzucić z panelu, ze śladem w audycie</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="E71" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F71" s="10" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="L71" s="11" t="inlineStr">
         <is>
-          <t>package.json (korzeń) — @eslint/js ^10.0.1 przy braku jakiegokolwiek eslint.config.* w korzeniu; libs/eslint-config/node_modules: eslint 10.9.0 obok @eslint/js 9.39.5; apps/api, apps/www, apps/client-panel, apps/status-page, libs/directadmin-sdk — eslint 9.39.5 | 2026-09-23: z korzenia zdjęte nieużywane @eslint/js ^10 i typescript-eslint; libs/eslint-config peer eslint ^9.39.5 (było &gt;=9 → auto-install dociągał 10.9.0); lockfile bez eslint 10; strażnik apps/api/src/test/eslint-jeden-major.spec.ts (deklaracje + peer + lockfile)</t>
+          <t>apps/api/src/common/audit/audit.actions.ts — PROVISIONING_JOB_DISCARDED_BY_ADMIN; provisioning-queue.service.ts — odrzucJob (getState() === failed, ślad przed job.remove(), audyt z subskrypcją, typem, liczbą prób, failedReason i powodem); provisioning-queue.admin.controller.ts — POST :id/odrzuc za @StaffPerm('PROVISIONING_MANAGE'); apps/admin-panel/.../provisioning-queue/ — actions.ts, odrzuc-button.tsx (dwa kliknięcia, powód ≥5 znaków, zdanie o nietkniętej subskrypcji), page.tsx; apps/api/src/test/odrzucenie-martwego-joba.spec.ts (13). BRAK: pierwszego odrzucenia na produkcji — dowód D3 jeszcze nie powstał.</t>
         </is>
       </c>
       <c r="M71" s="11" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="O71" s="11" t="inlineStr">
         <is>
-          <t>Odkryte 2026-08-28 przy DEP-01. Korzeń deklaruje @eslint/js ^10.0.1, którego peer to eslint ^10.0.0 — i to on wciąga eslint@10.9.0 do drzewa. Tymczasem KAŻDY pakiet, który realnie lintuje, ma 9.39.5. Najostrzej widać to wewnątrz libs/eslint-config, czyli wspólnej konfiguracji: node_modules/eslint = 10.9.0, node_modules/@eslint/js = 9.39.5 — dwie połowy jednego narzędzia z różnych majorów w jednym katalogu. | Korzeń NIE MA żadnego eslint.config.* i nie odpala lintera (pnpm lint = turbo run lint), więc te zależności nie robią nic poza wciąganiem majora, którego nikt nie używa. | To nie awaria — bramka jest zielona, 0 błędów. To BRAK KONTROLI: żaden strażnik nie sprawdza, czy major ESLinta jest jeden, tak jak do ENV-01 nic nie sprawdzało wersji Node. | DO ZROBIENIA: zdjąć z korzenia nieużywane @eslint/js i typescript-eslint albo cofnąć je do dziewiątki (rusza lockfile — osobny commit z pełną bramką), plus strażnik spójności majora na wzór wersja-node.spec.ts. | 2026-09-23: zrobione zgodnie z DO ZROBIENIA; lockfile zmieniony wyłącznie o usunięcie gałęzi eslint 10 (pnpm 9.5.0 --lockfile-only). Przed bramką lokalną: pnpm install.</t>
+          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 przy pierwszym odrzuceniu na produkcji — a to da się zrobić od razu po wdrożeniu, w odróżnieniu od Z-18, który czeka na węzeł. Decyzja właściciela produktu: dorobić akcję w panelu zamiast jednorazowego czyszczenia Redisa. | JAK TO WYSZŁO: X-30 naprawiło alerting, VerrisProvisioningQueueFailed zapalił się z prawdziwego powodu i wskazał cztery martwe joby (to z nich wyszło Z-18). Naturalny następny ruch — usunąć je — okazał się NIEWYKONALNY: panel ma przy nich wyłącznie „Retry", a kontroler administracyjny dokładnie dwa endpointy, listowanie i ponowienie. Retry nic nie daje, bo węzła nie ma: job padnie ponownie, podbije licznik prób i dołoży wpisy do audytu — cztery martwe joby zamieniają się w cztery martwe joby z dłuższą historią. Zostawało grzebanie w Redisie ręcznie, czyli zmiana stanu produkcyjnego dotyczącego subskrypcji klientów BEZ ŚLADU W AUDYCIE. | TO NIE JEST USTERKA TYCH CZTERECH JOBÓW, tylko luka w warstwie operatorskiej, która ujawni się ponownie przy pierwszym prawdziwym niepowodzeniu provisioningu — z tą różnicą, że wtedy po drugiej stronie będzie klient. | ROZWIĄZANIE: POST /admin/provisioning-queue/:id/odrzuc + przycisk „Odrzuć" obok Retry. TRZY REGUŁY: (1) TYLKO STAN failed — usunięcie joba aktywnego albo czekającego osierociłoby provisioning w trakcie, konto na węźle mogłoby powstać, a system przestałby o nim wiedzieć; ograniczenie siedzi w usłudze, nie w kontrolerze, bo to reguła o kolejce, nie o HTTP; (2) POWÓD WYMAGANY, tak samo jak przy retry — operacja bez powodu to operacja, której za pół roku nikt nie wyjaśni; (3) NAJPIERW ODCZYT, POTEM USUNIĘCIE — ślad zbierany PRZED job.remove(), bo po usunięciu nie ma już czego odczytać; zapisujemy subskrypcję, joba, typ, liczbę prób, ostatni błąd i powód. Po Z-18 ten ostatni błąd niesie PRAWDZIWĄ przyczynę, więc wpis ma realną wartość dowodową — jeszcze wczoraj zapisałby zdanie o brakującym pakiecie DirectAdmina, którego nigdy nie brakowało. | OSOBNA AKCJA AUDYTU (PROVISIONING_JOB_DISCARDED_BY_ADMIN), nie wariant retry: w raportach odrzucenie i ponowienie to dwie różne decyzje i nie wolno im się zlewać. | DWA KLIKNIĘCIA, NIE JEDNO: retry można cofnąć następnym retry, odrzucenia nie da się cofnąć wcale. Potwierdzenie jest po to, żeby ta różnica była wyczuwalna w palcach. | ZDANIE PRZY PRZYCISKU: „Usuwa wpis z kolejki bez możliwości cofnięcia. Subskrypcja zostaje nietknięta." Operator ma prawo założyć, że „odrzuć" anuluje zamówienie — nie anuluje. Musi to być napisane tam, gdzie się klika, a nie w dokumentacji, której nikt nie otworzy w trakcie incydentu. | Czerwieni się na starym kodzie: 11 z 13. | DWIE UWAGI O SAMYCH TESTACH: odczyty plików panelu są LENIWE, bo odczyt na poziomie describe wywalał cały plik testowy, zanim cokolwiek się policzyło — a wtedy nie wiadomo, ILE asercji się czerwieni, tylko że „nie skompilowało się"; asercja o warunku row.failedReason nie mierzy odległości w znakach, tylko relację między warunkiem a przyciskiem, bo wersja licząca znaki zepsuła się od dopisania komentarza i kusiło, żeby poszerzyć okno zamiast poprawić asercję — to byłoby naprawianie testu zamiast kodu. | CZEGO NIE OBEJMUJE: losu czterech subskrypcji, które dostały zwrot i status PENDING_PAYMENT (odrzucenie joba ich nie dotyka — osobne sprzątanie po stronie bazy); odrzucania hurtem — świadomie, bo przycisk „odrzuć wszystkie" jest wygodny dokładnie do momentu, w którym ktoś kliknie go na kolejce z prawdziwym zamówieniem. | JAK ZAMKNĄĆ: odrzucić jeden z czterech martwych jobów, obejrzeć wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie i sprawdzić, że verris_provisioning_queue_depth{state="failed"} spadło o jeden. Dokumentacja: docs/archiwum/zadania/X-32-odrzucenie-martwego-joba.md | 2026-09-22 D3: wlasciciel odrzucil martwy job przyciskiem 'Odrzuc' w panelu admina na produkcji (potwierdzenie wlasciciela; wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie).</t>
         </is>
       </c>
       <c r="P71" s="10" t="inlineStr">
@@ -6341,12 +6341,12 @@
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>M-08</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Anulowanie faktury (VOID) z panelu</t>
+          <t>W drzewie stoją dwa majory ESLinta naraz</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -6356,12 +6356,12 @@
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E72" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F72" s="10" t="n">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="L72" s="11" t="inlineStr">
         <is>
-          <t>billing/anulowanie.service.ts (POST /admin/invoices/:id/anuluj, BILLING_MANAGE); admin: invoices/void-button.tsx; test D2 anulowanie.service.spec.ts</t>
+          <t>package.json (korzeń) — @eslint/js ^10.0.1 przy braku jakiegokolwiek eslint.config.* w korzeniu; libs/eslint-config/node_modules: eslint 10.9.0 obok @eslint/js 9.39.5; apps/api, apps/www, apps/client-panel, apps/status-page, libs/directadmin-sdk — eslint 9.39.5 | 2026-09-23: z korzenia zdjęte nieużywane @eslint/js ^10 i typescript-eslint; libs/eslint-config peer eslint ^9.39.5 (było &gt;=9 → auto-install dociągał 10.9.0); lockfile bez eslint 10; strażnik apps/api/src/test/eslint-jeden-major.spec.ts (deklaracje + peer + lockfile)</t>
         </is>
       </c>
       <c r="M72" s="11" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="O72" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: anulować wolno tylko dokument nieopłacony (DRAFT/OPEN); opłacony, także z portfela, zmienia się korektą (M-06). Faktura Stripe unieważniana najpierw w Stripe, błąd = brak zmiany lokalnej. Numer zostaje (ciągłość), powód w audycie INVOICE_VOIDED.</t>
+          <t>Odkryte 2026-08-28 przy DEP-01. Korzeń deklaruje @eslint/js ^10.0.1, którego peer to eslint ^10.0.0 — i to on wciąga eslint@10.9.0 do drzewa. Tymczasem KAŻDY pakiet, który realnie lintuje, ma 9.39.5. Najostrzej widać to wewnątrz libs/eslint-config, czyli wspólnej konfiguracji: node_modules/eslint = 10.9.0, node_modules/@eslint/js = 9.39.5 — dwie połowy jednego narzędzia z różnych majorów w jednym katalogu. | Korzeń NIE MA żadnego eslint.config.* i nie odpala lintera (pnpm lint = turbo run lint), więc te zależności nie robią nic poza wciąganiem majora, którego nikt nie używa. | To nie awaria — bramka jest zielona, 0 błędów. To BRAK KONTROLI: żaden strażnik nie sprawdza, czy major ESLinta jest jeden, tak jak do ENV-01 nic nie sprawdzało wersji Node. | DO ZROBIENIA: zdjąć z korzenia nieużywane @eslint/js i typescript-eslint albo cofnąć je do dziewiątki (rusza lockfile — osobny commit z pełną bramką), plus strażnik spójności majora na wzór wersja-node.spec.ts. | 2026-09-23: zrobione zgodnie z DO ZROBIENIA; lockfile zmieniony wyłącznie o usunięcie gałęzi eslint 10 (pnpm 9.5.0 --lockfile-only). Przed bramką lokalną: pnpm install.</t>
         </is>
       </c>
       <c r="P72" s="10" t="inlineStr">
@@ -6419,12 +6419,12 @@
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>C-18</t>
+          <t>M-08</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>Konto FTP — zmiana hasła</t>
+          <t>Anulowanie faktury (VOID) z panelu</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -6434,7 +6434,7 @@
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
@@ -6465,12 +6465,12 @@
       </c>
       <c r="K73" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L73" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/hosting-ftp/:username/password (ZmienHasloFtpDto) → directadmin.service changeHostingFtpPassword (action=modify, katalog zachowany) + audyt HOSTING_FTP_PASSWORD_CHANGED; UI FtpTab — kluczyk przy koncie; test servers/zmiana-hasla-ftp.spec.ts</t>
+          <t>billing/anulowanie.service.ts (POST /admin/invoices/:id/anuluj, BILLING_MANAGE); admin: invoices/void-button.tsx; test D2 anulowanie.service.spec.ts</t>
         </is>
       </c>
       <c r="M73" s="11" t="inlineStr">
@@ -6480,12 +6480,12 @@
       </c>
       <c r="N73" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O73" s="11" t="inlineStr">
         <is>
-          <t>brak jakiejkolwiek ścieżki edycji istniejącego konta | Przy okazji body tworzenia konta FTP dostało klasę DTO (login, hasło, katalog bez „..”). OTWARTE do D3 (PB-21): format action=modify na żywym DA.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: anulować wolno tylko dokument nieopłacony (DRAFT/OPEN); opłacony, także z portfela, zmienia się korektą (M-06). Faktura Stripe unieważniana najpierw w Stripe, błąd = brak zmiany lokalnej. Numer zostaje (ciągłość), powód w audycie INVOICE_VOIDED.</t>
         </is>
       </c>
       <c r="P73" s="10" t="inlineStr">
@@ -6497,12 +6497,12 @@
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>C-18</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>Konto FTP — zmiana hasła</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="E74" s="10" t="inlineStr">
@@ -6524,7 +6524,7 @@
         <v>6</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
@@ -6533,22 +6533,22 @@
       </c>
       <c r="I74" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="J74" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="K74" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L74" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>2026-09-23 D1: POST /services/:id/hosting-ftp/:username/password (ZmienHasloFtpDto) → directadmin.service changeHostingFtpPassword (action=modify, katalog zachowany) + audyt HOSTING_FTP_PASSWORD_CHANGED; UI FtpTab — kluczyk przy koncie; test servers/zmiana-hasla-ftp.spec.ts</t>
         </is>
       </c>
       <c r="M74" s="11" t="inlineStr">
@@ -6558,12 +6558,12 @@
       </c>
       <c r="N74" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O74" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>brak jakiejkolwiek ścieżki edycji istniejącego konta | Przy okazji body tworzenia konta FTP dostało klasę DTO (login, hasło, katalog bez „..”). OTWARTE do D3 (PB-21): format action=modify na żywym DA.</t>
         </is>
       </c>
       <c r="P74" s="10" t="inlineStr">
@@ -6575,12 +6575,12 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>C-11</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>Spakowanie do archiwum</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -6590,12 +6590,12 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F75" s="10" t="n">
@@ -6621,12 +6621,12 @@
       </c>
       <c r="K75" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L75" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M75" s="11" t="inlineStr">
@@ -6636,12 +6636,12 @@
       </c>
       <c r="N75" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O75" s="11" t="inlineStr">
         <is>
-          <t>standard we wszystkich panelach | OTWARTE do D3 (PB-21): format action=compress na żywym DA.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P75" s="10" t="inlineStr">
@@ -6653,12 +6653,12 @@
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>NODE-03</t>
+          <t>C-11</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>Pojemność węzła nigdy się nie odświeża</t>
+          <t>Spakowanie do archiwum</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -6668,7 +6668,7 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="E76" s="10" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="L76" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: verris-lve.sh node_capacity (nproc, MemTotal, df /) w każdym raporcie, lve-agent/1.1; telemetry.dto NodeStatusDto.totalCpuCores/totalMemoryMb/totalDiskMb; telemetry.service aktualizuje Server; test telemetry/pojemnosc-wezla.spec.ts</t>
+          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych</t>
         </is>
       </c>
       <c r="M76" s="11" t="inlineStr">
@@ -6719,7 +6719,7 @@
       </c>
       <c r="O76" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Pojemność węzła nigdy się nie odświeża. `totalCpuCores`/`totalMemoryMb`/`totalDiskMb` ustawiane wyłącznie w handshake; telemetria ich nie aktualizuje — mimo komentarza w schemacie „reported via handshake / heartbeat”. Rozbudowa węzła nie dociera do `NodeSelector`. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Telemetria aktualizuje totalCpuCores/totalMemoryMb/totalDiskMb, nie tylko handshake. | Stary agent bez pól niczego nie zeruje. OTWARTE do D3 (PB-21): raport z agenta na żywym węźle i odświeżona pojemność w panelu admina. | 2026-09-25: pojemność z agenta trafia też do planera pojemności (admin → Product Ops): ryzyko liczone względem rdzeni i RAM węzła (CPU 2×/4× rdzeni, RAM 1×/1,5×; test ryzyko-pojemnosci.spec.ts), a opis „CPU 250%” zastąpiony „przydzielone limity: CPU 2,5 rdz. z N · RAM x z y GB” — wcześniej wyglądało jak zużycie ponad 100%.</t>
+          <t>standard we wszystkich panelach | OTWARTE do D3 (PB-21): format action=compress na żywym DA.</t>
         </is>
       </c>
       <c r="P76" s="10" t="inlineStr">
@@ -6731,31 +6731,31 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>PB-08</t>
+          <t>NODE-03</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
+          <t>Pojemność węzła nigdy się nie odświeża</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F77" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G77" s="10" t="n">
         <v>14</v>
@@ -6777,12 +6777,12 @@
       </c>
       <c r="K77" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L77" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-09-23 D1: verris-lve.sh node_capacity (nproc, MemTotal, df /) w każdym raporcie, lve-agent/1.1; telemetry.dto NodeStatusDto.totalCpuCores/totalMemoryMb/totalDiskMb; telemetry.service aktualizuje Server; test telemetry/pojemnosc-wezla.spec.ts</t>
         </is>
       </c>
       <c r="M77" s="11" t="inlineStr">
@@ -6792,12 +6792,12 @@
       </c>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Pojemność węzła nigdy się nie odświeża. `totalCpuCores`/`totalMemoryMb`/`totalDiskMb` ustawiane wyłącznie w handshake; telemetria ich nie aktualizuje — mimo komentarza w schemacie „reported via handshake / heartbeat”. Rozbudowa węzła nie dociera do `NodeSelector`. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Telemetria aktualizuje totalCpuCores/totalMemoryMb/totalDiskMb, nie tylko handshake. | Stary agent bez pól niczego nie zeruje. OTWARTE do D3 (PB-21): raport z agenta na żywym węźle i odświeżona pojemność w panelu admina. | 2026-09-25: pojemność z agenta trafia też do planera pojemności (admin → Product Ops): ryzyko liczone względem rdzeni i RAM węzła (CPU 2×/4× rdzeni, RAM 1×/1,5×; test ryzyko-pojemnosci.spec.ts), a opis „CPU 250%” zastąpiony „przydzielone limity: CPU 2,5 rdz. z N · RAM x z y GB” — wcześniej wyglądało jak zużycie ponad 100%.</t>
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr">
@@ -6809,12 +6809,12 @@
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>PB-27</t>
+          <t>PB-08</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
+          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
@@ -6829,11 +6829,11 @@
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G78" s="10" t="n">
         <v>14</v>
@@ -6870,12 +6870,12 @@
       </c>
       <c r="N78" s="11" t="inlineStr">
         <is>
-          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
+          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
         </is>
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr">
@@ -6887,12 +6887,12 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>PB-28</t>
+          <t>PB-27</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Rozliczenie poza Verris (całe konto)</t>
+          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
@@ -6911,7 +6911,7 @@
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G79" s="10" t="n">
         <v>14</v>
@@ -6948,12 +6948,12 @@
       </c>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
+          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
         </is>
       </c>
       <c r="O79" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P79" s="10" t="inlineStr">
@@ -6965,58 +6965,58 @@
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>X-41</t>
+          <t>PB-28</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
+          <t>Rozliczenie poza Verris (całe konto)</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E80" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H80" s="10" t="inlineStr">
         <is>
-          <t>Faza 3 — Wejście na rynek</t>
+          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
         </is>
       </c>
       <c r="I80" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J80" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K80" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L80" s="11" t="inlineStr">
         <is>
-          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M80" s="11" t="inlineStr">
@@ -7026,12 +7026,12 @@
       </c>
       <c r="N80" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
         </is>
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
+          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr">
@@ -7043,12 +7043,12 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>X-41</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
+          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
@@ -7094,7 +7094,7 @@
       </c>
       <c r="L81" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
+          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
         </is>
       </c>
       <c r="M81" s="11" t="inlineStr">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr">
@@ -7121,31 +7121,31 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>PB-22</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
+          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E82" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F82" s="10" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G82" s="10" t="n">
         <v>15</v>
@@ -7167,12 +7167,12 @@
       </c>
       <c r="K82" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
         </is>
       </c>
       <c r="M82" s="11" t="inlineStr">
@@ -7182,12 +7182,12 @@
       </c>
       <c r="N82" s="11" t="inlineStr">
         <is>
-          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O82" s="11" t="inlineStr">
         <is>
-          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr">
@@ -7199,34 +7199,34 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>PB-22</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Log egressu jest próbką, nie zapisem</t>
+          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F83" s="10" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G83" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H83" s="10" t="inlineStr">
         <is>
@@ -7235,22 +7235,22 @@
       </c>
       <c r="I83" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="J83" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="K83" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M83" s="11" t="inlineStr">
@@ -7260,12 +7260,12 @@
       </c>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
         </is>
       </c>
       <c r="O83" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
+          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr">
@@ -7277,12 +7277,12 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
+          <t>Log egressu jest próbką, nie zapisem</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -7323,12 +7323,12 @@
       </c>
       <c r="K84" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
@@ -7338,12 +7338,12 @@
       </c>
       <c r="N84" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O84" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr">
@@ -7355,12 +7355,12 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Tryb `--strict` jest atrapą</t>
+          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -7379,7 +7379,7 @@
         </is>
       </c>
       <c r="F85" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G85" s="10" t="n">
         <v>16</v>
@@ -7406,7 +7406,7 @@
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
+          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M85" s="11" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="O85" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr">
@@ -7433,12 +7433,12 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
+          <t>Tryb `--strict` jest atrapą</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -7479,12 +7479,12 @@
       </c>
       <c r="K86" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
+          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr">
@@ -7494,12 +7494,12 @@
       </c>
       <c r="N86" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O86" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr">
@@ -7511,12 +7511,12 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
+          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -7531,11 +7531,11 @@
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F87" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G87" s="10" t="n">
         <v>16</v>
@@ -7562,7 +7562,7 @@
       </c>
       <c r="L87" s="11" t="inlineStr">
         <is>
-          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
+          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
         </is>
       </c>
       <c r="M87" s="11" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="O87" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr">
@@ -7589,31 +7589,31 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>PB-23</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
+          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>16</v>
@@ -7635,12 +7635,12 @@
       </c>
       <c r="K88" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
         </is>
       </c>
       <c r="M88" s="11" t="inlineStr">
@@ -7650,12 +7650,12 @@
       </c>
       <c r="N88" s="11" t="inlineStr">
         <is>
-          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O88" s="11" t="inlineStr">
         <is>
-          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr">
@@ -7667,34 +7667,34 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>PB-23</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Podpisane DPA z subprocesorami (część)</t>
+          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G89" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H89" s="10" t="inlineStr">
         <is>
@@ -7703,22 +7703,22 @@
       </c>
       <c r="I89" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="J89" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="K89" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L89" s="11" t="inlineStr">
         <is>
-          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M89" s="11" t="inlineStr">
@@ -7728,12 +7728,12 @@
       </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
         </is>
       </c>
       <c r="O89" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
+          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr">
@@ -7745,31 +7745,31 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>PB-03</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Finalizacja dokumentów prawnych 1.0.0</t>
+          <t>Podpisane DPA z subprocesorami (część)</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>17</v>
@@ -7791,12 +7791,12 @@
       </c>
       <c r="K90" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L90" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
         </is>
       </c>
       <c r="M90" s="11" t="inlineStr">
@@ -7806,12 +7806,12 @@
       </c>
       <c r="N90" s="11" t="inlineStr">
         <is>
-          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7823,12 +7823,12 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>PB-04</t>
+          <t>PB-03</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
+          <t>Finalizacja dokumentów prawnych 1.0.0</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
@@ -7843,11 +7843,11 @@
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G91" s="10" t="n">
         <v>17</v>
@@ -7884,12 +7884,12 @@
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
+          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
+          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7901,34 +7901,34 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>N-16</t>
+          <t>PB-04</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>SLA z zapisanymi kredytami</t>
+          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H92" s="10" t="inlineStr">
         <is>
@@ -7937,37 +7937,37 @@
       </c>
       <c r="I92" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-21</t>
         </is>
       </c>
       <c r="J92" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="K92" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L92" s="11" t="inlineStr">
         <is>
-          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M92" s="11" t="inlineStr">
         <is>
-          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
+          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>N-16</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>SLA z zapisanymi kredytami</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
@@ -8025,27 +8025,27 @@
       </c>
       <c r="K93" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L93" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
         </is>
       </c>
       <c r="M93" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
         </is>
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8057,31 +8057,31 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>PB-07</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Treści i cennik na verris.pl</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>18</v>
@@ -8103,27 +8103,27 @@
       </c>
       <c r="K94" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M94" s="11" t="inlineStr">
         <is>
-          <t>PB-01 (cennik zależy od unit economics)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8135,12 +8135,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>PB-11</t>
+          <t>PB-07</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
+          <t>Treści i cennik na verris.pl</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8159,7 +8159,7 @@
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G95" s="10" t="n">
         <v>18</v>
@@ -8191,17 +8191,17 @@
       </c>
       <c r="M95" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-01 (cennik zależy od unit economics)</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
+          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
+          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,12 +8213,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>PB-21</t>
+          <t>PB-11</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>DNS platformy i poczty na serwerze testowym</t>
+          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8237,7 +8237,7 @@
         </is>
       </c>
       <c r="F96" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G96" s="10" t="n">
         <v>18</v>
@@ -8274,12 +8274,12 @@
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
+          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
+          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,12 +8291,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-24</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8315,7 +8315,7 @@
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>18</v>
@@ -8352,12 +8352,12 @@
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8369,12 +8369,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-25</t>
+          <t>PB-24</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>White label na węźle — klient nie widzi DirectAdmina</t>
+          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8393,7 +8393,7 @@
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G98" s="10" t="n">
         <v>18</v>
@@ -8430,12 +8430,12 @@
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
+          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
+          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8447,12 +8447,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-25</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>White label na węźle — klient nie widzi DirectAdmina</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8471,10 +8471,10 @@
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G99" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H99" s="10" t="inlineStr">
         <is>
@@ -8483,12 +8483,12 @@
       </c>
       <c r="I99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K99" s="10" t="inlineStr">
@@ -8503,17 +8503,17 @@
       </c>
       <c r="M99" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
+          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8525,12 +8525,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8545,7 +8545,7 @@
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F100" s="10" t="n">
@@ -8581,17 +8581,17 @@
       </c>
       <c r="M100" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8603,12 +8603,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8627,7 +8627,7 @@
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G101" s="10" t="n">
         <v>19</v>
@@ -8664,12 +8664,12 @@
       </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8681,12 +8681,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8705,20 +8705,24 @@
         </is>
       </c>
       <c r="F102" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G102" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H102" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H102" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I102" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J102" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K102" s="10" t="inlineStr">
@@ -8733,17 +8737,17 @@
       </c>
       <c r="M102" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8755,69 +8759,69 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G103" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H103" s="10" t="inlineStr"/>
       <c r="I103" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J103" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K103" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L103" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M103" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N103" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8829,12 +8833,12 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
@@ -8844,16 +8848,16 @@
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F104" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G104" s="10" t="n">
         <v>21</v>
@@ -8876,7 +8880,7 @@
       </c>
       <c r="L104" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M104" s="11" t="inlineStr">
@@ -8891,7 +8895,7 @@
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8903,12 +8907,12 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -8918,7 +8922,7 @@
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr">
@@ -8945,12 +8949,12 @@
       </c>
       <c r="K105" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L105" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M105" s="11" t="inlineStr">
@@ -8960,12 +8964,12 @@
       </c>
       <c r="N105" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O105" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr">
@@ -8977,12 +8981,12 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -8997,7 +9001,7 @@
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F106" s="10" t="n">
@@ -9024,7 +9028,7 @@
       </c>
       <c r="L106" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M106" s="11" t="inlineStr">
@@ -9039,7 +9043,7 @@
       </c>
       <c r="O106" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr">
@@ -9051,12 +9055,12 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -9066,12 +9070,12 @@
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F107" s="10" t="n">
@@ -9093,12 +9097,12 @@
       </c>
       <c r="K107" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L107" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M107" s="11" t="inlineStr">
@@ -9108,12 +9112,12 @@
       </c>
       <c r="N107" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O107" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr">
@@ -9125,31 +9129,31 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F108" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G108" s="10" t="n">
         <v>21</v>
@@ -9167,12 +9171,12 @@
       </c>
       <c r="K108" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L108" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>services.controller.ts:125</t>
         </is>
       </c>
       <c r="M108" s="11" t="inlineStr">
@@ -9182,12 +9186,12 @@
       </c>
       <c r="N108" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O108" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr">
@@ -9199,12 +9203,12 @@
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>PB-29</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C109" s="10" t="inlineStr">
@@ -9219,11 +9223,11 @@
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>KRYTYCZNY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F109" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G109" s="10" t="n">
         <v>21</v>
@@ -9256,12 +9260,12 @@
       </c>
       <c r="N109" s="11" t="inlineStr">
         <is>
-          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O109" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr">
@@ -9273,12 +9277,12 @@
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>PB-30</t>
+          <t>PB-29</t>
         </is>
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>Jeden plik wersji dla floty + test zgodności</t>
+          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
@@ -9293,7 +9297,7 @@
       </c>
       <c r="E110" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F110" s="10" t="n">
@@ -9330,12 +9334,12 @@
       </c>
       <c r="N110" s="11" t="inlineStr">
         <is>
-          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
+          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="O110" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
+          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr">
@@ -9347,12 +9351,12 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>PB-31</t>
+          <t>PB-30</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Pełna automatyzacja kreatora węzła</t>
+          <t>Jeden plik wersji dla floty + test zgodności</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
@@ -9371,7 +9375,7 @@
         </is>
       </c>
       <c r="F111" s="10" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G111" s="10" t="n">
         <v>21</v>
@@ -9404,12 +9408,12 @@
       </c>
       <c r="N111" s="11" t="inlineStr">
         <is>
-          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
+          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
         </is>
       </c>
       <c r="O111" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
+          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr">
@@ -9421,12 +9425,12 @@
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>PB-32</t>
+          <t>PB-31</t>
         </is>
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
-          <t>Aktualizacje węzłów falami</t>
+          <t>Pełna automatyzacja kreatora węzła</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -9441,11 +9445,11 @@
       </c>
       <c r="E112" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F112" s="10" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G112" s="10" t="n">
         <v>21</v>
@@ -9478,12 +9482,12 @@
       </c>
       <c r="N112" s="11" t="inlineStr">
         <is>
-          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
+          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
         </is>
       </c>
       <c r="O112" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
+          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
         </is>
       </c>
       <c r="P112" s="10" t="inlineStr">
@@ -9495,12 +9499,12 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>PB-33</t>
+          <t>PB-32</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>Wersje stosu floty w panelu + wyrównanie falą</t>
+          <t>Aktualizacje węzłów falami</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
@@ -9515,11 +9519,11 @@
       </c>
       <c r="E113" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F113" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G113" s="10" t="n">
         <v>21</v>
@@ -9552,12 +9556,12 @@
       </c>
       <c r="N113" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji w panelu → nowy węzeł instaluje ją, istniejące wyrównane falą; audyt zgodności zielony.</t>
+          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
         </is>
       </c>
       <c r="O113" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: strona „Wersje stosu floty” w panelu admina (DB, PHP, LiteSpeed, DirectAdmin) z dozwolonymi wartościami z oficjalnych list; zmiana obowiązuje nowe węzły od razu, „Wyrównaj flotę” aktualizuje istniejące falą (PHP/LiteSpeed przez CustomBuild, MariaDB po jednej wersji z kopią bazy — wymóg CloudLinux Governor). | 2026-09-26 ZROBIONE W KODZIE: manifest w bazie (StosWezlaService), strona Admin → Wersje stosu floty (dozwolone wartości z oficjalnych list, tabela zgodności), „Wyrównaj flotę” = fala z php1_release + łańcuch DB_UPGRADE krok po kroku z kopią; bootstrap i agent biorą manifest z bazy. Testy na PostgreSQL. Zostało: wyrównanie na węzłach (D3).</t>
+          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
         </is>
       </c>
       <c r="P113" s="10" t="inlineStr">
@@ -9569,12 +9573,12 @@
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>PB-35</t>
+          <t>PB-33</t>
         </is>
       </c>
       <c r="B114" s="11" t="inlineStr">
         <is>
-          <t>Automatyczna fala aktualizacji węzłów co tydzień</t>
+          <t>Wersje stosu floty w panelu + wyrównanie falą</t>
         </is>
       </c>
       <c r="C114" s="10" t="inlineStr">
@@ -9593,7 +9597,7 @@
         </is>
       </c>
       <c r="F114" s="10" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G114" s="10" t="n">
         <v>21</v>
@@ -9626,12 +9630,12 @@
       </c>
       <c r="N114" s="11" t="inlineStr">
         <is>
-          <t>Fala startuje sama w oknie; zatrzymanie widoczne w powiadomieniach admina.</t>
+          <t>Zmiana wersji w panelu → nowy węzeł instaluje ją, istniejące wyrównane falą; audyt zgodności zielony.</t>
         </is>
       </c>
       <c r="O114" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: fala rusza sama we wtorki o 4:00 (kanarek → reszta po jednym, błąd zatrzymuje, powiadomienie). Węzły same już niczego nie instalują (dnf-automatic tylko pobiera). | 2026-09-26 ZROBIONE W KODZIE: FalaTygodniowaScheduler (wtorek 4:00 Europe/Warsaw), zatrzymanie fali → powiadomienie adminów. Test na PostgreSQL.</t>
+          <t>Decyzja właściciela 2026-09-26: strona „Wersje stosu floty” w panelu admina (DB, PHP, LiteSpeed, DirectAdmin) z dozwolonymi wartościami z oficjalnych list; zmiana obowiązuje nowe węzły od razu, „Wyrównaj flotę” aktualizuje istniejące falą (PHP/LiteSpeed przez CustomBuild, MariaDB po jednej wersji z kopią bazy — wymóg CloudLinux Governor). | 2026-09-26 ZROBIONE W KODZIE: manifest w bazie (StosWezlaService), strona Admin → Wersje stosu floty (dozwolone wartości z oficjalnych list, tabela zgodności), „Wyrównaj flotę” = fala z php1_release + łańcuch DB_UPGRADE krok po kroku z kopią; bootstrap i agent biorą manifest z bazy. Testy na PostgreSQL. Zostało: wyrównanie na węzłach (D3).</t>
         </is>
       </c>
       <c r="P114" s="10" t="inlineStr">
@@ -9643,12 +9647,12 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>PB-36</t>
+          <t>PB-35</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>Podpisane skrypty węzła i klucz SSH ograniczony do control-plane</t>
+          <t>Automatyczna fala aktualizacji węzłów co tydzień</t>
         </is>
       </c>
       <c r="C115" s="10" t="inlineStr">
@@ -9663,11 +9667,11 @@
       </c>
       <c r="E115" s="10" t="inlineStr">
         <is>
-          <t>KRYTYCZNY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F115" s="10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G115" s="10" t="n">
         <v>21</v>
@@ -9700,12 +9704,12 @@
       </c>
       <c r="N115" s="11" t="inlineStr">
         <is>
-          <t>Niepodpisany/zmieniony skrypt odrzucony przez węzeł; authorized_keys zawiera tylko aktualny klucz z ograniczeniem IP.</t>
+          <t>Fala startuje sama w oknie; zatrzymanie widoczne w powiadomieniach admina.</t>
         </is>
       </c>
       <c r="O115" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: przed startem. Węzeł uruchamia tylko skrypty podpisane kluczem Verris (przejęte API nie daje roota na flocie); klucz SSH z from= na IP control-plane, stare klucze usuwane (dziś agent co minutę tylko dopisuje klucz). | 2026-09-26 ZROBIONE W KODZIE: podpis Ed25519 każdej odpowiedzi GET /agent/tasks/* (skrypty zadań, pakiety onboardu i strony domyślnej, manifest stosu, konfiguracja kopii, zlecenia, klucz deploy) — podpis obejmuje ścieżkę, id węzła, czas i SHA-256 treści (bez podmiany, przeniesienia na inną ścieżkę/węzeł, powtórki po 5 min). Węzeł pobiera wyłącznie przez /usr/local/bin/verris-fetch (openssl pkeyutl -verify), klucz publiczny przywozi bootstrap / instalacja agenta. Klucz deploy: jeden wpis from="VERRIS_CONTROL_PLANE_IPS" bez przekierowań, poprzedni usuwany (rotacja). API w produkcji nie wystartuje bez VERRIS_SCRIPT_SIGNING_KEY albo z kluczem deploy bez adresów control-plane. Test: prawdziwy verris-fetch vs serwer podpisujący (zmieniona treść / inna ścieżka / inny węzeł / stary podpis / brak podpisu → odrzucone) + smoke na lokalnym API. Do sprawdzenia na D3: openssl na CloudLinux 9, rotacja klucza deploy.</t>
+          <t>Decyzja właściciela 2026-09-26: fala rusza sama we wtorki o 4:00 (kanarek → reszta po jednym, błąd zatrzymuje, powiadomienie). Węzły same już niczego nie instalują (dnf-automatic tylko pobiera). | 2026-09-26 ZROBIONE W KODZIE: FalaTygodniowaScheduler (wtorek 4:00 Europe/Warsaw), zatrzymanie fali → powiadomienie adminów. Test na PostgreSQL.</t>
         </is>
       </c>
       <c r="P115" s="10" t="inlineStr">
@@ -9717,12 +9721,12 @@
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>PB-26</t>
+          <t>PB-36</t>
         </is>
       </c>
       <c r="B116" s="11" t="inlineStr">
         <is>
-          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
+          <t>Podpisane skrypty węzła i klucz SSH ograniczony do control-plane</t>
         </is>
       </c>
       <c r="C116" s="10" t="inlineStr">
@@ -9737,24 +9741,24 @@
       </c>
       <c r="E116" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F116" s="10" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G116" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H116" s="10" t="inlineStr"/>
       <c r="I116" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J116" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K116" s="10" t="inlineStr">
@@ -9774,12 +9778,12 @@
       </c>
       <c r="N116" s="11" t="inlineStr">
         <is>
-          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
+          <t>Niepodpisany/zmieniony skrypt odrzucony przez węzeł; authorized_keys zawiera tylko aktualny klucz z ograniczeniem IP.</t>
         </is>
       </c>
       <c r="O116" s="11" t="inlineStr">
         <is>
-          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
+          <t>Decyzja właściciela 2026-09-26: przed startem. Węzeł uruchamia tylko skrypty podpisane kluczem Verris (przejęte API nie daje roota na flocie); klucz SSH z from= na IP control-plane, stare klucze usuwane (dziś agent co minutę tylko dopisuje klucz). | 2026-09-26 ZROBIONE W KODZIE: podpis Ed25519 każdej odpowiedzi GET /agent/tasks/* (skrypty zadań, pakiety onboardu i strony domyślnej, manifest stosu, konfiguracja kopii, zlecenia, klucz deploy) — podpis obejmuje ścieżkę, id węzła, czas i SHA-256 treści (bez podmiany, przeniesienia na inną ścieżkę/węzeł, powtórki po 5 min). Węzeł pobiera wyłącznie przez /usr/local/bin/verris-fetch (openssl pkeyutl -verify), klucz publiczny przywozi bootstrap / instalacja agenta. Klucz deploy: jeden wpis from="VERRIS_CONTROL_PLANE_IPS" bez przekierowań, poprzedni usuwany (rotacja). API w produkcji nie wystartuje bez VERRIS_SCRIPT_SIGNING_KEY albo z kluczem deploy bez adresów control-plane. Test: prawdziwy verris-fetch vs serwer podpisujący (zmieniona treść / inna ścieżka / inny węzeł / stary podpis / brak podpisu → odrzucone) + smoke na lokalnym API. Do sprawdzenia na D3: openssl na CloudLinux 9, rotacja klucza deploy.</t>
         </is>
       </c>
       <c r="P116" s="10" t="inlineStr">
@@ -9791,12 +9795,12 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-26</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
         </is>
       </c>
       <c r="C117" s="10" t="inlineStr">
@@ -9811,11 +9815,11 @@
       </c>
       <c r="E117" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F117" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G117" s="10" t="n">
         <v>22</v>
@@ -9843,17 +9847,17 @@
       </c>
       <c r="M117" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N117" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
         </is>
       </c>
       <c r="O117" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr">
@@ -9865,12 +9869,12 @@
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B118" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
@@ -9889,7 +9893,7 @@
         </is>
       </c>
       <c r="F118" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G118" s="10" t="n">
         <v>22</v>
@@ -9917,28 +9921,102 @@
       </c>
       <c r="M118" s="11" t="inlineStr">
         <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N118" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O118" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P118" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G119" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H119" s="10" t="inlineStr"/>
+      <c r="I119" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J119" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K119" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L119" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M119" s="11" t="inlineStr">
+        <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N118" s="11" t="inlineStr">
+      <c r="N119" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O118" s="11" t="inlineStr">
+      <c r="O119" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P118" s="10" t="inlineStr">
+      <c r="P119" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P118"/>
-  <conditionalFormatting sqref="E2:E118">
+  <autoFilter ref="A1:P119"/>
+  <conditionalFormatting sqref="E2:E119">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -9958,7 +10036,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P118">
+  <conditionalFormatting sqref="P2:P119">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -10068,11 +10146,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A2,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A2,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -10113,11 +10191,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A3,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A3,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -10158,11 +10236,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A4,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A4,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -10203,11 +10281,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A5,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A5,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -10248,11 +10326,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A6,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A6,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -10293,11 +10371,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A7,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A7,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -10338,11 +10416,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A8,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A8,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -10383,11 +10461,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A9,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A9,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -10428,11 +10506,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A10,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A10,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -10473,11 +10551,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A11,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A11,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -10518,11 +10596,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A12,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A12,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -10563,11 +10641,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A13,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A13,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -10608,11 +10686,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A14,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A14,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -10653,11 +10731,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A15,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A15,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -10698,11 +10776,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A16,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A16,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -10743,11 +10821,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A17,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A17,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -10788,11 +10866,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A18,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A18,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -10833,11 +10911,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A19,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A19,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -10878,11 +10956,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A20,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A20,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -10919,11 +10997,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A21,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A21,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -10960,11 +11038,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A22,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A22,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -11001,11 +11079,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A23,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A23,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">
@@ -11042,11 +11120,11 @@
         </is>
       </c>
       <c r="F24" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$118,A24)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A24)</f>
         <v/>
       </c>
       <c r="G24" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$118,A24,'Backlog do startu'!$F$2:$F$118)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A24,'Backlog do startu'!$F$2:$F$119)</f>
         <v/>
       </c>
       <c r="H24" s="10" t="n">

</xml_diff>

<commit_message>
chore(audyt): tablice po PB-38 fala 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$120</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$22</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$119)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$120)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$119,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$119,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$120,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$120,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$119,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$120,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$119,"zrobione",'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$120,"zrobione",'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P119"/>
+  <dimension ref="A1:P120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4937,34 +4937,34 @@
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>PB-38</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>Rekordy SPF — kreator</t>
+          <t>Najnowsze stabilne wersje narzędzi i bibliotek przed startem</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E54" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F54" s="10" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H54" s="10" t="inlineStr">
         <is>
@@ -4973,22 +4973,22 @@
       </c>
       <c r="I54" s="10" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J54" s="10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K54" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L54" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: deliverability/mail-auth.ts (buildMailAuthChecks) + deliverability.service.ts (strefa DA + delegacja NS); UI app/dashboard/email/deliverability-panel.tsx podpięty w MailTab (zakładka Poczta); test mail-auth.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M54" s="11" t="inlineStr">
@@ -4998,12 +4998,12 @@
       </c>
       <c r="N54" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Bramka (lint, typecheck, testy) i testy integracyjne zielone na nowych wersjach; obrazy budują się w CI; wdrożenie produkcyjne bez błędów; Dependabot i strażnik EOL działają.</t>
         </is>
       </c>
       <c r="O54" s="11" t="inlineStr">
         <is>
-          <t>deliverability-panel.tsx:26 to komponent osierocony — nikt go nie importuje | KOD: kreator pokazuje stan z publicznego DNS i gotowy rekord — „Dodaj/Zamień rekord w DNS” gdy domena na NS Verris, inaczej do skopiowania u dostawcy DNS. Zalecany SPF to `v=spf1 a mx ip4:&lt;IP węzła&gt; ~all`. ZNALEZISKO: dotychczasowa podpowiedź include:_spf.verris.pl odwołuje się do nieistniejącego rekordu (NXDOMAIN) → SPF permerror; usunięta z podpowiedzi, presetu DNS i artykułów KB, a kreator wykrywa ją u klientów. OTWARTE do D3 (węzeł): zapis rekordu przez CMD_API_DNS_CONTROL.</t>
+          <t>Decyzja właściciela 2026-09-26 (formularz): Node 24 teraz, 26 po wejściu w LTS; TypeScript 6.0 teraz, 7.x gdy typescript-eslint go obsłuży; MinIO zostaje do węzła testowego (potem Hetzner Object Storage); Dependabot + raport w tablicy. Fala 1: Node 24, TS 6, pnpm 12, Debian 13, łatki (Next 16.3.6, Payload 3.90). Fala 2: NestJS 12, ESLint 10, SimpleWebAuthn 14, GraphQL 17. Fala 3: Postgres 18 (procedura z kopią), Redis 8, monitoring. Fala 4: Dependabot, strażnik EOL w CI, kafelek wersji.</t>
         </is>
       </c>
       <c r="P54" s="10" t="inlineStr">
@@ -5015,12 +5015,12 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>E-16</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Rekordy DKIM — konfiguracja</t>
+          <t>Rekordy SPF — kreator</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -5066,12 +5066,12 @@
       </c>
       <c r="L55" s="11" t="inlineStr">
         <is>
-          <t>deliverability/mail-auth.ts (akcja enable-dkim); servers/directadmin.service.ts enableHostingDkim; POST /services/:id/hosting-email/dkim; email/deliverability-panel.tsx; testy mail-auth.spec.ts, directadmin.narzedzia.spec.ts</t>
+          <t>2026-09-23 D1: deliverability/mail-auth.ts (buildMailAuthChecks) + deliverability.service.ts (strefa DA + delegacja NS); UI app/dashboard/email/deliverability-panel.tsx podpięty w MailTab (zakładka Poczta); test mail-auth.spec.ts</t>
         </is>
       </c>
       <c r="M55" s="11" t="inlineStr">
         <is>
-          <t>E-15 (ten sam panel dostarczalności)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N55" s="11" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O55" s="11" t="inlineStr">
         <is>
-          <t>j.w. | KOD: DKIM odczytywany ze strefy DA (DA dopisuje klucz sam przy włączonym DKIM). Brak klucza = link do zgłoszenia. OTWARTE: włączanie DKIM z panelu (komenda DA niepotwierdzona bez węzła) — D3 w sprincie 18. | 2026-09-25: KOD (D2) — „Włącz DKIM dla &lt;domena&gt;” w sekcji Dostarczalność zamiast „napisz zgłoszenie”. Komenda DA potwierdzona w dokumentacji (changelog 1.57.2): CMD_API_EMAIL_POP action=set_dkim&amp;domain=…&amp;enable=… — DA tworzy klucze i dopisuje rekord TXT do strefy. Tylko domena z konta usługi, konto zawieszone bez zmian, wpis w dzienniku (HOSTING_DKIM_ENABLED). Wyłączenia celowo brak: ponowne włączenie generuje nowe klucze i rekord u zewnętrznego DNS przestałby pasować. Przy DNS u innego dostawcy panel po włączeniu pokazuje rekord do skopiowania (istniejąca ścieżka „klucz w strefie”). D3: pierwsze włączenie na węźle. | 2026-09-25 (dokumentacja DirectAdmin „Exim → DKIM”): dkim=2 udostępnia włączanie DKIM użytkownikom per domena, dkim=1 generuje klucze automatycznie przy tworzeniu domeny (tylko gdy DNS jest lokalny). Profil węzła ustawia dkim=1 — przycisk w panelu pojawia się tylko dla domen bez klucza. D3 ma potwierdzić, że set_dkim działa przy dkim=1; jeśli nie — alternatywa z dokumentacji: scripts/dkim_create.sh &lt;domena&gt; po stronie węzła (zadanie agenta).</t>
+          <t>deliverability-panel.tsx:26 to komponent osierocony — nikt go nie importuje | KOD: kreator pokazuje stan z publicznego DNS i gotowy rekord — „Dodaj/Zamień rekord w DNS” gdy domena na NS Verris, inaczej do skopiowania u dostawcy DNS. Zalecany SPF to `v=spf1 a mx ip4:&lt;IP węzła&gt; ~all`. ZNALEZISKO: dotychczasowa podpowiedź include:_spf.verris.pl odwołuje się do nieistniejącego rekordu (NXDOMAIN) → SPF permerror; usunięta z podpowiedzi, presetu DNS i artykułów KB, a kreator wykrywa ją u klientów. OTWARTE do D3 (węzeł): zapis rekordu przez CMD_API_DNS_CONTROL.</t>
         </is>
       </c>
       <c r="P55" s="10" t="inlineStr">
@@ -5093,12 +5093,12 @@
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>E-17</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>Rekord DMARC — konfiguracja</t>
+          <t>Rekordy DKIM — konfiguracja</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -5144,12 +5144,12 @@
       </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: mail-auth.ts dmarcCheck (brak / p=none / kilka rekordów) + lib/dmarc.ts tuneDmarc (polityka + adres raportów) w deliverability-panel.tsx; testy mail-auth.spec.ts, dmarc.spec.ts</t>
+          <t>deliverability/mail-auth.ts (akcja enable-dkim); servers/directadmin.service.ts enableHostingDkim; POST /services/:id/hosting-email/dkim; email/deliverability-panel.tsx; testy mail-auth.spec.ts, directadmin.narzedzia.spec.ts</t>
         </is>
       </c>
       <c r="M56" s="11" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>E-15 (ten sam panel dostarczalności)</t>
         </is>
       </c>
       <c r="N56" s="11" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="O56" s="11" t="inlineStr">
         <is>
-          <t>j.w. | KOD: kreator DMARC — wybór polityki i opcjonalny adres raportów, zachowuje pozostałe tagi. Sugestia bez rua na verris.pl (raporty do obcej domeny wymagają rekordu autoryzacji). OTWARTE do D3: zapis do strefy DA.</t>
+          <t>j.w. | KOD: DKIM odczytywany ze strefy DA (DA dopisuje klucz sam przy włączonym DKIM). Brak klucza = link do zgłoszenia. OTWARTE: włączanie DKIM z panelu (komenda DA niepotwierdzona bez węzła) — D3 w sprincie 18. | 2026-09-25: KOD (D2) — „Włącz DKIM dla &lt;domena&gt;” w sekcji Dostarczalność zamiast „napisz zgłoszenie”. Komenda DA potwierdzona w dokumentacji (changelog 1.57.2): CMD_API_EMAIL_POP action=set_dkim&amp;domain=…&amp;enable=… — DA tworzy klucze i dopisuje rekord TXT do strefy. Tylko domena z konta usługi, konto zawieszone bez zmian, wpis w dzienniku (HOSTING_DKIM_ENABLED). Wyłączenia celowo brak: ponowne włączenie generuje nowe klucze i rekord u zewnętrznego DNS przestałby pasować. Przy DNS u innego dostawcy panel po włączeniu pokazuje rekord do skopiowania (istniejąca ścieżka „klucz w strefie”). D3: pierwsze włączenie na węźle. | 2026-09-25 (dokumentacja DirectAdmin „Exim → DKIM”): dkim=2 udostępnia włączanie DKIM użytkownikom per domena, dkim=1 generuje klucze automatycznie przy tworzeniu domeny (tylko gdy DNS jest lokalny). Profil węzła ustawia dkim=1 — przycisk w panelu pojawia się tylko dla domen bez klucza. D3 ma potwierdzić, że set_dkim działa przy dkim=1; jeśli nie — alternatywa z dokumentacji: scripts/dkim_create.sh &lt;domena&gt; po stronie węzła (zadanie agenta).</t>
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr">
@@ -5171,12 +5171,12 @@
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>E-05</t>
+          <t>E-17</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Zmiana quoty ISTNIEJĄCEJ skrzynki</t>
+          <t>Rekord DMARC — konfiguracja</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -5222,12 +5222,12 @@
       </c>
       <c r="L57" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/hosting-email/quota (ZmienRozmiarSkrzynkiDto 10–102400 MB) → directadmin.service changeHostingEmailQuota (CMD_API_POP action=modify bez passwd) + audyt HOSTING_EMAIL_QUOTA_CHANGED; UI MailTab — klik w rozmiar skrzynki</t>
+          <t>2026-09-23 D1: mail-auth.ts dmarcCheck (brak / p=none / kilka rekordów) + lib/dmarc.ts tuneDmarc (polityka + adres raportów) w deliverability-panel.tsx; testy mail-auth.spec.ts, dmarc.spec.ts</t>
         </is>
       </c>
       <c r="M57" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="N57" s="11" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="O57" s="11" t="inlineStr">
         <is>
-          <t>brak jakiejkolwiek ścieżki edycji — klient musi usunąć i odtworzyć skrzynkę | KOD: zmiana rozmiaru bez usuwania skrzynki. Przy okazji body tworzenia skrzynki i zmiany hasła dostały klasy DTO (wcześniej interfejs = zero walidacji na granicy zaufania). OTWARTE do D3: czy DA przy modify bez passwd zostawia hasło (komentarz ponytail).</t>
+          <t>j.w. | KOD: kreator DMARC — wybór polityki i opcjonalny adres raportów, zachowuje pozostałe tagi. Sugestia bez rua na verris.pl (raporty do obcej domeny wymagają rekordu autoryzacji). OTWARTE do D3: zapis do strefy DA.</t>
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr">
@@ -5249,12 +5249,12 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>M-26</t>
+          <t>E-05</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Usunięcie zapisanej karty przez klienta</t>
+          <t>Zmiana quoty ISTNIEJĄCEJ skrzynki</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
@@ -5295,12 +5295,12 @@
       </c>
       <c r="K58" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L58" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: DELETE /billing/payment-methods/:id (ParseUUIDPipe) → billing.service deleteMyPaymentMethod: Stripe detach, usunięcie wiersza, zerowanie karty domyślnej i auto-doładowania, audyt PAYMENT_METHOD_REMOVED; UI billing-extras-forms „Zapisane karty”; test usun-karte.spec.ts | 2026-09-23: zapis kart — billing.service handlePaymentMethodAttached/Detached (webhooki payment_method.attached/.detached, upsert po provider+providerRef, pierwsza karta domyślna); test D2 zapis-karty.spec.ts</t>
+          <t>2026-09-23 D1: POST /services/:id/hosting-email/quota (ZmienRozmiarSkrzynkiDto 10–102400 MB) → directadmin.service changeHostingEmailQuota (CMD_API_POP action=modify bez passwd) + audyt HOSTING_EMAIL_QUOTA_CHANGED; UI MailTab — klik w rozmiar skrzynki</t>
         </is>
       </c>
       <c r="M58" s="11" t="inlineStr">
@@ -5310,12 +5310,12 @@
       </c>
       <c r="N58" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O58" s="11" t="inlineStr">
         <is>
-          <t>wymóg konsumencki | KOD gotowy i przetestowany na atrapach. UWAGA: nic w API nie zapisuje dziś wierszy PaymentMethod (brak create/upsert) — lista kart jest zawsze pusta, więc usuwanie da się sprawdzić dopiero, gdy zapis kart zostanie podpięty (webhook Stripe po płatności kartą). | 2026-09-23: domknięty brakujący zapis — karta zapisana w Stripe (np. przy subskrypcji kartą) pojawia się w panelu, odpięta (także z dashboardu Stripe) znika i odpina się od auto-doładowania. WYMAGA OD WŁAŚCICIELA: dopisać zdarzenia payment_method.attached i payment_method.detached do endpointu webhooka w Stripe (DEPLOY.md, OPERATIONAL_CHECKLIST). Karty zapisane przed tą zmianą nie pojawią się wstecz. D3 przy pierwszej płatności kartą.</t>
+          <t>brak jakiejkolwiek ścieżki edycji — klient musi usunąć i odtworzyć skrzynkę | KOD: zmiana rozmiaru bez usuwania skrzynki. Przy okazji body tworzenia skrzynki i zmiany hasła dostały klasy DTO (wcześniej interfejs = zero walidacji na granicy zaufania). OTWARTE do D3: czy DA przy modify bez passwd zostawia hasło (komentarz ponytail).</t>
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr">
@@ -5327,58 +5327,58 @@
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>PB-17</t>
+          <t>M-26</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>Asystent v1: dymki, naprawy jednym kliknięciem, czat z danymi konta</t>
+          <t>Usunięcie zapisanej karty przez klienta</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G59" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
+          <t>Faza 1 — Rozliczenia i dowód odtworzenia</t>
         </is>
       </c>
       <c r="I59" s="10" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J59" s="10" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K59" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L59" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-09-23 D1: DELETE /billing/payment-methods/:id (ParseUUIDPipe) → billing.service deleteMyPaymentMethod: Stripe detach, usunięcie wiersza, zerowanie karty domyślnej i auto-doładowania, audyt PAYMENT_METHOD_REMOVED; UI billing-extras-forms „Zapisane karty”; test usun-karte.spec.ts | 2026-09-23: zapis kart — billing.service handlePaymentMethodAttached/Detached (webhooki payment_method.attached/.detached, upsert po provider+providerRef, pierwsza karta domyślna); test D2 zapis-karty.spec.ts</t>
         </is>
       </c>
       <c r="M59" s="11" t="inlineStr">
@@ -5388,12 +5388,12 @@
       </c>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>Co najmniej 5 reguł dymków z testami; każda naprawa ma cofnięcie i wpis audytu; czat odpowiada z kontekstem usługi; brak akcji destrukcyjnych w v1.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O59" s="11" t="inlineStr">
         <is>
-          <t>Dymki kontekstowe na regułach (bez kosztu AI): dysk, domena nie wskazuje na nas, SPF/DKIM, SSL wygasa, backup nieświeży — najwyżej jeden na ekran, „nie pokazuj więcej”. Naprawy jednym kliknięciem tylko dla akcji odwracalnych, z kartą podglądu skutku i „Cofnij”. Obecny czat (HostingAssistant, RAG) dostaje odczyt danych konta. Każda akcja w audycie. Diagnoza i naprawy po naszej stronie za darmo.</t>
+          <t>wymóg konsumencki | KOD gotowy i przetestowany na atrapach. UWAGA: nic w API nie zapisuje dziś wierszy PaymentMethod (brak create/upsert) — lista kart jest zawsze pusta, więc usuwanie da się sprawdzić dopiero, gdy zapis kart zostanie podpięty (webhook Stripe po płatności kartą). | 2026-09-23: domknięty brakujący zapis — karta zapisana w Stripe (np. przy subskrypcji kartą) pojawia się w panelu, odpięta (także z dashboardu Stripe) znika i odpina się od auto-doładowania. WYMAGA OD WŁAŚCICIELA: dopisać zdarzenia payment_method.attached i payment_method.detached do endpointu webhooka w Stripe (DEPLOY.md, OPERATIONAL_CHECKLIST). Karty zapisane przed tą zmianą nie pojawią się wstecz. D3 przy pierwszej płatności kartą.</t>
         </is>
       </c>
       <c r="P59" s="10" t="inlineStr">
@@ -5405,12 +5405,12 @@
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>PB-18</t>
+          <t>PB-17</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>Tickety v2: podgląd klienta, szablony ze zmiennymi, szkice odpowiedzi</t>
+          <t>Asystent v1: dymki, naprawy jednym kliknięciem, czat z danymi konta</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
@@ -5429,10 +5429,10 @@
         </is>
       </c>
       <c r="F60" s="10" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G60" s="10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
@@ -5441,12 +5441,12 @@
       </c>
       <c r="I60" s="10" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="J60" s="10" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K60" s="10" t="inlineStr">
@@ -5466,12 +5466,12 @@
       </c>
       <c r="N60" s="11" t="inlineStr">
         <is>
-          <t>Podgląd klienta bez przechodzenia między ekranami; szablony podstawiają zmienne z testem; szkic odpowiedzi dla 6 kategorii (DNS, SSL, poczta, płatność, migracja, awaria).</t>
+          <t>Co najmniej 5 reguł dymków z testami; każda naprawa ma cofnięcie i wpis audytu; czat odpowiada z kontekstem usługi; brak akcji destrukcyjnych w v1.</t>
         </is>
       </c>
       <c r="O60" s="11" t="inlineStr">
         <is>
-          <t>Panel staff: boczny podgląd klienta w tickecie (usługi, saldo, faktury/dokumenty, zdarzenia, historia zgłoszeń, health score); szablony odpowiedzi ze zmiennymi (imię, domena, usługa, termin) i kategoriami — rozbudowa canned responses; klasyfikacja zgłoszenia i szkic odpowiedzi z bazy wiedzy i danych konta (do akceptacji, bez auto-wysyłki w v2); akcje z ticketu z audytem; licznik SLA.</t>
+          <t>Dymki kontekstowe na regułach (bez kosztu AI): dysk, domena nie wskazuje na nas, SPF/DKIM, SSL wygasa, backup nieświeży — najwyżej jeden na ekran, „nie pokazuj więcej”. Naprawy jednym kliknięciem tylko dla akcji odwracalnych, z kartą podglądu skutku i „Cofnij”. Obecny czat (HostingAssistant, RAG) dostaje odczyt danych konta. Każda akcja w audycie. Diagnoza i naprawy po naszej stronie za darmo.</t>
         </is>
       </c>
       <c r="P60" s="10" t="inlineStr">
@@ -5483,34 +5483,34 @@
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>A-25</t>
+          <t>PB-18</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Ręczne zawieszenie usługi przez operatora</t>
+          <t>Tickety v2: podgląd klienta, szablony ze zmiennymi, szkice odpowiedzi</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F61" s="10" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="G61" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
@@ -5519,22 +5519,22 @@
       </c>
       <c r="I61" s="10" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="J61" s="10" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="K61" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L61" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: admin-panel subscriptions/[id]/suspend-form.tsx + suspend-actions.ts → POST /admin/subscriptions/:id/suspend (powód, notatka, potwierdzenie)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M61" s="11" t="inlineStr">
@@ -5544,12 +5544,12 @@
       </c>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Podgląd klienta bez przechodzenia między ekranami; szablony podstawiają zmienne z testem; szkic odpowiedzi dla 6 kategorii (DNS, SSL, poczta, płatność, migracja, awaria).</t>
         </is>
       </c>
       <c r="O61" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: endpoint działa i jest osiągalny (curl + DirectAdmin), auto-suspend za brak płatności działa. Brakuje UI, nie możliwości zatrzymania szkody. | UI zrobione. OTWARTE do D3 (PB-21, serwer testowy): zawieszenie konta w DirectAdminie na żywym węźle.</t>
+          <t>Panel staff: boczny podgląd klienta w tickecie (usługi, saldo, faktury/dokumenty, zdarzenia, historia zgłoszeń, health score); szablony odpowiedzi ze zmiennymi (imię, domena, usługa, termin) i kategoriami — rozbudowa canned responses; klasyfikacja zgłoszenia i szkic odpowiedzi z bazy wiedzy i danych konta (do akceptacji, bez auto-wysyłki w v2); akcje z ticketu z audytem; licznik SLA.</t>
         </is>
       </c>
       <c r="P61" s="10" t="inlineStr">
@@ -5561,12 +5561,12 @@
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>A-26</t>
+          <t>A-25</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Ręczne odwieszenie usługi przez operatora</t>
+          <t>Ręczne zawieszenie usługi przez operatora</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -5612,12 +5612,12 @@
       </c>
       <c r="L62" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: ten sam formularz — odwieszenie z opcją obciążenia za odnowienie (chargeRenewal)</t>
+          <t>2026-09-23 D1: admin-panel subscriptions/[id]/suspend-form.tsx + suspend-actions.ts → POST /admin/subscriptions/:id/suspend (powód, notatka, potwierdzenie)</t>
         </is>
       </c>
       <c r="M62" s="11" t="inlineStr">
         <is>
-          <t>A-25 (ten sam widok)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N62" s="11" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="O62" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: jak A-25, endpoint subscriptions.admin.controller.ts:210 działa z chargeRenewal. | UI zrobione. OTWARTE do D3 (PB-21): odwieszenie konta w DA na żywym węźle.</t>
+          <t>Skorygowane: endpoint działa i jest osiągalny (curl + DirectAdmin), auto-suspend za brak płatności działa. Brakuje UI, nie możliwości zatrzymania szkody. | UI zrobione. OTWARTE do D3 (PB-21, serwer testowy): zawieszenie konta w DirectAdminie na żywym węźle.</t>
         </is>
       </c>
       <c r="P62" s="10" t="inlineStr">
@@ -5639,12 +5639,12 @@
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>N-07</t>
+          <t>A-26</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Ręczne tworzenie incydentu na status page</t>
+          <t>Ręczne odwieszenie usługi przez operatora</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -5654,7 +5654,7 @@
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E63" s="10" t="inlineStr">
@@ -5685,27 +5685,27 @@
       </c>
       <c r="K63" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L63" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D2: admin-panel status/incidents/incident-compose.tsx → POST /admin/product-ops/incidents; przycisk „Rozwiąż” (PATCH incidents/:id status=RESOLVED); probe-ingest.service.ts isManualIncident; test status/incydent-reczny.spec.ts</t>
+          <t>2026-09-23 D1: ten sam formularz — odwieszenie z opcją obciążenia za odnowienie (chargeRenewal)</t>
         </is>
       </c>
       <c r="M63" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A-25 (ten sam widok)</t>
         </is>
       </c>
       <c r="N63" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O63" s="11" t="inlineStr">
         <is>
-          <t>w kryzysie nie ma jak zakomunikować awarii | ZNALEZISKO: incydent ogłoszony ręcznie zamykał się sam przy pierwszej udanej próbie monitora (w ciągu minut), więc komunikat o awarii, której monitor nie widzi, znikał ze status page. Teraz zamyka go tylko operator; zamknięcie wysyła webhook INCIDENT_RESOLVED i trafia do audytu.</t>
+          <t>Skorygowane: jak A-25, endpoint subscriptions.admin.controller.ts:210 działa z chargeRenewal. | UI zrobione. OTWARTE do D3 (PB-21): odwieszenie konta w DA na żywym węźle.</t>
         </is>
       </c>
       <c r="P63" s="10" t="inlineStr">
@@ -5717,12 +5717,12 @@
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>N-14</t>
+          <t>N-07</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>Cordon wysyłki poczty (auto-blokada spamu)</t>
+          <t>Ręczne tworzenie incydentu na status page</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="L64" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: admin-panel /deliverability (Blokady wysyłki poczty, link w menu) → GET/POST /admin/deliverability/cordons; lista z e-mailem i nazwą klienta</t>
+          <t>2026-09-23 D2: admin-panel status/incidents/incident-compose.tsx → POST /admin/product-ops/incidents; przycisk „Rozwiąż” (PATCH incidents/:id status=RESOLVED); probe-ingest.service.ts isManualIncident; test status/incydent-reczny.spec.ts</t>
         </is>
       </c>
       <c r="M64" s="11" t="inlineStr">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="O64" s="11" t="inlineStr">
         <is>
-          <t>mechanizm działa, operator nie może go zobaczyć ani zdjąć | Operator widzi kogo i dlaczego zablokowano oraz zdejmuje blokadę (ADMIN, z potwierdzeniem, audyt po stronie API).</t>
+          <t>w kryzysie nie ma jak zakomunikować awarii | ZNALEZISKO: incydent ogłoszony ręcznie zamykał się sam przy pierwszej udanej próbie monitora (w ciągu minut), więc komunikat o awarii, której monitor nie widzi, znikał ze status page. Teraz zamyka go tylko operator; zamknięcie wysyła webhook INCIDENT_RESOLVED i trafia do audytu.</t>
         </is>
       </c>
       <c r="P64" s="10" t="inlineStr">
@@ -5795,12 +5795,12 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>H-22</t>
+          <t>N-14</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>Panel odtwarzania w widocznym miejscu</t>
+          <t>Cordon wysyłki poczty (auto-blokada spamu)</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -5810,7 +5810,7 @@
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E65" s="10" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="L65" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: client-panel BackupsTab.tsx — sekcja „Kopie poza serwerem” (HostingOffsitePanel) w zakładce Kopie zapasowe; zdublowany panel przywracania usunięty z Zużycia zasobów (hosting-backup-restore-panel.tsx)</t>
+          <t>2026-09-23: admin-panel /deliverability (Blokady wysyłki poczty, link w menu) → GET/POST /admin/deliverability/cordons; lista z e-mailem i nazwą klienta</t>
         </is>
       </c>
       <c r="M65" s="11" t="inlineStr">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="O65" s="11" t="inlineStr">
         <is>
-          <t>klient w kryzysie tego nie znajdzie | Kopie off-site są tam, gdzie klient ich szuka w kryzysie; przywracanie jest w jednym miejscu, z potwierdzeniem domeną.</t>
+          <t>mechanizm działa, operator nie może go zobaczyć ani zdjąć | Operator widzi kogo i dlaczego zablokowano oraz zdejmuje blokadę (ADMIN, z potwierdzeniem, audyt po stronie API).</t>
         </is>
       </c>
       <c r="P65" s="10" t="inlineStr">
@@ -5873,12 +5873,12 @@
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>H-09</t>
+          <t>H-22</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Kopia bezpieczeństwa przed odtworzeniem</t>
+          <t>Panel odtwarzania w widocznym miejscu</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -5900,7 +5900,7 @@
         <v>6</v>
       </c>
       <c r="G66" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H66" s="10" t="inlineStr">
         <is>
@@ -5909,22 +5909,22 @@
       </c>
       <c r="I66" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J66" s="10" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K66" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L66" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
+          <t>2026-09-23: client-panel BackupsTab.tsx — sekcja „Kopie poza serwerem” (HostingOffsitePanel) w zakładce Kopie zapasowe; zdublowany panel przywracania usunięty z Zużycia zasobów (hosting-backup-restore-panel.tsx)</t>
         </is>
       </c>
       <c r="M66" s="11" t="inlineStr">
@@ -5934,12 +5934,12 @@
       </c>
       <c r="N66" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O66" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: hosting-restore.service.ts:167 tylko KOLEJKUJE backup w DA i nie czeka na wynik — destrukcyjne odtworzenie rusza mimo nieudanej kopii. Job dostaje COMPLETED (:182) w chwili przyjęcia zadania, nie po odtworzeniu. | Naprawione: nadpisywanie danych bez siatki. Status COMPLETED w panelu klienta opisany uczciwie („Odtwarzanie zlecone — serwer odtwarza dane w tle”), bo DA przyjmuje odtworzenie asynchronicznie. OTWARTE do D3 (PB-21): pełny przebieg na żywym DA i wykrycie końca odtwarzania.</t>
+          <t>klient w kryzysie tego nie znajdzie | Kopie off-site są tam, gdzie klient ich szuka w kryzysie; przywracanie jest w jednym miejscu, z potwierdzeniem domeną.</t>
         </is>
       </c>
       <c r="P66" s="10" t="inlineStr">
@@ -5951,12 +5951,12 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>H-17</t>
+          <t>H-09</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>Tryb restore skryptu odtwarzającego osiągalny z produktu</t>
+          <t>Kopia bezpieczeństwa przed odtworzeniem</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -5997,27 +5997,27 @@
       </c>
       <c r="K67" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L67" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: produktowa ścieżka odtwarzania z off-site = „Pobierz na serwer” (fetch, agent) + przywrócenie z listy kopii z kopią bezpieczeństwa (H-09) i potwierdzeniem domeną; tryb `restore` skryptu (DA type=admin, bez kopii bezpieczeństwa) celowo zostaje tylko w CLI/runbooku DR</t>
+          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
         </is>
       </c>
       <c r="M67" s="11" t="inlineStr">
         <is>
-          <t>H-20 (najpierw potwierdzone odtworzenie, potem wystawienie trybu w produkcie)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N67" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O67" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: tryb restore jest martwy z poziomu produktu, ale żywy z CLI (node-account-restore.sh:120-124) i udokumentowany w runbooku. | DO DECYZJI WŁAŚCICIELA: proponuję zamknąć jako PARYTET przez równoważną ścieżkę produktową — wystawienie trybu `restore` ominęłoby kopię bezpieczeństwa z H-09. Tryb restore działa też tylko przy istniejącym koncie na węźle, czyli dokładnie tam, gdzie wystarcza fetch + przywrócenie. | DECYZJA WŁAŚCICIELA 2026-09-23: zamknięte jako PARYTET — ścieżka produktowa (pobierz na serwer + przywrócenie z kopią bezpieczeństwa i potwierdzeniem domeną) daje ten sam efekt bezpieczniej; tryb restore skryptu zostaje wyłącznie w CLI/runbooku DR.</t>
+          <t>OSŁABIONE: hosting-restore.service.ts:167 tylko KOLEJKUJE backup w DA i nie czeka na wynik — destrukcyjne odtworzenie rusza mimo nieudanej kopii. Job dostaje COMPLETED (:182) w chwili przyjęcia zadania, nie po odtworzeniu. | Naprawione: nadpisywanie danych bez siatki. Status COMPLETED w panelu klienta opisany uczciwie („Odtwarzanie zlecone — serwer odtwarza dane w tle”), bo DA przyjmuje odtworzenie asynchronicznie. OTWARTE do D3 (PB-21): pełny przebieg na żywym DA i wykrycie końca odtwarzania.</t>
         </is>
       </c>
       <c r="P67" s="10" t="inlineStr">
@@ -6029,12 +6029,12 @@
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>G-20</t>
+          <t>H-17</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>Ochrona przed atakiem słownikowym na panel</t>
+          <t>Tryb restore skryptu odtwarzającego osiągalny z produktu</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="E68" s="10" t="inlineStr">
@@ -6080,12 +6080,12 @@
       </c>
       <c r="L68" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D2: common/guards/rate-limit.guard.spec.ts (6 testów: limit per IP, per e-mail z wielu IP, reset okna, zakresy i @SkipRateLimit, przepełnienie mapy, awaria Redisa)</t>
+          <t>2026-09-23: produktowa ścieżka odtwarzania z off-site = „Pobierz na serwer” (fetch, agent) + przywrócenie z listy kopii z kopią bezpieczeństwa (H-09) i potwierdzeniem domeną; tryb `restore` skryptu (DA type=admin, bez kopii bezpieczeństwa) celowo zostaje tylko w CLI/runbooku DR</t>
         </is>
       </c>
       <c r="M68" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>H-20 (najpierw potwierdzone odtworzenie, potem wystawienie trybu w produkcie)</t>
         </is>
       </c>
       <c r="N68" s="11" t="inlineStr">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>brak dowodu D2 na krytycznym guardzie | ZNALEZISKO przy pisaniu testów: w trybie pamięciowym przepełnienie mapy (50 tys. kluczy) czyściło WSZYSTKIE liczniki — losowe e-maile zerowały licznik prób logowania do atakowanego konta (fail-open). Teraz usuwane są tylko wygasłe, a przy pełnej mapie nowe klucze dostają 429 (fail-closed).</t>
+          <t>Skorygowane: tryb restore jest martwy z poziomu produktu, ale żywy z CLI (node-account-restore.sh:120-124) i udokumentowany w runbooku. | DO DECYZJI WŁAŚCICIELA: proponuję zamknąć jako PARYTET przez równoważną ścieżkę produktową — wystawienie trybu `restore` ominęłoby kopię bezpieczeństwa z H-09. Tryb restore działa też tylko przy istniejącym koncie na węźle, czyli dokładnie tam, gdzie wystarcza fetch + przywrócenie. | DECYZJA WŁAŚCICIELA 2026-09-23: zamknięte jako PARYTET — ścieżka produktowa (pobierz na serwer + przywrócenie z kopią bezpieczeństwa i potwierdzeniem domeną) daje ten sam efekt bezpieczniej; tryb restore skryptu zostaje wyłącznie w CLI/runbooku DR.</t>
         </is>
       </c>
       <c r="P68" s="10" t="inlineStr">
@@ -6107,12 +6107,12 @@
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>I-11</t>
+          <t>G-20</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Staging — publikacja na produkcję</t>
+          <t>Ochrona przed atakiem słownikowym na panel</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E69" s="10" t="inlineStr">
@@ -6153,12 +6153,12 @@
       </c>
       <c r="K69" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L69" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
+          <t>2026-09-23 D2: common/guards/rate-limit.guard.spec.ts (6 testów: limit per IP, per e-mail z wielu IP, reset okna, zakresy i @SkipRateLimit, przepełnienie mapy, awaria Redisa)</t>
         </is>
       </c>
       <c r="M69" s="11" t="inlineStr">
@@ -6168,12 +6168,12 @@
       </c>
       <c r="N69" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O69" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: node-staging-sync.sh:141-142 backup plików jest twardą bramką, ale :152-153 backup bazy LIVE jest best-effort — linia 158 robi wp db import na produkcji mimo braku kopii. | Naprawione: import bazy staging na produkcję mimo braku kopii bazy LIVE. OTWARTE do D3 (PB-21): publikacja stagingu na żywym węźle.</t>
+          <t>brak dowodu D2 na krytycznym guardzie | ZNALEZISKO przy pisaniu testów: w trybie pamięciowym przepełnienie mapy (50 tys. kluczy) czyściło WSZYSTKIE liczniki — losowe e-maile zerowały licznik prób logowania do atakowanego konta (fail-open). Teraz usuwane są tylko wygasłe, a przy pełnej mapie nowe klucze dostają 429 (fail-closed).</t>
         </is>
       </c>
       <c r="P69" s="10" t="inlineStr">
@@ -6185,12 +6185,12 @@
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>X-31</t>
+          <t>I-11</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>Kanał alertów daje znak życia (dead man's switch)</t>
+          <t>Staging — publikacja na produkcję</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -6200,19 +6200,19 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F70" s="10" t="n">
         <v>6</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H70" s="10" t="inlineStr">
         <is>
@@ -6221,22 +6221,22 @@
       </c>
       <c r="I70" s="10" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="J70" s="10" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="K70" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L70" s="11" t="inlineStr">
         <is>
-          <t>ops/observability/grafana/provisioning/alerting/rules.yaml — grupa verris_kanal_alertow, reguła VerrisKanalAlertowZyje (vector(1), for: 0s, oba stany awaryjne na Alerting, etykieta kanal: heartbeat); policies.yaml — gałąź object_matchers kanal=heartbeat, repeat_interval 24h; apps/api/src/test/routing-alertow.spec.ts (5 asercji X-31); docs/ops/GRAFANA_ALERTING.md §4. BRAK: pierwszego maila [FIRING:1] VerrisKanalAlertowZyje — dowód D3 jeszcze nie powstał.</t>
+          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
         </is>
       </c>
       <c r="M70" s="11" t="inlineStr">
@@ -6246,12 +6246,12 @@
       </c>
       <c r="N70" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O70" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 powstanie przy pierwszym mailu. Decyzja właściciela produktu: wariant „jeden mail na dobę". | PROBLEM: po naprawie X-30 alerty ucichną, a cisza będzie znaczyła „nic się nie pali" — i będzie wyglądała IDENTYCZNIE jak: Grafana padła, Postfix przestał przyjmować, mail.hvln.pl zaczął odrzucać albo wrzucać do spamu, ktoś zmienił adres w punkcie kontaktowym, polityka przestała pasować do etykiet. To dokładnie ta sama cisza, która przez miesiąc znaczyła „kopia bazy jest w porządku" (H-23) i kosztowała wszystkie kopie zapasowe. | ROZWIĄZANIE: VerrisKanalAlertowZyje — reguła vector(1), pali się ZAWSZE, jej BRAK jest sygnałem. for: 0s, noDataState: Alerting, execErrState: Alerting — nie da się jej „nie zapalić": normalnie warunek jest spełniony, a gdyby źródło danych przestało odpowiadać, oba stany awaryjne też prowadzą do Alerting. Milczenie ma znaczyć awarię, nigdy spokój. | JEDEN MAIL NA DOBĘ, NIE SZEŚĆ: osobna gałąź polityki na etykiecie kanal: heartbeat z repeat_interval 24h. Na domyślnej (4h) byłoby sześć dziennie, a alert przychodzący sześć razy dziennie przestaje być czytany po tygodniu — wtedy przestaje cokolwiek dawać, bo jego BRAK jest jedyną informacją, jaką niesie. Strażnik pilnuje osobno, że polityka domyślna NIE została przy okazji przestawiona na dobę: prawdziwy alarm ma się przypominać co cztery godziny. | HACZYK, KTÓRY TRZEBA NAZWAĆ: mail, którego się nie czyta, wraca do punktu wyjścia. Jeśli po tygodniu przestanie być zauważany, reguła przestaje działać — nie dlatego, że jest zepsuta, tylko dlatego, że przestała być czytana. Tego nie da się naprawić kodem. | CZEGO NIE OBEJMUJE: awarii całego serwera (heartbeat mieszka na tej samej maszynie co Grafana i milczy razem z nią — odporny byłby watchdog SPOZA naszej infrastruktury, pukany cronem; nie ma go i to świadoma decyzja, nie przeoczenie) ani poprawności pozostałych reguł (tego pilnuje bramka z X-30). | Czerwieni się na starym kodzie: 5 z 36. | Doszła lista DOPISANE_POZNIEJ, trzymana osobno od ALERTY: tamta odpowiada na pytanie „czy migracja czegoś nie zgubiła" i ma zostać zamrożona, ta na „czy ktoś czegoś po cichu nie dołożył". Dokumentacja: docs/archiwum/zadania/X-31-znak-zycia-kanalu-alertow.md | 2026-09-22 D3: wlasciciel potwierdza, ze mail [FIRING:1] VerrisKanalAlertowZyje przychodzi codziennie. Kanal alertow dziala koniec-do-konca.</t>
+          <t>OSŁABIONE: node-staging-sync.sh:141-142 backup plików jest twardą bramką, ale :152-153 backup bazy LIVE jest best-effort — linia 158 robi wp db import na produkcji mimo braku kopii. | Naprawione: import bazy staging na produkcję mimo braku kopii bazy LIVE. OTWARTE do D3 (PB-21): publikacja stagingu na żywym węźle.</t>
         </is>
       </c>
       <c r="P70" s="10" t="inlineStr">
@@ -6263,12 +6263,12 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>X-32</t>
+          <t>X-31</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>Martwy job da się odrzucić z panelu, ze śladem w audycie</t>
+          <t>Kanał alertów daje znak życia (dead man's switch)</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="L71" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/common/audit/audit.actions.ts — PROVISIONING_JOB_DISCARDED_BY_ADMIN; provisioning-queue.service.ts — odrzucJob (getState() === failed, ślad przed job.remove(), audyt z subskrypcją, typem, liczbą prób, failedReason i powodem); provisioning-queue.admin.controller.ts — POST :id/odrzuc za @StaffPerm('PROVISIONING_MANAGE'); apps/admin-panel/.../provisioning-queue/ — actions.ts, odrzuc-button.tsx (dwa kliknięcia, powód ≥5 znaków, zdanie o nietkniętej subskrypcji), page.tsx; apps/api/src/test/odrzucenie-martwego-joba.spec.ts (13). BRAK: pierwszego odrzucenia na produkcji — dowód D3 jeszcze nie powstał.</t>
+          <t>ops/observability/grafana/provisioning/alerting/rules.yaml — grupa verris_kanal_alertow, reguła VerrisKanalAlertowZyje (vector(1), for: 0s, oba stany awaryjne na Alerting, etykieta kanal: heartbeat); policies.yaml — gałąź object_matchers kanal=heartbeat, repeat_interval 24h; apps/api/src/test/routing-alertow.spec.ts (5 asercji X-31); docs/ops/GRAFANA_ALERTING.md §4. BRAK: pierwszego maila [FIRING:1] VerrisKanalAlertowZyje — dowód D3 jeszcze nie powstał.</t>
         </is>
       </c>
       <c r="M71" s="11" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="O71" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 przy pierwszym odrzuceniu na produkcji — a to da się zrobić od razu po wdrożeniu, w odróżnieniu od Z-18, który czeka na węzeł. Decyzja właściciela produktu: dorobić akcję w panelu zamiast jednorazowego czyszczenia Redisa. | JAK TO WYSZŁO: X-30 naprawiło alerting, VerrisProvisioningQueueFailed zapalił się z prawdziwego powodu i wskazał cztery martwe joby (to z nich wyszło Z-18). Naturalny następny ruch — usunąć je — okazał się NIEWYKONALNY: panel ma przy nich wyłącznie „Retry", a kontroler administracyjny dokładnie dwa endpointy, listowanie i ponowienie. Retry nic nie daje, bo węzła nie ma: job padnie ponownie, podbije licznik prób i dołoży wpisy do audytu — cztery martwe joby zamieniają się w cztery martwe joby z dłuższą historią. Zostawało grzebanie w Redisie ręcznie, czyli zmiana stanu produkcyjnego dotyczącego subskrypcji klientów BEZ ŚLADU W AUDYCIE. | TO NIE JEST USTERKA TYCH CZTERECH JOBÓW, tylko luka w warstwie operatorskiej, która ujawni się ponownie przy pierwszym prawdziwym niepowodzeniu provisioningu — z tą różnicą, że wtedy po drugiej stronie będzie klient. | ROZWIĄZANIE: POST /admin/provisioning-queue/:id/odrzuc + przycisk „Odrzuć" obok Retry. TRZY REGUŁY: (1) TYLKO STAN failed — usunięcie joba aktywnego albo czekającego osierociłoby provisioning w trakcie, konto na węźle mogłoby powstać, a system przestałby o nim wiedzieć; ograniczenie siedzi w usłudze, nie w kontrolerze, bo to reguła o kolejce, nie o HTTP; (2) POWÓD WYMAGANY, tak samo jak przy retry — operacja bez powodu to operacja, której za pół roku nikt nie wyjaśni; (3) NAJPIERW ODCZYT, POTEM USUNIĘCIE — ślad zbierany PRZED job.remove(), bo po usunięciu nie ma już czego odczytać; zapisujemy subskrypcję, joba, typ, liczbę prób, ostatni błąd i powód. Po Z-18 ten ostatni błąd niesie PRAWDZIWĄ przyczynę, więc wpis ma realną wartość dowodową — jeszcze wczoraj zapisałby zdanie o brakującym pakiecie DirectAdmina, którego nigdy nie brakowało. | OSOBNA AKCJA AUDYTU (PROVISIONING_JOB_DISCARDED_BY_ADMIN), nie wariant retry: w raportach odrzucenie i ponowienie to dwie różne decyzje i nie wolno im się zlewać. | DWA KLIKNIĘCIA, NIE JEDNO: retry można cofnąć następnym retry, odrzucenia nie da się cofnąć wcale. Potwierdzenie jest po to, żeby ta różnica była wyczuwalna w palcach. | ZDANIE PRZY PRZYCISKU: „Usuwa wpis z kolejki bez możliwości cofnięcia. Subskrypcja zostaje nietknięta." Operator ma prawo założyć, że „odrzuć" anuluje zamówienie — nie anuluje. Musi to być napisane tam, gdzie się klika, a nie w dokumentacji, której nikt nie otworzy w trakcie incydentu. | Czerwieni się na starym kodzie: 11 z 13. | DWIE UWAGI O SAMYCH TESTACH: odczyty plików panelu są LENIWE, bo odczyt na poziomie describe wywalał cały plik testowy, zanim cokolwiek się policzyło — a wtedy nie wiadomo, ILE asercji się czerwieni, tylko że „nie skompilowało się"; asercja o warunku row.failedReason nie mierzy odległości w znakach, tylko relację między warunkiem a przyciskiem, bo wersja licząca znaki zepsuła się od dopisania komentarza i kusiło, żeby poszerzyć okno zamiast poprawić asercję — to byłoby naprawianie testu zamiast kodu. | CZEGO NIE OBEJMUJE: losu czterech subskrypcji, które dostały zwrot i status PENDING_PAYMENT (odrzucenie joba ich nie dotyka — osobne sprzątanie po stronie bazy); odrzucania hurtem — świadomie, bo przycisk „odrzuć wszystkie" jest wygodny dokładnie do momentu, w którym ktoś kliknie go na kolejce z prawdziwym zamówieniem. | JAK ZAMKNĄĆ: odrzucić jeden z czterech martwych jobów, obejrzeć wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie i sprawdzić, że verris_provisioning_queue_depth{state="failed"} spadło o jeden. Dokumentacja: docs/archiwum/zadania/X-32-odrzucenie-martwego-joba.md | 2026-09-22 D3: wlasciciel odrzucil martwy job przyciskiem 'Odrzuc' w panelu admina na produkcji (potwierdzenie wlasciciela; wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie).</t>
+          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 powstanie przy pierwszym mailu. Decyzja właściciela produktu: wariant „jeden mail na dobę". | PROBLEM: po naprawie X-30 alerty ucichną, a cisza będzie znaczyła „nic się nie pali" — i będzie wyglądała IDENTYCZNIE jak: Grafana padła, Postfix przestał przyjmować, mail.hvln.pl zaczął odrzucać albo wrzucać do spamu, ktoś zmienił adres w punkcie kontaktowym, polityka przestała pasować do etykiet. To dokładnie ta sama cisza, która przez miesiąc znaczyła „kopia bazy jest w porządku" (H-23) i kosztowała wszystkie kopie zapasowe. | ROZWIĄZANIE: VerrisKanalAlertowZyje — reguła vector(1), pali się ZAWSZE, jej BRAK jest sygnałem. for: 0s, noDataState: Alerting, execErrState: Alerting — nie da się jej „nie zapalić": normalnie warunek jest spełniony, a gdyby źródło danych przestało odpowiadać, oba stany awaryjne też prowadzą do Alerting. Milczenie ma znaczyć awarię, nigdy spokój. | JEDEN MAIL NA DOBĘ, NIE SZEŚĆ: osobna gałąź polityki na etykiecie kanal: heartbeat z repeat_interval 24h. Na domyślnej (4h) byłoby sześć dziennie, a alert przychodzący sześć razy dziennie przestaje być czytany po tygodniu — wtedy przestaje cokolwiek dawać, bo jego BRAK jest jedyną informacją, jaką niesie. Strażnik pilnuje osobno, że polityka domyślna NIE została przy okazji przestawiona na dobę: prawdziwy alarm ma się przypominać co cztery godziny. | HACZYK, KTÓRY TRZEBA NAZWAĆ: mail, którego się nie czyta, wraca do punktu wyjścia. Jeśli po tygodniu przestanie być zauważany, reguła przestaje działać — nie dlatego, że jest zepsuta, tylko dlatego, że przestała być czytana. Tego nie da się naprawić kodem. | CZEGO NIE OBEJMUJE: awarii całego serwera (heartbeat mieszka na tej samej maszynie co Grafana i milczy razem z nią — odporny byłby watchdog SPOZA naszej infrastruktury, pukany cronem; nie ma go i to świadoma decyzja, nie przeoczenie) ani poprawności pozostałych reguł (tego pilnuje bramka z X-30). | Czerwieni się na starym kodzie: 5 z 36. | Doszła lista DOPISANE_POZNIEJ, trzymana osobno od ALERTY: tamta odpowiada na pytanie „czy migracja czegoś nie zgubiła" i ma zostać zamrożona, ta na „czy ktoś czegoś po cichu nie dołożył". Dokumentacja: docs/archiwum/zadania/X-31-znak-zycia-kanalu-alertow.md | 2026-09-22 D3: wlasciciel potwierdza, ze mail [FIRING:1] VerrisKanalAlertowZyje przychodzi codziennie. Kanal alertow dziala koniec-do-konca.</t>
         </is>
       </c>
       <c r="P71" s="10" t="inlineStr">
@@ -6341,12 +6341,12 @@
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>X-32</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>W drzewie stoją dwa majory ESLinta naraz</t>
+          <t>Martwy job da się odrzucić z panelu, ze śladem w audycie</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -6361,7 +6361,7 @@
       </c>
       <c r="E72" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F72" s="10" t="n">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="L72" s="11" t="inlineStr">
         <is>
-          <t>package.json (korzeń) — @eslint/js ^10.0.1 przy braku jakiegokolwiek eslint.config.* w korzeniu; libs/eslint-config/node_modules: eslint 10.9.0 obok @eslint/js 9.39.5; apps/api, apps/www, apps/client-panel, apps/status-page, libs/directadmin-sdk — eslint 9.39.5 | 2026-09-23: z korzenia zdjęte nieużywane @eslint/js ^10 i typescript-eslint; libs/eslint-config peer eslint ^9.39.5 (było &gt;=9 → auto-install dociągał 10.9.0); lockfile bez eslint 10; strażnik apps/api/src/test/eslint-jeden-major.spec.ts (deklaracje + peer + lockfile)</t>
+          <t>apps/api/src/common/audit/audit.actions.ts — PROVISIONING_JOB_DISCARDED_BY_ADMIN; provisioning-queue.service.ts — odrzucJob (getState() === failed, ślad przed job.remove(), audyt z subskrypcją, typem, liczbą prób, failedReason i powodem); provisioning-queue.admin.controller.ts — POST :id/odrzuc za @StaffPerm('PROVISIONING_MANAGE'); apps/admin-panel/.../provisioning-queue/ — actions.ts, odrzuc-button.tsx (dwa kliknięcia, powód ≥5 znaków, zdanie o nietkniętej subskrypcji), page.tsx; apps/api/src/test/odrzucenie-martwego-joba.spec.ts (13). BRAK: pierwszego odrzucenia na produkcji — dowód D3 jeszcze nie powstał.</t>
         </is>
       </c>
       <c r="M72" s="11" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="O72" s="11" t="inlineStr">
         <is>
-          <t>Odkryte 2026-08-28 przy DEP-01. Korzeń deklaruje @eslint/js ^10.0.1, którego peer to eslint ^10.0.0 — i to on wciąga eslint@10.9.0 do drzewa. Tymczasem KAŻDY pakiet, który realnie lintuje, ma 9.39.5. Najostrzej widać to wewnątrz libs/eslint-config, czyli wspólnej konfiguracji: node_modules/eslint = 10.9.0, node_modules/@eslint/js = 9.39.5 — dwie połowy jednego narzędzia z różnych majorów w jednym katalogu. | Korzeń NIE MA żadnego eslint.config.* i nie odpala lintera (pnpm lint = turbo run lint), więc te zależności nie robią nic poza wciąganiem majora, którego nikt nie używa. | To nie awaria — bramka jest zielona, 0 błędów. To BRAK KONTROLI: żaden strażnik nie sprawdza, czy major ESLinta jest jeden, tak jak do ENV-01 nic nie sprawdzało wersji Node. | DO ZROBIENIA: zdjąć z korzenia nieużywane @eslint/js i typescript-eslint albo cofnąć je do dziewiątki (rusza lockfile — osobny commit z pełną bramką), plus strażnik spójności majora na wzór wersja-node.spec.ts. | 2026-09-23: zrobione zgodnie z DO ZROBIENIA; lockfile zmieniony wyłącznie o usunięcie gałęzi eslint 10 (pnpm 9.5.0 --lockfile-only). Przed bramką lokalną: pnpm install.</t>
+          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 przy pierwszym odrzuceniu na produkcji — a to da się zrobić od razu po wdrożeniu, w odróżnieniu od Z-18, który czeka na węzeł. Decyzja właściciela produktu: dorobić akcję w panelu zamiast jednorazowego czyszczenia Redisa. | JAK TO WYSZŁO: X-30 naprawiło alerting, VerrisProvisioningQueueFailed zapalił się z prawdziwego powodu i wskazał cztery martwe joby (to z nich wyszło Z-18). Naturalny następny ruch — usunąć je — okazał się NIEWYKONALNY: panel ma przy nich wyłącznie „Retry", a kontroler administracyjny dokładnie dwa endpointy, listowanie i ponowienie. Retry nic nie daje, bo węzła nie ma: job padnie ponownie, podbije licznik prób i dołoży wpisy do audytu — cztery martwe joby zamieniają się w cztery martwe joby z dłuższą historią. Zostawało grzebanie w Redisie ręcznie, czyli zmiana stanu produkcyjnego dotyczącego subskrypcji klientów BEZ ŚLADU W AUDYCIE. | TO NIE JEST USTERKA TYCH CZTERECH JOBÓW, tylko luka w warstwie operatorskiej, która ujawni się ponownie przy pierwszym prawdziwym niepowodzeniu provisioningu — z tą różnicą, że wtedy po drugiej stronie będzie klient. | ROZWIĄZANIE: POST /admin/provisioning-queue/:id/odrzuc + przycisk „Odrzuć" obok Retry. TRZY REGUŁY: (1) TYLKO STAN failed — usunięcie joba aktywnego albo czekającego osierociłoby provisioning w trakcie, konto na węźle mogłoby powstać, a system przestałby o nim wiedzieć; ograniczenie siedzi w usłudze, nie w kontrolerze, bo to reguła o kolejce, nie o HTTP; (2) POWÓD WYMAGANY, tak samo jak przy retry — operacja bez powodu to operacja, której za pół roku nikt nie wyjaśni; (3) NAJPIERW ODCZYT, POTEM USUNIĘCIE — ślad zbierany PRZED job.remove(), bo po usunięciu nie ma już czego odczytać; zapisujemy subskrypcję, joba, typ, liczbę prób, ostatni błąd i powód. Po Z-18 ten ostatni błąd niesie PRAWDZIWĄ przyczynę, więc wpis ma realną wartość dowodową — jeszcze wczoraj zapisałby zdanie o brakującym pakiecie DirectAdmina, którego nigdy nie brakowało. | OSOBNA AKCJA AUDYTU (PROVISIONING_JOB_DISCARDED_BY_ADMIN), nie wariant retry: w raportach odrzucenie i ponowienie to dwie różne decyzje i nie wolno im się zlewać. | DWA KLIKNIĘCIA, NIE JEDNO: retry można cofnąć następnym retry, odrzucenia nie da się cofnąć wcale. Potwierdzenie jest po to, żeby ta różnica była wyczuwalna w palcach. | ZDANIE PRZY PRZYCISKU: „Usuwa wpis z kolejki bez możliwości cofnięcia. Subskrypcja zostaje nietknięta." Operator ma prawo założyć, że „odrzuć" anuluje zamówienie — nie anuluje. Musi to być napisane tam, gdzie się klika, a nie w dokumentacji, której nikt nie otworzy w trakcie incydentu. | Czerwieni się na starym kodzie: 11 z 13. | DWIE UWAGI O SAMYCH TESTACH: odczyty plików panelu są LENIWE, bo odczyt na poziomie describe wywalał cały plik testowy, zanim cokolwiek się policzyło — a wtedy nie wiadomo, ILE asercji się czerwieni, tylko że „nie skompilowało się"; asercja o warunku row.failedReason nie mierzy odległości w znakach, tylko relację między warunkiem a przyciskiem, bo wersja licząca znaki zepsuła się od dopisania komentarza i kusiło, żeby poszerzyć okno zamiast poprawić asercję — to byłoby naprawianie testu zamiast kodu. | CZEGO NIE OBEJMUJE: losu czterech subskrypcji, które dostały zwrot i status PENDING_PAYMENT (odrzucenie joba ich nie dotyka — osobne sprzątanie po stronie bazy); odrzucania hurtem — świadomie, bo przycisk „odrzuć wszystkie" jest wygodny dokładnie do momentu, w którym ktoś kliknie go na kolejce z prawdziwym zamówieniem. | JAK ZAMKNĄĆ: odrzucić jeden z czterech martwych jobów, obejrzeć wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie i sprawdzić, że verris_provisioning_queue_depth{state="failed"} spadło o jeden. Dokumentacja: docs/archiwum/zadania/X-32-odrzucenie-martwego-joba.md | 2026-09-22 D3: wlasciciel odrzucil martwy job przyciskiem 'Odrzuc' w panelu admina na produkcji (potwierdzenie wlasciciela; wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie).</t>
         </is>
       </c>
       <c r="P72" s="10" t="inlineStr">
@@ -6419,12 +6419,12 @@
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>M-08</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>Anulowanie faktury (VOID) z panelu</t>
+          <t>W drzewie stoją dwa majory ESLinta naraz</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -6434,12 +6434,12 @@
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F73" s="10" t="n">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="L73" s="11" t="inlineStr">
         <is>
-          <t>billing/anulowanie.service.ts (POST /admin/invoices/:id/anuluj, BILLING_MANAGE); admin: invoices/void-button.tsx; test D2 anulowanie.service.spec.ts</t>
+          <t>package.json (korzeń) — @eslint/js ^10.0.1 przy braku jakiegokolwiek eslint.config.* w korzeniu; libs/eslint-config/node_modules: eslint 10.9.0 obok @eslint/js 9.39.5; apps/api, apps/www, apps/client-panel, apps/status-page, libs/directadmin-sdk — eslint 9.39.5 | 2026-09-23: z korzenia zdjęte nieużywane @eslint/js ^10 i typescript-eslint; libs/eslint-config peer eslint ^9.39.5 (było &gt;=9 → auto-install dociągał 10.9.0); lockfile bez eslint 10; strażnik apps/api/src/test/eslint-jeden-major.spec.ts (deklaracje + peer + lockfile)</t>
         </is>
       </c>
       <c r="M73" s="11" t="inlineStr">
@@ -6485,7 +6485,7 @@
       </c>
       <c r="O73" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: anulować wolno tylko dokument nieopłacony (DRAFT/OPEN); opłacony, także z portfela, zmienia się korektą (M-06). Faktura Stripe unieważniana najpierw w Stripe, błąd = brak zmiany lokalnej. Numer zostaje (ciągłość), powód w audycie INVOICE_VOIDED.</t>
+          <t>Odkryte 2026-08-28 przy DEP-01. Korzeń deklaruje @eslint/js ^10.0.1, którego peer to eslint ^10.0.0 — i to on wciąga eslint@10.9.0 do drzewa. Tymczasem KAŻDY pakiet, który realnie lintuje, ma 9.39.5. Najostrzej widać to wewnątrz libs/eslint-config, czyli wspólnej konfiguracji: node_modules/eslint = 10.9.0, node_modules/@eslint/js = 9.39.5 — dwie połowy jednego narzędzia z różnych majorów w jednym katalogu. | Korzeń NIE MA żadnego eslint.config.* i nie odpala lintera (pnpm lint = turbo run lint), więc te zależności nie robią nic poza wciąganiem majora, którego nikt nie używa. | To nie awaria — bramka jest zielona, 0 błędów. To BRAK KONTROLI: żaden strażnik nie sprawdza, czy major ESLinta jest jeden, tak jak do ENV-01 nic nie sprawdzało wersji Node. | DO ZROBIENIA: zdjąć z korzenia nieużywane @eslint/js i typescript-eslint albo cofnąć je do dziewiątki (rusza lockfile — osobny commit z pełną bramką), plus strażnik spójności majora na wzór wersja-node.spec.ts. | 2026-09-23: zrobione zgodnie z DO ZROBIENIA; lockfile zmieniony wyłącznie o usunięcie gałęzi eslint 10 (pnpm 9.5.0 --lockfile-only). Przed bramką lokalną: pnpm install.</t>
         </is>
       </c>
       <c r="P73" s="10" t="inlineStr">
@@ -6497,12 +6497,12 @@
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>C-18</t>
+          <t>M-08</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>Konto FTP — zmiana hasła</t>
+          <t>Anulowanie faktury (VOID) z panelu</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="E74" s="10" t="inlineStr">
@@ -6543,12 +6543,12 @@
       </c>
       <c r="K74" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L74" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/hosting-ftp/:username/password (ZmienHasloFtpDto) → directadmin.service changeHostingFtpPassword (action=modify, katalog zachowany) + audyt HOSTING_FTP_PASSWORD_CHANGED; UI FtpTab — kluczyk przy koncie; test servers/zmiana-hasla-ftp.spec.ts</t>
+          <t>billing/anulowanie.service.ts (POST /admin/invoices/:id/anuluj, BILLING_MANAGE); admin: invoices/void-button.tsx; test D2 anulowanie.service.spec.ts</t>
         </is>
       </c>
       <c r="M74" s="11" t="inlineStr">
@@ -6558,12 +6558,12 @@
       </c>
       <c r="N74" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O74" s="11" t="inlineStr">
         <is>
-          <t>brak jakiejkolwiek ścieżki edycji istniejącego konta | Przy okazji body tworzenia konta FTP dostało klasę DTO (login, hasło, katalog bez „..”). OTWARTE do D3 (PB-21): format action=modify na żywym DA.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: anulować wolno tylko dokument nieopłacony (DRAFT/OPEN); opłacony, także z portfela, zmienia się korektą (M-06). Faktura Stripe unieważniana najpierw w Stripe, błąd = brak zmiany lokalnej. Numer zostaje (ciągłość), powód w audycie INVOICE_VOIDED.</t>
         </is>
       </c>
       <c r="P74" s="10" t="inlineStr">
@@ -6575,12 +6575,12 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>C-18</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>Konto FTP — zmiana hasła</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
@@ -6602,7 +6602,7 @@
         <v>6</v>
       </c>
       <c r="G75" s="10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H75" s="10" t="inlineStr">
         <is>
@@ -6611,22 +6611,22 @@
       </c>
       <c r="I75" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="J75" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="K75" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L75" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>2026-09-23 D1: POST /services/:id/hosting-ftp/:username/password (ZmienHasloFtpDto) → directadmin.service changeHostingFtpPassword (action=modify, katalog zachowany) + audyt HOSTING_FTP_PASSWORD_CHANGED; UI FtpTab — kluczyk przy koncie; test servers/zmiana-hasla-ftp.spec.ts</t>
         </is>
       </c>
       <c r="M75" s="11" t="inlineStr">
@@ -6636,12 +6636,12 @@
       </c>
       <c r="N75" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O75" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>brak jakiejkolwiek ścieżki edycji istniejącego konta | Przy okazji body tworzenia konta FTP dostało klasę DTO (login, hasło, katalog bez „..”). OTWARTE do D3 (PB-21): format action=modify na żywym DA.</t>
         </is>
       </c>
       <c r="P75" s="10" t="inlineStr">
@@ -6653,12 +6653,12 @@
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>C-11</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>Spakowanie do archiwum</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -6668,12 +6668,12 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E76" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F76" s="10" t="n">
@@ -6699,12 +6699,12 @@
       </c>
       <c r="K76" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L76" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M76" s="11" t="inlineStr">
@@ -6714,12 +6714,12 @@
       </c>
       <c r="N76" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O76" s="11" t="inlineStr">
         <is>
-          <t>standard we wszystkich panelach | OTWARTE do D3 (PB-21): format action=compress na żywym DA.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P76" s="10" t="inlineStr">
@@ -6731,12 +6731,12 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>NODE-03</t>
+          <t>C-11</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Pojemność węzła nigdy się nie odświeża</t>
+          <t>Spakowanie do archiwum</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -6746,7 +6746,7 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="L77" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: verris-lve.sh node_capacity (nproc, MemTotal, df /) w każdym raporcie, lve-agent/1.1; telemetry.dto NodeStatusDto.totalCpuCores/totalMemoryMb/totalDiskMb; telemetry.service aktualizuje Server; test telemetry/pojemnosc-wezla.spec.ts</t>
+          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych</t>
         </is>
       </c>
       <c r="M77" s="11" t="inlineStr">
@@ -6797,7 +6797,7 @@
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Pojemność węzła nigdy się nie odświeża. `totalCpuCores`/`totalMemoryMb`/`totalDiskMb` ustawiane wyłącznie w handshake; telemetria ich nie aktualizuje — mimo komentarza w schemacie „reported via handshake / heartbeat”. Rozbudowa węzła nie dociera do `NodeSelector`. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Telemetria aktualizuje totalCpuCores/totalMemoryMb/totalDiskMb, nie tylko handshake. | Stary agent bez pól niczego nie zeruje. OTWARTE do D3 (PB-21): raport z agenta na żywym węźle i odświeżona pojemność w panelu admina. | 2026-09-25: pojemność z agenta trafia też do planera pojemności (admin → Product Ops): ryzyko liczone względem rdzeni i RAM węzła (CPU 2×/4× rdzeni, RAM 1×/1,5×; test ryzyko-pojemnosci.spec.ts), a opis „CPU 250%” zastąpiony „przydzielone limity: CPU 2,5 rdz. z N · RAM x z y GB” — wcześniej wyglądało jak zużycie ponad 100%.</t>
+          <t>standard we wszystkich panelach | OTWARTE do D3 (PB-21): format action=compress na żywym DA.</t>
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr">
@@ -6809,31 +6809,31 @@
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>PB-08</t>
+          <t>NODE-03</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
+          <t>Pojemność węzła nigdy się nie odświeża</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G78" s="10" t="n">
         <v>14</v>
@@ -6855,12 +6855,12 @@
       </c>
       <c r="K78" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L78" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-09-23 D1: verris-lve.sh node_capacity (nproc, MemTotal, df /) w każdym raporcie, lve-agent/1.1; telemetry.dto NodeStatusDto.totalCpuCores/totalMemoryMb/totalDiskMb; telemetry.service aktualizuje Server; test telemetry/pojemnosc-wezla.spec.ts</t>
         </is>
       </c>
       <c r="M78" s="11" t="inlineStr">
@@ -6870,12 +6870,12 @@
       </c>
       <c r="N78" s="11" t="inlineStr">
         <is>
-          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Pojemność węzła nigdy się nie odświeża. `totalCpuCores`/`totalMemoryMb`/`totalDiskMb` ustawiane wyłącznie w handshake; telemetria ich nie aktualizuje — mimo komentarza w schemacie „reported via handshake / heartbeat”. Rozbudowa węzła nie dociera do `NodeSelector`. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Telemetria aktualizuje totalCpuCores/totalMemoryMb/totalDiskMb, nie tylko handshake. | Stary agent bez pól niczego nie zeruje. OTWARTE do D3 (PB-21): raport z agenta na żywym węźle i odświeżona pojemność w panelu admina. | 2026-09-25: pojemność z agenta trafia też do planera pojemności (admin → Product Ops): ryzyko liczone względem rdzeni i RAM węzła (CPU 2×/4× rdzeni, RAM 1×/1,5×; test ryzyko-pojemnosci.spec.ts), a opis „CPU 250%” zastąpiony „przydzielone limity: CPU 2,5 rdz. z N · RAM x z y GB” — wcześniej wyglądało jak zużycie ponad 100%.</t>
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr">
@@ -6887,12 +6887,12 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>PB-27</t>
+          <t>PB-08</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
+          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
@@ -6907,11 +6907,11 @@
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G79" s="10" t="n">
         <v>14</v>
@@ -6948,12 +6948,12 @@
       </c>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
+          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
         </is>
       </c>
       <c r="O79" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
         </is>
       </c>
       <c r="P79" s="10" t="inlineStr">
@@ -6965,12 +6965,12 @@
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>PB-28</t>
+          <t>PB-27</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Rozliczenie poza Verris (całe konto)</t>
+          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -6989,7 +6989,7 @@
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G80" s="10" t="n">
         <v>14</v>
@@ -7026,12 +7026,12 @@
       </c>
       <c r="N80" s="11" t="inlineStr">
         <is>
-          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
+          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
         </is>
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr">
@@ -7043,58 +7043,58 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>X-41</t>
+          <t>PB-28</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
+          <t>Rozliczenie poza Verris (całe konto)</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G81" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H81" s="10" t="inlineStr">
         <is>
-          <t>Faza 3 — Wejście na rynek</t>
+          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
         </is>
       </c>
       <c r="I81" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K81" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L81" s="11" t="inlineStr">
         <is>
-          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M81" s="11" t="inlineStr">
@@ -7104,12 +7104,12 @@
       </c>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
         </is>
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
+          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr">
@@ -7121,12 +7121,12 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>X-41</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
+          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E82" s="10" t="inlineStr">
@@ -7172,7 +7172,7 @@
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
+          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
         </is>
       </c>
       <c r="M82" s="11" t="inlineStr">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="O82" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr">
@@ -7199,31 +7199,31 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>PB-22</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
+          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F83" s="10" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G83" s="10" t="n">
         <v>15</v>
@@ -7245,12 +7245,12 @@
       </c>
       <c r="K83" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
         </is>
       </c>
       <c r="M83" s="11" t="inlineStr">
@@ -7260,12 +7260,12 @@
       </c>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O83" s="11" t="inlineStr">
         <is>
-          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr">
@@ -7277,34 +7277,34 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>PB-22</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Log egressu jest próbką, nie zapisem</t>
+          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F84" s="10" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H84" s="10" t="inlineStr">
         <is>
@@ -7313,22 +7313,22 @@
       </c>
       <c r="I84" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="J84" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="K84" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
@@ -7338,12 +7338,12 @@
       </c>
       <c r="N84" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
         </is>
       </c>
       <c r="O84" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
+          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr">
@@ -7355,12 +7355,12 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
+          <t>Log egressu jest próbką, nie zapisem</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -7401,12 +7401,12 @@
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M85" s="11" t="inlineStr">
@@ -7416,12 +7416,12 @@
       </c>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O85" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr">
@@ -7433,12 +7433,12 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>Tryb `--strict` jest atrapą</t>
+          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -7457,7 +7457,7 @@
         </is>
       </c>
       <c r="F86" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G86" s="10" t="n">
         <v>16</v>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
+          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr">
@@ -7499,7 +7499,7 @@
       </c>
       <c r="O86" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr">
@@ -7511,12 +7511,12 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
+          <t>Tryb `--strict` jest atrapą</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -7557,12 +7557,12 @@
       </c>
       <c r="K87" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L87" s="11" t="inlineStr">
         <is>
-          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
+          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
         </is>
       </c>
       <c r="M87" s="11" t="inlineStr">
@@ -7572,12 +7572,12 @@
       </c>
       <c r="N87" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O87" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr">
@@ -7589,12 +7589,12 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
+          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
@@ -7609,11 +7609,11 @@
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>16</v>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
+          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
         </is>
       </c>
       <c r="M88" s="11" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="O88" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr">
@@ -7667,31 +7667,31 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>PB-23</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
+          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G89" s="10" t="n">
         <v>16</v>
@@ -7713,12 +7713,12 @@
       </c>
       <c r="K89" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L89" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
         </is>
       </c>
       <c r="M89" s="11" t="inlineStr">
@@ -7728,12 +7728,12 @@
       </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O89" s="11" t="inlineStr">
         <is>
-          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr">
@@ -7745,34 +7745,34 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>PB-23</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Podpisane DPA z subprocesorami (część)</t>
+          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G90" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H90" s="10" t="inlineStr">
         <is>
@@ -7781,22 +7781,22 @@
       </c>
       <c r="I90" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="J90" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="K90" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L90" s="11" t="inlineStr">
         <is>
-          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M90" s="11" t="inlineStr">
@@ -7806,12 +7806,12 @@
       </c>
       <c r="N90" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
         </is>
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
+          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7823,31 +7823,31 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>PB-03</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Finalizacja dokumentów prawnych 1.0.0</t>
+          <t>Podpisane DPA z subprocesorami (część)</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G91" s="10" t="n">
         <v>17</v>
@@ -7869,12 +7869,12 @@
       </c>
       <c r="K91" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L91" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
         </is>
       </c>
       <c r="M91" s="11" t="inlineStr">
@@ -7884,12 +7884,12 @@
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7901,12 +7901,12 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>PB-04</t>
+          <t>PB-03</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
+          <t>Finalizacja dokumentów prawnych 1.0.0</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -7921,11 +7921,11 @@
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>17</v>
@@ -7962,12 +7962,12 @@
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
+          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
+          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7979,34 +7979,34 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>N-16</t>
+          <t>PB-04</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>SLA z zapisanymi kredytami</t>
+          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G93" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H93" s="10" t="inlineStr">
         <is>
@@ -8015,37 +8015,37 @@
       </c>
       <c r="I93" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-21</t>
         </is>
       </c>
       <c r="J93" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="K93" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L93" s="11" t="inlineStr">
         <is>
-          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M93" s="11" t="inlineStr">
         <is>
-          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
+          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8057,12 +8057,12 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>N-16</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>SLA z zapisanymi kredytami</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E94" s="10" t="inlineStr">
@@ -8103,27 +8103,27 @@
       </c>
       <c r="K94" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
         </is>
       </c>
       <c r="M94" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
         </is>
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8135,31 +8135,31 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>PB-07</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>Treści i cennik na verris.pl</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G95" s="10" t="n">
         <v>18</v>
@@ -8181,27 +8181,27 @@
       </c>
       <c r="K95" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L95" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M95" s="11" t="inlineStr">
         <is>
-          <t>PB-01 (cennik zależy od unit economics)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,12 +8213,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>PB-11</t>
+          <t>PB-07</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
+          <t>Treści i cennik na verris.pl</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8237,7 +8237,7 @@
         </is>
       </c>
       <c r="F96" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G96" s="10" t="n">
         <v>18</v>
@@ -8269,17 +8269,17 @@
       </c>
       <c r="M96" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-01 (cennik zależy od unit economics)</t>
         </is>
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
+          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
+          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,12 +8291,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-21</t>
+          <t>PB-11</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>DNS platformy i poczty na serwerze testowym</t>
+          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8315,7 +8315,7 @@
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>18</v>
@@ -8352,12 +8352,12 @@
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
+          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
+          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8369,12 +8369,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-24</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8393,7 +8393,7 @@
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G98" s="10" t="n">
         <v>18</v>
@@ -8430,12 +8430,12 @@
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8447,12 +8447,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-25</t>
+          <t>PB-24</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>White label na węźle — klient nie widzi DirectAdmina</t>
+          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8471,7 +8471,7 @@
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G99" s="10" t="n">
         <v>18</v>
@@ -8508,12 +8508,12 @@
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
+          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
+          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8525,12 +8525,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-25</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>White label na węźle — klient nie widzi DirectAdmina</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8549,10 +8549,10 @@
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G100" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H100" s="10" t="inlineStr">
         <is>
@@ -8561,12 +8561,12 @@
       </c>
       <c r="I100" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K100" s="10" t="inlineStr">
@@ -8581,17 +8581,17 @@
       </c>
       <c r="M100" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
+          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8603,12 +8603,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8623,7 +8623,7 @@
       </c>
       <c r="E101" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F101" s="10" t="n">
@@ -8659,17 +8659,17 @@
       </c>
       <c r="M101" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8681,12 +8681,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8705,7 +8705,7 @@
         </is>
       </c>
       <c r="F102" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G102" s="10" t="n">
         <v>19</v>
@@ -8742,12 +8742,12 @@
       </c>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8759,12 +8759,12 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8783,20 +8783,24 @@
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G103" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H103" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H103" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I103" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J103" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K103" s="10" t="inlineStr">
@@ -8811,17 +8815,17 @@
       </c>
       <c r="M103" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N103" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8833,69 +8837,69 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F104" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G104" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H104" s="10" t="inlineStr"/>
       <c r="I104" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J104" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K104" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L104" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M104" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8907,12 +8911,12 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -8922,16 +8926,16 @@
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F105" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G105" s="10" t="n">
         <v>21</v>
@@ -8954,7 +8958,7 @@
       </c>
       <c r="L105" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M105" s="11" t="inlineStr">
@@ -8969,7 +8973,7 @@
       </c>
       <c r="O105" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr">
@@ -8981,12 +8985,12 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -8996,7 +9000,7 @@
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E106" s="10" t="inlineStr">
@@ -9023,12 +9027,12 @@
       </c>
       <c r="K106" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L106" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M106" s="11" t="inlineStr">
@@ -9038,12 +9042,12 @@
       </c>
       <c r="N106" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O106" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr">
@@ -9055,12 +9059,12 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -9075,7 +9079,7 @@
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F107" s="10" t="n">
@@ -9102,7 +9106,7 @@
       </c>
       <c r="L107" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M107" s="11" t="inlineStr">
@@ -9117,7 +9121,7 @@
       </c>
       <c r="O107" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr">
@@ -9129,12 +9133,12 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -9144,12 +9148,12 @@
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F108" s="10" t="n">
@@ -9171,12 +9175,12 @@
       </c>
       <c r="K108" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L108" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M108" s="11" t="inlineStr">
@@ -9186,12 +9190,12 @@
       </c>
       <c r="N108" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O108" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr">
@@ -9203,31 +9207,31 @@
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C109" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F109" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G109" s="10" t="n">
         <v>21</v>
@@ -9245,12 +9249,12 @@
       </c>
       <c r="K109" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L109" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>services.controller.ts:125</t>
         </is>
       </c>
       <c r="M109" s="11" t="inlineStr">
@@ -9260,12 +9264,12 @@
       </c>
       <c r="N109" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O109" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr">
@@ -9277,12 +9281,12 @@
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>PB-29</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
@@ -9297,11 +9301,11 @@
       </c>
       <c r="E110" s="10" t="inlineStr">
         <is>
-          <t>KRYTYCZNY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F110" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G110" s="10" t="n">
         <v>21</v>
@@ -9334,12 +9338,12 @@
       </c>
       <c r="N110" s="11" t="inlineStr">
         <is>
-          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O110" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr">
@@ -9351,12 +9355,12 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>PB-30</t>
+          <t>PB-29</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Jeden plik wersji dla floty + test zgodności</t>
+          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
@@ -9371,7 +9375,7 @@
       </c>
       <c r="E111" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F111" s="10" t="n">
@@ -9408,12 +9412,12 @@
       </c>
       <c r="N111" s="11" t="inlineStr">
         <is>
-          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
+          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="O111" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
+          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr">
@@ -9425,12 +9429,12 @@
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>PB-31</t>
+          <t>PB-30</t>
         </is>
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
-          <t>Pełna automatyzacja kreatora węzła</t>
+          <t>Jeden plik wersji dla floty + test zgodności</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -9449,7 +9453,7 @@
         </is>
       </c>
       <c r="F112" s="10" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G112" s="10" t="n">
         <v>21</v>
@@ -9482,12 +9486,12 @@
       </c>
       <c r="N112" s="11" t="inlineStr">
         <is>
-          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
+          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
         </is>
       </c>
       <c r="O112" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
+          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
         </is>
       </c>
       <c r="P112" s="10" t="inlineStr">
@@ -9499,12 +9503,12 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>PB-32</t>
+          <t>PB-31</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>Aktualizacje węzłów falami</t>
+          <t>Pełna automatyzacja kreatora węzła</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
@@ -9519,11 +9523,11 @@
       </c>
       <c r="E113" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F113" s="10" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G113" s="10" t="n">
         <v>21</v>
@@ -9556,12 +9560,12 @@
       </c>
       <c r="N113" s="11" t="inlineStr">
         <is>
-          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
+          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
         </is>
       </c>
       <c r="O113" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
+          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
         </is>
       </c>
       <c r="P113" s="10" t="inlineStr">
@@ -9573,12 +9577,12 @@
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>PB-33</t>
+          <t>PB-32</t>
         </is>
       </c>
       <c r="B114" s="11" t="inlineStr">
         <is>
-          <t>Wersje stosu floty w panelu + wyrównanie falą</t>
+          <t>Aktualizacje węzłów falami</t>
         </is>
       </c>
       <c r="C114" s="10" t="inlineStr">
@@ -9593,11 +9597,11 @@
       </c>
       <c r="E114" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F114" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G114" s="10" t="n">
         <v>21</v>
@@ -9630,12 +9634,12 @@
       </c>
       <c r="N114" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji w panelu → nowy węzeł instaluje ją, istniejące wyrównane falą; audyt zgodności zielony.</t>
+          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
         </is>
       </c>
       <c r="O114" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: strona „Wersje stosu floty” w panelu admina (DB, PHP, LiteSpeed, DirectAdmin) z dozwolonymi wartościami z oficjalnych list; zmiana obowiązuje nowe węzły od razu, „Wyrównaj flotę” aktualizuje istniejące falą (PHP/LiteSpeed przez CustomBuild, MariaDB po jednej wersji z kopią bazy — wymóg CloudLinux Governor). | 2026-09-26 ZROBIONE W KODZIE: manifest w bazie (StosWezlaService), strona Admin → Wersje stosu floty (dozwolone wartości z oficjalnych list, tabela zgodności), „Wyrównaj flotę” = fala z php1_release + łańcuch DB_UPGRADE krok po kroku z kopią; bootstrap i agent biorą manifest z bazy. Testy na PostgreSQL. Zostało: wyrównanie na węzłach (D3).</t>
+          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
         </is>
       </c>
       <c r="P114" s="10" t="inlineStr">
@@ -9647,12 +9651,12 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>PB-35</t>
+          <t>PB-33</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>Automatyczna fala aktualizacji węzłów co tydzień</t>
+          <t>Wersje stosu floty w panelu + wyrównanie falą</t>
         </is>
       </c>
       <c r="C115" s="10" t="inlineStr">
@@ -9671,7 +9675,7 @@
         </is>
       </c>
       <c r="F115" s="10" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G115" s="10" t="n">
         <v>21</v>
@@ -9704,12 +9708,12 @@
       </c>
       <c r="N115" s="11" t="inlineStr">
         <is>
-          <t>Fala startuje sama w oknie; zatrzymanie widoczne w powiadomieniach admina.</t>
+          <t>Zmiana wersji w panelu → nowy węzeł instaluje ją, istniejące wyrównane falą; audyt zgodności zielony.</t>
         </is>
       </c>
       <c r="O115" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: fala rusza sama we wtorki o 4:00 (kanarek → reszta po jednym, błąd zatrzymuje, powiadomienie). Węzły same już niczego nie instalują (dnf-automatic tylko pobiera). | 2026-09-26 ZROBIONE W KODZIE: FalaTygodniowaScheduler (wtorek 4:00 Europe/Warsaw), zatrzymanie fali → powiadomienie adminów. Test na PostgreSQL.</t>
+          <t>Decyzja właściciela 2026-09-26: strona „Wersje stosu floty” w panelu admina (DB, PHP, LiteSpeed, DirectAdmin) z dozwolonymi wartościami z oficjalnych list; zmiana obowiązuje nowe węzły od razu, „Wyrównaj flotę” aktualizuje istniejące falą (PHP/LiteSpeed przez CustomBuild, MariaDB po jednej wersji z kopią bazy — wymóg CloudLinux Governor). | 2026-09-26 ZROBIONE W KODZIE: manifest w bazie (StosWezlaService), strona Admin → Wersje stosu floty (dozwolone wartości z oficjalnych list, tabela zgodności), „Wyrównaj flotę” = fala z php1_release + łańcuch DB_UPGRADE krok po kroku z kopią; bootstrap i agent biorą manifest z bazy. Testy na PostgreSQL. Zostało: wyrównanie na węzłach (D3).</t>
         </is>
       </c>
       <c r="P115" s="10" t="inlineStr">
@@ -9721,12 +9725,12 @@
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>PB-36</t>
+          <t>PB-35</t>
         </is>
       </c>
       <c r="B116" s="11" t="inlineStr">
         <is>
-          <t>Podpisane skrypty węzła i klucz SSH ograniczony do control-plane</t>
+          <t>Automatyczna fala aktualizacji węzłów co tydzień</t>
         </is>
       </c>
       <c r="C116" s="10" t="inlineStr">
@@ -9741,11 +9745,11 @@
       </c>
       <c r="E116" s="10" t="inlineStr">
         <is>
-          <t>KRYTYCZNY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F116" s="10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G116" s="10" t="n">
         <v>21</v>
@@ -9778,12 +9782,12 @@
       </c>
       <c r="N116" s="11" t="inlineStr">
         <is>
-          <t>Niepodpisany/zmieniony skrypt odrzucony przez węzeł; authorized_keys zawiera tylko aktualny klucz z ograniczeniem IP.</t>
+          <t>Fala startuje sama w oknie; zatrzymanie widoczne w powiadomieniach admina.</t>
         </is>
       </c>
       <c r="O116" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: przed startem. Węzeł uruchamia tylko skrypty podpisane kluczem Verris (przejęte API nie daje roota na flocie); klucz SSH z from= na IP control-plane, stare klucze usuwane (dziś agent co minutę tylko dopisuje klucz). | 2026-09-26 ZROBIONE W KODZIE: podpis Ed25519 każdej odpowiedzi GET /agent/tasks/* (skrypty zadań, pakiety onboardu i strony domyślnej, manifest stosu, konfiguracja kopii, zlecenia, klucz deploy) — podpis obejmuje ścieżkę, id węzła, czas i SHA-256 treści (bez podmiany, przeniesienia na inną ścieżkę/węzeł, powtórki po 5 min). Węzeł pobiera wyłącznie przez /usr/local/bin/verris-fetch (openssl pkeyutl -verify), klucz publiczny przywozi bootstrap / instalacja agenta. Klucz deploy: jeden wpis from="VERRIS_CONTROL_PLANE_IPS" bez przekierowań, poprzedni usuwany (rotacja). API w produkcji nie wystartuje bez VERRIS_SCRIPT_SIGNING_KEY albo z kluczem deploy bez adresów control-plane. Test: prawdziwy verris-fetch vs serwer podpisujący (zmieniona treść / inna ścieżka / inny węzeł / stary podpis / brak podpisu → odrzucone) + smoke na lokalnym API. Do sprawdzenia na D3: openssl na CloudLinux 9, rotacja klucza deploy.</t>
+          <t>Decyzja właściciela 2026-09-26: fala rusza sama we wtorki o 4:00 (kanarek → reszta po jednym, błąd zatrzymuje, powiadomienie). Węzły same już niczego nie instalują (dnf-automatic tylko pobiera). | 2026-09-26 ZROBIONE W KODZIE: FalaTygodniowaScheduler (wtorek 4:00 Europe/Warsaw), zatrzymanie fali → powiadomienie adminów. Test na PostgreSQL.</t>
         </is>
       </c>
       <c r="P116" s="10" t="inlineStr">
@@ -9795,12 +9799,12 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>PB-26</t>
+          <t>PB-36</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
+          <t>Podpisane skrypty węzła i klucz SSH ograniczony do control-plane</t>
         </is>
       </c>
       <c r="C117" s="10" t="inlineStr">
@@ -9815,24 +9819,24 @@
       </c>
       <c r="E117" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F117" s="10" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G117" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H117" s="10" t="inlineStr"/>
       <c r="I117" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J117" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K117" s="10" t="inlineStr">
@@ -9852,12 +9856,12 @@
       </c>
       <c r="N117" s="11" t="inlineStr">
         <is>
-          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
+          <t>Niepodpisany/zmieniony skrypt odrzucony przez węzeł; authorized_keys zawiera tylko aktualny klucz z ograniczeniem IP.</t>
         </is>
       </c>
       <c r="O117" s="11" t="inlineStr">
         <is>
-          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
+          <t>Decyzja właściciela 2026-09-26: przed startem. Węzeł uruchamia tylko skrypty podpisane kluczem Verris (przejęte API nie daje roota na flocie); klucz SSH z from= na IP control-plane, stare klucze usuwane (dziś agent co minutę tylko dopisuje klucz). | 2026-09-26 ZROBIONE W KODZIE: podpis Ed25519 każdej odpowiedzi GET /agent/tasks/* (skrypty zadań, pakiety onboardu i strony domyślnej, manifest stosu, konfiguracja kopii, zlecenia, klucz deploy) — podpis obejmuje ścieżkę, id węzła, czas i SHA-256 treści (bez podmiany, przeniesienia na inną ścieżkę/węzeł, powtórki po 5 min). Węzeł pobiera wyłącznie przez /usr/local/bin/verris-fetch (openssl pkeyutl -verify), klucz publiczny przywozi bootstrap / instalacja agenta. Klucz deploy: jeden wpis from="VERRIS_CONTROL_PLANE_IPS" bez przekierowań, poprzedni usuwany (rotacja). API w produkcji nie wystartuje bez VERRIS_SCRIPT_SIGNING_KEY albo z kluczem deploy bez adresów control-plane. Test: prawdziwy verris-fetch vs serwer podpisujący (zmieniona treść / inna ścieżka / inny węzeł / stary podpis / brak podpisu → odrzucone) + smoke na lokalnym API. Do sprawdzenia na D3: openssl na CloudLinux 9, rotacja klucza deploy.</t>
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr">
@@ -9869,12 +9873,12 @@
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-26</t>
         </is>
       </c>
       <c r="B118" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
@@ -9889,11 +9893,11 @@
       </c>
       <c r="E118" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F118" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G118" s="10" t="n">
         <v>22</v>
@@ -9921,17 +9925,17 @@
       </c>
       <c r="M118" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N118" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
         </is>
       </c>
       <c r="O118" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
         </is>
       </c>
       <c r="P118" s="10" t="inlineStr">
@@ -9943,12 +9947,12 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C119" s="10" t="inlineStr">
@@ -9967,7 +9971,7 @@
         </is>
       </c>
       <c r="F119" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G119" s="10" t="n">
         <v>22</v>
@@ -9995,28 +9999,102 @@
       </c>
       <c r="M119" s="11" t="inlineStr">
         <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N119" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O119" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P119" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F120" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G120" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H120" s="10" t="inlineStr"/>
+      <c r="I120" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J120" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K120" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L120" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M120" s="11" t="inlineStr">
+        <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N119" s="11" t="inlineStr">
+      <c r="N120" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O119" s="11" t="inlineStr">
+      <c r="O120" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P119" s="10" t="inlineStr">
+      <c r="P120" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P119"/>
-  <conditionalFormatting sqref="E2:E119">
+  <autoFilter ref="A1:P120"/>
+  <conditionalFormatting sqref="E2:E120">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -10036,7 +10114,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P119">
+  <conditionalFormatting sqref="P2:P120">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -10146,11 +10224,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A2,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A2,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -10191,11 +10269,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A3,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A3,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -10236,11 +10314,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A4,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A4,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -10281,11 +10359,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A5,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A5,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -10326,11 +10404,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A6,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A6,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -10371,11 +10449,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A7,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A7,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -10416,11 +10494,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A8,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A8,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -10461,11 +10539,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A9,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A9,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -10506,11 +10584,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A10,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A10,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -10551,11 +10629,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A11,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A11,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -10596,11 +10674,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A12,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A12,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -10641,11 +10719,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A13,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A13,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -10686,11 +10764,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A14,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A14,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -10731,11 +10809,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A15,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A15,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -10776,11 +10854,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A16,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A16,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -10821,11 +10899,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A17,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A17,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -10866,11 +10944,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A18,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A18,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -10911,11 +10989,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A19,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A19,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -10956,11 +11034,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A20,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A20,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -10997,11 +11075,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A21,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A21,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -11038,11 +11116,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A22,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A22,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -11079,11 +11157,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A23,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A23,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">
@@ -11120,11 +11198,11 @@
         </is>
       </c>
       <c r="F24" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$119,A24)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A24)</f>
         <v/>
       </c>
       <c r="G24" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$119,A24,'Backlog do startu'!$F$2:$F$119)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A24,'Backlog do startu'!$F$2:$F$120)</f>
         <v/>
       </c>
       <c r="H24" s="10" t="n">

</xml_diff>

<commit_message>
chore(audyt): tablice po PB-39
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$22</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$120)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$121)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$120,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$120,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$121,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$121,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$120,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$121,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$120,"zrobione",'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$121,"zrobione",'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P120"/>
+  <dimension ref="A1:P121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5015,34 +5015,34 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>PB-39</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Rekordy SPF — kreator</t>
+          <t>API i biblioteki jako ESM (Vitest, Prisma prisma-client)</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F55" s="10" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G55" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H55" s="10" t="inlineStr">
         <is>
@@ -5051,22 +5051,22 @@
       </c>
       <c r="I55" s="10" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J55" s="10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K55" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L55" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: deliverability/mail-auth.ts (buildMailAuthChecks) + deliverability.service.ts (strefa DA + delegacja NS); UI app/dashboard/email/deliverability-panel.tsx podpięty w MailTab (zakładka Poczta); test mail-auth.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M55" s="11" t="inlineStr">
@@ -5076,12 +5076,12 @@
       </c>
       <c r="N55" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Bramka i testy integracyjne zielone na Vitest; obraz API buduje się w CI; wdrożenie produkcyjne bez błędów; główne ścieżki działają po wdrożeniu.</t>
         </is>
       </c>
       <c r="O55" s="11" t="inlineStr">
         <is>
-          <t>deliverability-panel.tsx:26 to komponent osierocony — nikt go nie importuje | KOD: kreator pokazuje stan z publicznego DNS i gotowy rekord — „Dodaj/Zamień rekord w DNS” gdy domena na NS Verris, inaczej do skopiowania u dostawcy DNS. Zalecany SPF to `v=spf1 a mx ip4:&lt;IP węzła&gt; ~all`. ZNALEZISKO: dotychczasowa podpowiedź include:_spf.verris.pl odwołuje się do nieistniejącego rekordu (NXDOMAIN) → SPF permerror; usunięta z podpowiedzi, presetu DNS i artykułów KB, a kreator wykrywa ją u klientów. OTWARTE do D3 (węzeł): zapis rekordu przez CMD_API_DNS_CONTROL.</t>
+          <t>Decyzja właściciela 2026-09-26 (formularz): przechodzimy teraz, przed falą 3. ESM to domyślny format NestJS 12; znika eksperymentalna flaga Jesta; prisma-client-js jest wycofany.</t>
         </is>
       </c>
       <c r="P55" s="10" t="inlineStr">
@@ -5093,12 +5093,12 @@
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>E-16</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>Rekordy DKIM — konfiguracja</t>
+          <t>Rekordy SPF — kreator</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -5144,12 +5144,12 @@
       </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
-          <t>deliverability/mail-auth.ts (akcja enable-dkim); servers/directadmin.service.ts enableHostingDkim; POST /services/:id/hosting-email/dkim; email/deliverability-panel.tsx; testy mail-auth.spec.ts, directadmin.narzedzia.spec.ts</t>
+          <t>2026-09-23 D1: deliverability/mail-auth.ts (buildMailAuthChecks) + deliverability.service.ts (strefa DA + delegacja NS); UI app/dashboard/email/deliverability-panel.tsx podpięty w MailTab (zakładka Poczta); test mail-auth.spec.ts</t>
         </is>
       </c>
       <c r="M56" s="11" t="inlineStr">
         <is>
-          <t>E-15 (ten sam panel dostarczalności)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N56" s="11" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="O56" s="11" t="inlineStr">
         <is>
-          <t>j.w. | KOD: DKIM odczytywany ze strefy DA (DA dopisuje klucz sam przy włączonym DKIM). Brak klucza = link do zgłoszenia. OTWARTE: włączanie DKIM z panelu (komenda DA niepotwierdzona bez węzła) — D3 w sprincie 18. | 2026-09-25: KOD (D2) — „Włącz DKIM dla &lt;domena&gt;” w sekcji Dostarczalność zamiast „napisz zgłoszenie”. Komenda DA potwierdzona w dokumentacji (changelog 1.57.2): CMD_API_EMAIL_POP action=set_dkim&amp;domain=…&amp;enable=… — DA tworzy klucze i dopisuje rekord TXT do strefy. Tylko domena z konta usługi, konto zawieszone bez zmian, wpis w dzienniku (HOSTING_DKIM_ENABLED). Wyłączenia celowo brak: ponowne włączenie generuje nowe klucze i rekord u zewnętrznego DNS przestałby pasować. Przy DNS u innego dostawcy panel po włączeniu pokazuje rekord do skopiowania (istniejąca ścieżka „klucz w strefie”). D3: pierwsze włączenie na węźle. | 2026-09-25 (dokumentacja DirectAdmin „Exim → DKIM”): dkim=2 udostępnia włączanie DKIM użytkownikom per domena, dkim=1 generuje klucze automatycznie przy tworzeniu domeny (tylko gdy DNS jest lokalny). Profil węzła ustawia dkim=1 — przycisk w panelu pojawia się tylko dla domen bez klucza. D3 ma potwierdzić, że set_dkim działa przy dkim=1; jeśli nie — alternatywa z dokumentacji: scripts/dkim_create.sh &lt;domena&gt; po stronie węzła (zadanie agenta).</t>
+          <t>deliverability-panel.tsx:26 to komponent osierocony — nikt go nie importuje | KOD: kreator pokazuje stan z publicznego DNS i gotowy rekord — „Dodaj/Zamień rekord w DNS” gdy domena na NS Verris, inaczej do skopiowania u dostawcy DNS. Zalecany SPF to `v=spf1 a mx ip4:&lt;IP węzła&gt; ~all`. ZNALEZISKO: dotychczasowa podpowiedź include:_spf.verris.pl odwołuje się do nieistniejącego rekordu (NXDOMAIN) → SPF permerror; usunięta z podpowiedzi, presetu DNS i artykułów KB, a kreator wykrywa ją u klientów. OTWARTE do D3 (węzeł): zapis rekordu przez CMD_API_DNS_CONTROL.</t>
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr">
@@ -5171,12 +5171,12 @@
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>E-17</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Rekord DMARC — konfiguracja</t>
+          <t>Rekordy DKIM — konfiguracja</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -5222,12 +5222,12 @@
       </c>
       <c r="L57" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: mail-auth.ts dmarcCheck (brak / p=none / kilka rekordów) + lib/dmarc.ts tuneDmarc (polityka + adres raportów) w deliverability-panel.tsx; testy mail-auth.spec.ts, dmarc.spec.ts</t>
+          <t>deliverability/mail-auth.ts (akcja enable-dkim); servers/directadmin.service.ts enableHostingDkim; POST /services/:id/hosting-email/dkim; email/deliverability-panel.tsx; testy mail-auth.spec.ts, directadmin.narzedzia.spec.ts</t>
         </is>
       </c>
       <c r="M57" s="11" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>E-15 (ten sam panel dostarczalności)</t>
         </is>
       </c>
       <c r="N57" s="11" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="O57" s="11" t="inlineStr">
         <is>
-          <t>j.w. | KOD: kreator DMARC — wybór polityki i opcjonalny adres raportów, zachowuje pozostałe tagi. Sugestia bez rua na verris.pl (raporty do obcej domeny wymagają rekordu autoryzacji). OTWARTE do D3: zapis do strefy DA.</t>
+          <t>j.w. | KOD: DKIM odczytywany ze strefy DA (DA dopisuje klucz sam przy włączonym DKIM). Brak klucza = link do zgłoszenia. OTWARTE: włączanie DKIM z panelu (komenda DA niepotwierdzona bez węzła) — D3 w sprincie 18. | 2026-09-25: KOD (D2) — „Włącz DKIM dla &lt;domena&gt;” w sekcji Dostarczalność zamiast „napisz zgłoszenie”. Komenda DA potwierdzona w dokumentacji (changelog 1.57.2): CMD_API_EMAIL_POP action=set_dkim&amp;domain=…&amp;enable=… — DA tworzy klucze i dopisuje rekord TXT do strefy. Tylko domena z konta usługi, konto zawieszone bez zmian, wpis w dzienniku (HOSTING_DKIM_ENABLED). Wyłączenia celowo brak: ponowne włączenie generuje nowe klucze i rekord u zewnętrznego DNS przestałby pasować. Przy DNS u innego dostawcy panel po włączeniu pokazuje rekord do skopiowania (istniejąca ścieżka „klucz w strefie”). D3: pierwsze włączenie na węźle. | 2026-09-25 (dokumentacja DirectAdmin „Exim → DKIM”): dkim=2 udostępnia włączanie DKIM użytkownikom per domena, dkim=1 generuje klucze automatycznie przy tworzeniu domeny (tylko gdy DNS jest lokalny). Profil węzła ustawia dkim=1 — przycisk w panelu pojawia się tylko dla domen bez klucza. D3 ma potwierdzić, że set_dkim działa przy dkim=1; jeśli nie — alternatywa z dokumentacji: scripts/dkim_create.sh &lt;domena&gt; po stronie węzła (zadanie agenta).</t>
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr">
@@ -5249,12 +5249,12 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>E-05</t>
+          <t>E-17</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Zmiana quoty ISTNIEJĄCEJ skrzynki</t>
+          <t>Rekord DMARC — konfiguracja</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -5300,12 +5300,12 @@
       </c>
       <c r="L58" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/hosting-email/quota (ZmienRozmiarSkrzynkiDto 10–102400 MB) → directadmin.service changeHostingEmailQuota (CMD_API_POP action=modify bez passwd) + audyt HOSTING_EMAIL_QUOTA_CHANGED; UI MailTab — klik w rozmiar skrzynki</t>
+          <t>2026-09-23 D1: mail-auth.ts dmarcCheck (brak / p=none / kilka rekordów) + lib/dmarc.ts tuneDmarc (polityka + adres raportów) w deliverability-panel.tsx; testy mail-auth.spec.ts, dmarc.spec.ts</t>
         </is>
       </c>
       <c r="M58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="N58" s="11" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="O58" s="11" t="inlineStr">
         <is>
-          <t>brak jakiejkolwiek ścieżki edycji — klient musi usunąć i odtworzyć skrzynkę | KOD: zmiana rozmiaru bez usuwania skrzynki. Przy okazji body tworzenia skrzynki i zmiany hasła dostały klasy DTO (wcześniej interfejs = zero walidacji na granicy zaufania). OTWARTE do D3: czy DA przy modify bez passwd zostawia hasło (komentarz ponytail).</t>
+          <t>j.w. | KOD: kreator DMARC — wybór polityki i opcjonalny adres raportów, zachowuje pozostałe tagi. Sugestia bez rua na verris.pl (raporty do obcej domeny wymagają rekordu autoryzacji). OTWARTE do D3: zapis do strefy DA.</t>
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr">
@@ -5327,12 +5327,12 @@
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>M-26</t>
+          <t>E-05</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>Usunięcie zapisanej karty przez klienta</t>
+          <t>Zmiana quoty ISTNIEJĄCEJ skrzynki</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
@@ -5373,12 +5373,12 @@
       </c>
       <c r="K59" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L59" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: DELETE /billing/payment-methods/:id (ParseUUIDPipe) → billing.service deleteMyPaymentMethod: Stripe detach, usunięcie wiersza, zerowanie karty domyślnej i auto-doładowania, audyt PAYMENT_METHOD_REMOVED; UI billing-extras-forms „Zapisane karty”; test usun-karte.spec.ts | 2026-09-23: zapis kart — billing.service handlePaymentMethodAttached/Detached (webhooki payment_method.attached/.detached, upsert po provider+providerRef, pierwsza karta domyślna); test D2 zapis-karty.spec.ts</t>
+          <t>2026-09-23 D1: POST /services/:id/hosting-email/quota (ZmienRozmiarSkrzynkiDto 10–102400 MB) → directadmin.service changeHostingEmailQuota (CMD_API_POP action=modify bez passwd) + audyt HOSTING_EMAIL_QUOTA_CHANGED; UI MailTab — klik w rozmiar skrzynki</t>
         </is>
       </c>
       <c r="M59" s="11" t="inlineStr">
@@ -5388,12 +5388,12 @@
       </c>
       <c r="N59" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O59" s="11" t="inlineStr">
         <is>
-          <t>wymóg konsumencki | KOD gotowy i przetestowany na atrapach. UWAGA: nic w API nie zapisuje dziś wierszy PaymentMethod (brak create/upsert) — lista kart jest zawsze pusta, więc usuwanie da się sprawdzić dopiero, gdy zapis kart zostanie podpięty (webhook Stripe po płatności kartą). | 2026-09-23: domknięty brakujący zapis — karta zapisana w Stripe (np. przy subskrypcji kartą) pojawia się w panelu, odpięta (także z dashboardu Stripe) znika i odpina się od auto-doładowania. WYMAGA OD WŁAŚCICIELA: dopisać zdarzenia payment_method.attached i payment_method.detached do endpointu webhooka w Stripe (DEPLOY.md, OPERATIONAL_CHECKLIST). Karty zapisane przed tą zmianą nie pojawią się wstecz. D3 przy pierwszej płatności kartą.</t>
+          <t>brak jakiejkolwiek ścieżki edycji — klient musi usunąć i odtworzyć skrzynkę | KOD: zmiana rozmiaru bez usuwania skrzynki. Przy okazji body tworzenia skrzynki i zmiany hasła dostały klasy DTO (wcześniej interfejs = zero walidacji na granicy zaufania). OTWARTE do D3: czy DA przy modify bez passwd zostawia hasło (komentarz ponytail).</t>
         </is>
       </c>
       <c r="P59" s="10" t="inlineStr">
@@ -5405,58 +5405,58 @@
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>PB-17</t>
+          <t>M-26</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>Asystent v1: dymki, naprawy jednym kliknięciem, czat z danymi konta</t>
+          <t>Usunięcie zapisanej karty przez klienta</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F60" s="10" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G60" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
+          <t>Faza 1 — Rozliczenia i dowód odtworzenia</t>
         </is>
       </c>
       <c r="I60" s="10" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J60" s="10" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K60" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-09-23 D1: DELETE /billing/payment-methods/:id (ParseUUIDPipe) → billing.service deleteMyPaymentMethod: Stripe detach, usunięcie wiersza, zerowanie karty domyślnej i auto-doładowania, audyt PAYMENT_METHOD_REMOVED; UI billing-extras-forms „Zapisane karty”; test usun-karte.spec.ts | 2026-09-23: zapis kart — billing.service handlePaymentMethodAttached/Detached (webhooki payment_method.attached/.detached, upsert po provider+providerRef, pierwsza karta domyślna); test D2 zapis-karty.spec.ts</t>
         </is>
       </c>
       <c r="M60" s="11" t="inlineStr">
@@ -5466,12 +5466,12 @@
       </c>
       <c r="N60" s="11" t="inlineStr">
         <is>
-          <t>Co najmniej 5 reguł dymków z testami; każda naprawa ma cofnięcie i wpis audytu; czat odpowiada z kontekstem usługi; brak akcji destrukcyjnych w v1.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O60" s="11" t="inlineStr">
         <is>
-          <t>Dymki kontekstowe na regułach (bez kosztu AI): dysk, domena nie wskazuje na nas, SPF/DKIM, SSL wygasa, backup nieświeży — najwyżej jeden na ekran, „nie pokazuj więcej”. Naprawy jednym kliknięciem tylko dla akcji odwracalnych, z kartą podglądu skutku i „Cofnij”. Obecny czat (HostingAssistant, RAG) dostaje odczyt danych konta. Każda akcja w audycie. Diagnoza i naprawy po naszej stronie za darmo.</t>
+          <t>wymóg konsumencki | KOD gotowy i przetestowany na atrapach. UWAGA: nic w API nie zapisuje dziś wierszy PaymentMethod (brak create/upsert) — lista kart jest zawsze pusta, więc usuwanie da się sprawdzić dopiero, gdy zapis kart zostanie podpięty (webhook Stripe po płatności kartą). | 2026-09-23: domknięty brakujący zapis — karta zapisana w Stripe (np. przy subskrypcji kartą) pojawia się w panelu, odpięta (także z dashboardu Stripe) znika i odpina się od auto-doładowania. WYMAGA OD WŁAŚCICIELA: dopisać zdarzenia payment_method.attached i payment_method.detached do endpointu webhooka w Stripe (DEPLOY.md, OPERATIONAL_CHECKLIST). Karty zapisane przed tą zmianą nie pojawią się wstecz. D3 przy pierwszej płatności kartą.</t>
         </is>
       </c>
       <c r="P60" s="10" t="inlineStr">
@@ -5483,12 +5483,12 @@
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>PB-18</t>
+          <t>PB-17</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Tickety v2: podgląd klienta, szablony ze zmiennymi, szkice odpowiedzi</t>
+          <t>Asystent v1: dymki, naprawy jednym kliknięciem, czat z danymi konta</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -5507,10 +5507,10 @@
         </is>
       </c>
       <c r="F61" s="10" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G61" s="10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
@@ -5519,12 +5519,12 @@
       </c>
       <c r="I61" s="10" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="J61" s="10" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K61" s="10" t="inlineStr">
@@ -5544,12 +5544,12 @@
       </c>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>Podgląd klienta bez przechodzenia między ekranami; szablony podstawiają zmienne z testem; szkic odpowiedzi dla 6 kategorii (DNS, SSL, poczta, płatność, migracja, awaria).</t>
+          <t>Co najmniej 5 reguł dymków z testami; każda naprawa ma cofnięcie i wpis audytu; czat odpowiada z kontekstem usługi; brak akcji destrukcyjnych w v1.</t>
         </is>
       </c>
       <c r="O61" s="11" t="inlineStr">
         <is>
-          <t>Panel staff: boczny podgląd klienta w tickecie (usługi, saldo, faktury/dokumenty, zdarzenia, historia zgłoszeń, health score); szablony odpowiedzi ze zmiennymi (imię, domena, usługa, termin) i kategoriami — rozbudowa canned responses; klasyfikacja zgłoszenia i szkic odpowiedzi z bazy wiedzy i danych konta (do akceptacji, bez auto-wysyłki w v2); akcje z ticketu z audytem; licznik SLA.</t>
+          <t>Dymki kontekstowe na regułach (bez kosztu AI): dysk, domena nie wskazuje na nas, SPF/DKIM, SSL wygasa, backup nieświeży — najwyżej jeden na ekran, „nie pokazuj więcej”. Naprawy jednym kliknięciem tylko dla akcji odwracalnych, z kartą podglądu skutku i „Cofnij”. Obecny czat (HostingAssistant, RAG) dostaje odczyt danych konta. Każda akcja w audycie. Diagnoza i naprawy po naszej stronie za darmo.</t>
         </is>
       </c>
       <c r="P61" s="10" t="inlineStr">
@@ -5561,34 +5561,34 @@
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>A-25</t>
+          <t>PB-18</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Ręczne zawieszenie usługi przez operatora</t>
+          <t>Tickety v2: podgląd klienta, szablony ze zmiennymi, szkice odpowiedzi</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F62" s="10" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="G62" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
@@ -5597,22 +5597,22 @@
       </c>
       <c r="I62" s="10" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="J62" s="10" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="K62" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L62" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: admin-panel subscriptions/[id]/suspend-form.tsx + suspend-actions.ts → POST /admin/subscriptions/:id/suspend (powód, notatka, potwierdzenie)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M62" s="11" t="inlineStr">
@@ -5622,12 +5622,12 @@
       </c>
       <c r="N62" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Podgląd klienta bez przechodzenia między ekranami; szablony podstawiają zmienne z testem; szkic odpowiedzi dla 6 kategorii (DNS, SSL, poczta, płatność, migracja, awaria).</t>
         </is>
       </c>
       <c r="O62" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: endpoint działa i jest osiągalny (curl + DirectAdmin), auto-suspend za brak płatności działa. Brakuje UI, nie możliwości zatrzymania szkody. | UI zrobione. OTWARTE do D3 (PB-21, serwer testowy): zawieszenie konta w DirectAdminie na żywym węźle.</t>
+          <t>Panel staff: boczny podgląd klienta w tickecie (usługi, saldo, faktury/dokumenty, zdarzenia, historia zgłoszeń, health score); szablony odpowiedzi ze zmiennymi (imię, domena, usługa, termin) i kategoriami — rozbudowa canned responses; klasyfikacja zgłoszenia i szkic odpowiedzi z bazy wiedzy i danych konta (do akceptacji, bez auto-wysyłki w v2); akcje z ticketu z audytem; licznik SLA.</t>
         </is>
       </c>
       <c r="P62" s="10" t="inlineStr">
@@ -5639,12 +5639,12 @@
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>A-26</t>
+          <t>A-25</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Ręczne odwieszenie usługi przez operatora</t>
+          <t>Ręczne zawieszenie usługi przez operatora</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -5690,12 +5690,12 @@
       </c>
       <c r="L63" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: ten sam formularz — odwieszenie z opcją obciążenia za odnowienie (chargeRenewal)</t>
+          <t>2026-09-23 D1: admin-panel subscriptions/[id]/suspend-form.tsx + suspend-actions.ts → POST /admin/subscriptions/:id/suspend (powód, notatka, potwierdzenie)</t>
         </is>
       </c>
       <c r="M63" s="11" t="inlineStr">
         <is>
-          <t>A-25 (ten sam widok)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N63" s="11" t="inlineStr">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="O63" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: jak A-25, endpoint subscriptions.admin.controller.ts:210 działa z chargeRenewal. | UI zrobione. OTWARTE do D3 (PB-21): odwieszenie konta w DA na żywym węźle.</t>
+          <t>Skorygowane: endpoint działa i jest osiągalny (curl + DirectAdmin), auto-suspend za brak płatności działa. Brakuje UI, nie możliwości zatrzymania szkody. | UI zrobione. OTWARTE do D3 (PB-21, serwer testowy): zawieszenie konta w DirectAdminie na żywym węźle.</t>
         </is>
       </c>
       <c r="P63" s="10" t="inlineStr">
@@ -5717,12 +5717,12 @@
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>N-07</t>
+          <t>A-26</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>Ręczne tworzenie incydentu na status page</t>
+          <t>Ręczne odwieszenie usługi przez operatora</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E64" s="10" t="inlineStr">
@@ -5763,27 +5763,27 @@
       </c>
       <c r="K64" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L64" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D2: admin-panel status/incidents/incident-compose.tsx → POST /admin/product-ops/incidents; przycisk „Rozwiąż” (PATCH incidents/:id status=RESOLVED); probe-ingest.service.ts isManualIncident; test status/incydent-reczny.spec.ts</t>
+          <t>2026-09-23 D1: ten sam formularz — odwieszenie z opcją obciążenia za odnowienie (chargeRenewal)</t>
         </is>
       </c>
       <c r="M64" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A-25 (ten sam widok)</t>
         </is>
       </c>
       <c r="N64" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O64" s="11" t="inlineStr">
         <is>
-          <t>w kryzysie nie ma jak zakomunikować awarii | ZNALEZISKO: incydent ogłoszony ręcznie zamykał się sam przy pierwszej udanej próbie monitora (w ciągu minut), więc komunikat o awarii, której monitor nie widzi, znikał ze status page. Teraz zamyka go tylko operator; zamknięcie wysyła webhook INCIDENT_RESOLVED i trafia do audytu.</t>
+          <t>Skorygowane: jak A-25, endpoint subscriptions.admin.controller.ts:210 działa z chargeRenewal. | UI zrobione. OTWARTE do D3 (PB-21): odwieszenie konta w DA na żywym węźle.</t>
         </is>
       </c>
       <c r="P64" s="10" t="inlineStr">
@@ -5795,12 +5795,12 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>N-14</t>
+          <t>N-07</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>Cordon wysyłki poczty (auto-blokada spamu)</t>
+          <t>Ręczne tworzenie incydentu na status page</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="L65" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: admin-panel /deliverability (Blokady wysyłki poczty, link w menu) → GET/POST /admin/deliverability/cordons; lista z e-mailem i nazwą klienta</t>
+          <t>2026-09-23 D2: admin-panel status/incidents/incident-compose.tsx → POST /admin/product-ops/incidents; przycisk „Rozwiąż” (PATCH incidents/:id status=RESOLVED); probe-ingest.service.ts isManualIncident; test status/incydent-reczny.spec.ts</t>
         </is>
       </c>
       <c r="M65" s="11" t="inlineStr">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="O65" s="11" t="inlineStr">
         <is>
-          <t>mechanizm działa, operator nie może go zobaczyć ani zdjąć | Operator widzi kogo i dlaczego zablokowano oraz zdejmuje blokadę (ADMIN, z potwierdzeniem, audyt po stronie API).</t>
+          <t>w kryzysie nie ma jak zakomunikować awarii | ZNALEZISKO: incydent ogłoszony ręcznie zamykał się sam przy pierwszej udanej próbie monitora (w ciągu minut), więc komunikat o awarii, której monitor nie widzi, znikał ze status page. Teraz zamyka go tylko operator; zamknięcie wysyła webhook INCIDENT_RESOLVED i trafia do audytu.</t>
         </is>
       </c>
       <c r="P65" s="10" t="inlineStr">
@@ -5873,12 +5873,12 @@
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>H-22</t>
+          <t>N-14</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Panel odtwarzania w widocznym miejscu</t>
+          <t>Cordon wysyłki poczty (auto-blokada spamu)</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E66" s="10" t="inlineStr">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="L66" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: client-panel BackupsTab.tsx — sekcja „Kopie poza serwerem” (HostingOffsitePanel) w zakładce Kopie zapasowe; zdublowany panel przywracania usunięty z Zużycia zasobów (hosting-backup-restore-panel.tsx)</t>
+          <t>2026-09-23: admin-panel /deliverability (Blokady wysyłki poczty, link w menu) → GET/POST /admin/deliverability/cordons; lista z e-mailem i nazwą klienta</t>
         </is>
       </c>
       <c r="M66" s="11" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="O66" s="11" t="inlineStr">
         <is>
-          <t>klient w kryzysie tego nie znajdzie | Kopie off-site są tam, gdzie klient ich szuka w kryzysie; przywracanie jest w jednym miejscu, z potwierdzeniem domeną.</t>
+          <t>mechanizm działa, operator nie może go zobaczyć ani zdjąć | Operator widzi kogo i dlaczego zablokowano oraz zdejmuje blokadę (ADMIN, z potwierdzeniem, audyt po stronie API).</t>
         </is>
       </c>
       <c r="P66" s="10" t="inlineStr">
@@ -5951,12 +5951,12 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>H-09</t>
+          <t>H-22</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>Kopia bezpieczeństwa przed odtworzeniem</t>
+          <t>Panel odtwarzania w widocznym miejscu</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -5978,7 +5978,7 @@
         <v>6</v>
       </c>
       <c r="G67" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H67" s="10" t="inlineStr">
         <is>
@@ -5987,22 +5987,22 @@
       </c>
       <c r="I67" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J67" s="10" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K67" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L67" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
+          <t>2026-09-23: client-panel BackupsTab.tsx — sekcja „Kopie poza serwerem” (HostingOffsitePanel) w zakładce Kopie zapasowe; zdublowany panel przywracania usunięty z Zużycia zasobów (hosting-backup-restore-panel.tsx)</t>
         </is>
       </c>
       <c r="M67" s="11" t="inlineStr">
@@ -6012,12 +6012,12 @@
       </c>
       <c r="N67" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O67" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: hosting-restore.service.ts:167 tylko KOLEJKUJE backup w DA i nie czeka na wynik — destrukcyjne odtworzenie rusza mimo nieudanej kopii. Job dostaje COMPLETED (:182) w chwili przyjęcia zadania, nie po odtworzeniu. | Naprawione: nadpisywanie danych bez siatki. Status COMPLETED w panelu klienta opisany uczciwie („Odtwarzanie zlecone — serwer odtwarza dane w tle”), bo DA przyjmuje odtworzenie asynchronicznie. OTWARTE do D3 (PB-21): pełny przebieg na żywym DA i wykrycie końca odtwarzania.</t>
+          <t>klient w kryzysie tego nie znajdzie | Kopie off-site są tam, gdzie klient ich szuka w kryzysie; przywracanie jest w jednym miejscu, z potwierdzeniem domeną.</t>
         </is>
       </c>
       <c r="P67" s="10" t="inlineStr">
@@ -6029,12 +6029,12 @@
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>H-17</t>
+          <t>H-09</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>Tryb restore skryptu odtwarzającego osiągalny z produktu</t>
+          <t>Kopia bezpieczeństwa przed odtworzeniem</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -6075,27 +6075,27 @@
       </c>
       <c r="K68" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L68" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23: produktowa ścieżka odtwarzania z off-site = „Pobierz na serwer” (fetch, agent) + przywrócenie z listy kopii z kopią bezpieczeństwa (H-09) i potwierdzeniem domeną; tryb `restore` skryptu (DA type=admin, bez kopii bezpieczeństwa) celowo zostaje tylko w CLI/runbooku DR</t>
+          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
         </is>
       </c>
       <c r="M68" s="11" t="inlineStr">
         <is>
-          <t>H-20 (najpierw potwierdzone odtworzenie, potem wystawienie trybu w produkcie)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N68" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>Skorygowane: tryb restore jest martwy z poziomu produktu, ale żywy z CLI (node-account-restore.sh:120-124) i udokumentowany w runbooku. | DO DECYZJI WŁAŚCICIELA: proponuję zamknąć jako PARYTET przez równoważną ścieżkę produktową — wystawienie trybu `restore` ominęłoby kopię bezpieczeństwa z H-09. Tryb restore działa też tylko przy istniejącym koncie na węźle, czyli dokładnie tam, gdzie wystarcza fetch + przywrócenie. | DECYZJA WŁAŚCICIELA 2026-09-23: zamknięte jako PARYTET — ścieżka produktowa (pobierz na serwer + przywrócenie z kopią bezpieczeństwa i potwierdzeniem domeną) daje ten sam efekt bezpieczniej; tryb restore skryptu zostaje wyłącznie w CLI/runbooku DR.</t>
+          <t>OSŁABIONE: hosting-restore.service.ts:167 tylko KOLEJKUJE backup w DA i nie czeka na wynik — destrukcyjne odtworzenie rusza mimo nieudanej kopii. Job dostaje COMPLETED (:182) w chwili przyjęcia zadania, nie po odtworzeniu. | Naprawione: nadpisywanie danych bez siatki. Status COMPLETED w panelu klienta opisany uczciwie („Odtwarzanie zlecone — serwer odtwarza dane w tle”), bo DA przyjmuje odtworzenie asynchronicznie. OTWARTE do D3 (PB-21): pełny przebieg na żywym DA i wykrycie końca odtwarzania.</t>
         </is>
       </c>
       <c r="P68" s="10" t="inlineStr">
@@ -6107,12 +6107,12 @@
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>G-20</t>
+          <t>H-17</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Ochrona przed atakiem słownikowym na panel</t>
+          <t>Tryb restore skryptu odtwarzającego osiągalny z produktu</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="E69" s="10" t="inlineStr">
@@ -6158,12 +6158,12 @@
       </c>
       <c r="L69" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D2: common/guards/rate-limit.guard.spec.ts (6 testów: limit per IP, per e-mail z wielu IP, reset okna, zakresy i @SkipRateLimit, przepełnienie mapy, awaria Redisa)</t>
+          <t>2026-09-23: produktowa ścieżka odtwarzania z off-site = „Pobierz na serwer” (fetch, agent) + przywrócenie z listy kopii z kopią bezpieczeństwa (H-09) i potwierdzeniem domeną; tryb `restore` skryptu (DA type=admin, bez kopii bezpieczeństwa) celowo zostaje tylko w CLI/runbooku DR</t>
         </is>
       </c>
       <c r="M69" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>H-20 (najpierw potwierdzone odtworzenie, potem wystawienie trybu w produkcie)</t>
         </is>
       </c>
       <c r="N69" s="11" t="inlineStr">
@@ -6173,7 +6173,7 @@
       </c>
       <c r="O69" s="11" t="inlineStr">
         <is>
-          <t>brak dowodu D2 na krytycznym guardzie | ZNALEZISKO przy pisaniu testów: w trybie pamięciowym przepełnienie mapy (50 tys. kluczy) czyściło WSZYSTKIE liczniki — losowe e-maile zerowały licznik prób logowania do atakowanego konta (fail-open). Teraz usuwane są tylko wygasłe, a przy pełnej mapie nowe klucze dostają 429 (fail-closed).</t>
+          <t>Skorygowane: tryb restore jest martwy z poziomu produktu, ale żywy z CLI (node-account-restore.sh:120-124) i udokumentowany w runbooku. | DO DECYZJI WŁAŚCICIELA: proponuję zamknąć jako PARYTET przez równoważną ścieżkę produktową — wystawienie trybu `restore` ominęłoby kopię bezpieczeństwa z H-09. Tryb restore działa też tylko przy istniejącym koncie na węźle, czyli dokładnie tam, gdzie wystarcza fetch + przywrócenie. | DECYZJA WŁAŚCICIELA 2026-09-23: zamknięte jako PARYTET — ścieżka produktowa (pobierz na serwer + przywrócenie z kopią bezpieczeństwa i potwierdzeniem domeną) daje ten sam efekt bezpieczniej; tryb restore skryptu zostaje wyłącznie w CLI/runbooku DR.</t>
         </is>
       </c>
       <c r="P69" s="10" t="inlineStr">
@@ -6185,12 +6185,12 @@
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>I-11</t>
+          <t>G-20</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>Staging — publikacja na produkcję</t>
+          <t>Ochrona przed atakiem słownikowym na panel</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -6200,7 +6200,7 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E70" s="10" t="inlineStr">
@@ -6231,12 +6231,12 @@
       </c>
       <c r="K70" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L70" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
+          <t>2026-09-23 D2: common/guards/rate-limit.guard.spec.ts (6 testów: limit per IP, per e-mail z wielu IP, reset okna, zakresy i @SkipRateLimit, przepełnienie mapy, awaria Redisa)</t>
         </is>
       </c>
       <c r="M70" s="11" t="inlineStr">
@@ -6246,12 +6246,12 @@
       </c>
       <c r="N70" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O70" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: node-staging-sync.sh:141-142 backup plików jest twardą bramką, ale :152-153 backup bazy LIVE jest best-effort — linia 158 robi wp db import na produkcji mimo braku kopii. | Naprawione: import bazy staging na produkcję mimo braku kopii bazy LIVE. OTWARTE do D3 (PB-21): publikacja stagingu na żywym węźle.</t>
+          <t>brak dowodu D2 na krytycznym guardzie | ZNALEZISKO przy pisaniu testów: w trybie pamięciowym przepełnienie mapy (50 tys. kluczy) czyściło WSZYSTKIE liczniki — losowe e-maile zerowały licznik prób logowania do atakowanego konta (fail-open). Teraz usuwane są tylko wygasłe, a przy pełnej mapie nowe klucze dostają 429 (fail-closed).</t>
         </is>
       </c>
       <c r="P70" s="10" t="inlineStr">
@@ -6263,12 +6263,12 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>X-31</t>
+          <t>I-11</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>Kanał alertów daje znak życia (dead man's switch)</t>
+          <t>Staging — publikacja na produkcję</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -6278,19 +6278,19 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F71" s="10" t="n">
         <v>6</v>
       </c>
       <c r="G71" s="10" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H71" s="10" t="inlineStr">
         <is>
@@ -6299,22 +6299,22 @@
       </c>
       <c r="I71" s="10" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="J71" s="10" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="K71" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L71" s="11" t="inlineStr">
         <is>
-          <t>ops/observability/grafana/provisioning/alerting/rules.yaml — grupa verris_kanal_alertow, reguła VerrisKanalAlertowZyje (vector(1), for: 0s, oba stany awaryjne na Alerting, etykieta kanal: heartbeat); policies.yaml — gałąź object_matchers kanal=heartbeat, repeat_interval 24h; apps/api/src/test/routing-alertow.spec.ts (5 asercji X-31); docs/ops/GRAFANA_ALERTING.md §4. BRAK: pierwszego maila [FIRING:1] VerrisKanalAlertowZyje — dowód D3 jeszcze nie powstał.</t>
+          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
         </is>
       </c>
       <c r="M71" s="11" t="inlineStr">
@@ -6324,12 +6324,12 @@
       </c>
       <c r="N71" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O71" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 powstanie przy pierwszym mailu. Decyzja właściciela produktu: wariant „jeden mail na dobę". | PROBLEM: po naprawie X-30 alerty ucichną, a cisza będzie znaczyła „nic się nie pali" — i będzie wyglądała IDENTYCZNIE jak: Grafana padła, Postfix przestał przyjmować, mail.hvln.pl zaczął odrzucać albo wrzucać do spamu, ktoś zmienił adres w punkcie kontaktowym, polityka przestała pasować do etykiet. To dokładnie ta sama cisza, która przez miesiąc znaczyła „kopia bazy jest w porządku" (H-23) i kosztowała wszystkie kopie zapasowe. | ROZWIĄZANIE: VerrisKanalAlertowZyje — reguła vector(1), pali się ZAWSZE, jej BRAK jest sygnałem. for: 0s, noDataState: Alerting, execErrState: Alerting — nie da się jej „nie zapalić": normalnie warunek jest spełniony, a gdyby źródło danych przestało odpowiadać, oba stany awaryjne też prowadzą do Alerting. Milczenie ma znaczyć awarię, nigdy spokój. | JEDEN MAIL NA DOBĘ, NIE SZEŚĆ: osobna gałąź polityki na etykiecie kanal: heartbeat z repeat_interval 24h. Na domyślnej (4h) byłoby sześć dziennie, a alert przychodzący sześć razy dziennie przestaje być czytany po tygodniu — wtedy przestaje cokolwiek dawać, bo jego BRAK jest jedyną informacją, jaką niesie. Strażnik pilnuje osobno, że polityka domyślna NIE została przy okazji przestawiona na dobę: prawdziwy alarm ma się przypominać co cztery godziny. | HACZYK, KTÓRY TRZEBA NAZWAĆ: mail, którego się nie czyta, wraca do punktu wyjścia. Jeśli po tygodniu przestanie być zauważany, reguła przestaje działać — nie dlatego, że jest zepsuta, tylko dlatego, że przestała być czytana. Tego nie da się naprawić kodem. | CZEGO NIE OBEJMUJE: awarii całego serwera (heartbeat mieszka na tej samej maszynie co Grafana i milczy razem z nią — odporny byłby watchdog SPOZA naszej infrastruktury, pukany cronem; nie ma go i to świadoma decyzja, nie przeoczenie) ani poprawności pozostałych reguł (tego pilnuje bramka z X-30). | Czerwieni się na starym kodzie: 5 z 36. | Doszła lista DOPISANE_POZNIEJ, trzymana osobno od ALERTY: tamta odpowiada na pytanie „czy migracja czegoś nie zgubiła" i ma zostać zamrożona, ta na „czy ktoś czegoś po cichu nie dołożył". Dokumentacja: docs/archiwum/zadania/X-31-znak-zycia-kanalu-alertow.md | 2026-09-22 D3: wlasciciel potwierdza, ze mail [FIRING:1] VerrisKanalAlertowZyje przychodzi codziennie. Kanal alertow dziala koniec-do-konca.</t>
+          <t>OSŁABIONE: node-staging-sync.sh:141-142 backup plików jest twardą bramką, ale :152-153 backup bazy LIVE jest best-effort — linia 158 robi wp db import na produkcji mimo braku kopii. | Naprawione: import bazy staging na produkcję mimo braku kopii bazy LIVE. OTWARTE do D3 (PB-21): publikacja stagingu na żywym węźle.</t>
         </is>
       </c>
       <c r="P71" s="10" t="inlineStr">
@@ -6341,12 +6341,12 @@
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>X-32</t>
+          <t>X-31</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Martwy job da się odrzucić z panelu, ze śladem w audycie</t>
+          <t>Kanał alertów daje znak życia (dead man's switch)</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="L72" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/common/audit/audit.actions.ts — PROVISIONING_JOB_DISCARDED_BY_ADMIN; provisioning-queue.service.ts — odrzucJob (getState() === failed, ślad przed job.remove(), audyt z subskrypcją, typem, liczbą prób, failedReason i powodem); provisioning-queue.admin.controller.ts — POST :id/odrzuc za @StaffPerm('PROVISIONING_MANAGE'); apps/admin-panel/.../provisioning-queue/ — actions.ts, odrzuc-button.tsx (dwa kliknięcia, powód ≥5 znaków, zdanie o nietkniętej subskrypcji), page.tsx; apps/api/src/test/odrzucenie-martwego-joba.spec.ts (13). BRAK: pierwszego odrzucenia na produkcji — dowód D3 jeszcze nie powstał.</t>
+          <t>ops/observability/grafana/provisioning/alerting/rules.yaml — grupa verris_kanal_alertow, reguła VerrisKanalAlertowZyje (vector(1), for: 0s, oba stany awaryjne na Alerting, etykieta kanal: heartbeat); policies.yaml — gałąź object_matchers kanal=heartbeat, repeat_interval 24h; apps/api/src/test/routing-alertow.spec.ts (5 asercji X-31); docs/ops/GRAFANA_ALERTING.md §4. BRAK: pierwszego maila [FIRING:1] VerrisKanalAlertowZyje — dowód D3 jeszcze nie powstał.</t>
         </is>
       </c>
       <c r="M72" s="11" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="O72" s="11" t="inlineStr">
         <is>
-          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 przy pierwszym odrzuceniu na produkcji — a to da się zrobić od razu po wdrożeniu, w odróżnieniu od Z-18, który czeka na węzeł. Decyzja właściciela produktu: dorobić akcję w panelu zamiast jednorazowego czyszczenia Redisa. | JAK TO WYSZŁO: X-30 naprawiło alerting, VerrisProvisioningQueueFailed zapalił się z prawdziwego powodu i wskazał cztery martwe joby (to z nich wyszło Z-18). Naturalny następny ruch — usunąć je — okazał się NIEWYKONALNY: panel ma przy nich wyłącznie „Retry", a kontroler administracyjny dokładnie dwa endpointy, listowanie i ponowienie. Retry nic nie daje, bo węzła nie ma: job padnie ponownie, podbije licznik prób i dołoży wpisy do audytu — cztery martwe joby zamieniają się w cztery martwe joby z dłuższą historią. Zostawało grzebanie w Redisie ręcznie, czyli zmiana stanu produkcyjnego dotyczącego subskrypcji klientów BEZ ŚLADU W AUDYCIE. | TO NIE JEST USTERKA TYCH CZTERECH JOBÓW, tylko luka w warstwie operatorskiej, która ujawni się ponownie przy pierwszym prawdziwym niepowodzeniu provisioningu — z tą różnicą, że wtedy po drugiej stronie będzie klient. | ROZWIĄZANIE: POST /admin/provisioning-queue/:id/odrzuc + przycisk „Odrzuć" obok Retry. TRZY REGUŁY: (1) TYLKO STAN failed — usunięcie joba aktywnego albo czekającego osierociłoby provisioning w trakcie, konto na węźle mogłoby powstać, a system przestałby o nim wiedzieć; ograniczenie siedzi w usłudze, nie w kontrolerze, bo to reguła o kolejce, nie o HTTP; (2) POWÓD WYMAGANY, tak samo jak przy retry — operacja bez powodu to operacja, której za pół roku nikt nie wyjaśni; (3) NAJPIERW ODCZYT, POTEM USUNIĘCIE — ślad zbierany PRZED job.remove(), bo po usunięciu nie ma już czego odczytać; zapisujemy subskrypcję, joba, typ, liczbę prób, ostatni błąd i powód. Po Z-18 ten ostatni błąd niesie PRAWDZIWĄ przyczynę, więc wpis ma realną wartość dowodową — jeszcze wczoraj zapisałby zdanie o brakującym pakiecie DirectAdmina, którego nigdy nie brakowało. | OSOBNA AKCJA AUDYTU (PROVISIONING_JOB_DISCARDED_BY_ADMIN), nie wariant retry: w raportach odrzucenie i ponowienie to dwie różne decyzje i nie wolno im się zlewać. | DWA KLIKNIĘCIA, NIE JEDNO: retry można cofnąć następnym retry, odrzucenia nie da się cofnąć wcale. Potwierdzenie jest po to, żeby ta różnica była wyczuwalna w palcach. | ZDANIE PRZY PRZYCISKU: „Usuwa wpis z kolejki bez możliwości cofnięcia. Subskrypcja zostaje nietknięta." Operator ma prawo założyć, że „odrzuć" anuluje zamówienie — nie anuluje. Musi to być napisane tam, gdzie się klika, a nie w dokumentacji, której nikt nie otworzy w trakcie incydentu. | Czerwieni się na starym kodzie: 11 z 13. | DWIE UWAGI O SAMYCH TESTACH: odczyty plików panelu są LENIWE, bo odczyt na poziomie describe wywalał cały plik testowy, zanim cokolwiek się policzyło — a wtedy nie wiadomo, ILE asercji się czerwieni, tylko że „nie skompilowało się"; asercja o warunku row.failedReason nie mierzy odległości w znakach, tylko relację między warunkiem a przyciskiem, bo wersja licząca znaki zepsuła się od dopisania komentarza i kusiło, żeby poszerzyć okno zamiast poprawić asercję — to byłoby naprawianie testu zamiast kodu. | CZEGO NIE OBEJMUJE: losu czterech subskrypcji, które dostały zwrot i status PENDING_PAYMENT (odrzucenie joba ich nie dotyka — osobne sprzątanie po stronie bazy); odrzucania hurtem — świadomie, bo przycisk „odrzuć wszystkie" jest wygodny dokładnie do momentu, w którym ktoś kliknie go na kolejce z prawdziwym zamówieniem. | JAK ZAMKNĄĆ: odrzucić jeden z czterech martwych jobów, obejrzeć wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie i sprawdzić, że verris_provisioning_queue_depth{state="failed"} spadło o jeden. Dokumentacja: docs/archiwum/zadania/X-32-odrzucenie-martwego-joba.md | 2026-09-22 D3: wlasciciel odrzucil martwy job przyciskiem 'Odrzuc' w panelu admina na produkcji (potwierdzenie wlasciciela; wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie).</t>
+          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 powstanie przy pierwszym mailu. Decyzja właściciela produktu: wariant „jeden mail na dobę". | PROBLEM: po naprawie X-30 alerty ucichną, a cisza będzie znaczyła „nic się nie pali" — i będzie wyglądała IDENTYCZNIE jak: Grafana padła, Postfix przestał przyjmować, mail.hvln.pl zaczął odrzucać albo wrzucać do spamu, ktoś zmienił adres w punkcie kontaktowym, polityka przestała pasować do etykiet. To dokładnie ta sama cisza, która przez miesiąc znaczyła „kopia bazy jest w porządku" (H-23) i kosztowała wszystkie kopie zapasowe. | ROZWIĄZANIE: VerrisKanalAlertowZyje — reguła vector(1), pali się ZAWSZE, jej BRAK jest sygnałem. for: 0s, noDataState: Alerting, execErrState: Alerting — nie da się jej „nie zapalić": normalnie warunek jest spełniony, a gdyby źródło danych przestało odpowiadać, oba stany awaryjne też prowadzą do Alerting. Milczenie ma znaczyć awarię, nigdy spokój. | JEDEN MAIL NA DOBĘ, NIE SZEŚĆ: osobna gałąź polityki na etykiecie kanal: heartbeat z repeat_interval 24h. Na domyślnej (4h) byłoby sześć dziennie, a alert przychodzący sześć razy dziennie przestaje być czytany po tygodniu — wtedy przestaje cokolwiek dawać, bo jego BRAK jest jedyną informacją, jaką niesie. Strażnik pilnuje osobno, że polityka domyślna NIE została przy okazji przestawiona na dobę: prawdziwy alarm ma się przypominać co cztery godziny. | HACZYK, KTÓRY TRZEBA NAZWAĆ: mail, którego się nie czyta, wraca do punktu wyjścia. Jeśli po tygodniu przestanie być zauważany, reguła przestaje działać — nie dlatego, że jest zepsuta, tylko dlatego, że przestała być czytana. Tego nie da się naprawić kodem. | CZEGO NIE OBEJMUJE: awarii całego serwera (heartbeat mieszka na tej samej maszynie co Grafana i milczy razem z nią — odporny byłby watchdog SPOZA naszej infrastruktury, pukany cronem; nie ma go i to świadoma decyzja, nie przeoczenie) ani poprawności pozostałych reguł (tego pilnuje bramka z X-30). | Czerwieni się na starym kodzie: 5 z 36. | Doszła lista DOPISANE_POZNIEJ, trzymana osobno od ALERTY: tamta odpowiada na pytanie „czy migracja czegoś nie zgubiła" i ma zostać zamrożona, ta na „czy ktoś czegoś po cichu nie dołożył". Dokumentacja: docs/archiwum/zadania/X-31-znak-zycia-kanalu-alertow.md | 2026-09-22 D3: wlasciciel potwierdza, ze mail [FIRING:1] VerrisKanalAlertowZyje przychodzi codziennie. Kanal alertow dziala koniec-do-konca.</t>
         </is>
       </c>
       <c r="P72" s="10" t="inlineStr">
@@ -6419,12 +6419,12 @@
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>X-32</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>W drzewie stoją dwa majory ESLinta naraz</t>
+          <t>Martwy job da się odrzucić z panelu, ze śladem w audycie</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -6439,7 +6439,7 @@
       </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F73" s="10" t="n">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="L73" s="11" t="inlineStr">
         <is>
-          <t>package.json (korzeń) — @eslint/js ^10.0.1 przy braku jakiegokolwiek eslint.config.* w korzeniu; libs/eslint-config/node_modules: eslint 10.9.0 obok @eslint/js 9.39.5; apps/api, apps/www, apps/client-panel, apps/status-page, libs/directadmin-sdk — eslint 9.39.5 | 2026-09-23: z korzenia zdjęte nieużywane @eslint/js ^10 i typescript-eslint; libs/eslint-config peer eslint ^9.39.5 (było &gt;=9 → auto-install dociągał 10.9.0); lockfile bez eslint 10; strażnik apps/api/src/test/eslint-jeden-major.spec.ts (deklaracje + peer + lockfile)</t>
+          <t>apps/api/src/common/audit/audit.actions.ts — PROVISIONING_JOB_DISCARDED_BY_ADMIN; provisioning-queue.service.ts — odrzucJob (getState() === failed, ślad przed job.remove(), audyt z subskrypcją, typem, liczbą prób, failedReason i powodem); provisioning-queue.admin.controller.ts — POST :id/odrzuc za @StaffPerm('PROVISIONING_MANAGE'); apps/admin-panel/.../provisioning-queue/ — actions.ts, odrzuc-button.tsx (dwa kliknięcia, powód ≥5 znaków, zdanie o nietkniętej subskrypcji), page.tsx; apps/api/src/test/odrzucenie-martwego-joba.spec.ts (13). BRAK: pierwszego odrzucenia na produkcji — dowód D3 jeszcze nie powstał.</t>
         </is>
       </c>
       <c r="M73" s="11" t="inlineStr">
@@ -6485,7 +6485,7 @@
       </c>
       <c r="O73" s="11" t="inlineStr">
         <is>
-          <t>Odkryte 2026-08-28 przy DEP-01. Korzeń deklaruje @eslint/js ^10.0.1, którego peer to eslint ^10.0.0 — i to on wciąga eslint@10.9.0 do drzewa. Tymczasem KAŻDY pakiet, który realnie lintuje, ma 9.39.5. Najostrzej widać to wewnątrz libs/eslint-config, czyli wspólnej konfiguracji: node_modules/eslint = 10.9.0, node_modules/@eslint/js = 9.39.5 — dwie połowy jednego narzędzia z różnych majorów w jednym katalogu. | Korzeń NIE MA żadnego eslint.config.* i nie odpala lintera (pnpm lint = turbo run lint), więc te zależności nie robią nic poza wciąganiem majora, którego nikt nie używa. | To nie awaria — bramka jest zielona, 0 błędów. To BRAK KONTROLI: żaden strażnik nie sprawdza, czy major ESLinta jest jeden, tak jak do ENV-01 nic nie sprawdzało wersji Node. | DO ZROBIENIA: zdjąć z korzenia nieużywane @eslint/js i typescript-eslint albo cofnąć je do dziewiątki (rusza lockfile — osobny commit z pełną bramką), plus strażnik spójności majora na wzór wersja-node.spec.ts. | 2026-09-23: zrobione zgodnie z DO ZROBIENIA; lockfile zmieniony wyłącznie o usunięcie gałęzi eslint 10 (pnpm 9.5.0 --lockfile-only). Przed bramką lokalną: pnpm install.</t>
+          <t>Stan 2026-08-23: ZROBIONE W KODZIE (D2), D3 przy pierwszym odrzuceniu na produkcji — a to da się zrobić od razu po wdrożeniu, w odróżnieniu od Z-18, który czeka na węzeł. Decyzja właściciela produktu: dorobić akcję w panelu zamiast jednorazowego czyszczenia Redisa. | JAK TO WYSZŁO: X-30 naprawiło alerting, VerrisProvisioningQueueFailed zapalił się z prawdziwego powodu i wskazał cztery martwe joby (to z nich wyszło Z-18). Naturalny następny ruch — usunąć je — okazał się NIEWYKONALNY: panel ma przy nich wyłącznie „Retry", a kontroler administracyjny dokładnie dwa endpointy, listowanie i ponowienie. Retry nic nie daje, bo węzła nie ma: job padnie ponownie, podbije licznik prób i dołoży wpisy do audytu — cztery martwe joby zamieniają się w cztery martwe joby z dłuższą historią. Zostawało grzebanie w Redisie ręcznie, czyli zmiana stanu produkcyjnego dotyczącego subskrypcji klientów BEZ ŚLADU W AUDYCIE. | TO NIE JEST USTERKA TYCH CZTERECH JOBÓW, tylko luka w warstwie operatorskiej, która ujawni się ponownie przy pierwszym prawdziwym niepowodzeniu provisioningu — z tą różnicą, że wtedy po drugiej stronie będzie klient. | ROZWIĄZANIE: POST /admin/provisioning-queue/:id/odrzuc + przycisk „Odrzuć" obok Retry. TRZY REGUŁY: (1) TYLKO STAN failed — usunięcie joba aktywnego albo czekającego osierociłoby provisioning w trakcie, konto na węźle mogłoby powstać, a system przestałby o nim wiedzieć; ograniczenie siedzi w usłudze, nie w kontrolerze, bo to reguła o kolejce, nie o HTTP; (2) POWÓD WYMAGANY, tak samo jak przy retry — operacja bez powodu to operacja, której za pół roku nikt nie wyjaśni; (3) NAJPIERW ODCZYT, POTEM USUNIĘCIE — ślad zbierany PRZED job.remove(), bo po usunięciu nie ma już czego odczytać; zapisujemy subskrypcję, joba, typ, liczbę prób, ostatni błąd i powód. Po Z-18 ten ostatni błąd niesie PRAWDZIWĄ przyczynę, więc wpis ma realną wartość dowodową — jeszcze wczoraj zapisałby zdanie o brakującym pakiecie DirectAdmina, którego nigdy nie brakowało. | OSOBNA AKCJA AUDYTU (PROVISIONING_JOB_DISCARDED_BY_ADMIN), nie wariant retry: w raportach odrzucenie i ponowienie to dwie różne decyzje i nie wolno im się zlewać. | DWA KLIKNIĘCIA, NIE JEDNO: retry można cofnąć następnym retry, odrzucenia nie da się cofnąć wcale. Potwierdzenie jest po to, żeby ta różnica była wyczuwalna w palcach. | ZDANIE PRZY PRZYCISKU: „Usuwa wpis z kolejki bez możliwości cofnięcia. Subskrypcja zostaje nietknięta." Operator ma prawo założyć, że „odrzuć" anuluje zamówienie — nie anuluje. Musi to być napisane tam, gdzie się klika, a nie w dokumentacji, której nikt nie otworzy w trakcie incydentu. | Czerwieni się na starym kodzie: 11 z 13. | DWIE UWAGI O SAMYCH TESTACH: odczyty plików panelu są LENIWE, bo odczyt na poziomie describe wywalał cały plik testowy, zanim cokolwiek się policzyło — a wtedy nie wiadomo, ILE asercji się czerwieni, tylko że „nie skompilowało się"; asercja o warunku row.failedReason nie mierzy odległości w znakach, tylko relację między warunkiem a przyciskiem, bo wersja licząca znaki zepsuła się od dopisania komentarza i kusiło, żeby poszerzyć okno zamiast poprawić asercję — to byłoby naprawianie testu zamiast kodu. | CZEGO NIE OBEJMUJE: losu czterech subskrypcji, które dostały zwrot i status PENDING_PAYMENT (odrzucenie joba ich nie dotyka — osobne sprzątanie po stronie bazy); odrzucania hurtem — świadomie, bo przycisk „odrzuć wszystkie" jest wygodny dokładnie do momentu, w którym ktoś kliknie go na kolejce z prawdziwym zamówieniem. | JAK ZAMKNĄĆ: odrzucić jeden z czterech martwych jobów, obejrzeć wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie i sprawdzić, że verris_provisioning_queue_depth{state="failed"} spadło o jeden. Dokumentacja: docs/archiwum/zadania/X-32-odrzucenie-martwego-joba.md | 2026-09-22 D3: wlasciciel odrzucil martwy job przyciskiem 'Odrzuc' w panelu admina na produkcji (potwierdzenie wlasciciela; wpis PROVISIONING_JOB_DISCARDED_BY_ADMIN w audycie).</t>
         </is>
       </c>
       <c r="P73" s="10" t="inlineStr">
@@ -6497,12 +6497,12 @@
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>M-08</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>Anulowanie faktury (VOID) z panelu</t>
+          <t>W drzewie stoją dwa majory ESLinta naraz</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -6512,12 +6512,12 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E74" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F74" s="10" t="n">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="L74" s="11" t="inlineStr">
         <is>
-          <t>billing/anulowanie.service.ts (POST /admin/invoices/:id/anuluj, BILLING_MANAGE); admin: invoices/void-button.tsx; test D2 anulowanie.service.spec.ts</t>
+          <t>package.json (korzeń) — @eslint/js ^10.0.1 przy braku jakiegokolwiek eslint.config.* w korzeniu; libs/eslint-config/node_modules: eslint 10.9.0 obok @eslint/js 9.39.5; apps/api, apps/www, apps/client-panel, apps/status-page, libs/directadmin-sdk — eslint 9.39.5 | 2026-09-23: z korzenia zdjęte nieużywane @eslint/js ^10 i typescript-eslint; libs/eslint-config peer eslint ^9.39.5 (było &gt;=9 → auto-install dociągał 10.9.0); lockfile bez eslint 10; strażnik apps/api/src/test/eslint-jeden-major.spec.ts (deklaracje + peer + lockfile)</t>
         </is>
       </c>
       <c r="M74" s="11" t="inlineStr">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="O74" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: anulować wolno tylko dokument nieopłacony (DRAFT/OPEN); opłacony, także z portfela, zmienia się korektą (M-06). Faktura Stripe unieważniana najpierw w Stripe, błąd = brak zmiany lokalnej. Numer zostaje (ciągłość), powód w audycie INVOICE_VOIDED.</t>
+          <t>Odkryte 2026-08-28 przy DEP-01. Korzeń deklaruje @eslint/js ^10.0.1, którego peer to eslint ^10.0.0 — i to on wciąga eslint@10.9.0 do drzewa. Tymczasem KAŻDY pakiet, który realnie lintuje, ma 9.39.5. Najostrzej widać to wewnątrz libs/eslint-config, czyli wspólnej konfiguracji: node_modules/eslint = 10.9.0, node_modules/@eslint/js = 9.39.5 — dwie połowy jednego narzędzia z różnych majorów w jednym katalogu. | Korzeń NIE MA żadnego eslint.config.* i nie odpala lintera (pnpm lint = turbo run lint), więc te zależności nie robią nic poza wciąganiem majora, którego nikt nie używa. | To nie awaria — bramka jest zielona, 0 błędów. To BRAK KONTROLI: żaden strażnik nie sprawdza, czy major ESLinta jest jeden, tak jak do ENV-01 nic nie sprawdzało wersji Node. | DO ZROBIENIA: zdjąć z korzenia nieużywane @eslint/js i typescript-eslint albo cofnąć je do dziewiątki (rusza lockfile — osobny commit z pełną bramką), plus strażnik spójności majora na wzór wersja-node.spec.ts. | 2026-09-23: zrobione zgodnie z DO ZROBIENIA; lockfile zmieniony wyłącznie o usunięcie gałęzi eslint 10 (pnpm 9.5.0 --lockfile-only). Przed bramką lokalną: pnpm install.</t>
         </is>
       </c>
       <c r="P74" s="10" t="inlineStr">
@@ -6575,12 +6575,12 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>C-18</t>
+          <t>M-08</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>Konto FTP — zmiana hasła</t>
+          <t>Anulowanie faktury (VOID) z panelu</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
@@ -6621,12 +6621,12 @@
       </c>
       <c r="K75" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L75" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/hosting-ftp/:username/password (ZmienHasloFtpDto) → directadmin.service changeHostingFtpPassword (action=modify, katalog zachowany) + audyt HOSTING_FTP_PASSWORD_CHANGED; UI FtpTab — kluczyk przy koncie; test servers/zmiana-hasla-ftp.spec.ts</t>
+          <t>billing/anulowanie.service.ts (POST /admin/invoices/:id/anuluj, BILLING_MANAGE); admin: invoices/void-button.tsx; test D2 anulowanie.service.spec.ts</t>
         </is>
       </c>
       <c r="M75" s="11" t="inlineStr">
@@ -6636,12 +6636,12 @@
       </c>
       <c r="N75" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O75" s="11" t="inlineStr">
         <is>
-          <t>brak jakiejkolwiek ścieżki edycji istniejącego konta | Przy okazji body tworzenia konta FTP dostało klasę DTO (login, hasło, katalog bez „..”). OTWARTE do D3 (PB-21): format action=modify na żywym DA.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: anulować wolno tylko dokument nieopłacony (DRAFT/OPEN); opłacony, także z portfela, zmienia się korektą (M-06). Faktura Stripe unieważniana najpierw w Stripe, błąd = brak zmiany lokalnej. Numer zostaje (ciągłość), powód w audycie INVOICE_VOIDED.</t>
         </is>
       </c>
       <c r="P75" s="10" t="inlineStr">
@@ -6653,12 +6653,12 @@
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>C-18</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>Konto FTP — zmiana hasła</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -6668,7 +6668,7 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="E76" s="10" t="inlineStr">
@@ -6680,7 +6680,7 @@
         <v>6</v>
       </c>
       <c r="G76" s="10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H76" s="10" t="inlineStr">
         <is>
@@ -6689,22 +6689,22 @@
       </c>
       <c r="I76" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="J76" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="K76" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L76" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>2026-09-23 D1: POST /services/:id/hosting-ftp/:username/password (ZmienHasloFtpDto) → directadmin.service changeHostingFtpPassword (action=modify, katalog zachowany) + audyt HOSTING_FTP_PASSWORD_CHANGED; UI FtpTab — kluczyk przy koncie; test servers/zmiana-hasla-ftp.spec.ts</t>
         </is>
       </c>
       <c r="M76" s="11" t="inlineStr">
@@ -6714,12 +6714,12 @@
       </c>
       <c r="N76" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O76" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>brak jakiejkolwiek ścieżki edycji istniejącego konta | Przy okazji body tworzenia konta FTP dostało klasę DTO (login, hasło, katalog bez „..”). OTWARTE do D3 (PB-21): format action=modify na żywym DA.</t>
         </is>
       </c>
       <c r="P76" s="10" t="inlineStr">
@@ -6731,12 +6731,12 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>C-11</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Spakowanie do archiwum</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -6746,12 +6746,12 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F77" s="10" t="n">
@@ -6777,12 +6777,12 @@
       </c>
       <c r="K77" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L77" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M77" s="11" t="inlineStr">
@@ -6792,12 +6792,12 @@
       </c>
       <c r="N77" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>standard we wszystkich panelach | OTWARTE do D3 (PB-21): format action=compress na żywym DA.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr">
@@ -6809,12 +6809,12 @@
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>NODE-03</t>
+          <t>C-11</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>Pojemność węzła nigdy się nie odświeża</t>
+          <t>Spakowanie do archiwum</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="E78" s="10" t="inlineStr">
@@ -6860,7 +6860,7 @@
       </c>
       <c r="L78" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: verris-lve.sh node_capacity (nproc, MemTotal, df /) w każdym raporcie, lve-agent/1.1; telemetry.dto NodeStatusDto.totalCpuCores/totalMemoryMb/totalDiskMb; telemetry.service aktualizuje Server; test telemetry/pojemnosc-wezla.spec.ts</t>
+          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych</t>
         </is>
       </c>
       <c r="M78" s="11" t="inlineStr">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Pojemność węzła nigdy się nie odświeża. `totalCpuCores`/`totalMemoryMb`/`totalDiskMb` ustawiane wyłącznie w handshake; telemetria ich nie aktualizuje — mimo komentarza w schemacie „reported via handshake / heartbeat”. Rozbudowa węzła nie dociera do `NodeSelector`. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Telemetria aktualizuje totalCpuCores/totalMemoryMb/totalDiskMb, nie tylko handshake. | Stary agent bez pól niczego nie zeruje. OTWARTE do D3 (PB-21): raport z agenta na żywym węźle i odświeżona pojemność w panelu admina. | 2026-09-25: pojemność z agenta trafia też do planera pojemności (admin → Product Ops): ryzyko liczone względem rdzeni i RAM węzła (CPU 2×/4× rdzeni, RAM 1×/1,5×; test ryzyko-pojemnosci.spec.ts), a opis „CPU 250%” zastąpiony „przydzielone limity: CPU 2,5 rdz. z N · RAM x z y GB” — wcześniej wyglądało jak zużycie ponad 100%.</t>
+          <t>standard we wszystkich panelach | OTWARTE do D3 (PB-21): format action=compress na żywym DA.</t>
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr">
@@ -6887,31 +6887,31 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>PB-08</t>
+          <t>NODE-03</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
+          <t>Pojemność węzła nigdy się nie odświeża</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G79" s="10" t="n">
         <v>14</v>
@@ -6933,12 +6933,12 @@
       </c>
       <c r="K79" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L79" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-09-23 D1: verris-lve.sh node_capacity (nproc, MemTotal, df /) w każdym raporcie, lve-agent/1.1; telemetry.dto NodeStatusDto.totalCpuCores/totalMemoryMb/totalDiskMb; telemetry.service aktualizuje Server; test telemetry/pojemnosc-wezla.spec.ts</t>
         </is>
       </c>
       <c r="M79" s="11" t="inlineStr">
@@ -6948,12 +6948,12 @@
       </c>
       <c r="N79" s="11" t="inlineStr">
         <is>
-          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O79" s="11" t="inlineStr">
         <is>
-          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Pojemność węzła nigdy się nie odświeża. `totalCpuCores`/`totalMemoryMb`/`totalDiskMb` ustawiane wyłącznie w handshake; telemetria ich nie aktualizuje — mimo komentarza w schemacie „reported via handshake / heartbeat”. Rozbudowa węzła nie dociera do `NodeSelector`. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Telemetria aktualizuje totalCpuCores/totalMemoryMb/totalDiskMb, nie tylko handshake. | Stary agent bez pól niczego nie zeruje. OTWARTE do D3 (PB-21): raport z agenta na żywym węźle i odświeżona pojemność w panelu admina. | 2026-09-25: pojemność z agenta trafia też do planera pojemności (admin → Product Ops): ryzyko liczone względem rdzeni i RAM węzła (CPU 2×/4× rdzeni, RAM 1×/1,5×; test ryzyko-pojemnosci.spec.ts), a opis „CPU 250%” zastąpiony „przydzielone limity: CPU 2,5 rdz. z N · RAM x z y GB” — wcześniej wyglądało jak zużycie ponad 100%.</t>
         </is>
       </c>
       <c r="P79" s="10" t="inlineStr">
@@ -6965,12 +6965,12 @@
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>PB-27</t>
+          <t>PB-08</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
+          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -6985,11 +6985,11 @@
       </c>
       <c r="E80" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G80" s="10" t="n">
         <v>14</v>
@@ -7026,12 +7026,12 @@
       </c>
       <c r="N80" s="11" t="inlineStr">
         <is>
-          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
+          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
         </is>
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr">
@@ -7043,12 +7043,12 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>PB-28</t>
+          <t>PB-27</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Rozliczenie poza Verris (całe konto)</t>
+          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -7067,7 +7067,7 @@
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G81" s="10" t="n">
         <v>14</v>
@@ -7104,12 +7104,12 @@
       </c>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
+          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
         </is>
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr">
@@ -7121,58 +7121,58 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>X-41</t>
+          <t>PB-28</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
+          <t>Rozliczenie poza Verris (całe konto)</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E82" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F82" s="10" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H82" s="10" t="inlineStr">
         <is>
-          <t>Faza 3 — Wejście na rynek</t>
+          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
         </is>
       </c>
       <c r="I82" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J82" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K82" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M82" s="11" t="inlineStr">
@@ -7182,12 +7182,12 @@
       </c>
       <c r="N82" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
         </is>
       </c>
       <c r="O82" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
+          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr">
@@ -7199,12 +7199,12 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>X-41</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
+          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
+          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
         </is>
       </c>
       <c r="M83" s="11" t="inlineStr">
@@ -7265,7 +7265,7 @@
       </c>
       <c r="O83" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01.</t>
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr">
@@ -7277,31 +7277,31 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>PB-22</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
+          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F84" s="10" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G84" s="10" t="n">
         <v>15</v>
@@ -7323,12 +7323,12 @@
       </c>
       <c r="K84" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
@@ -7338,12 +7338,12 @@
       </c>
       <c r="N84" s="11" t="inlineStr">
         <is>
-          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O84" s="11" t="inlineStr">
         <is>
-          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41.</t>
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr">
@@ -7355,34 +7355,34 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>PB-22</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Log egressu jest próbką, nie zapisem</t>
+          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F85" s="10" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G85" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
@@ -7391,22 +7391,22 @@
       </c>
       <c r="I85" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="J85" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M85" s="11" t="inlineStr">
@@ -7416,12 +7416,12 @@
       </c>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
         </is>
       </c>
       <c r="O85" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
+          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr">
@@ -7433,12 +7433,12 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
+          <t>Log egressu jest próbką, nie zapisem</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -7479,12 +7479,12 @@
       </c>
       <c r="K86" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr">
@@ -7494,12 +7494,12 @@
       </c>
       <c r="N86" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O86" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr">
@@ -7511,12 +7511,12 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Tryb `--strict` jest atrapą</t>
+          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -7535,7 +7535,7 @@
         </is>
       </c>
       <c r="F87" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G87" s="10" t="n">
         <v>16</v>
@@ -7562,7 +7562,7 @@
       </c>
       <c r="L87" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
+          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M87" s="11" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="O87" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9).</t>
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr">
@@ -7589,12 +7589,12 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
+          <t>Tryb `--strict` jest atrapą</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
@@ -7635,12 +7635,12 @@
       </c>
       <c r="K88" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
+          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
         </is>
       </c>
       <c r="M88" s="11" t="inlineStr">
@@ -7650,12 +7650,12 @@
       </c>
       <c r="N88" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O88" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru.</t>
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr">
@@ -7667,12 +7667,12 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
+          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
@@ -7687,11 +7687,11 @@
       </c>
       <c r="E89" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G89" s="10" t="n">
         <v>16</v>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="L89" s="11" t="inlineStr">
         <is>
-          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
+          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
         </is>
       </c>
       <c r="M89" s="11" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="O89" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr">
@@ -7745,31 +7745,31 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>PB-23</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
+          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>16</v>
@@ -7791,12 +7791,12 @@
       </c>
       <c r="K90" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L90" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
         </is>
       </c>
       <c r="M90" s="11" t="inlineStr">
@@ -7806,12 +7806,12 @@
       </c>
       <c r="N90" s="11" t="inlineStr">
         <is>
-          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7823,34 +7823,34 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>PB-23</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Podpisane DPA z subprocesorami (część)</t>
+          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G91" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H91" s="10" t="inlineStr">
         <is>
@@ -7859,22 +7859,22 @@
       </c>
       <c r="I91" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="J91" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="K91" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L91" s="11" t="inlineStr">
         <is>
-          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M91" s="11" t="inlineStr">
@@ -7884,12 +7884,12 @@
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
+          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7901,31 +7901,31 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>PB-03</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Finalizacja dokumentów prawnych 1.0.0</t>
+          <t>Podpisane DPA z subprocesorami (część)</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>17</v>
@@ -7947,12 +7947,12 @@
       </c>
       <c r="K92" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L92" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
         </is>
       </c>
       <c r="M92" s="11" t="inlineStr">
@@ -7962,12 +7962,12 @@
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>PB-04</t>
+          <t>PB-03</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
+          <t>Finalizacja dokumentów prawnych 1.0.0</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -7999,11 +7999,11 @@
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G93" s="10" t="n">
         <v>17</v>
@@ -8040,12 +8040,12 @@
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
+          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
+          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8057,34 +8057,34 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>N-16</t>
+          <t>PB-04</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>SLA z zapisanymi kredytami</t>
+          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G94" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H94" s="10" t="inlineStr">
         <is>
@@ -8093,37 +8093,37 @@
       </c>
       <c r="I94" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-21</t>
         </is>
       </c>
       <c r="J94" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="K94" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
         <is>
-          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M94" s="11" t="inlineStr">
         <is>
-          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
+          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8135,12 +8135,12 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>N-16</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>SLA z zapisanymi kredytami</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8150,7 +8150,7 @@
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
@@ -8181,27 +8181,27 @@
       </c>
       <c r="K95" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L95" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
         </is>
       </c>
       <c r="M95" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
+          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja).</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,31 +8213,31 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>PB-07</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Treści i cennik na verris.pl</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E96" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F96" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G96" s="10" t="n">
         <v>18</v>
@@ -8259,27 +8259,27 @@
       </c>
       <c r="K96" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="L96" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M96" s="11" t="inlineStr">
         <is>
-          <t>PB-01 (cennik zależy od unit economics)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
+          <t>Wartość domyślna włączona albo check w live-readiness pilnuje konfiguracji — flaga nie może po cichu wyłączyć funkcji.</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15).</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,12 +8291,12 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-11</t>
+          <t>PB-07</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
+          <t>Treści i cennik na verris.pl</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8315,7 +8315,7 @@
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>18</v>
@@ -8347,17 +8347,17 @@
       </c>
       <c r="M97" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-01 (cennik zależy od unit economics)</t>
         </is>
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
+          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
+          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8369,12 +8369,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-21</t>
+          <t>PB-11</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>DNS platformy i poczty na serwerze testowym</t>
+          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8393,7 +8393,7 @@
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G98" s="10" t="n">
         <v>18</v>
@@ -8430,12 +8430,12 @@
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
+          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
+          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7.</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8447,12 +8447,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-24</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8471,7 +8471,7 @@
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G99" s="10" t="n">
         <v>18</v>
@@ -8508,12 +8508,12 @@
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle.</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8525,12 +8525,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>PB-25</t>
+          <t>PB-24</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>White label na węźle — klient nie widzi DirectAdmina</t>
+          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8549,7 +8549,7 @@
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G100" s="10" t="n">
         <v>18</v>
@@ -8586,12 +8586,12 @@
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
+          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
+          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8603,12 +8603,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-25</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>White label na węźle — klient nie widzi DirectAdmina</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8627,10 +8627,10 @@
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G101" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H101" s="10" t="inlineStr">
         <is>
@@ -8639,12 +8639,12 @@
       </c>
       <c r="I101" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="J101" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="K101" s="10" t="inlineStr">
@@ -8659,17 +8659,17 @@
       </c>
       <c r="M101" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
+          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz.</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8681,12 +8681,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8701,7 +8701,7 @@
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
@@ -8737,17 +8737,17 @@
       </c>
       <c r="M102" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8759,12 +8759,12 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8783,7 +8783,7 @@
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G103" s="10" t="n">
         <v>19</v>
@@ -8820,12 +8820,12 @@
       </c>
       <c r="N103" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”.</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8837,12 +8837,12 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
@@ -8861,20 +8861,24 @@
         </is>
       </c>
       <c r="F104" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G104" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H104" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H104" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I104" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J104" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K104" s="10" t="inlineStr">
@@ -8889,17 +8893,17 @@
       </c>
       <c r="M104" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8911,69 +8915,69 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F105" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G105" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H105" s="10" t="inlineStr"/>
       <c r="I105" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="J105" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="K105" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L105" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M105" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N105" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O105" s="11" t="inlineStr">
         <is>
-          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr">
@@ -8985,12 +8989,12 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -9000,16 +9004,16 @@
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F106" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G106" s="10" t="n">
         <v>21</v>
@@ -9032,7 +9036,7 @@
       </c>
       <c r="L106" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M106" s="11" t="inlineStr">
@@ -9047,7 +9051,7 @@
       </c>
       <c r="O106" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md</t>
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr">
@@ -9059,12 +9063,12 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -9074,7 +9078,7 @@
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr">
@@ -9101,12 +9105,12 @@
       </c>
       <c r="K107" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L107" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M107" s="11" t="inlineStr">
@@ -9116,12 +9120,12 @@
       </c>
       <c r="N107" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O107" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr">
@@ -9133,12 +9137,12 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -9153,7 +9157,7 @@
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F108" s="10" t="n">
@@ -9180,7 +9184,7 @@
       </c>
       <c r="L108" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu</t>
         </is>
       </c>
       <c r="M108" s="11" t="inlineStr">
@@ -9195,7 +9199,7 @@
       </c>
       <c r="O108" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr">
@@ -9207,12 +9211,12 @@
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C109" s="10" t="inlineStr">
@@ -9222,12 +9226,12 @@
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F109" s="10" t="n">
@@ -9249,12 +9253,12 @@
       </c>
       <c r="K109" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>b.d.</t>
         </is>
       </c>
       <c r="L109" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125</t>
+          <t>poza kodem panelu</t>
         </is>
       </c>
       <c r="M109" s="11" t="inlineStr">
@@ -9264,12 +9268,12 @@
       </c>
       <c r="N109" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
         </is>
       </c>
       <c r="O109" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr">
@@ -9281,31 +9285,31 @@
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E110" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F110" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G110" s="10" t="n">
         <v>21</v>
@@ -9323,12 +9327,12 @@
       </c>
       <c r="K110" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L110" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>services.controller.ts:125</t>
         </is>
       </c>
       <c r="M110" s="11" t="inlineStr">
@@ -9338,12 +9342,12 @@
       </c>
       <c r="N110" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O110" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr">
@@ -9355,12 +9359,12 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>PB-29</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
@@ -9375,11 +9379,11 @@
       </c>
       <c r="E111" s="10" t="inlineStr">
         <is>
-          <t>KRYTYCZNY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F111" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G111" s="10" t="n">
         <v>21</v>
@@ -9412,12 +9416,12 @@
       </c>
       <c r="N111" s="11" t="inlineStr">
         <is>
-          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O111" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr">
@@ -9429,12 +9433,12 @@
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>PB-30</t>
+          <t>PB-29</t>
         </is>
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
-          <t>Jeden plik wersji dla floty + test zgodności</t>
+          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -9449,7 +9453,7 @@
       </c>
       <c r="E112" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F112" s="10" t="n">
@@ -9486,12 +9490,12 @@
       </c>
       <c r="N112" s="11" t="inlineStr">
         <is>
-          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
+          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="O112" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
+          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="P112" s="10" t="inlineStr">
@@ -9503,12 +9507,12 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>PB-31</t>
+          <t>PB-30</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>Pełna automatyzacja kreatora węzła</t>
+          <t>Jeden plik wersji dla floty + test zgodności</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
@@ -9527,7 +9531,7 @@
         </is>
       </c>
       <c r="F113" s="10" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G113" s="10" t="n">
         <v>21</v>
@@ -9560,12 +9564,12 @@
       </c>
       <c r="N113" s="11" t="inlineStr">
         <is>
-          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
+          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
         </is>
       </c>
       <c r="O113" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
+          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
         </is>
       </c>
       <c r="P113" s="10" t="inlineStr">
@@ -9577,12 +9581,12 @@
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>PB-32</t>
+          <t>PB-31</t>
         </is>
       </c>
       <c r="B114" s="11" t="inlineStr">
         <is>
-          <t>Aktualizacje węzłów falami</t>
+          <t>Pełna automatyzacja kreatora węzła</t>
         </is>
       </c>
       <c r="C114" s="10" t="inlineStr">
@@ -9597,11 +9601,11 @@
       </c>
       <c r="E114" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F114" s="10" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G114" s="10" t="n">
         <v>21</v>
@@ -9634,12 +9638,12 @@
       </c>
       <c r="N114" s="11" t="inlineStr">
         <is>
-          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
+          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
         </is>
       </c>
       <c r="O114" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
+          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
         </is>
       </c>
       <c r="P114" s="10" t="inlineStr">
@@ -9651,12 +9655,12 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>PB-33</t>
+          <t>PB-32</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>Wersje stosu floty w panelu + wyrównanie falą</t>
+          <t>Aktualizacje węzłów falami</t>
         </is>
       </c>
       <c r="C115" s="10" t="inlineStr">
@@ -9671,11 +9675,11 @@
       </c>
       <c r="E115" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F115" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G115" s="10" t="n">
         <v>21</v>
@@ -9708,12 +9712,12 @@
       </c>
       <c r="N115" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji w panelu → nowy węzeł instaluje ją, istniejące wyrównane falą; audyt zgodności zielony.</t>
+          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
         </is>
       </c>
       <c r="O115" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: strona „Wersje stosu floty” w panelu admina (DB, PHP, LiteSpeed, DirectAdmin) z dozwolonymi wartościami z oficjalnych list; zmiana obowiązuje nowe węzły od razu, „Wyrównaj flotę” aktualizuje istniejące falą (PHP/LiteSpeed przez CustomBuild, MariaDB po jednej wersji z kopią bazy — wymóg CloudLinux Governor). | 2026-09-26 ZROBIONE W KODZIE: manifest w bazie (StosWezlaService), strona Admin → Wersje stosu floty (dozwolone wartości z oficjalnych list, tabela zgodności), „Wyrównaj flotę” = fala z php1_release + łańcuch DB_UPGRADE krok po kroku z kopią; bootstrap i agent biorą manifest z bazy. Testy na PostgreSQL. Zostało: wyrównanie na węzłach (D3).</t>
+          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
         </is>
       </c>
       <c r="P115" s="10" t="inlineStr">
@@ -9725,12 +9729,12 @@
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>PB-35</t>
+          <t>PB-33</t>
         </is>
       </c>
       <c r="B116" s="11" t="inlineStr">
         <is>
-          <t>Automatyczna fala aktualizacji węzłów co tydzień</t>
+          <t>Wersje stosu floty w panelu + wyrównanie falą</t>
         </is>
       </c>
       <c r="C116" s="10" t="inlineStr">
@@ -9749,7 +9753,7 @@
         </is>
       </c>
       <c r="F116" s="10" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G116" s="10" t="n">
         <v>21</v>
@@ -9782,12 +9786,12 @@
       </c>
       <c r="N116" s="11" t="inlineStr">
         <is>
-          <t>Fala startuje sama w oknie; zatrzymanie widoczne w powiadomieniach admina.</t>
+          <t>Zmiana wersji w panelu → nowy węzeł instaluje ją, istniejące wyrównane falą; audyt zgodności zielony.</t>
         </is>
       </c>
       <c r="O116" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: fala rusza sama we wtorki o 4:00 (kanarek → reszta po jednym, błąd zatrzymuje, powiadomienie). Węzły same już niczego nie instalują (dnf-automatic tylko pobiera). | 2026-09-26 ZROBIONE W KODZIE: FalaTygodniowaScheduler (wtorek 4:00 Europe/Warsaw), zatrzymanie fali → powiadomienie adminów. Test na PostgreSQL.</t>
+          <t>Decyzja właściciela 2026-09-26: strona „Wersje stosu floty” w panelu admina (DB, PHP, LiteSpeed, DirectAdmin) z dozwolonymi wartościami z oficjalnych list; zmiana obowiązuje nowe węzły od razu, „Wyrównaj flotę” aktualizuje istniejące falą (PHP/LiteSpeed przez CustomBuild, MariaDB po jednej wersji z kopią bazy — wymóg CloudLinux Governor). | 2026-09-26 ZROBIONE W KODZIE: manifest w bazie (StosWezlaService), strona Admin → Wersje stosu floty (dozwolone wartości z oficjalnych list, tabela zgodności), „Wyrównaj flotę” = fala z php1_release + łańcuch DB_UPGRADE krok po kroku z kopią; bootstrap i agent biorą manifest z bazy. Testy na PostgreSQL. Zostało: wyrównanie na węzłach (D3).</t>
         </is>
       </c>
       <c r="P116" s="10" t="inlineStr">
@@ -9799,12 +9803,12 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>PB-36</t>
+          <t>PB-35</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>Podpisane skrypty węzła i klucz SSH ograniczony do control-plane</t>
+          <t>Automatyczna fala aktualizacji węzłów co tydzień</t>
         </is>
       </c>
       <c r="C117" s="10" t="inlineStr">
@@ -9819,11 +9823,11 @@
       </c>
       <c r="E117" s="10" t="inlineStr">
         <is>
-          <t>KRYTYCZNY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F117" s="10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G117" s="10" t="n">
         <v>21</v>
@@ -9856,12 +9860,12 @@
       </c>
       <c r="N117" s="11" t="inlineStr">
         <is>
-          <t>Niepodpisany/zmieniony skrypt odrzucony przez węzeł; authorized_keys zawiera tylko aktualny klucz z ograniczeniem IP.</t>
+          <t>Fala startuje sama w oknie; zatrzymanie widoczne w powiadomieniach admina.</t>
         </is>
       </c>
       <c r="O117" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: przed startem. Węzeł uruchamia tylko skrypty podpisane kluczem Verris (przejęte API nie daje roota na flocie); klucz SSH z from= na IP control-plane, stare klucze usuwane (dziś agent co minutę tylko dopisuje klucz). | 2026-09-26 ZROBIONE W KODZIE: podpis Ed25519 każdej odpowiedzi GET /agent/tasks/* (skrypty zadań, pakiety onboardu i strony domyślnej, manifest stosu, konfiguracja kopii, zlecenia, klucz deploy) — podpis obejmuje ścieżkę, id węzła, czas i SHA-256 treści (bez podmiany, przeniesienia na inną ścieżkę/węzeł, powtórki po 5 min). Węzeł pobiera wyłącznie przez /usr/local/bin/verris-fetch (openssl pkeyutl -verify), klucz publiczny przywozi bootstrap / instalacja agenta. Klucz deploy: jeden wpis from="VERRIS_CONTROL_PLANE_IPS" bez przekierowań, poprzedni usuwany (rotacja). API w produkcji nie wystartuje bez VERRIS_SCRIPT_SIGNING_KEY albo z kluczem deploy bez adresów control-plane. Test: prawdziwy verris-fetch vs serwer podpisujący (zmieniona treść / inna ścieżka / inny węzeł / stary podpis / brak podpisu → odrzucone) + smoke na lokalnym API. Do sprawdzenia na D3: openssl na CloudLinux 9, rotacja klucza deploy.</t>
+          <t>Decyzja właściciela 2026-09-26: fala rusza sama we wtorki o 4:00 (kanarek → reszta po jednym, błąd zatrzymuje, powiadomienie). Węzły same już niczego nie instalują (dnf-automatic tylko pobiera). | 2026-09-26 ZROBIONE W KODZIE: FalaTygodniowaScheduler (wtorek 4:00 Europe/Warsaw), zatrzymanie fali → powiadomienie adminów. Test na PostgreSQL.</t>
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr">
@@ -9873,12 +9877,12 @@
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
         <is>
-          <t>PB-26</t>
+          <t>PB-36</t>
         </is>
       </c>
       <c r="B118" s="11" t="inlineStr">
         <is>
-          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
+          <t>Podpisane skrypty węzła i klucz SSH ograniczony do control-plane</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
@@ -9893,24 +9897,24 @@
       </c>
       <c r="E118" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F118" s="10" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G118" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H118" s="10" t="inlineStr"/>
       <c r="I118" s="10" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-01-18</t>
         </is>
       </c>
       <c r="J118" s="10" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2027-01-22</t>
         </is>
       </c>
       <c r="K118" s="10" t="inlineStr">
@@ -9930,12 +9934,12 @@
       </c>
       <c r="N118" s="11" t="inlineStr">
         <is>
-          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
+          <t>Niepodpisany/zmieniony skrypt odrzucony przez węzeł; authorized_keys zawiera tylko aktualny klucz z ograniczeniem IP.</t>
         </is>
       </c>
       <c r="O118" s="11" t="inlineStr">
         <is>
-          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
+          <t>Decyzja właściciela 2026-09-26: przed startem. Węzeł uruchamia tylko skrypty podpisane kluczem Verris (przejęte API nie daje roota na flocie); klucz SSH z from= na IP control-plane, stare klucze usuwane (dziś agent co minutę tylko dopisuje klucz). | 2026-09-26 ZROBIONE W KODZIE: podpis Ed25519 każdej odpowiedzi GET /agent/tasks/* (skrypty zadań, pakiety onboardu i strony domyślnej, manifest stosu, konfiguracja kopii, zlecenia, klucz deploy) — podpis obejmuje ścieżkę, id węzła, czas i SHA-256 treści (bez podmiany, przeniesienia na inną ścieżkę/węzeł, powtórki po 5 min). Węzeł pobiera wyłącznie przez /usr/local/bin/verris-fetch (openssl pkeyutl -verify), klucz publiczny przywozi bootstrap / instalacja agenta. Klucz deploy: jeden wpis from="VERRIS_CONTROL_PLANE_IPS" bez przekierowań, poprzedni usuwany (rotacja). API w produkcji nie wystartuje bez VERRIS_SCRIPT_SIGNING_KEY albo z kluczem deploy bez adresów control-plane. Test: prawdziwy verris-fetch vs serwer podpisujący (zmieniona treść / inna ścieżka / inny węzeł / stary podpis / brak podpisu → odrzucone) + smoke na lokalnym API. Do sprawdzenia na D3: openssl na CloudLinux 9, rotacja klucza deploy.</t>
         </is>
       </c>
       <c r="P118" s="10" t="inlineStr">
@@ -9947,12 +9951,12 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>PB-05</t>
+          <t>PB-26</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>Test end-to-end „pierwszy klient”</t>
+          <t>Otwarte testy (beta) z zaproszonymi użytkownikami</t>
         </is>
       </c>
       <c r="C119" s="10" t="inlineStr">
@@ -9967,11 +9971,11 @@
       </c>
       <c r="E119" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F119" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G119" s="10" t="n">
         <v>22</v>
@@ -9999,17 +10003,17 @@
       </c>
       <c r="M119" s="11" t="inlineStr">
         <is>
-          <t>wszystkie blokery zamknięte (sprint 8)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N119" s="11" t="inlineStr">
         <is>
-          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+          <t>Minimum 7 dni od pierwszej aktywnej usługi; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); ≥ 80% testerów z działającą stroną bez pomocy wsparcia; poprawki „przed GO” zamknięte. Dopiero potem PB-12.</t>
         </is>
       </c>
       <c r="O119" s="11" t="inlineStr">
         <is>
-          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+          <t>Prośba właściciela 2026-09-24: przed startem otwarte testy z osobami zaproszonymi przez właściciela, w ramach darmowego kredytu / okresu. Plan: docs/ops/BETA_TESTY.md — 10–20 osób (WordPress do przeniesienia, sklepy, osoby nietechniczne, agencje), kod FIXED_CREDIT 150 K na osobę (1 użycie, 14 dni), scenariusze od rejestracji po odtworzenie kopii i telefon, kanał: zgłoszenia z kategorią Beta. Po naszej stronie: generator kodów, kategoria zgłoszeń, mail zaproszenia, ankieta, widok testerów w panelu admina. | PRZYGOTOWANIE 2026-09-24 (D2): panel admina „Testy (beta)” — zaproszenie tworzy imienny kod BETA-XXXXXX (150 K, 1 użycie, 14 dni) i wysyła mail z instrukcją; lista testerów (stan kodu, konto, aktywne usługi, zgłoszenia Beta); temat „Testy (beta)” w panelu klienta tylko dla testera, znacznik Beta w panelu obsługi. Zostaje: ankieta końcowa (mailem), sama beta po węźle #1.</t>
         </is>
       </c>
       <c r="P119" s="10" t="inlineStr">
@@ -10021,12 +10025,12 @@
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
         <is>
-          <t>PB-12</t>
+          <t>PB-05</t>
         </is>
       </c>
       <c r="B120" s="11" t="inlineStr">
         <is>
-          <t>Runbook startu i decyzja GO</t>
+          <t>Test end-to-end „pierwszy klient”</t>
         </is>
       </c>
       <c r="C120" s="10" t="inlineStr">
@@ -10045,7 +10049,7 @@
         </is>
       </c>
       <c r="F120" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G120" s="10" t="n">
         <v>22</v>
@@ -10073,28 +10077,102 @@
       </c>
       <c r="M120" s="11" t="inlineStr">
         <is>
+          <t>wszystkie blokery zamknięte (sprint 8)</t>
+        </is>
+      </c>
+      <c r="N120" s="11" t="inlineStr">
+        <is>
+          <t>Zapisany przebieg z timestampami dla każdego kroku — to jest dowód poziomu D3, jedyny w całym projekcie. Każdy nieudany krok wraca do backlogu jako bloker.</t>
+        </is>
+      </c>
+      <c r="O120" s="11" t="inlineStr">
+        <is>
+          <t>Przejście całej ścieżki na produkcji jako realny klient: rejestracja, zakup, płatność, provisioning, migracja strony, wystawienie faktury, KSeF, backup, odtworzenie.</t>
+        </is>
+      </c>
+      <c r="P120" s="10" t="inlineStr">
+        <is>
+          <t>do zrobienia</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>PB-12</t>
+        </is>
+      </c>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>Runbook startu i decyzja GO</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>poza audytem</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>Praca spoza audytu</t>
+        </is>
+      </c>
+      <c r="E121" s="10" t="inlineStr">
+        <is>
+          <t>BLOKER BIZNESOWY</t>
+        </is>
+      </c>
+      <c r="F121" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G121" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H121" s="10" t="inlineStr"/>
+      <c r="I121" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="J121" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-29</t>
+        </is>
+      </c>
+      <c r="K121" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L121" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M121" s="11" t="inlineStr">
+        <is>
           <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
-      <c r="N120" s="11" t="inlineStr">
+      <c r="N121" s="11" t="inlineStr">
         <is>
           <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
-      <c r="O120" s="11" t="inlineStr">
+      <c r="O121" s="11" t="inlineStr">
         <is>
           <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
-      <c r="P120" s="10" t="inlineStr">
+      <c r="P121" s="10" t="inlineStr">
         <is>
           <t>do zrobienia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P120"/>
-  <conditionalFormatting sqref="E2:E120">
+  <autoFilter ref="A1:P121"/>
+  <conditionalFormatting sqref="E2:E121">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BLOKER STARTU"</formula>
     </cfRule>
@@ -10114,7 +10192,7 @@
       <formula>"ŚREDNI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P120">
+  <conditionalFormatting sqref="P2:P121">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"zrobione"</formula>
     </cfRule>
@@ -10224,11 +10302,11 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A2)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A2)</f>
         <v/>
       </c>
       <c r="G2" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A2,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A2,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H2" s="10" t="n">
@@ -10269,11 +10347,11 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A3)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A3)</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A3,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A3,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H3" s="10" t="n">
@@ -10314,11 +10392,11 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A4)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A4)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A4,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A4,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H4" s="10" t="n">
@@ -10359,11 +10437,11 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A5)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A5)</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A5,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A5,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H5" s="10" t="n">
@@ -10404,11 +10482,11 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A6)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A6)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A6,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A6,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H6" s="10" t="n">
@@ -10449,11 +10527,11 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A7)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A7)</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A7,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A7,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H7" s="10" t="n">
@@ -10494,11 +10572,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A8)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A8)</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A8,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A8,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H8" s="10" t="n">
@@ -10539,11 +10617,11 @@
         </is>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A9)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A9)</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A9,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A9,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H9" s="10" t="n">
@@ -10584,11 +10662,11 @@
         </is>
       </c>
       <c r="F10" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A10)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A10)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A10,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A10,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H10" s="10" t="n">
@@ -10629,11 +10707,11 @@
         </is>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A11)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A11)</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A11,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A11,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H11" s="10" t="n">
@@ -10674,11 +10752,11 @@
         </is>
       </c>
       <c r="F12" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A12)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A12)</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A12,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A12,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H12" s="10" t="n">
@@ -10719,11 +10797,11 @@
         </is>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A13)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A13)</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A13,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A13,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H13" s="10" t="n">
@@ -10764,11 +10842,11 @@
         </is>
       </c>
       <c r="F14" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A14)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A14)</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A14,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A14,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H14" s="10" t="n">
@@ -10809,11 +10887,11 @@
         </is>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A15)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A15)</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A15,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A15,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H15" s="10" t="n">
@@ -10854,11 +10932,11 @@
         </is>
       </c>
       <c r="F16" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A16)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A16)</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A16,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A16,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H16" s="10" t="n">
@@ -10899,11 +10977,11 @@
         </is>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A17)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A17)</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A17,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A17,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H17" s="10" t="n">
@@ -10944,11 +11022,11 @@
         </is>
       </c>
       <c r="F18" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A18)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A18)</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A18,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A18,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H18" s="10" t="n">
@@ -10989,11 +11067,11 @@
         </is>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A19)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A19)</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A19,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A19,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H19" s="10" t="n">
@@ -11034,11 +11112,11 @@
         </is>
       </c>
       <c r="F20" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A20)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A20)</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A20,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A20,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H20" s="10" t="n">
@@ -11075,11 +11153,11 @@
         </is>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A21)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A21)</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A21,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A21,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H21" s="10" t="n">
@@ -11116,11 +11194,11 @@
         </is>
       </c>
       <c r="F22" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A22)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A22)</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A22,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A22,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H22" s="10" t="n">
@@ -11157,11 +11235,11 @@
         </is>
       </c>
       <c r="F23" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A23)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A23)</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A23,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A23,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H23" s="10" t="n">
@@ -11198,11 +11276,11 @@
         </is>
       </c>
       <c r="F24" s="10">
-        <f>COUNTIF('Backlog do startu'!$G$2:$G$120,A24)</f>
+        <f>COUNTIF('Backlog do startu'!$G$2:$G$121,A24)</f>
         <v/>
       </c>
       <c r="G24" s="10">
-        <f>SUMIF('Backlog do startu'!$G$2:$G$120,A24,'Backlog do startu'!$F$2:$F$120)</f>
+        <f>SUMIF('Backlog do startu'!$G$2:$G$121,A24,'Backlog do startu'!$F$2:$F$121)</f>
         <v/>
       </c>
       <c r="H24" s="10" t="n">

</xml_diff>

<commit_message>
fix(www): zgoda z cookie odtwarzana przed GTM (GA4 u powracających), /specyfikacja opublikowana; audyt: PB-04, PB-06, PB-07 zamknięte
- GTM: tag Google odpala na Initialization z wymogiem analytics_storage, a zgoda z cookie wracała
  dopiero po gtm.js i page_view — powracający gość ze zgodą nie wysyłał nic do GA4
- PB-07: SPECYFIKACJA_OPUBLIKOWANA=true (treść zaakceptowana 27.09)
- audyt: PB-04, PB-06, PB-07 zamknięte; PB-08 i P-15 — stan

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -7031,7 +7031,7 @@
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty.</t>
+          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty. | 2026-09-27 SPRAWDZONE: kontener GTM-PJQNXCF5 w wersji 10 ma jeden tag Google (G-HHN0S0R777) — zdublowany GA4 wstrzymany przez właściciela. ZNALEZISKO: tag odpala na Initialization z wymogiem analytics_storage, a verris.pl odtwarzał zgodę z cookie dopiero PO gtm.js i page_view — powracający gość ze zgodą nie wysyłał nic do GA4 (tylko ccm/collect Ads). Poprawione w Analytics.tsx: zgoda z cookie odtwarzana przed GTM (jak w panelu). Zostaje: po wdrożeniu sprawdzić g/collect; nowy gość po kliknięciu „Akceptuj” — tag nie odpali do następnej odsłony (wyzwalacz Initialization) → dodać w GTM wyzwalacz zdarzenia verris_consent_update do tagu Google.</t>
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą.</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą. | 2026-09-27: właściciel — umowy powierzenia zaakceptowane przy zakładaniu kont (Hetzner, Openprovider, Cloudflare, Firmino; konta używane od wcześniejszego hostingu na Plesku), dokładnych dat nie pamięta. Cloudflare: DPA wchodzi z umową główną. Hetzner: umowę powierzenia zawiera się osobno w accounts.hetzner.com → Data protection — do potwierdzenia jednym spojrzeniem (data zawarcia widoczna na stronie), wtedy ZAMKNIĘTE.</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06).</t>
+          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06). | 2026-09-27 ZAMKNIĘTE: skrzynka abuse@verris.pl działa (przekierowanie na skrzynkę właściciela — potwierdzone przez właściciela 23.09 i 27.09); test zgłoszenia: formularz /zglos-naduzycie → ABUSE_REPORT_RECEIVED 24.09 (test-live-verris.pl, PHISHING) → decyzja w panelu obsługi 26.09 (N-13).</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8357,7 +8357,7 @@
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts.</t>
+          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts. | 2026-09-27 ZAMKNIĘTE: treści zaakceptowane przez właściciela; /specyfikacja włączona (SPECYFIKACJA_OPUBLIKOWANA=true: menu, sitemap), wiersze po D3 nadal ukryte (SPEC_PO_WERYFIKACJI); /funkcje/sla na produkcji.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8747,7 +8747,7 @@
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji.</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji. | 2026-09-27 ZAMKNIĘTE: treści zaakceptowane przez właściciela (docs/marketing/akceptacja-tresci-2026-09.md); /przenies-strone na produkcji (200).</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">

</xml_diff>

<commit_message>
audyt: tablice planu po decyzji zakresu 29.09
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1348</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="18">
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>44.9</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="19">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F78" s="10" t="n">
@@ -6855,12 +6855,12 @@
       </c>
       <c r="K78" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L78" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych; D3 t1 (d3.hvln.pl) 29.09: archiwum powstaje, ale panel mówi „nie udało się” (stara CMD_FILE_MANAGER zwraca 500 po wykonaniu) — poprawka 347e8ae (CMD_API_FILE_MANAGER)</t>
+          <t>2026-09-23 D1: POST /services/:id/files/compress → files.service compress (nazwa archiwum walidowana) → SDK compressEntries (schowek DA + action=compress) + audyt HOSTING_FILE_COMPRESSED; UI menedżera plików „Spakuj…” dla zaznaczonych; D3 t1 (d3.hvln.pl) 29.09: archiwum powstaje, ale panel mówi „nie udało się” (stara CMD_FILE_MANAGER zwraca 500 po wykonaniu) — poprawka 347e8ae (CMD_API_FILE_MANAGER); D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu: Spakuj z panelu → „Spakowano do archiwum”, verris-r2.tar.gz w katalogu (347e8ae: bez fałszywego błędu 500 starego endpointu)</t>
         </is>
       </c>
       <c r="M78" s="11" t="inlineStr">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="N78" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O78" s="11" t="inlineStr">
@@ -11317,7 +11317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11668,7 +11668,7 @@
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>C-05</t>
+          <t>C-17</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -11693,7 +11693,7 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Zmiana nazwy pliku/katalogu</t>
+          <t>Konto FTP — usunięcie</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -11716,14 +11716,14 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>files.controller.ts:81; D3 t1 (d3.hvln.pl) 29.09 FAIL: zmiana nazwy → „Wewnętrzny błąd serwera” (DA 1.710: old = sama nazwa, nie pełna ścieżka; sprawdzone na t1); poprawka 3434c1a czeka na wdrożenie</t>
+          <t>services.controller.ts:415; D3 t1 (d3.hvln.pl) 29.09: DA 1.710 zwraca listę FTP jako login@domena=ścieżka (nie user0/path0) — dodatkowe konta niewidoczne w panelu, więc bez usuwania i zmiany hasła; poprawka bcce42d czeka na wdrożenie; D3 na koncie dodatkowym</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>C-06</t>
+          <t>C-21</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Usuwanie plików (także zaznaczonych)</t>
+          <t>Dostęp SSH</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="I8" s="10" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
@@ -11771,14 +11771,14 @@
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>files.controller.ts:91; D3 t1 (d3.hvln.pl) 29.09 FAIL: „Usuń zaznaczone” → komunikat sukcesu, pliki zostają (DA 1.710 wymaga selectN = pełna ścieżka; sprawdzone na t1: nazwa → bez zmian, pełna ścieżka → usunięty); poprawka 464dd72 (SDK) czeka na wdrożenie; retest; 29.09: usuwanie pełnymi ścieżkami sprawdzone na t1 bezpośrednio w DA (6 elementów naraz); retest z panelu po wdrożeniu 347e8ae</t>
+          <t>ops/scripts/node-ssh-access.sh (zadanie SSH_ACCESS), subscriptions/ssh-access.service.ts, services.controller.ts :id/hosting-ssh(/keys), client-panel components/hosting/SshPanel.tsx (FTP → Dostęp SSH); test ssh-access.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>C-17</t>
+          <t>C-22</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Konto FTP — usunięcie</t>
+          <t>Zarządzanie kluczami SSH konta hostingowego</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -11813,11 +11813,11 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I9" s="10" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
@@ -11826,14 +11826,14 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:415; D3 t1 (d3.hvln.pl) 29.09: DA 1.710 zwraca listę FTP jako login@domena=ścieżka (nie user0/path0) — dodatkowe konta niewidoczne w panelu, więc bez usuwania i zmiany hasła; poprawka bcce42d czeka na wdrożenie; D3 na koncie dodatkowym</t>
+          <t>ops/scripts/node-ssh-access.sh (zadanie SSH_ACCESS), subscriptions/ssh-access.service.ts, services.controller.ts :id/hosting-ssh(/keys), client-panel components/hosting/SshPanel.tsx (FTP → Dostęp SSH); test ssh-access.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>C-21</t>
+          <t>C-25</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -11858,7 +11858,7 @@
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Dostęp SSH</t>
+          <t>Klonowanie repozytorium Git z panelu</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -11868,7 +11868,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I10" s="10" t="n">
@@ -11881,14 +11881,14 @@
       </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-ssh-access.sh (zadanie SSH_ACCESS), subscriptions/ssh-access.service.ts, services.controller.ts :id/hosting-ssh(/keys), client-panel components/hosting/SshPanel.tsx (FTP → Dostęp SSH); test ssh-access.service.spec.ts</t>
+          <t>ops/scripts/node-git-deploy.sh (zadanie GIT_DEPLOY: klucz ed25519 ~/.ssh/verris_deploy, git clone --depth 50 z odłożeniem dotychczasowych plików, pull --ff-only, HEAD w wyniku; jako klient), subscriptions/git-deploy.service.ts, :id/hosting-git(/key|/clone|/pull), panel GitRepoPanel.tsx (Deploy (Git) → Repozytorium strony); test git-deploy.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>C-22</t>
+          <t>C-26</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -11913,7 +11913,7 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Zarządzanie kluczami SSH konta hostingowego</t>
+          <t>Deploy z repozytorium (pull na żądanie)</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
@@ -11936,14 +11936,14 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-ssh-access.sh (zadanie SSH_ACCESS), subscriptions/ssh-access.service.ts, services.controller.ts :id/hosting-ssh(/keys), client-panel components/hosting/SshPanel.tsx (FTP → Dostęp SSH); test ssh-access.service.spec.ts</t>
+          <t>ops/scripts/node-git-deploy.sh (zadanie GIT_DEPLOY: klucz ed25519 ~/.ssh/verris_deploy, git clone --depth 50 z odłożeniem dotychczasowych plików, pull --ff-only, HEAD w wyniku; jako klient), subscriptions/git-deploy.service.ts, :id/hosting-git(/key|/clone|/pull), panel GitRepoPanel.tsx (Deploy (Git) → Repozytorium strony); test git-deploy.service.spec.ts; harmonogram: services.controller.ts:717, directadmin.service.ts createDeployJob</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>C-25</t>
+          <t>C-27</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -11968,7 +11968,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Klonowanie repozytorium Git z panelu</t>
+          <t>Webhook deploy z GitHuba</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -11978,7 +11978,7 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I12" s="10" t="n">
@@ -11991,14 +11991,14 @@
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-git-deploy.sh (zadanie GIT_DEPLOY: klucz ed25519 ~/.ssh/verris_deploy, git clone --depth 50 z odłożeniem dotychczasowych plików, pull --ff-only, HEAD w wyniku; jako klient), subscriptions/git-deploy.service.ts, :id/hosting-git(/key|/clone|/pull), panel GitRepoPanel.tsx (Deploy (Git) → Repozytorium strony); test git-deploy.service.spec.ts</t>
+          <t>subscriptions/git-webhook.controller.ts (POST /hooks/git/:token, bez logowania, limit), GitDeployService.utworzWebhook/usunWebhook/wyzwolWebhook (model GitWebhook: tylko skrót tokenu), :id/hosting-git-webhook(/delete), GitRepoPanel.tsx (adres pokazany raz, lista z datą ostatniego wywołania); test git-deploy.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>C-26</t>
+          <t>C-28</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -12023,7 +12023,7 @@
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Deploy z repozytorium (pull na żądanie)</t>
+          <t>Composer / narzędzia CLI przez SSH</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -12046,14 +12046,14 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-git-deploy.sh (zadanie GIT_DEPLOY: klucz ed25519 ~/.ssh/verris_deploy, git clone --depth 50 z odłożeniem dotychczasowych plików, pull --ff-only, HEAD w wyniku; jako klient), subscriptions/git-deploy.service.ts, :id/hosting-git(/key|/clone|/pull), panel GitRepoPanel.tsx (Deploy (Git) → Repozytorium strony); test git-deploy.service.spec.ts; harmonogram: services.controller.ts:717, directadmin.service.ts createDeployJob</t>
+          <t>zależne od C-21</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>C-27</t>
+          <t>D-08</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -12078,21 +12078,21 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Webhook deploy z GitHuba</t>
+          <t>Nadawanie uprawnień użytkownikowi bazy</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>D — Bazy danych</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I14" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J14" s="10" t="inlineStr">
         <is>
@@ -12101,14 +12101,14 @@
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/git-webhook.controller.ts (POST /hooks/git/:token, bez logowania, limit), GitDeployService.utworzWebhook/usunWebhook/wyzwolWebhook (model GitWebhook: tylko skrót tokenu), :id/hosting-git-webhook(/delete), GitRepoPanel.tsx (adres pokazany raz, lista z datą ostatniego wywołania); test git-deploy.service.spec.ts</t>
+          <t>ops/scripts/node-db-transfer.sh (privileges); db-transfer.service.ts zlecUprawnienia; DbUsers.tsx</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>C-28</t>
+          <t>D-12</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -12133,17 +12133,17 @@
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Composer / narzędzia CLI przez SSH</t>
+          <t>Import / eksport bazy z panelu</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>D — Bazy danych</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I15" s="10" t="n">
@@ -12156,14 +12156,14 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>zależne od C-21</t>
+          <t>ops/scripts/node-db-transfer.sh (zadanie DB_TRANSFER), subscriptions/db-transfer.service.ts, services.controller.ts :id/hosting-db-transfer|hosting-db-export|hosting-db-import, client-panel components/hosting/DbTransferPanel.tsx; testy db-transfer.service.spec.ts, agent-wezla-jedno-zrodlo.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>D-08</t>
+          <t>D-13</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -12188,7 +12188,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Nadawanie uprawnień użytkownikowi bazy</t>
+          <t>Kopia bazy na żądanie</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -12211,14 +12211,14 @@
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-db-transfer.sh (privileges); db-transfer.service.ts zlecUprawnienia; DbUsers.tsx</t>
+          <t>D-12: DbTransferPanel „Eksportuj bazę” (zadanie DB_TRANSFER export → ~/verris-bazy/&lt;baza&gt;-&lt;czas&gt;.sql.gz, pobranie z panelu)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>D-12</t>
+          <t>D-14</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -12243,7 +12243,7 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Import / eksport bazy z panelu</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -12253,11 +12253,11 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I17" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J17" s="10" t="inlineStr">
         <is>
@@ -12266,14 +12266,14 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-db-transfer.sh (zadanie DB_TRANSFER), subscriptions/db-transfer.service.ts, services.controller.ts :id/hosting-db-transfer|hosting-db-export|hosting-db-import, client-panel components/hosting/DbTransferPanel.tsx; testy db-transfer.service.spec.ts, agent-wezla-jedno-zrodlo.spec.ts</t>
+          <t>ops/scripts/node-pgsql.sh (zadanie PGSQL, migracja 20260925210000); subscriptions/pgsql.service.ts; services.controller.ts :id/hosting-pgsql; client-panel PgsqlPanel (zakładka Bazy danych); node-hosting-profile.sh (PostgreSQL 16 z AppStream, localhost, scram-sha-256); test pgsql.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>D-13</t>
+          <t>D-18</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -12298,7 +12298,7 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Kopia bazy na żądanie</t>
+          <t>Naprawa / optymalizacja tabel</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -12308,7 +12308,7 @@
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I18" s="10" t="n">
@@ -12321,14 +12321,14 @@
       </c>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>D-12: DbTransferPanel „Eksportuj bazę” (zadanie DB_TRANSFER export → ~/verris-bazy/&lt;baza&gt;-&lt;czas&gt;.sql.gz, pobranie z panelu)</t>
+          <t>ops/scripts/node-db-transfer.sh (repair/optimize); db-transfer.service.ts zlecKonserwacje; DbTransferPanel.tsx</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>D-14</t>
+          <t>K-04</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -12353,21 +12353,21 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>Logi dostępu WWW (access log)</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>D — Bazy danych</t>
+          <t>K — Statystyki, logi, limity</t>
         </is>
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I19" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J19" s="10" t="inlineStr">
         <is>
@@ -12376,14 +12376,14 @@
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-pgsql.sh (zadanie PGSQL, migracja 20260925210000); subscriptions/pgsql.service.ts; services.controller.ts :id/hosting-pgsql; client-panel PgsqlPanel (zakładka Bazy danych); node-hosting-profile.sh (PostgreSQL 16 z AppStream, localhost, scram-sha-256); test pgsql.service.spec.ts</t>
+          <t>GET /services/:id/hosting-logs (readHostingLog, DA CMD_SHOW_LOG type=log|error) + zakładka usługi „Logi WWW” (LogsTab.tsx); directadmin.logi.spec.ts (9 testów); subkonto: FILES_MANAGE</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>D-18</t>
+          <t>K-05</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -12408,21 +12408,21 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>Naprawa / optymalizacja tabel</t>
+          <t>Logi błędów PHP</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>D — Bazy danych</t>
+          <t>K — Statystyki, logi, limity</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I20" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J20" s="10" t="inlineStr">
         <is>
@@ -12431,14 +12431,14 @@
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-db-transfer.sh (repair/optimize); db-transfer.service.ts zlecKonserwacje; DbTransferPanel.tsx</t>
+          <t>GET /services/:id/hosting-logs (readHostingLog, DA CMD_SHOW_LOG type=log|error) + zakładka usługi „Logi WWW” (LogsTab.tsx); directadmin.logi.spec.ts (9 testów); subkonto: FILES_MANAGE</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>K-04</t>
+          <t>K-14</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -12463,7 +12463,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>Logi dostępu WWW (access log)</t>
+          <t>Wolne zapytania SQL</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -12473,7 +12473,7 @@
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I21" s="10" t="n">
@@ -12486,24 +12486,24 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>GET /services/:id/hosting-logs (readHostingLog, DA CMD_SHOW_LOG type=log|error) + zakładka usługi „Logi WWW” (LogsTab.tsx); directadmin.logi.spec.ts (9 testów); subkonto: FILES_MANAGE</t>
+          <t>ops/scripts/node-slow-sql.sh (zadanie SLOW_SQL, migracja 20260925200000); subscriptions/slow-sql.service.ts; services.controller.ts :id/hosting-slow-sql; client-panel SlowSqlPanel (zakładka Bazy danych); node-hosting-profile.sh (slow_query_log=1, long_query_time=2, logrotate); test slow-sql.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>K-05</t>
+          <t>D-15</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-02</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Wydajność: cache i skalowanie</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
@@ -12518,12 +12518,12 @@
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>Logi błędów PHP</t>
+          <t>Redis / cache obiektowy dla klienta</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>K — Statystyki, logi, limity</t>
+          <t>D — Bazy danych</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
@@ -12541,24 +12541,24 @@
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>GET /services/:id/hosting-logs (readHostingLog, DA CMD_SHOW_LOG type=log|error) + zakładka usługi „Logi WWW” (LogsTab.tsx); directadmin.logi.spec.ts (9 testów); subkonto: FILES_MANAGE</t>
+          <t>ops/scripts/node-redis.sh (zadanie REDIS_ACCESS: instancja na konto, tylko gniazdo ~/.verris-redis/redis.sock 0700, konfiguracja roota, CONFIG wyłączone, 64 MB, MemoryMax w systemd), subscriptions/redis-access.service.ts, :id/hosting-redis, panel RedisPanel.tsx (PHP i serwer); WordPress: node-wp-update.sh WPU_CACHE=redis-on/off (wtyczka Redis Object Cache, WP_REDIS_PATH, kontrola strony), WpUpdatesPanel.tsx; testy redis-access.service.spec.ts, wp-update.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>K-14</t>
+          <t>D-16</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-02</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Wydajność: cache i skalowanie</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -12573,12 +12573,12 @@
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>Wolne zapytania SQL</t>
+          <t>Memcached</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>K — Statystyki, logi, limity</t>
+          <t>D — Bazy danych</t>
         </is>
       </c>
       <c r="H23" s="10" t="inlineStr">
@@ -12596,14 +12596,14 @@
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-slow-sql.sh (zadanie SLOW_SQL, migracja 20260925200000); subscriptions/slow-sql.service.ts; services.controller.ts :id/hosting-slow-sql; client-panel SlowSqlPanel (zakładka Bazy danych); node-hosting-profile.sh (slow_query_log=1, long_query_time=2, logrotate); test slow-sql.service.spec.ts</t>
+          <t>ops/scripts/node-memcached.sh (zadanie MEMCACHED_ACCESS, migracja 20260925201000); redis-access.service.ts (silnik memcached); services.controller.ts :id/hosting-memcached; client-panel RedisPanel silnik="memcached" (zakładka PHP i serwer); node-hosting-profile.sh (pakiet memcached, usługa TCP wyłączona)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>D-15</t>
+          <t>J-03</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -12628,12 +12628,12 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Redis / cache obiektowy dla klienta</t>
+          <t>Cache obiektowy (Redis) dla WordPressa</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>D — Bazy danych</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
@@ -12658,7 +12658,7 @@
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>D-16</t>
+          <t>J-05</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -12683,12 +12683,12 @@
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Memcached</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>D — Bazy danych</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="H25" s="10" t="inlineStr">
@@ -12697,23 +12697,23 @@
         </is>
       </c>
       <c r="I25" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-memcached.sh (zadanie MEMCACHED_ACCESS, migracja 20260925201000); redis-access.service.ts (silnik memcached); services.controller.ts :id/hosting-memcached; client-panel RedisPanel silnik="memcached" (zakładka PHP i serwer); node-hosting-profile.sh (pakiet memcached, usługa TCP wyłączona)</t>
+          <t>na rynku PL płatny dodatek</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>J-03</t>
+          <t>J-06</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -12738,7 +12738,7 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Cache obiektowy (Redis) dla WordPressa</t>
+          <t>Optymalizacja obrazów</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -12748,7 +12748,7 @@
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I26" s="10" t="n">
@@ -12761,14 +12761,14 @@
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-redis.sh (zadanie REDIS_ACCESS: instancja na konto, tylko gniazdo ~/.verris-redis/redis.sock 0700, konfiguracja roota, CONFIG wyłączone, 64 MB, MemoryMax w systemd), subscriptions/redis-access.service.ts, :id/hosting-redis, panel RedisPanel.tsx (PHP i serwer); WordPress: node-wp-update.sh WPU_CACHE=redis-on/off (wtyczka Redis Object Cache, WP_REDIS_PATH, kontrola strony), WpUpdatesPanel.tsx; testy redis-access.service.spec.ts, wp-update.service.spec.ts</t>
+          <t>ops/scripts/node-image-optimize.sh (zadanie IMAGE_OPTIMIZE, migracja 20260925211000); subscriptions/obrazy.service.ts; services.controller.ts :id/hosting-images; client-panel ObrazyPanel (widok strony → Pliki); profil węzła: jpegoptim, optipng (EPEL); test obrazy.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>J-05</t>
+          <t>J-07</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>Dedykowany adres IP</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -12803,37 +12803,37 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I27" s="10" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>na rynku PL płatny dodatek</t>
+          <t>addons — jako dodatek typu workorder</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>J-06</t>
+          <t>H-03</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Wydajność: cache i skalowanie</t>
+          <t>Backup: granularność i retencja</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
@@ -12848,21 +12848,21 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>Optymalizacja obrazów</t>
+          <t>Konfigurowalna retencja kopii</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I28" s="10" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="J28" s="10" t="inlineStr">
         <is>
@@ -12871,24 +12871,24 @@
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-image-optimize.sh (zadanie IMAGE_OPTIMIZE, migracja 20260925211000); subscriptions/obrazy.service.ts; services.controller.ts :id/hosting-images; client-panel ObrazyPanel (widok strony → Pliki); profil węzła: jpegoptim, optipng (EPEL); test obrazy.service.spec.ts</t>
+          <t>services.controller.ts:926; D3 t1 (d3.hvln.pl) 29.09: DA 1.710 robi .tar.zst z datą epoch — retencja pomijała .tar.zst, a przy dacie NaN sortowała po nazwie (Sep &gt; Oct = kasowanie najnowszych); poprawka 8f7b043 + test; retest po wdrożeniu</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>J-07</t>
+          <t>H-04</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Wydajność: cache i skalowanie</t>
+          <t>Backup: granularność i retencja</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
@@ -12903,21 +12903,21 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Dedykowany adres IP</t>
+          <t>Retencja co najmniej 28 dni w cenie</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I29" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J29" s="10" t="inlineStr">
         <is>
@@ -12926,14 +12926,14 @@
       </c>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>addons — jako dodatek typu workorder</t>
+          <t>off-site: 30 dni (node-offsite-backup.sh:101); libs/contracts/src/kopie.ts; hosting-offsite-panel.tsx; test kopie-30-dni.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>H-03</t>
+          <t>H-10</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>Konfigurowalna retencja kopii</t>
+          <t>Odtworzenie pojedynczego pliku</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
@@ -12972,7 +12972,7 @@
         </is>
       </c>
       <c r="I30" s="10" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J30" s="10" t="inlineStr">
         <is>
@@ -12981,14 +12981,14 @@
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:926; D3 t1 (d3.hvln.pl) 29.09: DA 1.710 robi .tar.zst z datą epoch — retencja pomijała .tar.zst, a przy dacie NaN sortowała po nazwie (Sep &gt; Oct = kasowanie najnowszych); poprawka 8f7b043 + test; retest po wdrożeniu</t>
+          <t>ops/scripts/node-file-restore.sh (zadanie FILE_RESTORE, list/extract jako klient), subscriptions/file-restore.service.ts, services.controller.ts :id/hosting-file-restore(/list|/extract), client-panel components/hosting/ArchiveBrowser.tsx (Kopie → Pliki); test file-restore.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>H-04</t>
+          <t>H-11</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>Retencja co najmniej 28 dni w cenie</t>
+          <t>Podgląd zawartości archiwum przed odtworzeniem</t>
         </is>
       </c>
       <c r="G31" s="10" t="inlineStr">
@@ -13036,14 +13036,14 @@
       </c>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>off-site: 30 dni (node-offsite-backup.sh:101); libs/contracts/src/kopie.ts; hosting-offsite-panel.tsx; test kopie-30-dni.spec.ts</t>
+          <t>ops/scripts/node-file-restore.sh (zadanie FILE_RESTORE, list/extract jako klient), subscriptions/file-restore.service.ts, services.controller.ts :id/hosting-file-restore(/list|/extract), client-panel components/hosting/ArchiveBrowser.tsx (Kopie → Pliki); test file-restore.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>H-10</t>
+          <t>H-13</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
@@ -13068,7 +13068,7 @@
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>Odtworzenie pojedynczego pliku</t>
+          <t>Pobranie archiwum kopii lokalnie</t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr">
@@ -13078,11 +13078,11 @@
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I32" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J32" s="10" t="inlineStr">
         <is>
@@ -13091,14 +13091,14 @@
       </c>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-file-restore.sh (zadanie FILE_RESTORE, list/extract jako klient), subscriptions/file-restore.service.ts, services.controller.ts :id/hosting-file-restore(/list|/extract), client-panel components/hosting/ArchiveBrowser.tsx (Kopie → Pliki); test file-restore.service.spec.ts</t>
+          <t>files/files.service.ts downloadStream; files.controller.ts GET download-stream; client app/api/services/[id]/files/download/route.ts; BackupsTab.tsx „Pobierz”; test files.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>H-11</t>
+          <t>H-14</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
@@ -13123,7 +13123,7 @@
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Podgląd zawartości archiwum przed odtworzeniem</t>
+          <t>Kopia off-site (poza węzłem)</t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
@@ -13133,11 +13133,11 @@
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" s="10" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="J33" s="10" t="inlineStr">
         <is>
@@ -13146,14 +13146,14 @@
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-file-restore.sh (zadanie FILE_RESTORE, list/extract jako klient), subscriptions/file-restore.service.ts, services.controller.ts :id/hosting-file-restore(/list|/extract), client-panel components/hosting/ArchiveBrowser.tsx (Kopie → Pliki); test file-restore.service.spec.ts</t>
+          <t>ops/scripts/node-offsite-backup.sh:93-97 (rclone crypt → S3); D3 t1 (d3.hvln.pl) 29.09: nocny przebieg 03:54 accounts=2, archiwum konta d3 widoczne w panelu (D4 — test odtworzenia — nadal otwarte)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>H-13</t>
+          <t>H-16</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
@@ -13178,7 +13178,7 @@
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>Pobranie archiwum kopii lokalnie</t>
+          <t>ODTWORZENIE KONTA NA INNY WĘZEŁ</t>
         </is>
       </c>
       <c r="G34" s="10" t="inlineStr">
@@ -13188,11 +13188,11 @@
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I34" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
@@ -13201,14 +13201,14 @@
       </c>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>files/files.service.ts downloadStream; files.controller.ts GET download-stream; client app/api/services/[id]/files/download/route.ts; BackupsTab.tsx „Pobierz”; test files.service.spec.ts</t>
+          <t>subscriptions/odtworzenie-na-wezle.service.ts; admin subskrypcja → odtworzenie-na-wezle-panel.tsx; ops/scripts/node-account-restore.sh (OFR_MODE=restore, OFR_SOURCE_PREFIX, OFR_IP); node-tasks.service.ts completeTaskFromNode (przepięcie konta); test odtworzenie-na-wezle.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>H-14</t>
+          <t>H-18</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>Kopia off-site (poza węzłem)</t>
+          <t>Odtworzenie konta przez operatora z panelu</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
@@ -13243,11 +13243,11 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I35" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
@@ -13256,24 +13256,24 @@
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-offsite-backup.sh:93-97 (rclone crypt → S3); D3 t1 (d3.hvln.pl) 29.09: nocny przebieg 03:54 accounts=2, archiwum konta d3 widoczne w panelu (D4 — test odtworzenia — nadal otwarte)</t>
+          <t>admin: Subskrypcje → usługa → „Odtworzenie konta z kopii” (restore-panel.tsx): lista kopii (nowe GET admin/subscriptions/:id/hosting-backups), zakres, kopia bezpieczeństwa domyślnie, potwierdzenie domeną, status ostatniego odtworzenia → POST admin/subscriptions/:id/hosting-restore (SUBSCRIPTIONS_MANAGE); D3 t1 (d3.hvln.pl) 29.09 FAIL: panel operatora „Na koncie nie ma kopii do odtworzenia” mimo archiwum w /backups — ten sam parser co H-05; poprawka 8f7b043 czeka na wdrożenie; retest z odtworzeniem</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>H-16</t>
+          <t>M-33</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>Rozliczenia: dokończenie</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
@@ -13288,21 +13288,21 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>ODTWORZENIE KONTA NA INNY WĘZEŁ</t>
+          <t>Dodatki płatne (IP, wsparcie priorytetowe)</t>
         </is>
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I36" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
@@ -13311,24 +13311,24 @@
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/odtworzenie-na-wezle.service.ts; admin subskrypcja → odtworzenie-na-wezle-panel.tsx; ops/scripts/node-account-restore.sh (OFR_MODE=restore, OFR_SOURCE_PREFIX, OFR_IP); node-tasks.service.ts completeTaskFromNode (przepięcie konta); test odtworzenie-na-wezle.service.spec.ts</t>
+          <t>addon.service.ts:120 — 2 z 3 to workorder do BOK</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>H-18</t>
+          <t>N-21</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>Wsparcie i ops: kolejka abuse</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
@@ -13343,17 +13343,17 @@
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Odtworzenie konta przez operatora z panelu</t>
+          <t>Wsparcie telefoniczne</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="H37" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I37" s="10" t="n">
@@ -13361,29 +13361,29 @@
       </c>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>admin: Subskrypcje → usługa → „Odtworzenie konta z kopii” (restore-panel.tsx): lista kopii (nowe GET admin/subscriptions/:id/hosting-backups), zakres, kopia bezpieczeństwa domyślnie, potwierdzenie domeną, status ostatniego odtworzenia → POST admin/subscriptions/:id/hosting-restore (SUBSCRIPTIONS_MANAGE); D3 t1 (d3.hvln.pl) 29.09 FAIL: panel operatora „Na koncie nie ma kopii do odtworzenia” mimo archiwum w /backups — ten sam parser co H-05; poprawka 8f7b043 czeka na wdrożenie; retest z odtworzeniem</t>
+          <t>poza produktem</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>M-33</t>
+          <t>PROD-01</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>E-14</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Rozliczenia: dokończenie</t>
+          <t>Wsparcie i ops: kolejka abuse</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
@@ -13398,21 +13398,21 @@
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>Dodatki płatne (IP, wsparcie priorytetowe)</t>
+          <t>Instalator węzła bez udziału administratora</t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I38" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J38" s="10" t="inlineStr">
         <is>
@@ -13421,29 +13421,29 @@
       </c>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>addon.service.ts:120 — 2 z 3 to workorder do BOK</t>
+          <t>docs/archiwum/zadania/PROD-01-instalator-wezla-bez-czlowieka.md; stan: bootstrap v2 + kreator węzła (Q-14) — kroki CloudLinux/DA/LiteSpeed nadal ręczne</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>N-21</t>
+          <t>I-04</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Wsparcie i ops: kolejka abuse</t>
+          <t>WordPress Toolkit</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -13453,52 +13453,52 @@
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>Wsparcie telefoniczne</t>
+          <t>Automatyczne aktualizacje WordPressa</t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I39" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>poza produktem</t>
+          <t>ops/scripts/node-wp-update.sh (zadanie WP_UPDATE, check/update jako klient), subscriptions/wp-update.service.ts, wp-auto-update.scheduler.ts (codziennie 3:20), model WpAutoUpdate, services.controller.ts :id/hosting-wp-updates(/check|/run|/auto), client-panel components/hosting/WpUpdatesPanel.tsx (strona → WordPress); test wp-update.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>PROD-01</t>
+          <t>I-05</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Wsparcie i ops: kolejka abuse</t>
+          <t>WordPress Toolkit</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
@@ -13508,21 +13508,21 @@
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>Instalator węzła bez udziału administratora</t>
+          <t>Aktualizacje wtyczek i motywów z panelu</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I40" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J40" s="10" t="inlineStr">
         <is>
@@ -13531,14 +13531,14 @@
       </c>
       <c r="K40" s="11" t="inlineStr">
         <is>
-          <t>docs/archiwum/zadania/PROD-01-instalator-wezla-bez-czlowieka.md; stan: bootstrap v2 + kreator węzła (Q-14) — kroki CloudLinux/DA/LiteSpeed nadal ręczne</t>
+          <t>ops/scripts/node-wp-update.sh (zadanie WP_UPDATE, check/update jako klient), subscriptions/wp-update.service.ts, wp-auto-update.scheduler.ts (codziennie 3:20), model WpAutoUpdate, services.controller.ts :id/hosting-wp-updates(/check|/run|/auto), client-panel components/hosting/WpUpdatesPanel.tsx (strona → WordPress); test wp-update.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-07</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
@@ -13563,7 +13563,7 @@
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Automatyczne aktualizacje WordPressa</t>
+          <t>Skanowanie podatności WordPressa</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
@@ -13573,11 +13573,11 @@
       </c>
       <c r="H41" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I41" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
@@ -13586,14 +13586,14 @@
       </c>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-wp-update.sh (zadanie WP_UPDATE, check/update jako klient), subscriptions/wp-update.service.ts, wp-auto-update.scheduler.ts (codziennie 3:20), model WpAutoUpdate, services.controller.ts :id/hosting-wp-updates(/check|/run|/auto), client-panel components/hosting/WpUpdatesPanel.tsx (strona → WordPress); test wp-update.service.spec.ts</t>
+          <t>subscriptions/wp-podatnosci.service.ts (Wordfence Scanner Feed v3, cron 05:40, tabela WpPodatnosc, migracja 20260925190000); wp-update.service.ts opis/przeglad → podatnosci; client-panel WpUpdatesPanel/WpOverviewPanel; test wp-podatnosci.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>I-05</t>
+          <t>I-13</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>Aktualizacje wtyczek i motywów z panelu</t>
+          <t>Klonowanie strony między domenami</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
@@ -13641,14 +13641,14 @@
       </c>
       <c r="K42" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-wp-update.sh (zadanie WP_UPDATE, check/update jako klient), subscriptions/wp-update.service.ts, wp-auto-update.scheduler.ts (codziennie 3:20), model WpAutoUpdate, services.controller.ts :id/hosting-wp-updates(/check|/run|/auto), client-panel components/hosting/WpUpdatesPanel.tsx (strona → WordPress); test wp-update.service.spec.ts</t>
+          <t>ops/scripts/node-site-clone.sh (zadanie SITE_CLONE: cp -a jako klient, cel odkładany obok z unikalną nazwą, WordPress: zrzut → nowa baza, wp-config.php kopii, search-replace adresów), subscriptions/site-clone.service.ts (nowa baza w DA dla WP), :id/hosting-site-clone, panel SiteClonePanel.tsx (strona → Pliki → Kopia strony na inną domenę); test site-clone.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>I-07</t>
+          <t>I-16</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
@@ -13673,7 +13673,7 @@
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>Skanowanie podatności WordPressa</t>
+          <t>WP-CLI</t>
         </is>
       </c>
       <c r="G43" s="10" t="inlineStr">
@@ -13687,7 +13687,7 @@
         </is>
       </c>
       <c r="I43" s="10" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="J43" s="10" t="inlineStr">
         <is>
@@ -13696,24 +13696,24 @@
       </c>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/wp-podatnosci.service.ts (Wordfence Scanner Feed v3, cron 05:40, tabela WpPodatnosc, migracja 20260925190000); wp-update.service.ts opis/przeglad → podatnosci; client-panel WpUpdatesPanel/WpOverviewPanel; test wp-podatnosci.service.spec.ts</t>
+          <t>używane wewnętrznie przy WP_INSTALL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>I-13</t>
+          <t>A-06</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>E-03</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>WordPress Toolkit</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
@@ -13728,21 +13728,21 @@
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>Klonowanie strony między domenami</t>
+          <t>Zmiana document root domeny</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I44" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J44" s="10" t="inlineStr">
         <is>
@@ -13751,24 +13751,24 @@
       </c>
       <c r="K44" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-site-clone.sh (zadanie SITE_CLONE: cp -a jako klient, cel odkładany obok z unikalną nazwą, WordPress: zrzut → nowa baza, wp-config.php kopii, search-replace adresów), subscriptions/site-clone.service.ts (nowa baza w DA dla WP), :id/hosting-site-clone, panel SiteClonePanel.tsx (strona → Pliki → Kopia strony na inną domenę); test site-clone.service.spec.ts</t>
+          <t>servers/docroot.ts; servers/directadmin.service.ts getHostingDocroot/setHostingDocroot; GET/POST /services/:id/hosting-docroot; client components/hosting/DocrootPanel.tsx; test servers/docroot.spec.ts; D3 t1 28.09: odczyt zawsze błąd — GET CMD_API_CUSTOM_HTTPD zwraca surową treść .cust_httpd → docroot.ts trescCustomHttpd; retest</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>I-16</t>
+          <t>A-08</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>E-03</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>WordPress Toolkit</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
@@ -13783,12 +13783,12 @@
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>WP-CLI</t>
+          <t>Rejestracja domeny z panelu</t>
         </is>
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H45" s="10" t="inlineStr">
@@ -13797,23 +13797,23 @@
         </is>
       </c>
       <c r="I45" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K45" s="11" t="inlineStr">
         <is>
-          <t>używane wewnętrznie przy WP_INSTALL</t>
+          <t>domains.controller.ts:118</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>A-06</t>
+          <t>A-09</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -13838,7 +13838,7 @@
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>Zmiana document root domeny</t>
+          <t>Transfer domeny (kod authinfo)</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
@@ -13848,27 +13848,27 @@
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I46" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J46" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
-          <t>servers/docroot.ts; servers/directadmin.service.ts getHostingDocroot/setHostingDocroot; GET/POST /services/:id/hosting-docroot; client components/hosting/DocrootPanel.tsx; test servers/docroot.spec.ts; D3 t1 28.09: odczyt zawsze błąd — GET CMD_API_CUSTOM_HTTPD zwraca surową treść .cust_httpd → docroot.ts trescCustomHttpd; retest</t>
+          <t>POST /domains/:id/registrar/authcode (A-09, tylko właściciel konta, 5/h, audyt DOMAIN_AUTHCODE_REVEALED bez kodu) → OpenProvider GET /v1/domains/{id}/authcode; panel: Domeny → domena → „Transfer i abonent” → Pokaż kod; transfer PRZYCHODZĄCY: formularz z danymi abonenta i oświadczeniem; test domains/abonent-domeny.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>A-08</t>
+          <t>A-10</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
@@ -13893,7 +13893,7 @@
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
-          <t>Rejestracja domeny z panelu</t>
+          <t>Odnowienie domeny przez klienta</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
@@ -13907,7 +13907,7 @@
         </is>
       </c>
       <c r="I47" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J47" s="10" t="inlineStr">
         <is>
@@ -13916,14 +13916,14 @@
       </c>
       <c r="K47" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:118</t>
+          <t>panel: Domeny → domena → „Odnowienie domeny” (domain-renew-box.tsx: okres → cena z nowego POST domains/:id/registrar/renew-quote → potwierdzenie → POST domains/:id/registrar/renew, obciążenie portfela, zwrot przy błędzie rejestratora); liczba lat walidowana 1–10 (wcześniej body bez walidacji)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>A-09</t>
+          <t>A-12</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
-          <t>Transfer domeny (kod authinfo)</t>
+          <t>Cennik rejestracji na 1–10 lat</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr">
@@ -13958,11 +13958,11 @@
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I48" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J48" s="10" t="inlineStr">
         <is>
@@ -13971,14 +13971,14 @@
       </c>
       <c r="K48" s="11" t="inlineStr">
         <is>
-          <t>POST /domains/:id/registrar/authcode (A-09, tylko właściciel konta, 5/h, audyt DOMAIN_AUTHCODE_REVEALED bez kodu) → OpenProvider GET /v1/domains/{id}/authcode; panel: Domeny → domena → „Transfer i abonent” → Pokaż kod; transfer PRZYCHODZĄCY: formularz z danymi abonenta i oświadczeniem; test domains/abonent-domeny.spec.ts</t>
+          <t>POST domains/registrar/quote-periods (domain-registrar.service.ts quotePeriods — ceny brutto dla 1, 2, 3, 5 i 10 lat + cena odnowienia/rok) → kreator zakupu: krok „Okres” z ceną każdego wariantu (domain-purchase-wizard.tsx YEAR_OPTIONS)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>A-10</t>
+          <t>A-13</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -14003,7 +14003,7 @@
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>Odnowienie domeny przez klienta</t>
+          <t>Zmiana danych abonenta domeny</t>
         </is>
       </c>
       <c r="G49" s="10" t="inlineStr">
@@ -14013,11 +14013,11 @@
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I49" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J49" s="10" t="inlineStr">
         <is>
@@ -14026,14 +14026,14 @@
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>panel: Domeny → domena → „Odnowienie domeny” (domain-renew-box.tsx: okres → cena z nowego POST domains/:id/registrar/renew-quote → potwierdzenie → POST domains/:id/registrar/renew, obciążenie portfela, zwrot przy błędzie rejestratora); liczba lat walidowana 1–10 (wcześniej body bez walidacji)</t>
+          <t>GET/PUT /domains/:id/registrar/registrant (tylko właściciel konta) → OpenProvider /v1/customers/{handle}; rejestracja i transfer zakładają uchwyt klienta (POST /v1/customers) przed obciążeniem portfela; panel: kreator zakupu, zamówienie hostingu z domeną, transfer, strona domeny; test domains/abonent-domeny.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>A-12</t>
+          <t>A-14</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -14058,7 +14058,7 @@
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>Cennik rejestracji na 1–10 lat</t>
+          <t>Ukrycie danych WHOIS / domain privacy</t>
         </is>
       </c>
       <c r="G50" s="10" t="inlineStr">
@@ -14068,7 +14068,7 @@
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I50" s="10" t="n">
@@ -14076,19 +14076,19 @@
       </c>
       <c r="J50" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>POST domains/registrar/quote-periods (domain-registrar.service.ts quotePeriods — ceny brutto dla 1, 2, 3, 5 i 10 lat + cena odnowienia/rok) → kreator zakupu: krok „Okres” z ceną każdego wariantu (domain-purchase-wizard.tsx YEAR_OPTIONS)</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-24: po starcie — u OpenProvider ukrycie WHOIS to usługa płatna per domena, a dla osób fizycznych z .pl rejestr i tak nie publikuje danych; wracamy przy sprzedaży domen, gdy znane będą koszty.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>A-13</t>
+          <t>A-15</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
@@ -14113,7 +14113,7 @@
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>Zmiana danych abonenta domeny</t>
+          <t>Blokada transferu domeny (transfer lock)</t>
         </is>
       </c>
       <c r="G51" s="10" t="inlineStr">
@@ -14123,11 +14123,11 @@
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I51" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J51" s="10" t="inlineStr">
         <is>
@@ -14136,24 +14136,24 @@
       </c>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>GET/PUT /domains/:id/registrar/registrant (tylko właściciel konta) → OpenProvider /v1/customers/{handle}; rejestracja i transfer zakładają uchwyt klienta (POST /v1/customers) przed obciążeniem portfela; panel: kreator zakupu, zamówienie hostingu z domeną, transfer, strona domeny; test domains/abonent-domeny.spec.ts</t>
+          <t>POST /domains/:id/registrar/lock → OpenProvider PUT /v1/domains/{id} {is_locked}; stan w Domain.transferLock + audyt DOMAIN_TRANSFER_LOCKED/UNLOCKED; panel: strona domeny „Transfer i abonent”; test domains/abonent-domeny.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>A-14</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-05</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Katalog aplikacji</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
@@ -14163,52 +14163,52 @@
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>Ukrycie danych WHOIS / domain privacy</t>
+          <t>Autoinstalator aplikacji</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I52" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J52" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-24: po starcie — u OpenProvider ukrycie WHOIS to usługa płatna per domena, a dla osób fizycznych z .pl rejestr i tak nie publikuje danych; wracamy przy sprzedaży domen, gdy znane będą koszty.</t>
+          <t>app-install.service.ts CATALOG (Nextcloud, PrestaShop, Joomla, MediaWiki); ops/scripts/node-app-install.sh; test test/instalator-aplikacji-katalog.spec.ts; D3 t1 28.09: WordPress 1-click na t1 — WP_INSTALL zakończone (kolejka ~3 min), strona po zmianie NS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>A-15</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Poczta: filtry, kalendarz, limity</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
@@ -14218,17 +14218,17 @@
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
         <is>
-          <t>Blokada transferu domeny (transfer lock)</t>
+          <t>Reguły filtrowania poczty (Sieve)</t>
         </is>
       </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
@@ -14237,33 +14237,33 @@
         </is>
       </c>
       <c r="I53" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J53" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>POST /domains/:id/registrar/lock → OpenProvider PUT /v1/domains/{id} {is_locked}; stan w Domain.transferLock + audyt DOMAIN_TRANSFER_LOCKED/UNLOCKED; panel: strona domeny „Transfer i abonent”; test domains/abonent-domeny.spec.ts</t>
+          <t>ops/scripts/node-hosting-profile.sh (da build dovecot_pigeonhole); client-panel MailTab.tsx (Filtry w webmailu)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>E-05</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Katalog aplikacji</t>
+          <t>Poczta: filtry, kalendarz, limity</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
@@ -14278,12 +14278,12 @@
       </c>
       <c r="F54" s="11" t="inlineStr">
         <is>
-          <t>Autoinstalator aplikacji</t>
+          <t>Webmail — auto-logowanie (SSO)</t>
         </is>
       </c>
       <c r="G54" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="H54" s="10" t="inlineStr">
@@ -14292,7 +14292,7 @@
         </is>
       </c>
       <c r="I54" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J54" s="10" t="inlineStr">
         <is>
@@ -14301,21 +14301,21 @@
       </c>
       <c r="K54" s="11" t="inlineStr">
         <is>
-          <t>app-install.service.ts CATALOG (Nextcloud, PrestaShop, Joomla, MediaWiki); ops/scripts/node-app-install.sh; test test/instalator-aplikacji-katalog.spec.ts; D3 t1 28.09: WordPress 1-click na t1 — WP_INSTALL zakończone (kolejka ~3 min), strona po zmianie NS</t>
+          <t>services.controller.ts — POST /services/:id/hosting-sso-url (wspólna trasa z D-11); MailTab.tsx:68; D3 t1 (d3.hvln.pl) 29.09: SSO działa do DA, nie do webmaila (jak E-13); retest po f8cfd8d; 29.09: przycisk „Webmail →” w Verris prowadzi do listy skrzynek DA (drugi klik); poprawka 3434c1a — prosto do Roundcube tokenem z CMD_WEBMAIL_LOGIN</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
+          <t>E-21</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
           <t>E-10</t>
         </is>
       </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t>E-10</t>
-        </is>
-      </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
           <t>Poczta: filtry, kalendarz, limity</t>
@@ -14333,7 +14333,7 @@
       </c>
       <c r="F55" s="11" t="inlineStr">
         <is>
-          <t>Catch-all</t>
+          <t>Samodzielny import skrzynek przez IMAP</t>
         </is>
       </c>
       <c r="G55" s="10" t="inlineStr">
@@ -14347,7 +14347,7 @@
         </is>
       </c>
       <c r="I55" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J55" s="10" t="inlineStr">
         <is>
@@ -14356,14 +14356,14 @@
       </c>
       <c r="K55" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:585; D3 t1 (d3.hvln.pl) 28.09 FAIL: CMD_API_EMAIL_CATCH_ALL 500 — pakiet bez catchall=ON; poprawka e047077 (pakiety) + wypchnięcie pakietów na flotę; retest</t>
+          <t>subscriptions/migration-orchestrator.service.ts createBundle (IMAP_SYNC, imapsync w node-migration-worker.sh); migrations/migration-wizard.tsx tryb tylkoPoczta; MailTab.tsx „Przenieś pocztę z innego serwera”; test migration-orchestrator.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>E-11</t>
+          <t>E-23</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
@@ -14388,7 +14388,7 @@
       </c>
       <c r="F56" s="11" t="inlineStr">
         <is>
-          <t>Filtr antyspamowy (próg + tag)</t>
+          <t>Kalendarz i kontakty (CalDAV/CardDAV)</t>
         </is>
       </c>
       <c r="G56" s="10" t="inlineStr">
@@ -14398,11 +14398,11 @@
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I56" s="10" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J56" s="10" t="inlineStr">
         <is>
@@ -14411,14 +14411,14 @@
       </c>
       <c r="K56" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:599; D3 t1 (d3.hvln.pl) 28.09 FAIL: „Spamd nie jest uruchomiony” — węzeł bez filtra; poprawka e047077 (rspamd w profilu) + uruchomienie profilu; retest; 29.09 po profilu: rspamd działa, odczyt filtra w panelu OK (5.0, tag), zapis → błąd DA (required_hits, blacklist/whitelist) — poprawka 2495c13, sprawdzona na t1 bezpośrednio</t>
+          <t>node-hosting-profile.sh (Radicale 3.8.1 w venv, verris-radicale.service, verris-dav-backup); security-hardening-baseline.sh (5232/tcp); client-panel MailTab (adres i instrukcja); test kalendarz-kontakty.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-24</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
@@ -14443,7 +14443,7 @@
       </c>
       <c r="F57" s="11" t="inlineStr">
         <is>
-          <t>Reguły filtrowania poczty (Sieve)</t>
+          <t>2FA dla webmaila</t>
         </is>
       </c>
       <c r="G57" s="10" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I57" s="10" t="n">
@@ -14461,34 +14461,34 @@
       </c>
       <c r="J57" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K57" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-hosting-profile.sh (da build dovecot_pigeonhole); client-panel MailTab.tsx (Filtry w webmailu)</t>
+          <t>cyber_Folks ma nawet 2FA dla IMAP/SMTP</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>E-14</t>
+          <t>G-08</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Bezpieczeństwo jako funkcja</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
@@ -14498,52 +14498,52 @@
       </c>
       <c r="F58" s="11" t="inlineStr">
         <is>
-          <t>Webmail — auto-logowanie (SSO)</t>
+          <t>Sprzedaż certyfikatów DV/OV/EV</t>
         </is>
       </c>
       <c r="G58" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I58" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J58" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K58" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts — POST /services/:id/hosting-sso-url (wspólna trasa z D-11); MailTab.tsx:68; D3 t1 (d3.hvln.pl) 29.09: SSO działa do DA, nie do webmaila (jak E-13); retest po f8cfd8d; 29.09: przycisk „Webmail →” w Verris prowadzi do listy skrzynek DA (drugi klik); poprawka 3434c1a — prosto do Roundcube tokenem z CMD_WEBMAIL_LOGIN</t>
+          <t>wszystkie 5 hostingów PL to sprzedaje</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>E-19</t>
+          <t>G-09</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Bezpieczeństwo jako funkcja</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
@@ -14553,21 +14553,21 @@
       </c>
       <c r="F59" s="11" t="inlineStr">
         <is>
-          <t>Podgląd kolejki i logów dostarczania</t>
+          <t>WAF — włączenie i tryb pracy</t>
         </is>
       </c>
       <c r="G59" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I59" s="10" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="J59" s="10" t="inlineStr">
         <is>
@@ -14576,29 +14576,29 @@
       </c>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-mail-log.sh (zadanie MAIL_LOG: log exima mainlog + mainlog.1, tylko wiadomości z nadawcą lub odbiorcą w domenach usługi — lista domen z API), subscriptions/mail-log.service.ts, :id/hosting-mail-log, panel MailLogPanel.tsx (Poczta → Dziennik dostarczania); test mail-log.service.spec.ts</t>
+          <t>services.controller.ts:203</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>E-21</t>
+          <t>G-12</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Bezpieczeństwo jako funkcja</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E60" s="10" t="inlineStr">
@@ -14608,12 +14608,12 @@
       </c>
       <c r="F60" s="11" t="inlineStr">
         <is>
-          <t>Samodzielny import skrzynek przez IMAP</t>
+          <t>Czyszczenie zainfekowanych plików</t>
         </is>
       </c>
       <c r="G60" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="H60" s="10" t="inlineStr">
@@ -14622,38 +14622,38 @@
         </is>
       </c>
       <c r="I60" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J60" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K60" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/migration-orchestrator.service.ts createBundle (IMAP_SYNC, imapsync w node-migration-worker.sh); migrations/migration-wizard.tsx tryb tylkoPoczta; MailTab.tsx „Przenieś pocztę z innego serwera”; test migration-orchestrator.service.spec.ts</t>
+          <t xml:space="preserve"> | DECYZJA WŁAŚCICIELA 2026-09-25: na start darmowy ImunifyAV (wykrywanie, G-11), czyszczenie robi obsługa na zgłoszenie; płatny ImunifyAV+ po starcie (wybór „po starcie”).</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>E-23</t>
+          <t>G-21</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Bezpieczeństwo jako funkcja</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
@@ -14663,17 +14663,17 @@
       </c>
       <c r="F61" s="11" t="inlineStr">
         <is>
-          <t>Kalendarz i kontakty (CalDAV/CardDAV)</t>
+          <t>Anty-DDoS</t>
         </is>
       </c>
       <c r="G61" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I61" s="10" t="n">
@@ -14686,29 +14686,29 @@
       </c>
       <c r="K61" s="11" t="inlineStr">
         <is>
-          <t>node-hosting-profile.sh (Radicale 3.8.1 w venv, verris-radicale.service, verris-dav-backup); security-hardening-baseline.sh (5232/tcp); client-panel MailTab (adres i instrukcja); test kalendarz-kontakty.spec.ts</t>
+          <t>ops/docs/DDOS.md; Hetzner DDoS Protection (L3/L4, w cenie); RateLimitGuard + Turnstile (L7 panel/API); LiteSpeed Per-Client Throttling (węzeł, onboarding)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>E-24</t>
+          <t>O-05</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-07</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Reseller jako produkt</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
@@ -14718,47 +14718,47 @@
       </c>
       <c r="F62" s="11" t="inlineStr">
         <is>
-          <t>2FA dla webmaila</t>
+          <t>Reseller — przegląd klientów</t>
         </is>
       </c>
       <c r="G62" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>O — Multi-user i reseller</t>
         </is>
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I62" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J62" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="K62" s="11" t="inlineStr">
         <is>
-          <t>cyber_Folks ma nawet 2FA dla IMAP/SMTP</t>
+          <t>reseller-klienci.service.ts + reseller.controller.ts (5 tras), reseller-klient.tsx; reseller-klienci.int-spec.ts (6 testów na PostgreSQL)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>G-08</t>
+          <t>O-07</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-07</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Bezpieczeństwo jako funkcja</t>
+          <t>Reseller jako produkt</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
@@ -14773,12 +14773,12 @@
       </c>
       <c r="F63" s="11" t="inlineStr">
         <is>
-          <t>Sprzedaż certyfikatów DV/OV/EV</t>
+          <t>Reseller — ustawianie własnej marży</t>
         </is>
       </c>
       <c r="G63" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>O — Multi-user i reseller</t>
         </is>
       </c>
       <c r="H63" s="10" t="inlineStr">
@@ -14791,29 +14791,29 @@
       </c>
       <c r="J63" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>wszystkie 5 hostingów PL to sprzedaje</t>
+          <t>reseller.controller.ts POST me/markup → reseller.service.ts setMarkup (0–300%, audyt RESELLER_MARKUP_CHANGED); reseller-client.tsx „Twój narzut”; test reseller.apply.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>G-09</t>
+          <t>P-12</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-08</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Bezpieczeństwo jako funkcja</t>
+          <t>Dostępność i zgodność w produkcie</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
@@ -14828,47 +14828,47 @@
       </c>
       <c r="F64" s="11" t="inlineStr">
         <is>
-          <t>WAF — włączenie i tryb pracy</t>
+          <t>Dostępność panelu wg WCAG 2.1 AA (EAA)</t>
         </is>
       </c>
       <c r="G64" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I64" s="10" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J64" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="K64" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:203</t>
+          <t>eslint.config.mjs w 4 aplikacjach: jsx-a11y recommended jako błędy (34 reguły); 76 → 0 znalezisk (client 52, admin 17, staff 6, www 1); client-panel/src/lib/kontrast-tokenow.spec.ts; ops/qa/a11y-nazwy-kontrolek.js</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>G-12</t>
+          <t>P-14</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-08</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Bezpieczeństwo jako funkcja</t>
+          <t>Dostępność i zgodność w produkcie</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
@@ -14883,17 +14883,17 @@
       </c>
       <c r="F65" s="11" t="inlineStr">
         <is>
-          <t>Czyszczenie zainfekowanych plików</t>
+          <t>Certyfikacja ISO 27001</t>
         </is>
       </c>
       <c r="G65" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="H65" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I65" s="10" t="n">
@@ -14906,24 +14906,24 @@
       </c>
       <c r="K65" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | DECYZJA WŁAŚCICIELA 2026-09-25: na start darmowy ImunifyAV (wykrywanie, G-11), czyszczenie robi obsługa na zgłoszenie; płatny ImunifyAV+ po starcie (wybór „po starcie”).</t>
+          <t>home.pl i nazwa.pl mają — element przetargowy w B2B</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>G-21</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-11</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Bezpieczeństwo jako funkcja</t>
+          <t>DNS: DNSSEC i zarządzanie strefą</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
@@ -14938,12 +14938,12 @@
       </c>
       <c r="F66" s="11" t="inlineStr">
         <is>
-          <t>Anty-DDoS</t>
+          <t>DNSSEC</t>
         </is>
       </c>
       <c r="G66" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>F — DNS</t>
         </is>
       </c>
       <c r="H66" s="10" t="inlineStr">
@@ -14952,7 +14952,7 @@
         </is>
       </c>
       <c r="I66" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J66" s="10" t="inlineStr">
         <is>
@@ -14961,24 +14961,24 @@
       </c>
       <c r="K66" s="11" t="inlineStr">
         <is>
-          <t>ops/docs/DDOS.md; Hetzner DDoS Protection (L3/L4, w cenie); RateLimitGuard + Turnstile (L7 panel/API); LiteSpeed Per-Client Throttling (węzeł, onboarding)</t>
+          <t>servers/directadmin.service.ts getHostingDnssec/enableHostingDnssec/disableHostingDnssec; services.controller.ts :id/hosting-dns/dnssec; client-panel components/hosting/DnssecPanel.tsx; ops/scripts/node-hosting-profile.sh dnssec=1; test directadmin.dnssec.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>O-05</t>
+          <t>F-11</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>E-07</t>
+          <t>E-11</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Reseller jako produkt</t>
+          <t>DNS: DNSSEC i zarządzanie strefą</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
@@ -14993,12 +14993,12 @@
       </c>
       <c r="F67" s="11" t="inlineStr">
         <is>
-          <t>Reseller — przegląd klientów</t>
+          <t>Zmiana TTL rekordów</t>
         </is>
       </c>
       <c r="G67" s="10" t="inlineStr">
         <is>
-          <t>O — Multi-user i reseller</t>
+          <t>F — DNS</t>
         </is>
       </c>
       <c r="H67" s="10" t="inlineStr">
@@ -15007,33 +15007,33 @@
         </is>
       </c>
       <c r="I67" s="10" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="J67" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K67" s="11" t="inlineStr">
         <is>
-          <t>reseller-klienci.service.ts + reseller.controller.ts (5 tras), reseller-klient.tsx; reseller-klienci.int-spec.ts (6 testów na PostgreSQL)</t>
+          <t>dns-manager.tsx:287,349 — pole TTL w formularzu rekordu → UtworzRekordDnsDto.ttl (60–86400) → directadmin.service createHostingDnsRecord ttl</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>O-07</t>
+          <t>F-12</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>E-07</t>
+          <t>E-11</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Reseller jako produkt</t>
+          <t>DNS: DNSSEC i zarządzanie strefą</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
@@ -15048,12 +15048,12 @@
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>Reseller — ustawianie własnej marży</t>
+          <t>Anycast DNS</t>
         </is>
       </c>
       <c r="G68" s="10" t="inlineStr">
         <is>
-          <t>O — Multi-user i reseller</t>
+          <t>F — DNS</t>
         </is>
       </c>
       <c r="H68" s="10" t="inlineStr">
@@ -15062,33 +15062,33 @@
         </is>
       </c>
       <c r="I68" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J68" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K68" s="11" t="inlineStr">
         <is>
-          <t>reseller.controller.ts POST me/markup → reseller.service.ts setMarkup (0–300%, audyt RESELLER_MARKUP_CHANGED); reseller-client.tsx „Twój narzut”; test reseller.apply.spec.ts</t>
+          <t>tylko nazwa.pl na rynku PL</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>P-12</t>
+          <t>L-08</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>E-08</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Dostępność i zgodność w produkcie</t>
+          <t>Automatyzacja: API zapisu i webhooki</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
@@ -15103,12 +15103,12 @@
       </c>
       <c r="F69" s="11" t="inlineStr">
         <is>
-          <t>Dostępność panelu wg WCAG 2.1 AA (EAA)</t>
+          <t>Publiczne API — zapis</t>
         </is>
       </c>
       <c r="G69" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>L — Automatyzacja</t>
         </is>
       </c>
       <c r="H69" s="10" t="inlineStr">
@@ -15121,29 +15121,29 @@
       </c>
       <c r="J69" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K69" s="11" t="inlineStr">
         <is>
-          <t>eslint.config.mjs w 4 aplikacjach: jsx-a11y recommended jako błędy (34 reguły); 76 → 0 znalezisk (client 52, admin 17, staff 6, www 1); client-panel/src/lib/kontrast-tokenow.spec.ts; ops/qa/a11y-nazwy-kontrolek.js</t>
+          <t>subscriptions/public-api-write.controller.ts (api/v1/services/:id/dns GET/POST, /dns/delete, /deploy GET/POST; zakresy dns:read, dns:write, deploy:write w api-scopes.ts; te same serwisy i walidacja co panel), opis w panelu api-tokens-client.tsx; test public-api-write.controller.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>P-14</t>
+          <t>L-10</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>E-08</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Dostępność i zgodność w produkcie</t>
+          <t>Automatyzacja: API zapisu i webhooki</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
@@ -15158,12 +15158,12 @@
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>Certyfikacja ISO 27001</t>
+          <t>Webhooki dla klienta</t>
         </is>
       </c>
       <c r="G70" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>L — Automatyzacja</t>
         </is>
       </c>
       <c r="H70" s="10" t="inlineStr">
@@ -15172,33 +15172,33 @@
         </is>
       </c>
       <c r="I70" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J70" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K70" s="11" t="inlineStr">
         <is>
-          <t>home.pl i nazwa.pl mają — element przetargowy w B2B</t>
+          <t>client-webhooks/ (serwis, kontroler users/me/webhooks, moduł globalny); node-tasks.service.ts → poZadaniu; api-tokens/webhooks-client.tsx; migracja 20260924242000_client_webhooks; test client-webhooks.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>F-06</t>
+          <t>L-11</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>E-11</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>DNS: DNSSEC i zarządzanie strefą</t>
+          <t>Automatyzacja: API zapisu i webhooki</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
@@ -15213,12 +15213,12 @@
       </c>
       <c r="F71" s="11" t="inlineStr">
         <is>
-          <t>DNSSEC</t>
+          <t>Asystent AI w panelu</t>
         </is>
       </c>
       <c r="G71" s="10" t="inlineStr">
         <is>
-          <t>F — DNS</t>
+          <t>L — Automatyzacja</t>
         </is>
       </c>
       <c r="H71" s="10" t="inlineStr">
@@ -15227,33 +15227,33 @@
         </is>
       </c>
       <c r="I71" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J71" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K71" s="11" t="inlineStr">
         <is>
-          <t>servers/directadmin.service.ts getHostingDnssec/enableHostingDnssec/disableHostingDnssec; services.controller.ts :id/hosting-dns/dnssec; client-panel components/hosting/DnssecPanel.tsx; ops/scripts/node-hosting-profile.sh dnssec=1; test directadmin.dnssec.spec.ts</t>
+          <t>ai-modele.ts; ai-provider.service.ts; ai-ustawienia.admin.controller.ts; admin /settings/ai</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>F-11</t>
+          <t>L-12</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>E-11</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>DNS: DNSSEC i zarządzanie strefą</t>
+          <t>Automatyzacja: API zapisu i webhooki</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
@@ -15268,17 +15268,17 @@
       </c>
       <c r="F72" s="11" t="inlineStr">
         <is>
-          <t>Zmiana TTL rekordów</t>
+          <t>Prognoza zużycia zasobów (AI)</t>
         </is>
       </c>
       <c r="G72" s="10" t="inlineStr">
         <is>
-          <t>F — DNS</t>
+          <t>L — Automatyzacja</t>
         </is>
       </c>
       <c r="H72" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I72" s="10" t="n">
@@ -15286,113 +15286,113 @@
       </c>
       <c r="J72" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K72" s="11" t="inlineStr">
         <is>
-          <t>dns-manager.tsx:287,349 — pole TTL w formularzu rekordu → UtworzRekordDnsDto.ttl (60–86400) → directadmin.service createHostingDnsRecord ttl</t>
+          <t>hosting-forecast-actions.ts:7; fallback ServiceForecastPanel.tsx:97</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>F-12</t>
+          <t>NODE-01</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>E-11</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>DNS: DNSSEC i zarządzanie strefą</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>Anycast DNS</t>
+          <t>Dwie niepołączone ścieżki dodania węzła w tym samym panelu</t>
         </is>
       </c>
       <c r="G73" s="10" t="inlineStr">
         <is>
-          <t>F — DNS</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H73" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I73" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J73" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="K73" s="11" t="inlineStr">
         <is>
-          <t>tylko nazwa.pl na rynku PL</t>
+          <t>node-wizard.tsx (krok „Instalacja (bootstrap v2)” z NodeBootstrapProgress), /nodes/init → przekierowanie, NODE_ONBOARD_RUNBOOK.md jedynym runbookiem</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>L-08</t>
+          <t>Q-05</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>E-13</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Automatyzacja: API zapisu i webhooki</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E74" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>Publiczne API — zapis</t>
+          <t>E-mail marketing wbudowany w panel</t>
         </is>
       </c>
       <c r="G74" s="10" t="inlineStr">
         <is>
-          <t>L — Automatyzacja</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I74" s="10" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="J74" s="10" t="inlineStr">
         <is>
@@ -15401,49 +15401,49 @@
       </c>
       <c r="K74" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/public-api-write.controller.ts (api/v1/services/:id/dns GET/POST, /dns/delete, /deploy GET/POST; zakresy dns:read, dns:write, deploy:write w api-scopes.ts; te same serwisy i walidacja co panel), opis w panelu api-tokens-client.tsx; test public-api-write.controller.spec.ts</t>
+          <t>email-marketing.controller.ts:36,81,119,139</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>L-10</t>
+          <t>Q-06</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>E-13</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Automatyzacja: API zapisu i webhooki</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F75" s="11" t="inlineStr">
         <is>
-          <t>Webhooki dla klienta</t>
+          <t>VPS / cloud w tym samym panelu</t>
         </is>
       </c>
       <c r="G75" s="10" t="inlineStr">
         <is>
-          <t>L — Automatyzacja</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H75" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I75" s="10" t="n">
@@ -15451,104 +15451,100 @@
       </c>
       <c r="J75" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K75" s="11" t="inlineStr">
         <is>
-          <t>client-webhooks/ (serwis, kontroler users/me/webhooks, moduł globalny); node-tasks.service.ts → poZadaniu; api-tokens/webhooks-client.tsx; migracja 20260924242000_client_webhooks; test client-webhooks.service.spec.ts</t>
+          <t>vps.controller.ts:53,59,69; HETZNER_API_TOKEN</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>L-11</t>
+          <t>Q-07</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>E-13</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Automatyzacja: API zapisu i webhooki</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E76" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>Asystent AI w panelu</t>
+          <t>VPS — konsola / VNC</t>
         </is>
       </c>
       <c r="G76" s="10" t="inlineStr">
         <is>
-          <t>L — Automatyzacja</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H76" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I76" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J76" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
-        </is>
-      </c>
-      <c r="K76" s="11" t="inlineStr">
-        <is>
-          <t>ai-modele.ts; ai-provider.service.ts; ai-ustawienia.admin.controller.ts; admin /settings/ai</t>
-        </is>
-      </c>
+          <t>BRAK</t>
+        </is>
+      </c>
+      <c r="K76" s="11" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>L-12</t>
+          <t>Q-08</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>E-13</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Automatyzacja: API zapisu i webhooki</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F77" s="11" t="inlineStr">
         <is>
-          <t>Prognoza zużycia zasobów (AI)</t>
+          <t>VPS — snapshoty i rebuild</t>
         </is>
       </c>
       <c r="G77" s="10" t="inlineStr">
         <is>
-          <t>L — Automatyzacja</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H77" s="10" t="inlineStr">
@@ -15557,23 +15553,19 @@
         </is>
       </c>
       <c r="I77" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J77" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
-        </is>
-      </c>
-      <c r="K77" s="11" t="inlineStr">
-        <is>
-          <t>hosting-forecast-actions.ts:7; fallback ServiceForecastPanel.tsx:97</t>
-        </is>
-      </c>
+          <t>BRAK</t>
+        </is>
+      </c>
+      <c r="K77" s="11" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>NODE-01</t>
+          <t>Q-14</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
@@ -15598,7 +15590,7 @@
       </c>
       <c r="F78" s="11" t="inlineStr">
         <is>
-          <t>Dwie niepołączone ścieżki dodania węzła w tym samym panelu</t>
+          <t>Kreator uruchomienia węzła</t>
         </is>
       </c>
       <c r="G78" s="10" t="inlineStr">
@@ -15608,7 +15600,7 @@
       </c>
       <c r="H78" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I78" s="10" t="n">
@@ -15616,284 +15608,17 @@
       </c>
       <c r="J78" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K78" s="11" t="inlineStr">
         <is>
-          <t>node-wizard.tsx (krok „Instalacja (bootstrap v2)” z NodeBootstrapProgress), /nodes/init → przekierowanie, NODE_ONBOARD_RUNBOOK.md jedynym runbookiem</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="10" t="inlineStr">
-        <is>
-          <t>Q-05</t>
-        </is>
-      </c>
-      <c r="B79" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C79" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D79" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E79" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F79" s="11" t="inlineStr">
-        <is>
-          <t>E-mail marketing wbudowany w panel</t>
-        </is>
-      </c>
-      <c r="G79" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H79" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I79" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J79" s="10" t="inlineStr">
-        <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K79" s="11" t="inlineStr">
-        <is>
-          <t>email-marketing.controller.ts:36,81,119,139</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="10" t="inlineStr">
-        <is>
-          <t>Q-06</t>
-        </is>
-      </c>
-      <c r="B80" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C80" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D80" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E80" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F80" s="11" t="inlineStr">
-        <is>
-          <t>VPS / cloud w tym samym panelu</t>
-        </is>
-      </c>
-      <c r="G80" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H80" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNIA</t>
-        </is>
-      </c>
-      <c r="I80" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J80" s="10" t="inlineStr">
-        <is>
-          <t>FLAGA</t>
-        </is>
-      </c>
-      <c r="K80" s="11" t="inlineStr">
-        <is>
-          <t>vps.controller.ts:53,59,69; HETZNER_API_TOKEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="10" t="inlineStr">
-        <is>
-          <t>Q-07</t>
-        </is>
-      </c>
-      <c r="B81" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C81" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D81" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E81" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F81" s="11" t="inlineStr">
-        <is>
-          <t>VPS — konsola / VNC</t>
-        </is>
-      </c>
-      <c r="G81" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H81" s="10" t="inlineStr">
-        <is>
-          <t>NISKA</t>
-        </is>
-      </c>
-      <c r="I81" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J81" s="10" t="inlineStr">
-        <is>
-          <t>BRAK</t>
-        </is>
-      </c>
-      <c r="K81" s="11" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="10" t="inlineStr">
-        <is>
-          <t>Q-08</t>
-        </is>
-      </c>
-      <c r="B82" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C82" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D82" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E82" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F82" s="11" t="inlineStr">
-        <is>
-          <t>VPS — snapshoty i rebuild</t>
-        </is>
-      </c>
-      <c r="G82" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H82" s="10" t="inlineStr">
-        <is>
-          <t>NISKA</t>
-        </is>
-      </c>
-      <c r="I82" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J82" s="10" t="inlineStr">
-        <is>
-          <t>BRAK</t>
-        </is>
-      </c>
-      <c r="K82" s="11" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="10" t="inlineStr">
-        <is>
-          <t>Q-14</t>
-        </is>
-      </c>
-      <c r="B83" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C83" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D83" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E83" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F83" s="11" t="inlineStr">
-        <is>
-          <t>Kreator uruchomienia węzła</t>
-        </is>
-      </c>
-      <c r="G83" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H83" s="10" t="inlineStr">
-        <is>
-          <t>WYSOKA</t>
-        </is>
-      </c>
-      <c r="I83" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J83" s="10" t="inlineStr">
-        <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K83" s="11" t="inlineStr">
-        <is>
           <t>node-wizard.tsx:277,288 — realnie tylko init + bootstrap; 7 z 9 kroków to treść runbooka (wizard-content.ts:21-40)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83"/>
+  <autoFilter ref="A1:K78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
audyt: tablice planu (plan-startowy) zsynchronizowane z macierzą — 75,0% planu, 90,0% kod gotowy
Wcześniejsze commity audytu dodawały tylko audyt/ i audyt-parytetu-2026-08/, więc
VERRIS_PLAN_DASHBOARD.html, PLAN_SPRINTOW i backlog w git zostały na 66,1%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>68</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1224</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="18">
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>40.8</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="19">
@@ -4515,12 +4515,12 @@
       </c>
       <c r="K48" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L48" s="11" t="inlineStr">
         <is>
-          <t>2026-09-22 D1: components/hosting/DnsZoneSection.tsx — edytor strefy w zakladce Domeny huba uslugi (wybor domeny, DnsManager z onChanged); dns-manager.tsx typy A/AAAA/CNAME/MX/TXT/SRV/NS/CAA; API subscriptions/dto/hosting-dns.dto.ts (whitelista typow, wzorzec nazwy, zakaz znakow sterujacych, TTL 60-86400) + assertDomainOnSubscription przy odczycie/dodaniu/usunieciu; test hosting-dns-dto.spec.ts; D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu 13:00 (panel klienta): CAA 0 issue "letsencrypt.org" dodany z panelu i widoczny w strefie; SRV nie sprawdzany; usuwanie/zmiana takich rekordów — poprawka 3b508f6</t>
+          <t>2026-09-22 D1: components/hosting/DnsZoneSection.tsx — edytor strefy w zakladce Domeny huba uslugi (wybor domeny, DnsManager z onChanged); dns-manager.tsx typy A/AAAA/CNAME/MX/TXT/SRV/NS/CAA; API subscriptions/dto/hosting-dns.dto.ts (whitelista typow, wzorzec nazwy, zakaz znakow sterujacych, TTL 60-86400) + assertDomainOnSubscription przy odczycie/dodaniu/usunieciu; test hosting-dns-dto.spec.ts; D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu 13:00 (panel klienta): CAA 0 issue "letsencrypt.org" dodany z panelu i widoczny w strefie; SRV nie sprawdzany; usuwanie/zmiana takich rekordów — poprawka 3b508f6; D3 t1 29.09 (panel klienta, d3.hvln.pl): CAA dodany wcześniej; SRV _sip._tcp „10 5 5060 mail.d3.hvln.pl.” dodany i usunięty z panelu (wartość ze spacjami, bez duplikatu), licznik 15→16→15</t>
         </is>
       </c>
       <c r="M48" s="11" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="N48" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O48" s="11" t="inlineStr">
@@ -6075,12 +6075,12 @@
       </c>
       <c r="K68" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L68" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts</t>
+          <t>2026-09-23 D1: hosting-restore.service.ts takeSafetyBackup — odtwarzanie rusza dopiero, gdy na liście kopii pojawi się NOWE archiwum (do 15 min), inaczej FAILED „dane nie zostały zmienione”; nieczytelna lista = odmowa; test hosting-restore.safety.spec.ts; D3 t1 29.09 (panel klienta, d3.hvln.pl): „Przywróć” z backup-Sep-29-2026-3 (pliki + bazy, kopia bezpieczeństwa zaznaczona) → najpierw powstała nowa kopia backup-Sep-29-2026-4, dopiero potem DA dostał restore; strona po odtworzeniu 200</t>
         </is>
       </c>
       <c r="M68" s="11" t="inlineStr">
@@ -6090,7 +6090,7 @@
       </c>
       <c r="N68" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O68" s="11" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="L71" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts</t>
+          <t>2026-09-23 D1: node-staging-sync.sh TO_LIVE — eksport bazy LIVE i niepusty plik kopii są twardą bramką (die) przed db import; retencja po udanej kopii; strażnik src/test/staging-publikacja-z-kopia.spec.ts; D3 t1 29.09 (panel klienta, d3.hvln.pl): pierwsze „Utwórz kopię roboczą” → błąd: DA 1.710 zakłada subdomenę jako domains/staging.&lt;domena&gt;/public_html, skrypt szukał public_html/staging; poprawka d93c86e (plus sprzątanie bazy stg z nieudanej próby) czeka na push</t>
         </is>
       </c>
       <c r="M71" s="11" t="inlineStr">
@@ -9179,12 +9179,12 @@
       </c>
       <c r="K108" s="10" t="inlineStr">
         <is>
-          <t>b.d.</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L108" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu; D3 t1 29.09 (panel klienta, d3.hvln.pl): LiteSpeed Enterprise (Server: LiteSpeed), CacheRoot z profilu [OK], strona główna WordPressa z x-litespeed-cache: hit</t>
         </is>
       </c>
       <c r="M108" s="11" t="inlineStr">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="N108" s="11" t="inlineStr">
         <is>
-          <t>Stan zweryfikowany na produkcji z timestampem (poziom D3), wynik zapisany w repo.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O108" s="11" t="inlineStr">
@@ -9258,7 +9258,7 @@
       </c>
       <c r="L109" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu</t>
+          <t>poza kodem panelu; D3 t1 29.09 (panel klienta, d3.hvln.pl): brak alt-svc, połączenia po h2 — firewalld nie przepuszczał UDP 443; poprawka 68c7e95 (profil + hardening) czeka na push i profil</t>
         </is>
       </c>
       <c r="M109" s="11" t="inlineStr">
@@ -11317,7 +11317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11393,7 +11393,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
@@ -11418,7 +11418,7 @@
       </c>
       <c r="F2" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP per katalog</t>
+          <t>Aplikacje Node.js</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
@@ -11432,7 +11432,7 @@
         </is>
       </c>
       <c r="I2" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J2" s="10" t="inlineStr">
         <is>
@@ -11441,14 +11441,14 @@
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-htaccess.sh (HT_DIR, HT_PHP); htaccess.service.ts phpKatalogu; services.controller.ts :id/hosting-htaccess/php-dir; client-panel PhpKatalogPanel (widok strony → PHP i serwer); test htaccess.service.spec.ts</t>
+          <t>ops/scripts/node-app-selector.sh (zadanie APP_SELECTOR); subscriptions/app-selector.service.ts; services.controller.ts :id/hosting-apps; client-panel components/hosting/AplikacjeSelektorPanel.tsx (zakładka Aplikacje); node-hosting-profile.sh (alt-nodejs/alt-python + selektory włączone); testy test/aplikacje-selektor.spec.ts, app-selector.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
@@ -11473,7 +11473,7 @@
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>Włączanie/wyłączanie rozszerzeń PHP</t>
+          <t>Aplikacje Python</t>
         </is>
       </c>
       <c r="G3" s="10" t="inlineStr">
@@ -11483,11 +11483,11 @@
       </c>
       <c r="H3" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I3" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J3" s="10" t="inlineStr">
         <is>
@@ -11496,14 +11496,14 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-php-info.sh (selektor); ops/scripts/node-php-apply.sh (PHP_EXT_ENABLE/DISABLE); subscriptions/php.service.ts setExtensionsForSubscription; POST /services/:id/hosting-php/extensions; client PhpInfoPanel.tsx; testy php.service.spec.ts, php-info.service.spec.ts</t>
+          <t>ops/scripts/node-app-selector.sh (zadanie APP_SELECTOR); subscriptions/app-selector.service.ts; services.controller.ts :id/hosting-apps; client-panel components/hosting/AplikacjeSelektorPanel.tsx (zakładka Aplikacje); node-hosting-profile.sh (alt-nodejs/alt-python + selektory włączone); testy test/aplikacje-selektor.spec.ts, app-selector.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-19</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -11528,7 +11528,7 @@
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Aplikacje Node.js</t>
+          <t>Kreator stron WWW</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
@@ -11542,23 +11542,23 @@
         </is>
       </c>
       <c r="I4" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-app-selector.sh (zadanie APP_SELECTOR); subscriptions/app-selector.service.ts; services.controller.ts :id/hosting-apps; client-panel components/hosting/AplikacjeSelektorPanel.tsx (zakładka Aplikacje); node-hosting-profile.sh (alt-nodejs/alt-python + selektory włączone); testy test/aplikacje-selektor.spec.ts, app-selector.service.spec.ts</t>
+          <t>SiteBuilderTab.tsx usunięty 2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>C-17</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -11583,21 +11583,21 @@
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Aplikacje Python</t>
+          <t>Konto FTP — usunięcie</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I5" s="10" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
@@ -11606,14 +11606,14 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-app-selector.sh (zadanie APP_SELECTOR); subscriptions/app-selector.service.ts; services.controller.ts :id/hosting-apps; client-panel components/hosting/AplikacjeSelektorPanel.tsx (zakładka Aplikacje); node-hosting-profile.sh (alt-nodejs/alt-python + selektory włączone); testy test/aplikacje-selektor.spec.ts, app-selector.service.spec.ts</t>
+          <t>services.controller.ts:415; D3 t1 (d3.hvln.pl) 29.09: DA 1.710 zwraca listę FTP jako login@domena=ścieżka (nie user0/path0) — dodatkowe konta niewidoczne w panelu, więc bez usuwania i zmiany hasła; poprawka bcce42d czeka na wdrożenie; D3 na koncie dodatkowym</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>B-19</t>
+          <t>C-27</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -11638,12 +11638,12 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Kreator stron WWW</t>
+          <t>Webhook deploy z GitHuba</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>C — Pliki, FTP, SSH, Git</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -11656,19 +11656,19 @@
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>SiteBuilderTab.tsx usunięty 2026-09-25</t>
+          <t>subscriptions/git-webhook.controller.ts (POST /hooks/git/:token, bez logowania, limit), GitDeployService.utworzWebhook/usunWebhook/wyzwolWebhook (model GitWebhook: tylko skrót tokenu), :id/hosting-git-webhook(/delete), GitRepoPanel.tsx (adres pokazany raz, lista z datą ostatniego wywołania); test git-deploy.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>C-17</t>
+          <t>C-28</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -11693,7 +11693,7 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Konto FTP — usunięcie</t>
+          <t>Composer / narzędzia CLI przez SSH</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -11707,7 +11707,7 @@
         </is>
       </c>
       <c r="I7" s="10" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
@@ -11716,14 +11716,14 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:415; D3 t1 (d3.hvln.pl) 29.09: DA 1.710 zwraca listę FTP jako login@domena=ścieżka (nie user0/path0) — dodatkowe konta niewidoczne w panelu, więc bez usuwania i zmiany hasła; poprawka bcce42d czeka na wdrożenie; D3 na koncie dodatkowym</t>
+          <t>zależne od C-21</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>C-21</t>
+          <t>D-08</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -11748,21 +11748,21 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Dostęp SSH</t>
+          <t>Nadawanie uprawnień użytkownikowi bazy</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>D — Bazy danych</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I8" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
@@ -11771,14 +11771,14 @@
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-ssh-access.sh (zadanie SSH_ACCESS), subscriptions/ssh-access.service.ts, services.controller.ts :id/hosting-ssh(/keys), client-panel components/hosting/SshPanel.tsx (FTP → Dostęp SSH); test ssh-access.service.spec.ts; D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu (panel klienta): włączenie SSH z panelu → DA ssh=ON; logowania z zewnątrz nie sprawdziłem (brak ruchu TCP/22 ze środowiska testowego) — do potwierdzenia przez właściciela</t>
+          <t>ops/scripts/node-db-transfer.sh (privileges); db-transfer.service.ts zlecUprawnienia; DbUsers.tsx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>C-22</t>
+          <t>D-14</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -11803,21 +11803,21 @@
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Zarządzanie kluczami SSH konta hostingowego</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>D — Bazy danych</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I9" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
@@ -11826,24 +11826,24 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-ssh-access.sh (zadanie SSH_ACCESS), subscriptions/ssh-access.service.ts, services.controller.ts :id/hosting-ssh(/keys), client-panel components/hosting/SshPanel.tsx (FTP → Dostęp SSH); test ssh-access.service.spec.ts; D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu (panel klienta): klucz publiczny z panelu → blok Verris w ~/.ssh/authorized_keys; logowanie kluczem do potwierdzenia (jak C-21); D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu 13:00 (panel klienta): klucz testowy usunięty z panelu (blok Verris w authorized_keys aktualizowany)</t>
+          <t>ops/scripts/node-pgsql.sh (zadanie PGSQL, migracja 20260925210000); subscriptions/pgsql.service.ts; services.controller.ts :id/hosting-pgsql; client-panel PgsqlPanel (zakładka Bazy danych); node-hosting-profile.sh (PostgreSQL 16 z AppStream, localhost, scram-sha-256); test pgsql.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>C-25</t>
+          <t>D-16</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-02</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Wydajność: cache i skalowanie</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -11858,17 +11858,17 @@
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Klonowanie repozytorium Git z panelu</t>
+          <t>Memcached</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>D — Bazy danych</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I10" s="10" t="n">
@@ -11881,24 +11881,24 @@
       </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-git-deploy.sh (zadanie GIT_DEPLOY: klucz ed25519 ~/.ssh/verris_deploy, git clone --depth 50 z odłożeniem dotychczasowych plików, pull --ff-only, HEAD w wyniku; jako klient), subscriptions/git-deploy.service.ts, :id/hosting-git(/key|/clone|/pull), panel GitRepoPanel.tsx (Deploy (Git) → Repozytorium strony); test git-deploy.service.spec.ts</t>
+          <t>ops/scripts/node-memcached.sh (zadanie MEMCACHED_ACCESS, migracja 20260925201000); redis-access.service.ts (silnik memcached); services.controller.ts :id/hosting-memcached; client-panel RedisPanel silnik="memcached" (zakładka PHP i serwer); node-hosting-profile.sh (pakiet memcached, usługa TCP wyłączona)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>C-26</t>
+          <t>J-05</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-02</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Wydajność: cache i skalowanie</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -11913,47 +11913,47 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Deploy z repozytorium (pull na żądanie)</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-git-deploy.sh (zadanie GIT_DEPLOY: klucz ed25519 ~/.ssh/verris_deploy, git clone --depth 50 z odłożeniem dotychczasowych plików, pull --ff-only, HEAD w wyniku; jako klient), subscriptions/git-deploy.service.ts, :id/hosting-git(/key|/clone|/pull), panel GitRepoPanel.tsx (Deploy (Git) → Repozytorium strony); test git-deploy.service.spec.ts; harmonogram: services.controller.ts:717, directadmin.service.ts createDeployJob</t>
+          <t>na rynku PL płatny dodatek</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>C-27</t>
+          <t>J-07</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-02</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Wydajność: cache i skalowanie</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -11968,21 +11968,21 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Webhook deploy z GitHuba</t>
+          <t>Dedykowany adres IP</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I12" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
@@ -11991,24 +11991,24 @@
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/git-webhook.controller.ts (POST /hooks/git/:token, bez logowania, limit), GitDeployService.utworzWebhook/usunWebhook/wyzwolWebhook (model GitWebhook: tylko skrót tokenu), :id/hosting-git-webhook(/delete), GitRepoPanel.tsx (adres pokazany raz, lista z datą ostatniego wywołania); test git-deploy.service.spec.ts</t>
+          <t>addons — jako dodatek typu workorder</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>C-28</t>
+          <t>H-03</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Backup: granularność i retencja</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -12023,21 +12023,21 @@
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Composer / narzędzia CLI przez SSH</t>
+          <t>Konfigurowalna retencja kopii</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>C — Pliki, FTP, SSH, Git</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I13" s="10" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
@@ -12046,24 +12046,24 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>zależne od C-21</t>
+          <t>services.controller.ts:926; D3 t1 (d3.hvln.pl) 29.09: DA 1.710 robi .tar.zst z datą epoch — retencja pomijała .tar.zst, a przy dacie NaN sortowała po nazwie (Sep &gt; Oct = kasowanie najnowszych); poprawka 8f7b043 + test; retest po wdrożeniu</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>D-08</t>
+          <t>H-04</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Backup: granularność i retencja</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -12078,21 +12078,21 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Nadawanie uprawnień użytkownikowi bazy</t>
+          <t>Retencja co najmniej 28 dni w cenie</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>D — Bazy danych</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I14" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J14" s="10" t="inlineStr">
         <is>
@@ -12101,24 +12101,24 @@
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-db-transfer.sh (privileges); db-transfer.service.ts zlecUprawnienia; DbUsers.tsx</t>
+          <t>off-site: 30 dni (node-offsite-backup.sh:101); libs/contracts/src/kopie.ts; hosting-offsite-panel.tsx; test kopie-30-dni.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>D-13</t>
+          <t>H-14</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Backup: granularność i retencja</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -12133,21 +12133,21 @@
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Kopia bazy na żądanie</t>
+          <t>Kopia off-site (poza węzłem)</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>D — Bazy danych</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I15" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J15" s="10" t="inlineStr">
         <is>
@@ -12156,24 +12156,24 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>D-12: DbTransferPanel „Eksportuj bazę” (zadanie DB_TRANSFER export → ~/verris-bazy/&lt;baza&gt;-&lt;czas&gt;.sql.gz, pobranie z panelu)</t>
+          <t>ops/scripts/node-offsite-backup.sh:93-97 (rclone crypt → S3); D3 t1 (d3.hvln.pl) 29.09: nocny przebieg 03:54 accounts=2, archiwum konta d3 widoczne w panelu (D4 — test odtworzenia — nadal otwarte)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>D-14</t>
+          <t>H-16</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Runtime, pliki i diagnostyka</t>
+          <t>Backup: granularność i retencja</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -12188,17 +12188,17 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>ODTWORZENIE KONTA NA INNY WĘZEŁ</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>D — Bazy danych</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I16" s="10" t="n">
@@ -12211,24 +12211,24 @@
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-pgsql.sh (zadanie PGSQL, migracja 20260925210000); subscriptions/pgsql.service.ts; services.controller.ts :id/hosting-pgsql; client-panel PgsqlPanel (zakładka Bazy danych); node-hosting-profile.sh (PostgreSQL 16 z AppStream, localhost, scram-sha-256); test pgsql.service.spec.ts</t>
+          <t>subscriptions/odtworzenie-na-wezle.service.ts; admin subskrypcja → odtworzenie-na-wezle-panel.tsx; ops/scripts/node-account-restore.sh (OFR_MODE=restore, OFR_SOURCE_PREFIX, OFR_IP); node-tasks.service.ts completeTaskFromNode (przepięcie konta); test odtworzenie-na-wezle.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>D-16</t>
+          <t>H-18</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Wydajność: cache i skalowanie</t>
+          <t>Backup: granularność i retencja</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -12243,21 +12243,21 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Memcached</t>
+          <t>Odtworzenie konta przez operatora z panelu</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>D — Bazy danych</t>
+          <t>H — Backup i odtwarzanie</t>
         </is>
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I17" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J17" s="10" t="inlineStr">
         <is>
@@ -12266,24 +12266,24 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-memcached.sh (zadanie MEMCACHED_ACCESS, migracja 20260925201000); redis-access.service.ts (silnik memcached); services.controller.ts :id/hosting-memcached; client-panel RedisPanel silnik="memcached" (zakładka PHP i serwer); node-hosting-profile.sh (pakiet memcached, usługa TCP wyłączona)</t>
+          <t>admin: Subskrypcje → usługa → „Odtworzenie konta z kopii” (restore-panel.tsx): lista kopii (nowe GET admin/subscriptions/:id/hosting-backups), zakres, kopia bezpieczeństwa domyślnie, potwierdzenie domeną, status ostatniego odtworzenia → POST admin/subscriptions/:id/hosting-restore (SUBSCRIPTIONS_MANAGE); D3 t1 (d3.hvln.pl) 29.09 FAIL: panel operatora „Na koncie nie ma kopii do odtworzenia” mimo archiwum w /backups — ten sam parser co H-05; poprawka 8f7b043 czeka na wdrożenie; retest z odtworzeniem</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>J-05</t>
+          <t>M-33</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Wydajność: cache i skalowanie</t>
+          <t>Rozliczenia: dokończenie</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -12298,12 +12298,12 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>Dodatki płatne (IP, wsparcie priorytetowe)</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>M — Rozliczenia</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
@@ -12312,33 +12312,33 @@
         </is>
       </c>
       <c r="I18" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>na rynku PL płatny dodatek</t>
+          <t>addon.service.ts:120 — 2 z 3 to workorder do BOK</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>J-06</t>
+          <t>N-21</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Wydajność: cache i skalowanie</t>
+          <t>Wsparcie i ops: kolejka abuse</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -12353,47 +12353,47 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>Optymalizacja obrazów</t>
+          <t>Wsparcie telefoniczne</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I19" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J19" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-image-optimize.sh (zadanie IMAGE_OPTIMIZE, migracja 20260925211000); subscriptions/obrazy.service.ts; services.controller.ts :id/hosting-images; client-panel ObrazyPanel (widok strony → Pliki); profil węzła: jpegoptim, optipng (EPEL); test obrazy.service.spec.ts</t>
+          <t>poza produktem</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>J-07</t>
+          <t>PROD-01</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Wydajność: cache i skalowanie</t>
+          <t>Wsparcie i ops: kolejka abuse</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -12408,21 +12408,21 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>Dedykowany adres IP</t>
+          <t>Instalator węzła bez udziału administratora</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I20" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J20" s="10" t="inlineStr">
         <is>
@@ -12431,29 +12431,29 @@
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>addons — jako dodatek typu workorder</t>
+          <t>docs/archiwum/zadania/PROD-01-instalator-wezla-bez-czlowieka.md; stan: bootstrap v2 + kreator węzła (Q-14) — kroki CloudLinux/DA/LiteSpeed nadal ręczne</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>H-03</t>
+          <t>I-04</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>WordPress Toolkit</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -12463,12 +12463,12 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>Konfigurowalna retencja kopii</t>
+          <t>Automatyczne aktualizacje WordPressa</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
@@ -12477,7 +12477,7 @@
         </is>
       </c>
       <c r="I21" s="10" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J21" s="10" t="inlineStr">
         <is>
@@ -12486,29 +12486,29 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:926; D3 t1 (d3.hvln.pl) 29.09: DA 1.710 robi .tar.zst z datą epoch — retencja pomijała .tar.zst, a przy dacie NaN sortowała po nazwie (Sep &gt; Oct = kasowanie najnowszych); poprawka 8f7b043 + test; retest po wdrożeniu</t>
+          <t>ops/scripts/node-wp-update.sh (zadanie WP_UPDATE, check/update jako klient), subscriptions/wp-update.service.ts, wp-auto-update.scheduler.ts (codziennie 3:20), model WpAutoUpdate, services.controller.ts :id/hosting-wp-updates(/check|/run|/auto), client-panel components/hosting/WpUpdatesPanel.tsx (strona → WordPress); test wp-update.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>H-04</t>
+          <t>I-05</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>WordPress Toolkit</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -12518,17 +12518,17 @@
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>Retencja co najmniej 28 dni w cenie</t>
+          <t>Aktualizacje wtyczek i motywów z panelu</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I22" s="10" t="n">
@@ -12541,29 +12541,29 @@
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>off-site: 30 dni (node-offsite-backup.sh:101); libs/contracts/src/kopie.ts; hosting-offsite-panel.tsx; test kopie-30-dni.spec.ts</t>
+          <t>ops/scripts/node-wp-update.sh (zadanie WP_UPDATE, check/update jako klient), subscriptions/wp-update.service.ts, wp-auto-update.scheduler.ts (codziennie 3:20), model WpAutoUpdate, services.controller.ts :id/hosting-wp-updates(/check|/run|/auto), client-panel components/hosting/WpUpdatesPanel.tsx (strona → WordPress); test wp-update.service.spec.ts; D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu (panel klienta): Sprawdź aktualizacje → rdzeń 7.1.2, 3 wtyczki, 4 motywy, wszystko aktualne (aktualizacji do wykonania nie było)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>H-10</t>
+          <t>I-07</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>WordPress Toolkit</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -12573,21 +12573,21 @@
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>Odtworzenie pojedynczego pliku</t>
+          <t>Skanowanie podatności WordPressa</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I23" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J23" s="10" t="inlineStr">
         <is>
@@ -12596,29 +12596,29 @@
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-file-restore.sh (zadanie FILE_RESTORE, list/extract jako klient), subscriptions/file-restore.service.ts, services.controller.ts :id/hosting-file-restore(/list|/extract), client-panel components/hosting/ArchiveBrowser.tsx (Kopie → Pliki); test file-restore.service.spec.ts</t>
+          <t>subscriptions/wp-podatnosci.service.ts (Wordfence Scanner Feed v3, cron 05:40, tabela WpPodatnosc, migracja 20260925190000); wp-update.service.ts opis/przeglad → podatnosci; client-panel WpUpdatesPanel/WpOverviewPanel; test wp-podatnosci.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>H-11</t>
+          <t>I-13</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>WordPress Toolkit</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
@@ -12628,17 +12628,17 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Podgląd zawartości archiwum przed odtworzeniem</t>
+          <t>Klonowanie strony między domenami</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I24" s="10" t="n">
@@ -12651,29 +12651,29 @@
       </c>
       <c r="K24" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-file-restore.sh (zadanie FILE_RESTORE, list/extract jako klient), subscriptions/file-restore.service.ts, services.controller.ts :id/hosting-file-restore(/list|/extract), client-panel components/hosting/ArchiveBrowser.tsx (Kopie → Pliki); test file-restore.service.spec.ts; D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu 13:00 (panel klienta): FAIL: podgląd katalogu „domains” w kopii → „Operacja nie powiodła się” (SIGPIPE tar przy &gt;2000 wpisach + pipefail); poprawka befd7f4 czeka na push</t>
+          <t>ops/scripts/node-site-clone.sh (zadanie SITE_CLONE: cp -a jako klient, cel odkładany obok z unikalną nazwą, WordPress: zrzut → nowa baza, wp-config.php kopii, search-replace adresów), subscriptions/site-clone.service.ts (nowa baza w DA dla WP), :id/hosting-site-clone, panel SiteClonePanel.tsx (strona → Pliki → Kopia strony na inną domenę); test site-clone.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>H-13</t>
+          <t>I-16</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>WordPress Toolkit</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
@@ -12683,12 +12683,12 @@
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Pobranie archiwum kopii lokalnie</t>
+          <t>WP-CLI</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>I — Aplikacje i WordPress</t>
         </is>
       </c>
       <c r="H25" s="10" t="inlineStr">
@@ -12706,29 +12706,29 @@
       </c>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>files/files.service.ts downloadStream; files.controller.ts GET download-stream; client app/api/services/[id]/files/download/route.ts; BackupsTab.tsx „Pobierz”; test files.service.spec.ts</t>
+          <t>używane wewnętrznie przy WP_INSTALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>H-14</t>
+          <t>A-08</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
@@ -12738,52 +12738,52 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Kopia off-site (poza węzłem)</t>
+          <t>Rejestracja domeny z panelu</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I26" s="10" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J26" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-offsite-backup.sh:93-97 (rclone crypt → S3); D3 t1 (d3.hvln.pl) 29.09: nocny przebieg 03:54 accounts=2, archiwum konta d3 widoczne w panelu (D4 — test odtworzenia — nadal otwarte)</t>
+          <t>domains.controller.ts:118</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>H-16</t>
+          <t>A-09</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
@@ -12793,12 +12793,12 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>ODTWORZENIE KONTA NA INNY WĘZEŁ</t>
+          <t>Transfer domeny (kod authinfo)</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H27" s="10" t="inlineStr">
@@ -12807,38 +12807,38 @@
         </is>
       </c>
       <c r="I27" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/odtworzenie-na-wezle.service.ts; admin subskrypcja → odtworzenie-na-wezle-panel.tsx; ops/scripts/node-account-restore.sh (OFR_MODE=restore, OFR_SOURCE_PREFIX, OFR_IP); node-tasks.service.ts completeTaskFromNode (przepięcie konta); test odtworzenie-na-wezle.service.spec.ts</t>
+          <t>POST /domains/:id/registrar/authcode (A-09, tylko właściciel konta, 5/h, audyt DOMAIN_AUTHCODE_REVEALED bez kodu) → OpenProvider GET /v1/domains/{id}/authcode; panel: Domeny → domena → „Transfer i abonent” → Pokaż kod; transfer PRZYCHODZĄCY: formularz z danymi abonenta i oświadczeniem; test domains/abonent-domeny.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>H-18</t>
+          <t>A-10</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Backup: granularność i retencja</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
@@ -12848,17 +12848,17 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>Odtworzenie konta przez operatora z panelu</t>
+          <t>Odnowienie domeny przez klienta</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>H — Backup i odtwarzanie</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I28" s="10" t="n">
@@ -12866,34 +12866,34 @@
       </c>
       <c r="J28" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>admin: Subskrypcje → usługa → „Odtworzenie konta z kopii” (restore-panel.tsx): lista kopii (nowe GET admin/subscriptions/:id/hosting-backups), zakres, kopia bezpieczeństwa domyślnie, potwierdzenie domeną, status ostatniego odtworzenia → POST admin/subscriptions/:id/hosting-restore (SUBSCRIPTIONS_MANAGE); D3 t1 (d3.hvln.pl) 29.09 FAIL: panel operatora „Na koncie nie ma kopii do odtworzenia” mimo archiwum w /backups — ten sam parser co H-05; poprawka 8f7b043 czeka na wdrożenie; retest z odtworzeniem</t>
+          <t>panel: Domeny → domena → „Odnowienie domeny” (domain-renew-box.tsx: okres → cena z nowego POST domains/:id/registrar/renew-quote → potwierdzenie → POST domains/:id/registrar/renew, obciążenie portfela, zwrot przy błędzie rejestratora); liczba lat walidowana 1–10 (wcześniej body bez walidacji)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>M-33</t>
+          <t>A-12</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>E-14</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Rozliczenia: dokończenie</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
@@ -12903,52 +12903,52 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Dodatki płatne (IP, wsparcie priorytetowe)</t>
+          <t>Cennik rejestracji na 1–10 lat</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>M — Rozliczenia</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I29" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>addon.service.ts:120 — 2 z 3 to workorder do BOK</t>
+          <t>POST domains/registrar/quote-periods (domain-registrar.service.ts quotePeriods — ceny brutto dla 1, 2, 3, 5 i 10 lat + cena odnowienia/rok) → kreator zakupu: krok „Okres” z ceną każdego wariantu (domain-purchase-wizard.tsx YEAR_OPTIONS)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>N-21</t>
+          <t>A-13</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Wsparcie i ops: kolejka abuse</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -12958,52 +12958,52 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>Wsparcie telefoniczne</t>
+          <t>Zmiana danych abonenta domeny</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I30" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>poza produktem</t>
+          <t>GET/PUT /domains/:id/registrar/registrant (tylko właściciel konta) → OpenProvider /v1/customers/{handle}; rejestracja i transfer zakładają uchwyt klienta (POST /v1/customers) przed obciążeniem portfela; panel: kreator zakupu, zamówienie hostingu z domeną, transfer, strona domeny; test domains/abonent-domeny.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>PROD-01</t>
+          <t>A-14</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>E-15</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Wsparcie i ops: kolejka abuse</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -13013,47 +13013,47 @@
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>Instalator węzła bez udziału administratora</t>
+          <t>Ukrycie danych WHOIS / domain privacy</t>
         </is>
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H31" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I31" s="10" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="J31" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>docs/archiwum/zadania/PROD-01-instalator-wezla-bez-czlowieka.md; stan: bootstrap v2 + kreator węzła (Q-14) — kroki CloudLinux/DA/LiteSpeed nadal ręczne</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-24: po starcie — u OpenProvider ukrycie WHOIS to usługa płatna per domena, a dla osób fizycznych z .pl rejestr i tak nie publikuje danych; wracamy przy sprzedaży domen, gdy znane będą koszty.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>A-15</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>E-03</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>WordPress Toolkit</t>
+          <t>Domeny jako produkt</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -13068,47 +13068,47 @@
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>Automatyczne aktualizacje WordPressa</t>
+          <t>Blokada transferu domeny (transfer lock)</t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I32" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J32" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-wp-update.sh (zadanie WP_UPDATE, check/update jako klient), subscriptions/wp-update.service.ts, wp-auto-update.scheduler.ts (codziennie 3:20), model WpAutoUpdate, services.controller.ts :id/hosting-wp-updates(/check|/run|/auto), client-panel components/hosting/WpUpdatesPanel.tsx (strona → WordPress); test wp-update.service.spec.ts</t>
+          <t>POST /domains/:id/registrar/lock → OpenProvider PUT /v1/domains/{id} {is_locked}; stan w Domain.transferLock + audyt DOMAIN_TRANSFER_LOCKED/UNLOCKED; panel: strona domeny „Transfer i abonent”; test domains/abonent-domeny.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>I-05</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>E-03</t>
+          <t>E-05</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>WordPress Toolkit</t>
+          <t>Katalog aplikacji</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -13118,12 +13118,12 @@
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Aktualizacje wtyczek i motywów z panelu</t>
+          <t>Autoinstalator aplikacji</t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
@@ -13133,7 +13133,7 @@
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I33" s="10" t="n">
@@ -13146,24 +13146,24 @@
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-wp-update.sh (zadanie WP_UPDATE, check/update jako klient), subscriptions/wp-update.service.ts, wp-auto-update.scheduler.ts (codziennie 3:20), model WpAutoUpdate, services.controller.ts :id/hosting-wp-updates(/check|/run|/auto), client-panel components/hosting/WpUpdatesPanel.tsx (strona → WordPress); test wp-update.service.spec.ts; D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu (panel klienta): Sprawdź aktualizacje → rdzeń 7.1.2, 3 wtyczki, 4 motywy, wszystko aktualne (aktualizacji do wykonania nie było)</t>
+          <t>app-install.service.ts CATALOG (Nextcloud, PrestaShop, Joomla, MediaWiki); ops/scripts/node-app-install.sh; test test/instalator-aplikacji-katalog.spec.ts; D3 t1 28.09: WordPress 1-click na t1 — WP_INSTALL zakończone (kolejka ~3 min), strona po zmianie NS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>I-07</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>E-03</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>WordPress Toolkit</t>
+          <t>Poczta: filtry, kalendarz, limity</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
@@ -13173,17 +13173,17 @@
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>Skanowanie podatności WordPressa</t>
+          <t>Reguły filtrowania poczty (Sieve)</t>
         </is>
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="H34" s="10" t="inlineStr">
@@ -13192,7 +13192,7 @@
         </is>
       </c>
       <c r="I34" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
@@ -13201,24 +13201,24 @@
       </c>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/wp-podatnosci.service.ts (Wordfence Scanner Feed v3, cron 05:40, tabela WpPodatnosc, migracja 20260925190000); wp-update.service.ts opis/przeglad → podatnosci; client-panel WpUpdatesPanel/WpOverviewPanel; test wp-podatnosci.service.spec.ts</t>
+          <t>ops/scripts/node-hosting-profile.sh (da build dovecot_pigeonhole); client-panel MailTab.tsx (Filtry w webmailu); D3 t1 29.09: `da build dovecot_pigeonhole` w DA 1.710 niewspierane („use da build dovecot”) — profil poprawiony w 98e6f24 (pigeonhole=yes + da build dovecot), czeka na profil</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>I-13</t>
+          <t>E-21</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>E-03</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>WordPress Toolkit</t>
+          <t>Poczta: filtry, kalendarz, limity</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
@@ -13228,17 +13228,17 @@
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>Klonowanie strony między domenami</t>
+          <t>Samodzielny import skrzynek przez IMAP</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="H35" s="10" t="inlineStr">
@@ -13247,7 +13247,7 @@
         </is>
       </c>
       <c r="I35" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
@@ -13256,24 +13256,24 @@
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-site-clone.sh (zadanie SITE_CLONE: cp -a jako klient, cel odkładany obok z unikalną nazwą, WordPress: zrzut → nowa baza, wp-config.php kopii, search-replace adresów), subscriptions/site-clone.service.ts (nowa baza w DA dla WP), :id/hosting-site-clone, panel SiteClonePanel.tsx (strona → Pliki → Kopia strony na inną domenę); test site-clone.service.spec.ts</t>
+          <t>subscriptions/migration-orchestrator.service.ts createBundle (IMAP_SYNC, imapsync w node-migration-worker.sh); migrations/migration-wizard.tsx tryb tylkoPoczta; MailTab.tsx „Przenieś pocztę z innego serwera”; test migration-orchestrator.service.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>I-16</t>
+          <t>E-23</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>E-03</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>WordPress Toolkit</t>
+          <t>Poczta: filtry, kalendarz, limity</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
@@ -13283,26 +13283,26 @@
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>WP-CLI</t>
+          <t>Kalendarz i kontakty (CalDAV/CardDAV)</t>
         </is>
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I36" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
@@ -13311,24 +13311,24 @@
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>używane wewnętrznie przy WP_INSTALL</t>
+          <t>node-hosting-profile.sh (Radicale 3.8.1 w venv, verris-radicale.service, verris-dav-backup); security-hardening-baseline.sh (5232/tcp); client-panel MailTab (adres i instrukcja); test kalendarz-kontakty.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>A-06</t>
+          <t>E-24</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Poczta: filtry, kalendarz, limity</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
@@ -13338,17 +13338,17 @@
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Zmiana document root domeny</t>
+          <t>2FA dla webmaila</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>E — Poczta</t>
         </is>
       </c>
       <c r="H37" s="10" t="inlineStr">
@@ -13357,58 +13357,58 @@
         </is>
       </c>
       <c r="I37" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>servers/docroot.ts; servers/directadmin.service.ts getHostingDocroot/setHostingDocroot; GET/POST /services/:id/hosting-docroot; client components/hosting/DocrootPanel.tsx; test servers/docroot.spec.ts; D3 t1 28.09: odczyt zawsze błąd — GET CMD_API_CUSTOM_HTTPD zwraca surową treść .cust_httpd → docroot.ts trescCustomHttpd; retest</t>
+          <t>cyber_Folks ma nawet 2FA dla IMAP/SMTP</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>A-08</t>
+          <t>G-08</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Bezpieczeństwo jako funkcja</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>Rejestracja domeny z panelu</t>
+          <t>Sprzedaż certyfikatów DV/OV/EV</t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I38" s="10" t="n">
@@ -13416,104 +13416,104 @@
       </c>
       <c r="J38" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:118</t>
+          <t>wszystkie 5 hostingów PL to sprzedaje</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>A-09</t>
+          <t>G-12</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Bezpieczeństwo jako funkcja</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>Transfer domeny (kod authinfo)</t>
+          <t>Czyszczenie zainfekowanych plików</t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I39" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>POST /domains/:id/registrar/authcode (A-09, tylko właściciel konta, 5/h, audyt DOMAIN_AUTHCODE_REVEALED bez kodu) → OpenProvider GET /v1/domains/{id}/authcode; panel: Domeny → domena → „Transfer i abonent” → Pokaż kod; transfer PRZYCHODZĄCY: formularz z danymi abonenta i oświadczeniem; test domains/abonent-domeny.spec.ts</t>
+          <t xml:space="preserve"> | DECYZJA WŁAŚCICIELA 2026-09-25: na start darmowy ImunifyAV (wykrywanie, G-11), czyszczenie robi obsługa na zgłoszenie; płatny ImunifyAV+ po starcie (wybór „po starcie”).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>A-10</t>
+          <t>G-21</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Bezpieczeństwo jako funkcja</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>Odnowienie domeny przez klienta</t>
+          <t>Anty-DDoS</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="H40" s="10" t="inlineStr">
@@ -13522,53 +13522,53 @@
         </is>
       </c>
       <c r="I40" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J40" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K40" s="11" t="inlineStr">
         <is>
-          <t>panel: Domeny → domena → „Odnowienie domeny” (domain-renew-box.tsx: okres → cena z nowego POST domains/:id/registrar/renew-quote → potwierdzenie → POST domains/:id/registrar/renew, obciążenie portfela, zwrot przy błędzie rejestratora); liczba lat walidowana 1–10 (wcześniej body bez walidacji)</t>
+          <t>ops/docs/DDOS.md; Hetzner DDoS Protection (L3/L4, w cenie); RateLimitGuard + Turnstile (L7 panel/API); LiteSpeed Per-Client Throttling (węzeł, onboarding)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>A-12</t>
+          <t>O-05</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-07</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Reseller jako produkt</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Cennik rejestracji na 1–10 lat</t>
+          <t>Reseller — przegląd klientów</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>O — Multi-user i reseller</t>
         </is>
       </c>
       <c r="H41" s="10" t="inlineStr">
@@ -13577,58 +13577,58 @@
         </is>
       </c>
       <c r="I41" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>POST domains/registrar/quote-periods (domain-registrar.service.ts quotePeriods — ceny brutto dla 1, 2, 3, 5 i 10 lat + cena odnowienia/rok) → kreator zakupu: krok „Okres” z ceną każdego wariantu (domain-purchase-wizard.tsx YEAR_OPTIONS)</t>
+          <t>reseller-klienci.service.ts + reseller.controller.ts (5 tras), reseller-klient.tsx; reseller-klienci.int-spec.ts (6 testów na PostgreSQL)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>A-13</t>
+          <t>O-07</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-07</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Reseller jako produkt</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>Zmiana danych abonenta domeny</t>
+          <t>Reseller — ustawianie własnej marży</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>O — Multi-user i reseller</t>
         </is>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I42" s="10" t="n">
@@ -13636,144 +13636,144 @@
       </c>
       <c r="J42" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K42" s="11" t="inlineStr">
         <is>
-          <t>GET/PUT /domains/:id/registrar/registrant (tylko właściciel konta) → OpenProvider /v1/customers/{handle}; rejestracja i transfer zakładają uchwyt klienta (POST /v1/customers) przed obciążeniem portfela; panel: kreator zakupu, zamówienie hostingu z domeną, transfer, strona domeny; test domains/abonent-domeny.spec.ts</t>
+          <t>reseller.controller.ts POST me/markup → reseller.service.ts setMarkup (0–300%, audyt RESELLER_MARKUP_CHANGED); reseller-client.tsx „Twój narzut”; test reseller.apply.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>A-14</t>
+          <t>P-12</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-08</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Dostępność i zgodność w produkcie</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>Ukrycie danych WHOIS / domain privacy</t>
+          <t>Dostępność panelu wg WCAG 2.1 AA (EAA)</t>
         </is>
       </c>
       <c r="G43" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="H43" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I43" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-24: po starcie — u OpenProvider ukrycie WHOIS to usługa płatna per domena, a dla osób fizycznych z .pl rejestr i tak nie publikuje danych; wracamy przy sprzedaży domen, gdy znane będą koszty.</t>
+          <t>eslint.config.mjs w 4 aplikacjach: jsx-a11y recommended jako błędy (34 reguły); 76 → 0 znalezisk (client 52, admin 17, staff 6, www 1); client-panel/src/lib/kontrast-tokenow.spec.ts; ops/qa/a11y-nazwy-kontrolek.js</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>A-15</t>
+          <t>P-14</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-08</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Domeny jako produkt</t>
+          <t>Dostępność i zgodność w produkcie</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>Blokada transferu domeny (transfer lock)</t>
+          <t>Certyfikacja ISO 27001</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I44" s="10" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J44" s="10" t="inlineStr">
         <is>
-          <t>FLAGA</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K44" s="11" t="inlineStr">
         <is>
-          <t>POST /domains/:id/registrar/lock → OpenProvider PUT /v1/domains/{id} {is_locked}; stan w Domain.transferLock + audyt DOMAIN_TRANSFER_LOCKED/UNLOCKED; panel: strona domeny „Transfer i abonent”; test domains/abonent-domeny.spec.ts</t>
+          <t>home.pl i nazwa.pl mają — element przetargowy w B2B</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>F-12</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>E-05</t>
+          <t>E-11</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Katalog aplikacji</t>
+          <t>DNS: DNSSEC i zarządzanie strefą</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
@@ -13783,52 +13783,52 @@
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>Autoinstalator aplikacji</t>
+          <t>Anycast DNS</t>
         </is>
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>I — Aplikacje i WordPress</t>
+          <t>F — DNS</t>
         </is>
       </c>
       <c r="H45" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I45" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="K45" s="11" t="inlineStr">
         <is>
-          <t>app-install.service.ts CATALOG (Nextcloud, PrestaShop, Joomla, MediaWiki); ops/scripts/node-app-install.sh; test test/instalator-aplikacji-katalog.spec.ts; D3 t1 28.09: WordPress 1-click na t1 — WP_INSTALL zakończone (kolejka ~3 min), strona po zmianie NS</t>
+          <t>tylko nazwa.pl na rynku PL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>L-08</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Automatyzacja: API zapisu i webhooki</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E46" s="10" t="inlineStr">
@@ -13838,12 +13838,12 @@
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>Reguły filtrowania poczty (Sieve)</t>
+          <t>Publiczne API — zapis</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>L — Automatyzacja</t>
         </is>
       </c>
       <c r="H46" s="10" t="inlineStr">
@@ -13852,7 +13852,7 @@
         </is>
       </c>
       <c r="I46" s="10" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J46" s="10" t="inlineStr">
         <is>
@@ -13861,29 +13861,29 @@
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/node-hosting-profile.sh (da build dovecot_pigeonhole); client-panel MailTab.tsx (Filtry w webmailu)</t>
+          <t>subscriptions/public-api-write.controller.ts (api/v1/services/:id/dns GET/POST, /dns/delete, /deploy GET/POST; zakresy dns:read, dns:write, deploy:write w api-scopes.ts; te same serwisy i walidacja co panel), opis w panelu api-tokens-client.tsx; test public-api-write.controller.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>E-21</t>
+          <t>L-11</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Automatyzacja: API zapisu i webhooki</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
@@ -13893,12 +13893,12 @@
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
-          <t>Samodzielny import skrzynek przez IMAP</t>
+          <t>Asystent AI w panelu</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>L — Automatyzacja</t>
         </is>
       </c>
       <c r="H47" s="10" t="inlineStr">
@@ -13911,34 +13911,34 @@
       </c>
       <c r="J47" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K47" s="11" t="inlineStr">
         <is>
-          <t>subscriptions/migration-orchestrator.service.ts createBundle (IMAP_SYNC, imapsync w node-migration-worker.sh); migrations/migration-wizard.tsx tryb tylkoPoczta; MailTab.tsx „Przenieś pocztę z innego serwera”; test migration-orchestrator.service.spec.ts</t>
+          <t>ai-modele.ts; ai-provider.service.ts; ai-ustawienia.admin.controller.ts; admin /settings/ai</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>E-23</t>
+          <t>L-12</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Automatyzacja: API zapisu i webhooki</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="E48" s="10" t="inlineStr">
@@ -13948,12 +13948,12 @@
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
-          <t>Kalendarz i kontakty (CalDAV/CardDAV)</t>
+          <t>Prognoza zużycia zasobów (AI)</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>L — Automatyzacja</t>
         </is>
       </c>
       <c r="H48" s="10" t="inlineStr">
@@ -13962,58 +13962,58 @@
         </is>
       </c>
       <c r="I48" s="10" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="J48" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K48" s="11" t="inlineStr">
         <is>
-          <t>node-hosting-profile.sh (Radicale 3.8.1 w venv, verris-radicale.service, verris-dav-backup); security-hardening-baseline.sh (5232/tcp); client-panel MailTab (adres i instrukcja); test kalendarz-kontakty.spec.ts</t>
+          <t>hosting-forecast-actions.ts:7; fallback ServiceForecastPanel.tsx:97</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>E-24</t>
+          <t>NODE-01</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Poczta: filtry, kalendarz, limity</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>2FA dla webmaila</t>
+          <t>Dwie niepołączone ścieżki dodania węzła w tym samym panelu</t>
         </is>
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
-          <t>E — Poczta</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="I49" s="10" t="n">
@@ -14021,104 +14021,104 @@
       </c>
       <c r="J49" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>cyber_Folks ma nawet 2FA dla IMAP/SMTP</t>
+          <t>node-wizard.tsx (krok „Instalacja (bootstrap v2)” z NodeBootstrapProgress), /nodes/init → przekierowanie, NODE_ONBOARD_RUNBOOK.md jedynym runbookiem</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>G-08</t>
+          <t>Q-05</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Bezpieczeństwo jako funkcja</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>Sprzedaż certyfikatów DV/OV/EV</t>
+          <t>E-mail marketing wbudowany w panel</t>
         </is>
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I50" s="10" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="J50" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>wszystkie 5 hostingów PL to sprzedaje</t>
+          <t>email-marketing.controller.ts:36,81,119,139</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>G-12</t>
+          <t>Q-06</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Bezpieczeństwo jako funkcja</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>Czyszczenie zainfekowanych plików</t>
+          <t>VPS / cloud w tym samym panelu</t>
         </is>
       </c>
       <c r="G51" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H51" s="10" t="inlineStr">
@@ -14127,168 +14127,160 @@
         </is>
       </c>
       <c r="I51" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J51" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>FLAGA</t>
         </is>
       </c>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | DECYZJA WŁAŚCICIELA 2026-09-25: na start darmowy ImunifyAV (wykrywanie, G-11), czyszczenie robi obsługa na zgłoszenie; płatny ImunifyAV+ po starcie (wybór „po starcie”).</t>
+          <t>vps.controller.ts:53,59,69; HETZNER_API_TOKEN</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>G-21</t>
+          <t>Q-07</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Bezpieczeństwo jako funkcja</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>Anty-DDoS</t>
+          <t>VPS — konsola / VNC</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I52" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J52" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K52" s="11" t="inlineStr">
-        <is>
-          <t>ops/docs/DDOS.md; Hetzner DDoS Protection (L3/L4, w cenie); RateLimitGuard + Turnstile (L7 panel/API); LiteSpeed Per-Client Throttling (węzeł, onboarding)</t>
-        </is>
-      </c>
+          <t>BRAK</t>
+        </is>
+      </c>
+      <c r="K52" s="11" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>O-05</t>
+          <t>Q-08</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>E-07</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Reseller jako produkt</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
         <is>
-          <t>Reseller — przegląd klientów</t>
+          <t>VPS — snapshoty i rebuild</t>
         </is>
       </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
-          <t>O — Multi-user i reseller</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>NISKA</t>
         </is>
       </c>
       <c r="I53" s="10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="J53" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
-        </is>
-      </c>
-      <c r="K53" s="11" t="inlineStr">
-        <is>
-          <t>reseller-klienci.service.ts + reseller.controller.ts (5 tras), reseller-klient.tsx; reseller-klienci.int-spec.ts (6 testów na PostgreSQL)</t>
-        </is>
-      </c>
+          <t>BRAK</t>
+        </is>
+      </c>
+      <c r="K53" s="11" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>O-07</t>
+          <t>Q-14</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>E-07</t>
+          <t>E-16</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Reseller jako produkt</t>
+          <t>Rozszerzenia oferty</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="E54" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>NISKI</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
         <is>
-          <t>Reseller — ustawianie własnej marży</t>
+          <t>Kreator uruchomienia węzła</t>
         </is>
       </c>
       <c r="G54" s="10" t="inlineStr">
         <is>
-          <t>O — Multi-user i reseller</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="H54" s="10" t="inlineStr">
         <is>
-          <t>NISKA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="I54" s="10" t="n">
@@ -14301,829 +14293,12 @@
       </c>
       <c r="K54" s="11" t="inlineStr">
         <is>
-          <t>reseller.controller.ts POST me/markup → reseller.service.ts setMarkup (0–300%, audyt RESELLER_MARKUP_CHANGED); reseller-client.tsx „Twój narzut”; test reseller.apply.spec.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="10" t="inlineStr">
-        <is>
-          <t>P-12</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t>E-08</t>
-        </is>
-      </c>
-      <c r="C55" s="11" t="inlineStr">
-        <is>
-          <t>Dostępność i zgodność w produkcie</t>
-        </is>
-      </c>
-      <c r="D55" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F55" s="11" t="inlineStr">
-        <is>
-          <t>Dostępność panelu wg WCAG 2.1 AA (EAA)</t>
-        </is>
-      </c>
-      <c r="G55" s="10" t="inlineStr">
-        <is>
-          <t>P — Zgodność</t>
-        </is>
-      </c>
-      <c r="H55" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNIA</t>
-        </is>
-      </c>
-      <c r="I55" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="J55" s="10" t="inlineStr">
-        <is>
-          <t>DZIAŁA</t>
-        </is>
-      </c>
-      <c r="K55" s="11" t="inlineStr">
-        <is>
-          <t>eslint.config.mjs w 4 aplikacjach: jsx-a11y recommended jako błędy (34 reguły); 76 → 0 znalezisk (client 52, admin 17, staff 6, www 1); client-panel/src/lib/kontrast-tokenow.spec.ts; ops/qa/a11y-nazwy-kontrolek.js</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="10" t="inlineStr">
-        <is>
-          <t>P-14</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>E-08</t>
-        </is>
-      </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>Dostępność i zgodność w produkcie</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E56" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F56" s="11" t="inlineStr">
-        <is>
-          <t>Certyfikacja ISO 27001</t>
-        </is>
-      </c>
-      <c r="G56" s="10" t="inlineStr">
-        <is>
-          <t>P — Zgodność</t>
-        </is>
-      </c>
-      <c r="H56" s="10" t="inlineStr">
-        <is>
-          <t>NISKA</t>
-        </is>
-      </c>
-      <c r="I56" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="J56" s="10" t="inlineStr">
-        <is>
-          <t>BRAK</t>
-        </is>
-      </c>
-      <c r="K56" s="11" t="inlineStr">
-        <is>
-          <t>home.pl i nazwa.pl mają — element przetargowy w B2B</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="10" t="inlineStr">
-        <is>
-          <t>F-06</t>
-        </is>
-      </c>
-      <c r="B57" s="10" t="inlineStr">
-        <is>
-          <t>E-11</t>
-        </is>
-      </c>
-      <c r="C57" s="11" t="inlineStr">
-        <is>
-          <t>DNS: DNSSEC i zarządzanie strefą</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F57" s="11" t="inlineStr">
-        <is>
-          <t>DNSSEC</t>
-        </is>
-      </c>
-      <c r="G57" s="10" t="inlineStr">
-        <is>
-          <t>F — DNS</t>
-        </is>
-      </c>
-      <c r="H57" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNIA</t>
-        </is>
-      </c>
-      <c r="I57" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J57" s="10" t="inlineStr">
-        <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K57" s="11" t="inlineStr">
-        <is>
-          <t>servers/directadmin.service.ts getHostingDnssec/enableHostingDnssec/disableHostingDnssec; services.controller.ts :id/hosting-dns/dnssec; client-panel components/hosting/DnssecPanel.tsx; ops/scripts/node-hosting-profile.sh dnssec=1; test directadmin.dnssec.spec.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="10" t="inlineStr">
-        <is>
-          <t>F-11</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>E-11</t>
-        </is>
-      </c>
-      <c r="C58" s="11" t="inlineStr">
-        <is>
-          <t>DNS: DNSSEC i zarządzanie strefą</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E58" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F58" s="11" t="inlineStr">
-        <is>
-          <t>Zmiana TTL rekordów</t>
-        </is>
-      </c>
-      <c r="G58" s="10" t="inlineStr">
-        <is>
-          <t>F — DNS</t>
-        </is>
-      </c>
-      <c r="H58" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNIA</t>
-        </is>
-      </c>
-      <c r="I58" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="J58" s="10" t="inlineStr">
-        <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K58" s="11" t="inlineStr">
-        <is>
-          <t>dns-manager.tsx:287,349 — pole TTL w formularzu rekordu → UtworzRekordDnsDto.ttl (60–86400) → directadmin.service createHostingDnsRecord ttl; D3 t1 (d3.hvln.pl) 29.09 po wdrożeniu 13:00 (panel klienta): FAIL: zmiana TTL rekordu → „zapisano”, TTL bez zmian (panel: dodaj+usuń); do tego usuwanie rekordów ze spacją w wartości (MX/TXT/CAA/SRV) nie działało (kodowanie „+”); poprawka 3b508f6 (DA action=edit, %20) czeka na push</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="10" t="inlineStr">
-        <is>
-          <t>F-12</t>
-        </is>
-      </c>
-      <c r="B59" s="10" t="inlineStr">
-        <is>
-          <t>E-11</t>
-        </is>
-      </c>
-      <c r="C59" s="11" t="inlineStr">
-        <is>
-          <t>DNS: DNSSEC i zarządzanie strefą</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E59" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F59" s="11" t="inlineStr">
-        <is>
-          <t>Anycast DNS</t>
-        </is>
-      </c>
-      <c r="G59" s="10" t="inlineStr">
-        <is>
-          <t>F — DNS</t>
-        </is>
-      </c>
-      <c r="H59" s="10" t="inlineStr">
-        <is>
-          <t>NISKA</t>
-        </is>
-      </c>
-      <c r="I59" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="J59" s="10" t="inlineStr">
-        <is>
-          <t>BRAK</t>
-        </is>
-      </c>
-      <c r="K59" s="11" t="inlineStr">
-        <is>
-          <t>tylko nazwa.pl na rynku PL</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="10" t="inlineStr">
-        <is>
-          <t>L-08</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>E-13</t>
-        </is>
-      </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>Automatyzacja: API zapisu i webhooki</t>
-        </is>
-      </c>
-      <c r="D60" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E60" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F60" s="11" t="inlineStr">
-        <is>
-          <t>Publiczne API — zapis</t>
-        </is>
-      </c>
-      <c r="G60" s="10" t="inlineStr">
-        <is>
-          <t>L — Automatyzacja</t>
-        </is>
-      </c>
-      <c r="H60" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNIA</t>
-        </is>
-      </c>
-      <c r="I60" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="J60" s="10" t="inlineStr">
-        <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K60" s="11" t="inlineStr">
-        <is>
-          <t>subscriptions/public-api-write.controller.ts (api/v1/services/:id/dns GET/POST, /dns/delete, /deploy GET/POST; zakresy dns:read, dns:write, deploy:write w api-scopes.ts; te same serwisy i walidacja co panel), opis w panelu api-tokens-client.tsx; test public-api-write.controller.spec.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="10" t="inlineStr">
-        <is>
-          <t>L-10</t>
-        </is>
-      </c>
-      <c r="B61" s="10" t="inlineStr">
-        <is>
-          <t>E-13</t>
-        </is>
-      </c>
-      <c r="C61" s="11" t="inlineStr">
-        <is>
-          <t>Automatyzacja: API zapisu i webhooki</t>
-        </is>
-      </c>
-      <c r="D61" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E61" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F61" s="11" t="inlineStr">
-        <is>
-          <t>Webhooki dla klienta</t>
-        </is>
-      </c>
-      <c r="G61" s="10" t="inlineStr">
-        <is>
-          <t>L — Automatyzacja</t>
-        </is>
-      </c>
-      <c r="H61" s="10" t="inlineStr">
-        <is>
-          <t>NISKA</t>
-        </is>
-      </c>
-      <c r="I61" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J61" s="10" t="inlineStr">
-        <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K61" s="11" t="inlineStr">
-        <is>
-          <t>client-webhooks/ (serwis, kontroler users/me/webhooks, moduł globalny); node-tasks.service.ts → poZadaniu; api-tokens/webhooks-client.tsx; migracja 20260924242000_client_webhooks; test client-webhooks.service.spec.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="10" t="inlineStr">
-        <is>
-          <t>L-11</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>E-13</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Automatyzacja: API zapisu i webhooki</t>
-        </is>
-      </c>
-      <c r="D62" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E62" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F62" s="11" t="inlineStr">
-        <is>
-          <t>Asystent AI w panelu</t>
-        </is>
-      </c>
-      <c r="G62" s="10" t="inlineStr">
-        <is>
-          <t>L — Automatyzacja</t>
-        </is>
-      </c>
-      <c r="H62" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNIA</t>
-        </is>
-      </c>
-      <c r="I62" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="J62" s="10" t="inlineStr">
-        <is>
-          <t>FLAGA</t>
-        </is>
-      </c>
-      <c r="K62" s="11" t="inlineStr">
-        <is>
-          <t>ai-modele.ts; ai-provider.service.ts; ai-ustawienia.admin.controller.ts; admin /settings/ai</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="10" t="inlineStr">
-        <is>
-          <t>L-12</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t>E-13</t>
-        </is>
-      </c>
-      <c r="C63" s="11" t="inlineStr">
-        <is>
-          <t>Automatyzacja: API zapisu i webhooki</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
-        <is>
-          <t>Q3 2027</t>
-        </is>
-      </c>
-      <c r="E63" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNI</t>
-        </is>
-      </c>
-      <c r="F63" s="11" t="inlineStr">
-        <is>
-          <t>Prognoza zużycia zasobów (AI)</t>
-        </is>
-      </c>
-      <c r="G63" s="10" t="inlineStr">
-        <is>
-          <t>L — Automatyzacja</t>
-        </is>
-      </c>
-      <c r="H63" s="10" t="inlineStr">
-        <is>
-          <t>NISKA</t>
-        </is>
-      </c>
-      <c r="I63" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="J63" s="10" t="inlineStr">
-        <is>
-          <t>FLAGA</t>
-        </is>
-      </c>
-      <c r="K63" s="11" t="inlineStr">
-        <is>
-          <t>hosting-forecast-actions.ts:7; fallback ServiceForecastPanel.tsx:97</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="10" t="inlineStr">
-        <is>
-          <t>NODE-01</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E64" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F64" s="11" t="inlineStr">
-        <is>
-          <t>Dwie niepołączone ścieżki dodania węzła w tym samym panelu</t>
-        </is>
-      </c>
-      <c r="G64" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H64" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNIA</t>
-        </is>
-      </c>
-      <c r="I64" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J64" s="10" t="inlineStr">
-        <is>
-          <t>DZIAŁA</t>
-        </is>
-      </c>
-      <c r="K64" s="11" t="inlineStr">
-        <is>
-          <t>node-wizard.tsx (krok „Instalacja (bootstrap v2)” z NodeBootstrapProgress), /nodes/init → przekierowanie, NODE_ONBOARD_RUNBOOK.md jedynym runbookiem</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="10" t="inlineStr">
-        <is>
-          <t>Q-05</t>
-        </is>
-      </c>
-      <c r="B65" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C65" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D65" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E65" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F65" s="11" t="inlineStr">
-        <is>
-          <t>E-mail marketing wbudowany w panel</t>
-        </is>
-      </c>
-      <c r="G65" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H65" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I65" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="10" t="inlineStr">
-        <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K65" s="11" t="inlineStr">
-        <is>
-          <t>email-marketing.controller.ts:36,81,119,139</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="10" t="inlineStr">
-        <is>
-          <t>Q-06</t>
-        </is>
-      </c>
-      <c r="B66" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C66" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D66" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E66" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F66" s="11" t="inlineStr">
-        <is>
-          <t>VPS / cloud w tym samym panelu</t>
-        </is>
-      </c>
-      <c r="G66" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H66" s="10" t="inlineStr">
-        <is>
-          <t>ŚREDNIA</t>
-        </is>
-      </c>
-      <c r="I66" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J66" s="10" t="inlineStr">
-        <is>
-          <t>FLAGA</t>
-        </is>
-      </c>
-      <c r="K66" s="11" t="inlineStr">
-        <is>
-          <t>vps.controller.ts:53,59,69; HETZNER_API_TOKEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="10" t="inlineStr">
-        <is>
-          <t>Q-07</t>
-        </is>
-      </c>
-      <c r="B67" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C67" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D67" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E67" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F67" s="11" t="inlineStr">
-        <is>
-          <t>VPS — konsola / VNC</t>
-        </is>
-      </c>
-      <c r="G67" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H67" s="10" t="inlineStr">
-        <is>
-          <t>NISKA</t>
-        </is>
-      </c>
-      <c r="I67" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J67" s="10" t="inlineStr">
-        <is>
-          <t>BRAK</t>
-        </is>
-      </c>
-      <c r="K67" s="11" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="10" t="inlineStr">
-        <is>
-          <t>Q-08</t>
-        </is>
-      </c>
-      <c r="B68" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C68" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D68" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E68" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F68" s="11" t="inlineStr">
-        <is>
-          <t>VPS — snapshoty i rebuild</t>
-        </is>
-      </c>
-      <c r="G68" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H68" s="10" t="inlineStr">
-        <is>
-          <t>NISKA</t>
-        </is>
-      </c>
-      <c r="I68" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J68" s="10" t="inlineStr">
-        <is>
-          <t>BRAK</t>
-        </is>
-      </c>
-      <c r="K68" s="11" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="10" t="inlineStr">
-        <is>
-          <t>Q-14</t>
-        </is>
-      </c>
-      <c r="B69" s="10" t="inlineStr">
-        <is>
-          <t>E-16</t>
-        </is>
-      </c>
-      <c r="C69" s="11" t="inlineStr">
-        <is>
-          <t>Rozszerzenia oferty</t>
-        </is>
-      </c>
-      <c r="D69" s="10" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E69" s="10" t="inlineStr">
-        <is>
-          <t>NISKI</t>
-        </is>
-      </c>
-      <c r="F69" s="11" t="inlineStr">
-        <is>
-          <t>Kreator uruchomienia węzła</t>
-        </is>
-      </c>
-      <c r="G69" s="10" t="inlineStr">
-        <is>
-          <t>Q — Przewaga</t>
-        </is>
-      </c>
-      <c r="H69" s="10" t="inlineStr">
-        <is>
-          <t>WYSOKA</t>
-        </is>
-      </c>
-      <c r="I69" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="J69" s="10" t="inlineStr">
-        <is>
-          <t>CZĘŚCIOWE</t>
-        </is>
-      </c>
-      <c r="K69" s="11" t="inlineStr">
-        <is>
           <t>node-wizard.tsx:277,288 — realnie tylko init + bootstrap; 7 z 9 kroków to treść runbooka (wizard-content.ts:21-40)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K69"/>
+  <autoFilter ref="A1:K54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Plan: harmonogram startu wariant A — beta wewnętrzna, AX102 9.11, GO 4–8.01.2027
Decyzja właściciela 04.10. Sprinty po zmianie dostają własny poniedziałek (konfiguracja.json
→ daty_sprintow), tablica układa je po dacie, koniec planu liczony ze sprintu z PB-12.
Nowe PB-40 (beta wewnętrzna na t1), PB-12 + PB-10 w sprincie 20, PB-26 + PB-05 w 22.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016StkFDdndcxTDp7ed2cv1W
</commit_message>
<xml_diff>
--- a/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
+++ b/plan-startowy-2026-08/VERRIS_BACKLOG_STARTOWY.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poza zakresem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog do startu'!$A$1:$P$122</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sprinty'!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Po starcie'!$A$1:$K$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Poza zakresem'!$A$1:$D$22</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTA('Backlog do startu'!$A$2:$A$121)</f>
+        <f>COUNTA('Backlog do startu'!$A$2:$A$122)</f>
         <v/>
       </c>
     </row>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUM('Backlog do startu'!$F$2:$F$121)</f>
+        <f>SUM('Backlog do startu'!$F$2:$F$122)</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF('Backlog do startu'!$E$2:$E$121,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$121,"BLOKER BIZNESOWY")</f>
+        <f>COUNTIF('Backlog do startu'!$E$2:$E$122,"BLOKER STARTU")+COUNTIF('Backlog do startu'!$E$2:$E$122,"BLOKER BIZNESOWY")</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Backlog do startu'!$P$2:$P$121,"zrobione")</f>
+        <f>COUNTIF('Backlog do startu'!$P$2:$P$122,"zrobione")</f>
         <v/>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>SUMIF('Backlog do startu'!$P$2:$P$121,"zrobione",'Backlog do startu'!$F$2:$F$121)</f>
+        <f>SUMIF('Backlog do startu'!$P$2:$P$122,"zrobione",'Backlog do startu'!$F$2:$F$122)</f>
         <v/>
       </c>
     </row>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P121"/>
+  <dimension ref="A1:P122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6767,12 +6767,12 @@
       </c>
       <c r="I77" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J77" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K77" s="10" t="inlineStr">
@@ -6845,12 +6845,12 @@
       </c>
       <c r="I78" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J78" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K78" s="10" t="inlineStr">
@@ -6923,12 +6923,12 @@
       </c>
       <c r="I79" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J79" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K79" s="10" t="inlineStr">
@@ -6965,12 +6965,12 @@
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>PB-08</t>
+          <t>PB-40</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
+          <t>Beta wewnętrzna na węźle testowym t1</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -6985,11 +6985,11 @@
       </c>
       <c r="E80" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G80" s="10" t="n">
         <v>14</v>
@@ -7001,12 +7001,12 @@
       </c>
       <c r="I80" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J80" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K80" s="10" t="inlineStr">
@@ -7026,12 +7026,12 @@
       </c>
       <c r="N80" s="11" t="inlineStr">
         <is>
-          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
+          <t>Wszystkie 8 scenariuszy przejście bez pomocy; zero otwartych błędów krytycznych (dane, pieniądze, dostęp); poprawki „przed AX102” zamknięte, reszta rozpisana na „przed GO” i „po starcie”.</t>
         </is>
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty. | 2026-09-27 SPRAWDZONE: kontener GTM-PJQNXCF5 w wersji 10 ma jeden tag Google (G-HHN0S0R777) — zdublowany GA4 wstrzymany przez właściciela. ZNALEZISKO: tag odpala na Initialization z wymogiem analytics_storage, a verris.pl odtwarzał zgodę z cookie dopiero PO gtm.js i page_view — powracający gość ze zgodą nie wysyłał nic do GA4 (tylko ccm/collect Ads). Poprawione w Analytics.tsx: zgoda z cookie odtwarzana przed GTM (jak w panelu). Zostaje: po wdrożeniu sprawdzić g/collect; nowy gość po kliknięciu „Akceptuj” — tag nie odpali do następnej odsłony (wyzwalacz Initialization) → dodać w GTM wyzwalacz zdarzenia verris_consent_update do tagu Google. | 2026-09-27: GTM wersja 11 opublikowana — tag Google odpala też na verris_consent_update (nowy gość liczony od razu po zgodzie); strona pcha zdarzenie tylko przy zmianie decyzji. Dowód problemu z GA4: ostatnie 7 dni — Panel klienta 354 wyświetlenia, verris.pl 2. W przeglądarce właściciela zapytania do Google kończą się 503 (blokada sieci/rozszerzenia) — weryfikacja po wdrożeniu w GA4 → Czas rzeczywisty z innego urządzenia. | 2026-09-27 PO WDROŻENIU (przeglądarka bez rozszerzeń, zgoda „Akceptuj wszystkie”): nowy gość — page_view do region1.analytics.google.com/g/collect od razu po zgodzie (gcs=G111, tag na verris_consent_update); powracający gość na /cennik — consent update przed gtm.js, page_view z gcs=G111; ciasteczka _ga i _ga_HHN0S0R777 ustawione. 503 z przeglądarki właściciela to blokada po jego stronie (rozszerzenie/sieć), nie strona. Zostaje: odsłona widoczna w GA4 → Czas rzeczywisty (właściciel) i zakup przy pierwszej prawdziwej płatności.</t>
+          <t>Przed zakupem AX102 właściciel i 2–3 zaufane osoby przechodzą scenariusze testerów z docs/ops/BETA_TESTY.md na t1 (decyzja 2026-09-29: otwarta beta dopiero po poprawnej wewnętrznej). Termin 19.10–6.11.2026.</t>
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr">
@@ -7043,12 +7043,12 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>PB-27</t>
+          <t>PB-08</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
+          <t>Pomiar: Consent Mode v2 + GTM + dedup event_id</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -7063,11 +7063,11 @@
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G81" s="10" t="n">
         <v>14</v>
@@ -7079,12 +7079,12 @@
       </c>
       <c r="I81" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K81" s="10" t="inlineStr">
@@ -7104,12 +7104,12 @@
       </c>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
+          <t>Zdarzenie zakupu dociera raz, nie dwa. Consent Mode nie blokuje pomiaru po zgodzie. Zweryfikowane w GTM Preview i w raporcie.</t>
         </is>
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji. | SPRAWDZONE NA PRODUKCJI 26.09 (22:35): na koncie testowym właściciela (mailtest-verris.pl) ustawiona cena 5 zł + rabat autoskalowania 20% z powodem, potem zmiana 5 → 6 — powód widoczny w adminie, klient widzi 6,00 zł/mies. Zostaje: odnowienie z tą ceną 22.10.2026 (samo się sprawdzi).</t>
+          <t>Wdrożenie ustaleń z audytu pomiaru: www linkuje, panel działa, deduplikacja po event_id, cookie Domain=.verris.pl. | PRZEGLĄD GTM 2026-09-23 (tylko odczyt): (1) DWA tagi Google z tym samym G-HHN0S0R777 na „Initialization - All Pages” („GA4” i „GA4 – Config”) — podwójna konfiguracja, ryzyko podwójnych page_view; prawdopodobnie to jest „Pilne” w jakości kontenera. Do zrobienia przez właściciela: wstrzymać „GA4” (starszy, bez wymogu zgody analytics_storage), zostawić „GA4 – Config”, opublikować. (2) GA4 – purchase: transaction_id/value/currency z ecommerce.* — poprawnie; dedup Meta po event_id purchase-&lt;id&gt;. (3) Consent: default → update przed gtm.js, user_data tylko hash SHA-256. (4) Zakup D3 wymaga prawdziwej płatności — do sprawdzenia przy pierwszym realnym zakupie. (5) W przeglądarce właściciela endpointy Google (collect) odpowiadają 503 — sprawdzić blokadę po stronie sieci/rozszerzenia; potwierdzić w GA4 → Czas rzeczywisty. | 2026-09-27 SPRAWDZONE: kontener GTM-PJQNXCF5 w wersji 10 ma jeden tag Google (G-HHN0S0R777) — zdublowany GA4 wstrzymany przez właściciela. ZNALEZISKO: tag odpala na Initialization z wymogiem analytics_storage, a verris.pl odtwarzał zgodę z cookie dopiero PO gtm.js i page_view — powracający gość ze zgodą nie wysyłał nic do GA4 (tylko ccm/collect Ads). Poprawione w Analytics.tsx: zgoda z cookie odtwarzana przed GTM (jak w panelu). Zostaje: po wdrożeniu sprawdzić g/collect; nowy gość po kliknięciu „Akceptuj” — tag nie odpali do następnej odsłony (wyzwalacz Initialization) → dodać w GTM wyzwalacz zdarzenia verris_consent_update do tagu Google. | 2026-09-27: GTM wersja 11 opublikowana — tag Google odpala też na verris_consent_update (nowy gość liczony od razu po zgodzie); strona pcha zdarzenie tylko przy zmianie decyzji. Dowód problemu z GA4: ostatnie 7 dni — Panel klienta 354 wyświetlenia, verris.pl 2. W przeglądarce właściciela zapytania do Google kończą się 503 (blokada sieci/rozszerzenia) — weryfikacja po wdrożeniu w GA4 → Czas rzeczywisty z innego urządzenia. | 2026-09-27 PO WDROŻENIU (przeglądarka bez rozszerzeń, zgoda „Akceptuj wszystkie”): nowy gość — page_view do region1.analytics.google.com/g/collect od razu po zgodzie (gcs=G111, tag na verris_consent_update); powracający gość na /cennik — consent update przed gtm.js, page_view z gcs=G111; ciasteczka _ga i _ga_HHN0S0R777 ustawione. 503 z przeglądarki właściciela to blokada po jego stronie (rozszerzenie/sieć), nie strona. Zostaje: odsłona widoczna w GA4 → Czas rzeczywisty (właściciel) i zakup przy pierwszej prawdziwej płatności.</t>
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr">
@@ -7121,12 +7121,12 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>PB-28</t>
+          <t>PB-27</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Rozliczenie poza Verris (całe konto)</t>
+          <t>Indywidualne warunki usługi: cena i autoskalowanie</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
@@ -7145,7 +7145,7 @@
         </is>
       </c>
       <c r="F82" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G82" s="10" t="n">
         <v>14</v>
@@ -7157,12 +7157,12 @@
       </c>
       <c r="I82" s="10" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J82" s="10" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K82" s="10" t="inlineStr">
@@ -7182,12 +7182,12 @@
       </c>
       <c r="N82" s="11" t="inlineStr">
         <is>
-          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
+          <t>Operator zakłada usługę z własną ceną; odnowienie pobiera tę cenę; autoskalowanie liczone z rabatem; każda zmiana w dzienniku audytu z autorem i powodem; test na PostgreSQL.</t>
         </is>
       </c>
       <c r="O82" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
+          <t>Decyzja właściciela 2026-09-26: operator (admin albo pracownik z uprawnieniem „Indywidualne warunki”) zakłada usługę na istniejącym lub nowym koncie i ustawia jej własną cenę (kwota albo rabat o X zł) oraz rabat na autoskalowanie o X%; warunki trzymają się usługi także przy odnowieniach. Stan 2026-09-26: operator nie może założyć usługi, ceny nie da się zmienić, odnowienie zawsze wraca do ceny katalogowej (promo.service.ts:266), stawki autoskalowania są globalne (AutoscalingPriceRule); błąd: kody rabatowe nie zapisują „appliesToRenewals” (promo.service.ts:157). | 2026-09-26 ZROBIONE W KODZIE: individualPrice + autoscalingDiscountPct na usłudze (odnowienia, bloki autoskalowania, limit wydatków, mail), POST /admin/custom-terms/user/:id/service (także plan ukryty), PATCH …/subscription/:id, uprawnienie CUSTOM_TERMS_MANAGE, sekcja w panelu admina i obsługi, audyt z powodem; poprawiony zapis appliesToRenewals kodów. Testy na PostgreSQL. Zostało: przejście na produkcji. | SPRAWDZONE NA PRODUKCJI 26.09 (22:35): na koncie testowym właściciela (mailtest-verris.pl) ustawiona cena 5 zł + rabat autoskalowania 20% z powodem, potem zmiana 5 → 6 — powód widoczny w adminie, klient widzi 6,00 zł/mies. Zostaje: odnowienie z tą ceną 22.10.2026 (samo się sprawdzi).</t>
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr">
@@ -7199,58 +7199,58 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>X-41</t>
+          <t>PB-28</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
+          <t>Rozliczenie poza Verris (całe konto)</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>X — Infrastruktura jakości</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F83" s="10" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G83" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H83" s="10" t="inlineStr">
         <is>
-          <t>Faza 3 — Wejście na rynek</t>
+          <t>Faza 2 — Odzyskanie funkcji-widm i luki pierwszego tygodnia</t>
         </is>
       </c>
       <c r="I83" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J83" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K83" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
-          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M83" s="11" t="inlineStr">
@@ -7260,12 +7260,12 @@
       </c>
       <c r="N83" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Flaga na koncie ustawiana z panelu admina/obsługi; testy: brak obciążeń, przedłużanie okresu, brak maili, brak blokady, raport zużycia autoskalowania.</t>
         </is>
       </c>
       <c r="O83" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01. | 2026-09-28: sieć danych (verris_internal) internal:true — Postgres, Valkey, MinIO, Loki, eksportery, Alloy bez internetu; API/www wychodzą przez verris_public (dotąd trasa domyślna szła przez sieć danych). Przejście: prod-siec-danych-izolacja.sh (93e0b8d, test na replice stosu). Allowlista domen dla API odrzucona: migrator, monitoring i webhooki łączą się z dowolnymi hostami klientów. | 2026-09-28 D3 NA PRODUKCJI (08:47): verris_internal internal=true; z kontenera API postgres/redis/minio → 172.18.x (sieć danych), API → api.stripe.com 200, postgres → 1.1.1.1:443 brak połączenia. Incydent przy przejściu: Compose zgubił aliasy usług (EAI_AGAIN) i nieudany minio-bootstrap zatrzymał API — ok. 10 min bez API (08:35–08:45); naprawione przepięciem z --alias, skrypt poprawiony (64409dc).</t>
+          <t>Decyzja właściciela 2026-09-26: klient oznaczony „rozliczany przez właściciela” — system nie pobiera opłat, nie blokuje za brak płatności, sam przedłuża okresy, nie wysyła maili o saldzie/odnowieniu, nie wystawia faktur; klient nie widzi portfela ani płatności; autoskalowanie działa bez pobierania, zużycie w raporcie do faktury właściciela. Stan 2026-09-26: tryb MANUAL istnieje tylko w bazie, nie da się go ustawić, okres się nie przedłuża, maile i autoskalowanie dalej działają jak u płacącego. | 2026-09-26 ZROBIONE W KODZIE: User.billingOutside + usługi MANUAL (przełącznik w transakcji, odmowa przy karcie cyklicznej); odnowienia przedłużają bez obciążenia, bez przypomnień/maili o saldzie/proformy/karencji; autoskalowanie bez pobierania z zestawieniem miesięcznym; panel klienta bez portfela, płatności i zamawiania. Testy na PostgreSQL. Zostało: przejście na produkcji.</t>
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr">
@@ -7277,12 +7277,12 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>X-41</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
+          <t>Hardening egressu wisi w łańcuchu OUTPUT, a ruch kontenerów idzie przez FORWARD</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -7292,7 +7292,7 @@
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>X — Infrastruktura jakości</t>
         </is>
       </c>
       <c r="E84" s="10" t="inlineStr">
@@ -7313,12 +7313,12 @@
       </c>
       <c r="I84" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J84" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="K84" s="10" t="inlineStr">
@@ -7328,7 +7328,7 @@
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
+          <t>obserwacja wpięta w DOCKER-USER, 1674 pakiety zliczone, 0 DROP/REJECT</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="O84" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41. | 2026-09-28: resolwery IPv6 Hetznera w liście DNS; pomiar DNS-KTO: zapytania wysyła tylko rspamd do 127.0.0.53 — wyjątek po właścicielu niepotrzebny (plik pusty) — 94cfe2c.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-25 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Cały hardening egressu wisi w łańcuchu OUTPUT. Ruch kontenerów idzie przez FORWARD → DOCKER-USER, więc egress całego produktu był poza zasięgiem zabezpieczenia, które wyglądało, jakby go obejmowało. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Obserwacja w DOCKER-USER juz stoi (1674 pakiety, 0 DROP). Zostaje egzekwowanie: przeniesienie regul z OUTPUT do FORWARD/DOCKER-USER razem z SEC-01. | 2026-09-28: sieć danych (verris_internal) internal:true — Postgres, Valkey, MinIO, Loki, eksportery, Alloy bez internetu; API/www wychodzą przez verris_public (dotąd trasa domyślna szła przez sieć danych). Przejście: prod-siec-danych-izolacja.sh (93e0b8d, test na replice stosu). Allowlista domen dla API odrzucona: migrator, monitoring i webhooki łączą się z dowolnymi hostami klientów. | 2026-09-28 D3 NA PRODUKCJI (08:47): verris_internal internal=true; z kontenera API postgres/redis/minio → 172.18.x (sieć danych), API → api.stripe.com 200, postgres → 1.1.1.1:443 brak połączenia. Incydent przy przejściu: Compose zgubił aliasy usług (EAI_AGAIN) i nieudany minio-bootstrap zatrzymał API — ok. 10 min bez API (08:35–08:45); naprawione przepięciem z --alias, skrypt poprawiony (64409dc).</t>
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr">
@@ -7355,31 +7355,31 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>PB-22</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
+          <t>Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F85" s="10" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G85" s="10" t="n">
         <v>15</v>
@@ -7391,22 +7391,22 @@
       </c>
       <c r="I85" s="10" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J85" s="10" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ops/scripts/security-control-plane-egress.sh — zbuduj_zbior_z_pliku (verris_egress_dns / verris_egress_smtp z ops/etc/verris/security/egress-allow-{dns,smtp}.txt), apply_strict_allowlist: DROP dla NOWYCH 53 udp/tcp i 25/465/587 poza listą, warunek wstępny strict obejmuje DNS i SMTP; test D2 egress-strict-naprawde-blokuje.spec.ts (SEC-03)</t>
         </is>
       </c>
       <c r="M85" s="11" t="inlineStr">
@@ -7416,12 +7416,12 @@
       </c>
       <c r="N85" s="11" t="inlineStr">
         <is>
-          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O85" s="11" t="inlineStr">
         <is>
-          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Ruch poza TCP/80 i TCP/443 — DNS (UDP/53), SMTP — nie jest objęty ani obserwacją z X-41, ani trybem strict. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Rozszerzenie obserwacji i trybu strict na UDP/53 i SMTP — nowe lancuchy, nowe zbiory, nowy zakres testu. | 2026-09-23: host (OUTPUT) — pomiar obejmuje każdy port od SEC-05; strict rozszerzony o DNS (resolwery Hetznera 185.12.64.1/2) i SMTP (przekaźnik poznan.hvln.pl) na podstawie --pomiar z 2026-09-23. Pomiar liczy już tylko TCP SYN (skaner SSH wyglądał jak ruch wychodzący). Zostaje: włączenie strict na prod (nie przed 2026-09-29) = D3; kontenery (FORWARD) — w X-41. | 2026-09-28: resolwery IPv6 Hetznera w liście DNS; pomiar DNS-KTO: zapytania wysyła tylko rspamd do 127.0.0.53 — wyjątek po właścicielu niepotrzebny (plik pusty) — 94cfe2c.</t>
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr">
@@ -7433,34 +7433,34 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>PB-22</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>Log egressu jest próbką, nie zapisem</t>
+          <t>Badge na stronę v2 — interaktywne i użyteczne dla klienta</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t>G — SSL i bezpieczeństwo</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E86" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F86" s="10" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G86" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H86" s="10" t="inlineStr">
         <is>
@@ -7469,22 +7469,22 @@
       </c>
       <c r="I86" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J86" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="K86" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr">
@@ -7494,12 +7494,12 @@
       </c>
       <c r="N86" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Badge widoczne na prod na domenie klienta; pieczęć znika przy niespełnionych warunkach; kliknięcia polecenia liczone; testy D2 zielone.</t>
         </is>
       </c>
       <c r="O86" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
+          <t>Zgłoszenie właściciela 2026-09-23: stare badge wyglądały źle i nic nie robiły (uptime pokazywał stan węzła, embed EKO blokowany przez X-Frame-Options/CORP). Nowy zestaw wg makiet: pieczęć zaufania (SSL, dostępność 30 dni, dane w UE, weryfikacja), dostępność na żywo z monitora strony, polecenie z prowizją (program partnerski), EKO SVG. Zakładka „Badge na stronę” w usłudze.</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr">
@@ -7511,12 +7511,12 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
+          <t>Log egressu jest próbką, nie zapisem</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -7547,12 +7547,12 @@
       </c>
       <c r="I87" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J87" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K87" s="10" t="inlineStr">
@@ -7562,7 +7562,7 @@
       </c>
       <c r="L87" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
+          <t>ops/scripts/security-control-plane-egress.sh — apply_egress_seen: lancuch VERRIS_EGRESS_SEEN (pierwszy w OUTPUT) dopisuje KAZDE nowe polaczenie TCP/UDP do ipset verris_egress_seen (hash:ip,port, okno 7 dni, bez -m limit); apply_forward_observe — to samo dla kontenerow (verris_egress_seen_fwd); --pomiar — raport z ipset z flaga allowlisty; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M87" s="11" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="O87" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9). | 2026-09-28: te same zwolnienia mostków (lo, docker0, br-+) w ip6tables — 94cfe2c. | 2026-10-01 INCYDENT I POPRAWKA (bc40703): VERRIS_ANTISCAN (iptables i ip6tables) nie zwalniał lo/docker0/br-+ — docker-proxy obsługujący klientów IPv6 otwiera nowe połączenie hosta do kontenera na 443, licznik anty-skanu się wyczerpał i DROP odciął cały IPv6 panelu i API (t1 bez sygnału ok. 1,5 h). Wyjątki dopisane w kodzie (test egress-strict-naprawde-blokuje.spec.ts) i na żywo na control-plane; po zmianie IPv6 lokalnie i z t1 → 200, sygnał i manifest z t1 wróciły.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: obserwowalność. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Log egressu jest próbką, nie zapisem. Licznik iptables pokazuje ~1,81 mln pakietów przez łańcuch strict, a w journalu jest 1796 wpisów z 48 h — reguła logująca ma ogranicznik częstotliwości. Nieobecność celu w tym logu nie dowodzi, że host tam nie chodzi. Każda allowlista budowana na tym odczycie jest niepełna z definicji. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zdjecie ogranicznika czestotliwosci z reguly logujacej albo przejscie na nflog z licznikami. WARUNEK WSTEPNY dla SEC-06: allowlista budowana na probce jest niepelna z definicji. | 2026-09-22 KOD (D1): zamiast zdejmowac ogranicznik z LOG (dysk/journal pod kazdym polaczeniem) — zapis celow w ipset w pamieci jadra. Obecnosc celu pewna, liczniki orientacyjne. D3: wlaczenie na control-plane (przebieg domyslny) i --pomiar po dobie. | 2026-09-22 D3: wlaczone na control-plane (09:23 UTC, przebieg domyslny po wdrozeniu 5c3fe99); --pomiar po kilku minutach pokazal pierwszy cel: 169.254.169.254,tcp:80 (metadane chmury, 2 nowe polaczenia) — cel, ktorego probkowany log nie wykazal. Pomiar kontenerow (FORWARD) wlaczy sie przy nastepnym --obserwuj-kontenery.</t>
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr">
@@ -7589,12 +7589,12 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Tryb `--strict` jest atrapą</t>
+          <t>Host rozmawia z kontenerami przez OUTPUT — ruch wewnętrzny liczony jako egress</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
@@ -7613,7 +7613,7 @@
         </is>
       </c>
       <c r="F88" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>16</v>
@@ -7625,22 +7625,22 @@
       </c>
       <c r="I88" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J88" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K88" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
+          <t>security-control-plane-egress.sh — RETURN dla -o lo/docker0/br-+ w VERRIS_EGRESS_STRICT i br-+ w VERRIS_EGRESS_BOGON przed DROP; test apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts</t>
         </is>
       </c>
       <c r="M88" s="11" t="inlineStr">
@@ -7650,12 +7650,12 @@
       </c>
       <c r="N88" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O88" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru. | 2026-09-28: strict także po IPv6 (REJECT → natychmiastowe przejście na IPv4), warunek pomiaru obu rodzin przed pierwszą regułą; verris-egress.service odtwarza tryb i pomiar po restarcie (dotąd restart zdejmował cały hardening) — 94cfe2c. | 2026-09-28 D3 (09:07): przebieg domyślny z ipv6=1 — pomiar verris_egress_seen6, bogony/IOC/log/anty-skan w ip6tables; verris-egress.service active (enabled). Zbiory IPv6: https6 71, dns6 2, smtp6 1. Strict jeszcze wyłączony — decyzja po pomiarze 30.09.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Host rozmawia z kontenerami przez OUTPUT. W logu egressu są wpisy `DST=172.19.0.3` na portach 443 i 80 — czyli ruch host → kontener. Reguła `DROP` trybu strict odrzuca wszystko spoza ipsetu, a adresy sieci Dockera w ipsecie nie są i być nie powinny. Włączenie strict bez wyjątku dla `172.16.0.0/12` zerwałoby to połączenie. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Wyjatek dla 172.16.0.0/12 w regule OUTPUT. Sama zmiana jest mala, ale bez niej wlaczenie strict zrywa polaczenie host-kontener. | 2026-09-22 KOD (D1): wyjatek po interfejsie (mostki Dockera), nie po CIDR — 172.16.0.0/12 zostaje w bogonach dla ruchu, ktory NIE idzie do kontenera. Przy okazji: lancuch BOGON zwalnial tylko docker0, a sieci compose to br-&lt;id&gt; w 172.18-172.20 — host-&gt;kontener na 443 wpadlby w DROP bogonow. D3 przy wlaczeniu strict (sprint 9). | 2026-09-28: te same zwolnienia mostków (lo, docker0, br-+) w ip6tables — 94cfe2c. | 2026-10-01 INCYDENT I POPRAWKA (bc40703): VERRIS_ANTISCAN (iptables i ip6tables) nie zwalniał lo/docker0/br-+ — docker-proxy obsługujący klientów IPv6 otwiera nowe połączenie hosta do kontenera na 443, licznik anty-skanu się wyczerpał i DROP odciął cały IPv6 panelu i API (t1 bez sygnału ok. 1,5 h). Wyjątki dopisane w kodzie (test egress-strict-naprawde-blokuje.spec.ts) i na żywo na control-plane; po zmianie IPv6 lokalnie i z t1 → 200, sygnał i manifest z t1 wróciły.</t>
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr">
@@ -7667,12 +7667,12 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
+          <t>Tryb `--strict` jest atrapą</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
@@ -7703,22 +7703,22 @@
       </c>
       <c r="I89" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J89" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K89" s="10" t="inlineStr">
         <is>
-          <t>BRAK</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L89" s="11" t="inlineStr">
         <is>
-          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
+          <t>security-control-plane-egress.sh — apply_strict_allowlist: DROP bez testu cgroup, kontrola po fakcie (iptables -S; brak reguly = exit 1), warunek wstepny sprawdz_pomiar_przed_strict (&gt;= POMIAR_MIN_DNI dni pomiaru i zero celow 80/443 spoza allowlisty, inaczej exit 1 z lista celow), --wymus-strict; security-install-verris-security.sh — usuniete automatyczne --strict || true; test behawioralny apps/api/src/test/egress-strict-naprawde-blokuje.spec.ts (prawdziwy skrypt na atrapach iptables/ipset, te same flagi powloki)</t>
         </is>
       </c>
       <c r="M89" s="11" t="inlineStr">
@@ -7728,12 +7728,12 @@
       </c>
       <c r="N89" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O89" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Tryb `--strict` jest atrapą. Trzy niezależne wyciszenia jedno po drugim: reguła `DROP` zagnieżdżona w teście dopasowania cgroup (na tym jądrze niedostępnego), skrypt kończy się `WARN` i kodem 0, a instalator woła go z `|| true`. Wyjątek cgroup miał przepuszczać ruch kontenerów — który do OUTPUT w ogóle nie dociera (patrz X-41). | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: DROP musi realnie obowiazywac: przebudowa security-control-plane-egress.sh bez zagniezdzenia w tescie cgroup, bez "|| true" w instalatorze, plus straznik zachowaniowy na wzor X-34 (atrapa wielkosci produkcyjnej, te same flagi powloki). | 2026-09-22 KOD (D1): trzy wyciszenia usuniete. Wyjatek cgroup byl zbedny — ruch kontenerow nie przechodzi przez OUTPUT (X-41). Strict przestal byc nieszkodliwy, dlatego warunek wstepny laczy SEC-05 (pomiar) z SEC-06 (allowlista z tego, co host robi): nie da sie go wlaczyc na slepo. D3 dopiero przy wlaczeniu na control-plane w sprincie 9, po tygodniu pomiaru. | 2026-09-28: strict także po IPv6 (REJECT → natychmiastowe przejście na IPv4), warunek pomiaru obu rodzin przed pierwszą regułą; verris-egress.service odtwarza tryb i pomiar po restarcie (dotąd restart zdejmował cały hardening) — 94cfe2c. | 2026-09-28 D3 (09:07): przebieg domyślny z ipv6=1 — pomiar verris_egress_seen6, bogony/IOC/log/anty-skan w ip6tables; verris-egress.service active (enabled). Zbiory IPv6: https6 71, dns6 2, smtp6 1. Strict jeszcze wyłączony — decyzja po pomiarze 30.09.</t>
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr">
@@ -7745,12 +7745,12 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
+          <t>Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -7765,11 +7765,11 @@
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>16</v>
@@ -7781,12 +7781,12 @@
       </c>
       <c r="I90" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J90" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K90" s="10" t="inlineStr">
@@ -7796,7 +7796,7 @@
       </c>
       <c r="L90" s="11" t="inlineStr">
         <is>
-          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
+          <t>ipset test verris_egress_https na 4 celach z logu egressu</t>
         </is>
       </c>
       <c r="M90" s="11" t="inlineStr">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="O90" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / firewall. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Allowlista pokrywa to, o czym ktoś pomyślał, nie to, co host robi. Test `ipset` na celach z rzeczywistego ruchu: `sogo-repo.alinto.org` — BRAK, `static.77.118.180.157.clients.your-server.de` (120 pakietów, nierozpoznany) — BRAK. GitHub i `sa-update.surbl.org` — JEST. Włączenie `--strict` dziś odcięłoby repozytorium pakietów SOGo i nieznany host Hetznera. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Okres obserwacji na pelnym logu (po SEC-05) i zbudowanie allowlisty z tego, co host robi, a nie z tego, o czym ktos pomyslal. Koszt to glownie czas obserwacji, nie kod. | 2026-09-22 POMIAR RUSZYL (SEC-05, D3). Pierwszy cel spoza allowlisty: 169.254.169.254:80 — metadane chmury, siec link-local. Z hosta odcina go VERRIS_EGRESS_BOGON, wiec --pomiar oznacza go jako 'bogon' i nie liczy do warunku strict. OTWARTE PYTANIE (SSRF): kontenery ida przez FORWARD, gdzie bogonow nie ma — jesli z kontenera API da sie odpytac 169.254.169.254, to kazda funkcja pobierajaca URL od klienta (webhooki, sondy statusu, migrator) moze byc droga do metadanych serwera. Do sprawdzenia jednym poleceniem z kontenera; wynik decyduje, czy blokada metadanych w DOCKER-USER idzie przed sprint 9.</t>
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr">
@@ -7823,31 +7823,31 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>PB-23</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
+          <t>Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>G — SSL i bezpieczeństwo</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G91" s="10" t="n">
         <v>16</v>
@@ -7859,22 +7859,22 @@
       </c>
       <c r="I91" s="10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J91" s="10" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K91" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BRAK</t>
         </is>
       </c>
       <c r="L91" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>`egress-allow-hostnames.txt`; ipset `verris_egress_https` = 65 wpisów</t>
         </is>
       </c>
       <c r="M91" s="11" t="inlineStr">
@@ -7884,12 +7884,12 @@
       </c>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O91" s="11" t="inlineStr">
         <is>
-          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: egress / płatności. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: Stripe jest w allowliście wyłącznie po nazwie, a ipset powstaje z rozwiązania nazw. Adresy Stripe rotują (198.137.x / 198.202.x), więc zbiór starzeje się między uruchomieniami. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Odswiezanie ipsetu z opublikowanej listy adresow Stripe zamiast jednorazowego rozwiazania nazw; cron plus check w live-readiness. | ANALIZA 2026-09-23: Stripe woła wyłącznie API w kontenerze (FORWARD), którego strict hosta (OUTPUT) nie dotyczy, a X-41 nie ogranicza kontenerom 80/443 (decyzja: tam chronią strażniki SSRF w aplikacji). Pomiar hosta z 2026-09-22/23 nie ma żadnego celu Stripe. Jeśli pomiar 7-dniowy (29.09) to potwierdzi — pozycja NIE DOTYCZY; wpisy Stripe w allowliście hosta zostają tylko dla ręcznego ops/scripts/uzgodnij-platnosci-stripe.mjs.</t>
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr">
@@ -7901,34 +7901,34 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>PB-23</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Podpisane DPA z subprocesorami (część)</t>
+          <t>Każdy widok osiągalny z menu (klient, admin, staff)</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>P — Zgodność</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H92" s="10" t="inlineStr">
         <is>
@@ -7937,22 +7937,22 @@
       </c>
       <c r="I92" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J92" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K92" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L92" s="11" t="inlineStr">
         <is>
-          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M92" s="11" t="inlineStr">
@@ -7962,12 +7962,12 @@
       </c>
       <c r="N92" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Lista tras vs menu dla trzech paneli bez luk; test-strażnik czerwony po dodaniu trasy bez wejścia w nawigacji.</t>
         </is>
       </c>
       <c r="O92" s="11" t="inlineStr">
         <is>
-          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą. | 2026-09-27: właściciel — umowy powierzenia zaakceptowane przy zakładaniu kont (Hetzner, Openprovider, Cloudflare, Firmino; konta używane od wcześniejszego hostingu na Plesku), dokładnych dat nie pamięta. Cloudflare: DPA wchodzi z umową główną. Hetzner: umowę powierzenia zawiera się osobno w accounts.hetzner.com → Data protection — do potwierdzenia jednym spojrzeniem (data zawarcia widoczna na stronie), wtedy ZAMKNIĘTE. | 2026-09-27 ZAMKNIĘTE: Hetzner — DPA v1.2 zawarta 27.09.2026 (klient K0265867421, Załącznik 1 z użytkownikami końcowymi stron i poczty klientów; PDF u właściciela); Openprovider, Cloudflare, Firmino — zaakceptowane przy rejestracji (właściciel); Stripe, AWS — z umowy głównej. Tracker: docs/legal/dpa-subprocessors-tracking.md.</t>
+          <t>Zasada właściciela 2026-09-23: żaden ekran nie może wymagać szukania po panelu. Przegląd wszystkich tras (page.tsx) w trzech panelach i ich wejść w menu/zakładkach; widoki bez wejścia dostają miejsce w menu albo zakładkę w logicznym rodzicu; strażnik w CI: każda trasa z page.tsx ma odnośnik w konfiguracji nawigacji albo jest na jawnej liście wyjątków (szczegóły rekordu, kroki kreatora) z uzasadnieniem. | WYNIK 2026-09-23: przegląd 60 tras klienta, 57 admina, 12 staff — brak widoków bez wejścia. Stare adresy klienta (/dashboard/apps, /backups, /cron, /databases, /dns, /email, /file-manager, /ftp, /php, /ssl, /domains/registrar) to przekierowania na zakładki usługi; strony auth z maili na liście wyjątków. Strażnik: apps/api/src/test/widoki-w-nawigacji.spec.ts (sprawdzony: sztuczna ukryta strona w admin i kliencie → czerwony).</t>
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr">
@@ -7979,31 +7979,31 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>PB-03</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>Finalizacja dokumentów prawnych 1.0.0</t>
+          <t>Podpisane DPA z subprocesorami (część)</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>P — Zgodność</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
-          <t>BLOKER BIZNESOWY</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G93" s="10" t="n">
         <v>17</v>
@@ -8015,22 +8015,22 @@
       </c>
       <c r="I93" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="J93" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="K93" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L93" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docs/legal/dpa-subprocessors-tracking.md — tabela statusow po korekcie 2026-09-19. Stripe i AWS: DPA obowiazuje z mocy umowy glownej. Hetzner i Openprovider: akceptacja w panelu, jeszcze nie wykonana. Cloudflare: mechanizm do potwierdzenia.</t>
         </is>
       </c>
       <c r="M93" s="11" t="inlineStr">
@@ -8040,12 +8040,12 @@
       </c>
       <c r="N93" s="11" t="inlineStr">
         <is>
-          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O93" s="11" t="inlineStr">
         <is>
-          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>POTWIERDZONE jako bloker, dowód poprawiony: tracker istnieje (wcześniejszy zapis „brak w repo” był fałszywy), ale ani jedno DPA nie jest podpisane — Stripe, dostawca VPS, dostawca backupu off-site, OpenProvider. Bez tego DPA podpisywane z klientem jest niekompletne. | KOREKTA 2026-09-19: naklad M (16 h) -&gt; S (6 h) i pozycja w calosci w sprincie 4. Zalozenie "zalezy od tempa dostawcow, nie od nas" bylo NIEPRAWDZIWE i kosztowalo cztery tygodnie w planie: P-15 bylo rozbite na sprinty 4 i 10, przez co domkniecie blokerow stalo na 2026-11-02. Sprawdzone u zrodla: u zadnego z pieciu dostawcow nie trzeba nikogo prosic — trzy DPA obowiazuja z mocy umowy glownej (Stripe, AWS, warunkowo Cloudflare), dwa akceptuje sie kliknieciem w panelu (Hetzner accounts.hetzner.com/account/dpa, Openprovider control panel). Jedyna praca wlasna to Zalacznik 1 do DPA Hetznera: kategorie danych i krag osob, w tym UZYTKOWNICY KONCOWI SERWISOW KLIENTOW — najlatwiejsza do pominiecia i najwieksza grupa. Rownolegle poprawiona lista subprocesorow, ktora byla nieaktualna od 2026-07-07: wymieniala "dostawca VPS (OVH/Hetzner)" i "dostawca backupu" jako nierozstrzygniete oraz reCAPTCHA zamiast Turnstile. | 2026-09-23: dopisany Streamsoft Firmino (program księgowy, akceptacja w Ustawienia → RODO → Umowa powierzenia); OpenAI poza listą — AI wyłączone na start; ClouDNS przy zakupie w sprincie 18. | 2026-09-23: właściciel potwierdził akceptację umów powierzenia i uruchomienie skrzynek; dowody (numery umów / zrzuty z paneli) do dopisania w trackerze przy weryfikacji przed startem. | 2026-09-25: doszli OpenAI Ireland Ltd i Anthropic Ireland, Limited (asystent AI) — DPA z SCC obowiązuje z akceptacją umowy przy założeniu konta API; Polityka prywatności 1.0.3 w drafts/privacy.md do publikacji przed wpisaniem kluczy. Do DPA z klientami (Zał. 2) nie wchodzą. | 2026-09-27: właściciel — umowy powierzenia zaakceptowane przy zakładaniu kont (Hetzner, Openprovider, Cloudflare, Firmino; konta używane od wcześniejszego hostingu na Plesku), dokładnych dat nie pamięta. Cloudflare: DPA wchodzi z umową główną. Hetzner: umowę powierzenia zawiera się osobno w accounts.hetzner.com → Data protection — do potwierdzenia jednym spojrzeniem (data zawarcia widoczna na stronie), wtedy ZAMKNIĘTE. | 2026-09-27 ZAMKNIĘTE: Hetzner — DPA v1.2 zawarta 27.09.2026 (klient K0265867421, Załącznik 1 z użytkownikami końcowymi stron i poczty klientów; PDF u właściciela); Openprovider, Cloudflare, Firmino — zaakceptowane przy rejestracji (właściciel); Stripe, AWS — z umowy głównej. Tracker: docs/legal/dpa-subprocessors-tracking.md.</t>
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr">
@@ -8057,12 +8057,12 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>PB-04</t>
+          <t>PB-03</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
+          <t>Finalizacja dokumentów prawnych 1.0.0</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8077,11 +8077,11 @@
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>17</v>
@@ -8093,12 +8093,12 @@
       </c>
       <c r="I94" s="10" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="J94" s="10" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="K94" s="10" t="inlineStr">
@@ -8118,12 +8118,12 @@
       </c>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
+          <t>Wszystkie dokumenty w statusie opublikowanym z numerem wersji i datą. Panel /legal nie pokazuje ani jednego „Dokument w przygotowaniu”.</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06). | 2026-09-27 ZAMKNIĘTE: skrzynka abuse@verris.pl działa (przekierowanie na skrzynkę właściciela — potwierdzone przez właściciela 23.09 i 27.09); test zgłoszenia: formularz /zglos-naduzycie → ABUSE_REPORT_RECEIVED 24.09 (test-live-verris.pl, PHISHING) → decyzja w panelu obsługi 26.09 (N-13).</t>
+          <t>Regulamin, polityka prywatności, SLA, DPA, polityka cookies — wyjście z DRAFT-u, wersjonowanie i publikacja w panelu. | 2026-09-23: decyzje właściciela — publikacja bez zewnętrznego przeglądu, raz, tuż przed pierwszym klientem; kontakt @verris.pl + telefon; Firmino (Streamsoft) dopisany do polityki i listy; AI wyłączone na start; §9 ust. 4 regulaminu (faktury z programu księgowego) — regulamin 1.2.0, polityka 1.0.2. Zostaje: §10 ust. 5 (kopie kont) po D3 węzła, ClouDNS po zakupie, akceptacje DPA (Hetzner, Openprovider, Cloudflare, Firmino), skrzynki kontakt@/rodo@/abuse@/security@. | 2026-09-26: pakiet publikacji — rozjazdy wersji (nagłówki 1.2.0/1.0.3/1.0.0, stopki z lipca, skrypt publikuje jako 1.2.0) → propozycja: wszystko 1.0.0 z datą publikacji; tekst §10 ust. 5 z miejscami na wartości z D3; wiersz ClouDNS (Cloud DNS Ltd., Sofia — DPA do potwierdzenia u dostawcy); lista kroków — docs/legal/drafts/DO_ZATWIERDZENIA_PB-03_publikacja-1.0.0.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr">
@@ -8135,34 +8135,34 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>N-16</t>
+          <t>PB-04</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>SLA z zapisanymi kredytami</t>
+          <t>Procedura obsługi nadużyć (abuse) — dokument</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>N — Wsparcie i ops</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G95" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H95" s="10" t="inlineStr">
         <is>
@@ -8171,37 +8171,37 @@
       </c>
       <c r="I95" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="J95" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="K95" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L95" s="11" t="inlineStr">
         <is>
-          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M95" s="11" t="inlineStr">
         <is>
-          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N95" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Dokument w ops/docs z właścicielem i czasami reakcji. Test: zgłoszenie wysłane na abuse@ trafia do kogoś i ma odpowiedź w deklarowanym czasie.</t>
         </is>
       </c>
       <c r="O95" s="11" t="inlineStr">
         <is>
-          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja). | 2026-09-27 KOD (31e5b2f): wyłączenie konserwacji tylko dla prac zapowiedzianych ≥48 h wcześniej i tylko w zapowiedzianych godzinach (§15 ust. 7); nieudane uznanie portfela zwalnia miesiąc do ponowienia. Test sla-kredyty.int-spec.ts. Rekompensaty na produkcji nadal wyłączone. | 2026-09-28 DECYZJA WŁAŚCICIELA: rekompensaty „na wniosek” wg regulaminu (bez automatu); tekst na verris.pl, blogu i w kampaniach poprawiony w 14 miejscach (46976c6).</t>
+          <t>Adres abuse@ obsługiwany, ścieżka od zgłoszenia do reakcji, czasy reakcji, kto decyduje o zawieszeniu, wzory odpowiedzi do CERT i rejestratorów. | 2026-09-23: dokument ops/docs/ABUSE.md — właściciel, źródła zgłoszeń, kategorie P0/P1/P2 z czasami (potwierdzenie 4 h/24 h/24 h, działanie 24 h/48 h/5 dni rob.), ścieżka krok po kroku z narzędziami panelu (A-25/A-26, N-14), kto decyduje, szablony A–D (w tym DSA art. 17 i odpowiedź dla Hetznera/CERT), test kwartalny. Zostaje: skrzynka abuse@verris.pl i test zgłoszenia (definicja ukończenia); formularz w stopce z landingiem (PB-06). | 2026-09-27 ZAMKNIĘTE: skrzynka abuse@verris.pl działa (przekierowanie na skrzynkę właściciela — potwierdzone przez właściciela 23.09 i 27.09); test zgłoszenia: formularz /zglos-naduzycie → ABUSE_REPORT_RECEIVED 24.09 (test-live-verris.pl, PHISHING) → decyzja w panelu obsługi 26.09 (N-13).</t>
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr">
@@ -8213,12 +8213,12 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>A-11</t>
+          <t>N-16</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Wyszukiwarka wolnych domen</t>
+          <t>SLA z zapisanymi kredytami</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>A — Domeny i konta</t>
+          <t>N — Wsparcie i ops</t>
         </is>
       </c>
       <c r="E96" s="10" t="inlineStr">
@@ -8249,12 +8249,12 @@
       </c>
       <c r="I96" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J96" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K96" s="10" t="inlineStr">
@@ -8264,12 +8264,12 @@
       </c>
       <c r="L96" s="11" t="inlineStr">
         <is>
-          <t>domains.controller.ts:54</t>
+          <t>sla-credit.scheduler.ts — wylicz() (progi §15, miesiąc kalendarzowy, okna konserwacyjne, 1 wypłata/usługę/miesiąc) + run() za flagą; GET /admin/sla/podglad + admin Ustawienia platformy → Podgląd kredytów SLA; live-readiness sla_credits (fail, gdy wyłączone); testy D2 sla-credit.scheduler.spec.ts + sla-credit.wylicz.spec.ts</t>
         </is>
       </c>
       <c r="M96" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-03 (kredyty SLA muszą być zgodne z opublikowanym regulaminem)</t>
         </is>
       </c>
       <c r="N96" s="11" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15). | 2026-09-27 PRODUKCJA po b0a556f: wyszukiwarka działa — „hvln-test-verris” → 32 wolne warianty z ceną rejestracji i odnowienia (brutto). Przyczyna „wszystko zajęte”: OpenProvider zwraca wyniki w innej kolejności niż w zapytaniu — dopasowanie po nazwie domeny, zapytania po 15 końcówek. Zostaje do pełnego testu z węzłem (decyzja właściciela). | 2026-10-04: D3 (sandbox OpenProvidera (api.sandbox.openprovider.nl), panel klienta prod, klient d3 czasowo na portfelu) — wyszukiwarka: 26 z 32 końcówek z cenami brutto. Po drodze: paczka 15 TLD „wszystko albo nic” gubiła .pl/.com, gdy jedna końcówka wisiała (.online/.shop &gt;40 s w sandboxie) → 36b8bca/9199355/99e38ec (limit 6 s, pojedynczo po błędzie paczki, budżet panelu 40 s); końcówki bez odpowiedzi „Nie sprawdzono” zamiast „Zajęta” → 9eb936d4.</t>
+          <t>OSŁABIONE: funkcja jest domyślnie martwa, a live-readiness nie ma checka SLA — flaga może zostać wyłączona bez żadnego sygnału. Regulamin obiecuje kredyty, kod ich nie nalicza. | 2026-09-23: kod liczył już według progów §15 (przepisany wcześniej), brakowało sygnału i podglądu. Dodane: podgląd bez zapisu na prawdziwych danych sond (do obejrzenia przed włączeniem) i blokujący check live-readiness — regulamin 1.1.0+ obiecuje rekompensatę automatyczną, więc wyłączona flaga nie może przejść niezauważona. Zostaje: obejrzeć podgląd na danych z działającego węzła i włączyć sla.creditsEnabled (sprint 18). | 2026-09-25: verris.pl w wielu miejscach obiecuje automatyczne rekompensaty — zostaje, ale preflight GO-LIVE blokuje start, dopóki sla.creditsEnabled≠1 (product-ops preflight, test preflight.spec.ts). | DECYZJA WŁAŚCICIELA 2026-09-25: włączamy rekompensaty na start — właściciel ustawia w panelu admina (Ustawienia → Platforma → Kredyty SLA) sla.creditsEnabled=1; preflight wtedy przejdzie. | Zamknięte 2026-09-25: właściciel włączył sla.creditsEnabled; admin → Gotowość do startu LIVE po deployu #160: „Rekompensaty SLA (automatyczne) — Włączone” (D3, produkcja). | 2026-09-27 KOD (31e5b2f): wyłączenie konserwacji tylko dla prac zapowiedzianych ≥48 h wcześniej i tylko w zapowiedzianych godzinach (§15 ust. 7); nieudane uznanie portfela zwalnia miesiąc do ponowienia. Test sla-kredyty.int-spec.ts. Rekompensaty na produkcji nadal wyłączone. | 2026-09-28 DECYZJA WŁAŚCICIELA: rekompensaty „na wniosek” wg regulaminu (bez automatu); tekst na verris.pl, blogu i w kampaniach poprawiony w 14 miejscach (46976c6).</t>
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr">
@@ -8291,31 +8291,31 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>PB-07</t>
+          <t>A-11</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>Treści i cennik na verris.pl</t>
+          <t>Wyszukiwarka wolnych domen</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>A — Domeny i konta</t>
         </is>
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>18</v>
@@ -8327,37 +8327,37 @@
       </c>
       <c r="I97" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J97" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K97" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L97" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>domains.controller.ts:54</t>
         </is>
       </c>
       <c r="M97" s="11" t="inlineStr">
         <is>
-          <t>PB-01 (cennik zależy od unit economics)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N97" s="11" t="inlineStr">
         <is>
-          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O97" s="11" t="inlineStr">
         <is>
-          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts. | 2026-09-27 ZAMKNIĘTE: treści zaakceptowane przez właściciela; /specyfikacja włączona (SPECYFIKACJA_OPUBLIKOWANA=true: menu, sitemap), wiersze po D3 nadal ukryte (SPEC_PO_WERYFIKACJI); /funkcje/sla na produkcji.</t>
+          <t>DECYZJA WŁAŚCICIELA 2026-09-23: konfiguracja OpenProvider (REGISTRAR_PROVIDER + dane API w .env.prod, wpisuje właściciel) razem z zakupem węzła w sprincie 18; do tego czasu wyszukiwarka za flagą. | 2026-09-25: preflight GO-LIVE blokuje start bez REGISTRAR_PROVIDER (strona oferuje rejestrację domen). Wyszukiwarka na verris.pl prowadzi do /dashboard/domains/buy?domain=… i panel wpisuje nazwę w wyszukiwarkę (wcześniej nazwa przepadała). /domeny: „bez blokad transferu” → blokadę włączasz i zdejmujesz sam (A-15). | 2026-09-27 PRODUKCJA po b0a556f: wyszukiwarka działa — „hvln-test-verris” → 32 wolne warianty z ceną rejestracji i odnowienia (brutto). Przyczyna „wszystko zajęte”: OpenProvider zwraca wyniki w innej kolejności niż w zapytaniu — dopasowanie po nazwie domeny, zapytania po 15 końcówek. Zostaje do pełnego testu z węzłem (decyzja właściciela). | 2026-10-04: D3 (sandbox OpenProvidera (api.sandbox.openprovider.nl), panel klienta prod, klient d3 czasowo na portfelu) — wyszukiwarka: 26 z 32 końcówek z cenami brutto. Po drodze: paczka 15 TLD „wszystko albo nic” gubiła .pl/.com, gdy jedna końcówka wisiała (.online/.shop &gt;40 s w sandboxie) → 36b8bca/9199355/99e38ec (limit 6 s, pojedynczo po błędzie paczki, budżet panelu 40 s); końcówki bez odpowiedzi „Nie sprawdzono” zamiast „Zajęta” → 9eb936d4.</t>
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr">
@@ -8369,12 +8369,12 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>PB-11</t>
+          <t>PB-07</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
+          <t>Treści i cennik na verris.pl</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8393,7 +8393,7 @@
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G98" s="10" t="n">
         <v>18</v>
@@ -8405,12 +8405,12 @@
       </c>
       <c r="I98" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J98" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K98" s="10" t="inlineStr">
@@ -8425,17 +8425,17 @@
       </c>
       <c r="M98" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-01 (cennik zależy od unit economics)</t>
         </is>
       </c>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
+          <t>Cennik zgodny z wynikiem PB-01. Specyfikacja techniczna publiczna, jak u cyber_Folks — to jest element zaufania, którego rynek oczekuje.</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
         <is>
-          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7. | 2026-09-27 PRODUKCJA (D4): Alerting → Contact points → Test: mail „[FIRING:1] TestAlert Grafana” od „Verris Alerts” dotarł na dominik@hvln.pl (21:10). Zamknięte.</t>
+          <t>Strona główna, cennik, specyfikacja techniczna pakietu, strona SLA. Narracja: cena stała, bez skoku po roku. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: /specyfikacja (tylko wiersze DZIAŁA; wiersze po D3 za SPEC_PO_WERYFIKACJI), ukryta flagą SPECYFIKACJA_OPUBLIKOWANA (404, poza menu i sitemapą). SLA: /funkcje/sla istnieje. Przy okazji: skrypt prod-sync-server-da-packages.sh dałby planowi verris-hosting limity starter — poprawione + test parytetu z da-package-spec.ts. | 2026-09-27 ZAMKNIĘTE: treści zaakceptowane przez właściciela; /specyfikacja włączona (SPECYFIKACJA_OPUBLIKOWANA=true: menu, sitemap), wiersze po D3 nadal ukryte (SPEC_PO_WERYFIKACJI); /funkcje/sla na produkcji.</t>
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr">
@@ -8447,12 +8447,12 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>PB-21</t>
+          <t>PB-11</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>DNS platformy i poczty na serwerze testowym</t>
+          <t>Bus factor: drugi kanał alertów i procedura zastępstwa</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8471,7 +8471,7 @@
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G99" s="10" t="n">
         <v>18</v>
@@ -8483,12 +8483,12 @@
       </c>
       <c r="I99" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J99" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K99" s="10" t="inlineStr">
@@ -8508,12 +8508,12 @@
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
+          <t>Alert testowy dociera dwoma kanałami. Dokument zastępstwa zawiera dostęp awaryjny i listę rzeczy, które muszą się dziać codziennie.</t>
         </is>
       </c>
       <c r="O99" s="11" t="inlineStr">
         <is>
-          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle. | ZAMKNIĘTE 2026-10-04 (D3 t1): NS platformy ns3/ns4.verris.pl (delegacja d3.hvln.pl, „Tryb NS: poprawny”); rekord dodany/usunięty bez duplikatu (F-01/F-02 30.09, usunięcie _dmarc 04.10 — serial strefy 2026100401); rozmiar skrzynki bez zmiany hasła (E-05); DKIM ze strefy, SPF/DMARC z kreatora (E-15/16/17); verris.pl jeden DMARC (p=none usunięty w OVH przez właściciela); decyzja: bez _spf.verris.pl (docs/VERRIS.md, 8bb0ea30). Przy okazji: raport poczty czytał strefę z cache resolvera (TTL 3600) — poprawka e7b47f48; naprawa asystenta (PB-17) do powtórki po wdrożeniu.</t>
+          <t>Alerty na więcej niż jeden adres, przetestowane. Dokument: co robi ktoś inny, gdy Ciebie nie ma przez tydzień. | 2026-09-23: Telegram jako drugi kanał w tym samym punkcie kontaktowym Grafany co e-mail (błąd jednego nie blokuje drugiego; znak życia X-31 raz dziennie też na Telegram); compose przekazuje TELEGRAM_BOT_TOKEN/CHAT_ID; strażnik routing-alertow.spec.ts (PB-11). Zastępcy nie ma (decyzja właściciela) — procedura awarii z telefonu w docs/ops/INCIDENT_RESPONSE.md; szukanie zastępcy po starcie. Zostaje: bot Telegrama + token w .env.prod i test alertu (D3). | DECYZJA WŁAŚCICIELA 2026-09-23: Telegram usunięty — alerty wyłącznie e-mailem. Konsekwencja: jeden kanał, więc awaria poczty (SMTP, skrzynka) wycisza też alerty; znak życia X-31 raz dziennie jest jedynym sposobem, by to zauważyć (brak maila = coś nie działa). Powrót do drugiego kanału: odtworzyć z commita 7d63cd7. | 2026-09-27 PRODUKCJA (D4): Alerting → Contact points → Test: mail „[FIRING:1] TestAlert Grafana” od „Verris Alerts” dotarł na dominik@hvln.pl (21:10). Zamknięte.</t>
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr">
@@ -8525,12 +8525,12 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>PB-24</t>
+          <t>PB-21</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
+          <t>DNS platformy i poczty na serwerze testowym</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8549,7 +8549,7 @@
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G100" s="10" t="n">
         <v>18</v>
@@ -8561,12 +8561,12 @@
       </c>
       <c r="I100" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K100" s="10" t="inlineStr">
@@ -8586,12 +8586,12 @@
       </c>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
+          <t>Na serwerze testowym: rekord dodany i usunięty z panelu bez duplikatu; zmiana rozmiaru skrzynki zostawia hasło; kreator poczty pokazuje DKIM ze strefy i zapisuje SPF/DMARC; verris.pl ma jeden DMARC; decyzja o _spf.verris.pl zapisana w docs/VERRIS.md. Po D3 F-01/F-02, E-05, E-15/16/17 przechodzą w macierzy na PARYTET.</t>
         </is>
       </c>
       <c r="O100" s="11" t="inlineStr">
         <is>
-          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
+          <t>Odłożone decyzją właściciela 2026-09-23 do chwili, gdy jest serwer testowy. (1) Decyzja: wspólny rekord _spf.verris.pl (include platformy, łatwa zmiana IP) albo zostajemy przy a/mx/ip4 per klient — dziś _spf.verris.pl nie istnieje. (2) verris.pl w OVH: dwa rekordy DMARC (p=none i p=quarantine) — odbiorcy ignorują oba; zostawić jeden. (3) Nameservery platformy (hosting.ns1/ns2) ustawione — od nich zależy, czy kreator poczty proponuje zapis do strefy. (4) D3 na żywym DirectAdminie: dodanie i usunięcie rekordu (CMD_API_DNS_CONTROL, edycja create-then-delete), zmiana rozmiaru skrzynki bez passwd, klucz DKIM w strefie po włączeniu DKIM. (5) Naprawy asystenta PB-17 (SPF/DMARC jednym kliknięciem + Cofnij) na żywej strefie. (6) Zawieszenie i odwieszenie usługi z panelu admina (A-25/A-26) na żywym koncie DA. (7) Sprint 12–14 na żywym węźle: kopia bezpieczeństwa przed odtworzeniem (H-09), publikacja stagingu z kopią bazy (I-11), zmiana hasła FTP (C-18), pakowanie plików (C-11), pojemność węzła z agenta lve-agent/1.1 (NODE-03). (8) PB-22: pieczęć zaufania na działającej stronie klienta (D3) — tprstudio.pl wygasła 2026-09-23, więc pełną pieczęć sprawdzamy dopiero na stronie na nowym węźle. | ZAMKNIĘTE 2026-10-04 (D3 t1): NS platformy ns3/ns4.verris.pl (delegacja d3.hvln.pl, „Tryb NS: poprawny”); rekord dodany/usunięty bez duplikatu (F-01/F-02 30.09, usunięcie _dmarc 04.10 — serial strefy 2026100401); rozmiar skrzynki bez zmiany hasła (E-05); DKIM ze strefy, SPF/DMARC z kreatora (E-15/16/17); verris.pl jeden DMARC (p=none usunięty w OVH przez właściciela); decyzja: bez _spf.verris.pl (docs/VERRIS.md, 8bb0ea30). Przy okazji: raport poczty czytał strefę z cache resolvera (TTL 3600) — poprawka e7b47f48; naprawa asystenta (PB-17) do powtórki po wdrożeniu.</t>
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr">
@@ -8603,12 +8603,12 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>PB-25</t>
+          <t>PB-24</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>White label na węźle — klient nie widzi DirectAdmina</t>
+          <t>KSC/NIS2: wpis do wykazu podmiotów kluczowych</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8627,7 +8627,7 @@
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G101" s="10" t="n">
         <v>18</v>
@@ -8639,12 +8639,12 @@
       </c>
       <c r="I101" s="10" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J101" s="10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K101" s="10" t="inlineStr">
@@ -8664,12 +8664,12 @@
       </c>
       <c r="N101" s="11" t="inlineStr">
         <is>
-          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
+          <t>Wpis w wykazie przed upływem 6 miesięcy od pierwszej domeny/DNS dla klienta; termin zapisany w tym zadaniu z datą.</t>
         </is>
       </c>
       <c r="O101" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz. | ZAMKNIĘTE 2026-10-04 (D3 na węźle testowym t1; na węźle #1 to samo przychodzi z profilu — kontrola w PB-02): phpMyAdmin z panelu (jednorazowy link) i webmail bez nazwy/portu DirectAdmina; linki do panelu DA puste z API; zawieszone konto → „Strona tymczasowo niedostępna” (verris-suspended-page), odwieszenie bez obciążenia; nowa poddomena wl3.d3.hvln.pl → „Witamy na stronie … hosting verris” po haku subdomain_create_post (b2ead35 + 0f7f032 dla układu DA 1.710). Uwaga: adres phpMyAdmin/webmaila to nazwa węzła (t1.verris.pl).</t>
+          <t>Wg FAQ KSC (cyber.gov.pl) podmiot świadczący usługi rejestracji nazw domen i dostawca usług DNS = podmiot kluczowy niezależnie od wielkości. Decyzja właściciela 2026-09-23: wpis w ciągu 6 miesięcy od uruchomienia sprzedaży domen / DNS dla klientów (sprint 18/19), nie przed 3.10.2026 — ryzyko przyjęte świadomie. Materiał: docs/legal/nis2-ksc-assessment.md (10 obszarów art. 21). Do zrobienia: data uruchomienia usług → termin wpisu; osoba kontaktowa ds. cyberbezpieczeństwa; kontakt 24/7 do incydentów; procedura zgłaszania incydentów do CSIRT (24 h / 72 h). | 2026-09-25: procedura zgłaszania incydentu poważnego w docs/ops/INCIDENT_RESPONSE.md (24 h wczesne ostrzeżenie / 72 h zgłoszenie / sprawozdanie końcowe w miesiąc — NIS2 art. 23; S46; rejestr docs/ops/incydenty/; test kwartalny; klienci i RODO równolegle). nis2-ksc-assessment.md poprawione wg komunikatu MC: wejście w życie 10.04.2026 (było 3.04), wykaz-ksc.gov.pl, S46 od 12.06.2026, koniec okresu dostosowawczego 3.04.2027, audyt do 3.04.2028; DNS/rejestracja domen = kluczowy niezależnie od wielkości (art. 5 ust. 1 pkt 4), termin wpisu 6 mies. od spełnienia przesłanek (art. 7c ust. 1). Zostaje (właściciel): potwierdzić osobę do kontaktów i telefon 24/7 we wniosku, skrzynka security@, konto S46 po wpisie. | 2026-09-26: projekt wniosku do Wykazu KSC — pola wg FAQ KSC pyt. 2.10 (wypełnione / do uzupełnienia przez właściciela: e-Doręczenia, IP po zakupie węzła, telefon 24/7, PESEL administratora S46 tylko w formularzu), termin od przesłanki, osobny wątek art. 16b (reseller domen) — docs/legal/drafts/DO_ZATWIERDZENIA_PB-24_wniosek-ksc.md (DO ZATWIERDZENIA, nic nie opublikowane/złożone).</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
@@ -8681,12 +8681,12 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>PB-06</t>
+          <t>PB-25</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Landing /przenies-strone</t>
+          <t>White label na węźle — klient nie widzi DirectAdmina</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8705,10 +8705,10 @@
         </is>
       </c>
       <c r="F102" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G102" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H102" s="10" t="inlineStr">
         <is>
@@ -8717,12 +8717,12 @@
       </c>
       <c r="I102" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J102" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K102" s="10" t="inlineStr">
@@ -8737,17 +8737,17 @@
       </c>
       <c r="M102" s="11" t="inlineStr">
         <is>
-          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
+          <t>Na węźle #1: logowanie do panelu hostingowego, phpMyAdmin i webmaila z panelu klienta nie pokazuje nazwy ani portu DirectAdmina; nowa domena i konto zawieszone pokazują strony Verris; zrzuty w dowodzie.</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji. | 2026-09-27 ZAMKNIĘTE: treści zaakceptowane przez właściciela (docs/marketing/akceptacja-tresci-2026-09.md); /przenies-strone na produkcji (200).</t>
+          <t>Decyzja właściciela 2026-09-24: pełny white label. Teksty dla klienta (verris.pl, panel, maile, dokumenty prawne) wyczyszczone tego dnia i pilnowane strażnikiem bez-nazwy-directadmina.spec.ts. Na węźle zostaje: panel hostingowy pod własną nazwą na 443 zamiast host:2222 (proxy), branding Evolution wg ops/docs/DA_EVOLUTION_BRANDING.md, phpMyAdmin i webmail pod własną nazwą, własne strony domyślne (nowa domena, konto zawieszone, wspólny IP), przegląd maili systemowych DA wysyłanych do użytkowników. Nie twierdzimy, że silnik hostingu jest nasz. | ZAMKNIĘTE 2026-10-04 (D3 na węźle testowym t1; na węźle #1 to samo przychodzi z profilu — kontrola w PB-02): phpMyAdmin z panelu (jednorazowy link) i webmail bez nazwy/portu DirectAdmina; linki do panelu DA puste z API; zawieszone konto → „Strona tymczasowo niedostępna” (verris-suspended-page), odwieszenie bez obciążenia; nowa poddomena wl3.d3.hvln.pl → „Witamy na stronie … hosting verris” po haku subdomain_create_post (b2ead35 + 0f7f032 dla układu DA 1.710). Uwaga: adres phpMyAdmin/webmaila to nazwa węzła (t1.verris.pl).</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr">
@@ -8759,12 +8759,12 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>PB-09</t>
+          <t>PB-06</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>Baza wiedzy — 20 artykułów startowych</t>
+          <t>Landing /przenies-strone</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8779,7 +8779,7 @@
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
@@ -8795,12 +8795,12 @@
       </c>
       <c r="I103" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J103" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K103" s="10" t="inlineStr">
@@ -8815,17 +8815,17 @@
       </c>
       <c r="M103" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-07 (landing korzysta z ustalonego cennika)</t>
         </is>
       </c>
       <c r="N103" s="11" t="inlineStr">
         <is>
-          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
+          <t>Strona opublikowana, pomiar działa, formularz i CTA prowadzą do rejestracji. Żadne twierdzenie na stronie nie jest oznaczone w macierzy jako LUKA lub ATRAPA.</t>
         </is>
       </c>
       <c r="O103" s="11" t="inlineStr">
         <is>
-          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”. | 2026-09-27 ZAMKNIĘTE: seed na produkcji (13 kategorii, 1 nowy artykuł, 37 odświeżonych). Uwaga: rejestracja-domeny i transfer-domeny opisują funkcję aktywną po włączeniu OpenProvider (A-08/A-09).</t>
+          <t>Strona docelowa kampanii Google Ads na osi migracji. Treść oparta na realnych przewagach z audytu, nie na obietnicach. | 2026-09-25 PRZYGOTOWANE DO AKCEPTACJI: audyt 38 twierdzeń (/, /hosting, /cennik, /przenies-strone) wobec macierzy — 13 poprawionych (tryb ECO to polityka kopii, nie skalowanie; Apple/Google Pay niewłączone; przypomnienia 7/3/1 dzień; rezygnacja z odnowienia w dwóch kliknięciach; zwrot przez wsparcie; domena nie odnowi się bez decyzji). Rabat na start zostaje (decyzja właściciela) — przekaz: odnowienie zawsze po cenie z cennika. Lista w docs/marketing/akceptacja-tresci-2026-09.md. Pomiar: generate_lead po wysłaniu formularza migracji (GTM, Consent Mode v2). Publikacja po akceptacji. | 2026-09-27 ZAMKNIĘTE: treści zaakceptowane przez właściciela (docs/marketing/akceptacja-tresci-2026-09.md); /przenies-strone na produkcji (200).</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr">
@@ -8837,12 +8837,12 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>PB-19</t>
+          <t>PB-09</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
+          <t>Baza wiedzy — 20 artykułów startowych</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
@@ -8861,7 +8861,7 @@
         </is>
       </c>
       <c r="F104" s="10" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G104" s="10" t="n">
         <v>19</v>
@@ -8873,12 +8873,12 @@
       </c>
       <c r="I104" s="10" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J104" s="10" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K104" s="10" t="inlineStr">
@@ -8898,12 +8898,12 @@
       </c>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
+          <t>20 artykułów opublikowanych i zaindeksowanych do asystenta AI. Każdy opisuje funkcję, która w macierzy ma status DZIAŁA.</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
         <is>
-          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
+          <t>Artykuły pokrywające najczęstsze pytania pierwszego tygodnia: skierowanie domeny, SSL, poczta, FTP, backup, migracja, faktury. | 2026-09-23: seed ma 37 artykułów (apps/api/src/cli/seed-kb-cms.ts, indeksowane do asystenta). Przegląd twierdzeń wobec macierzy: usunięte obietnice funkcji, których nie ma lub nie są gotowe — SFTP/SSH (C-21 CZĘŚCIOWE; teraz FTPS), VPS i osobna poczta (Q-06 FLAGA), włączanie rozszerzeń PHP i CloudLinux Selector (B-04 BRAK), phpinfo w panelu (B-06), białe/czarne listy antyspamu (E-12), kopia przy forwarderze, „wildcard płatny”; faktury opisane zgodnie z §9 ust. 4 (dokument rozliczeniowy + faktura z programu księgowego). ZOSTAJE: rejestracja-domeny i transfer-domeny opisują A-08/A-09 (FLAGA) — prawdziwe dopiero po włączeniu rejestratora (A-11, sprint 18); uruchomić seed na produkcji (node apps/api/dist-cli/cli/seed-kb-cms.js) — nadpisuje tylko artykuły autorstwa „Zespół Verris”. | 2026-09-27 ZAMKNIĘTE: seed na produkcji (13 kategorii, 1 nowy artykuł, 37 odświeżonych). Uwaga: rejestracja-domeny i transfer-domeny opisują funkcję aktywną po włączeniu OpenProvider (A-08/A-09).</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">
@@ -8915,12 +8915,12 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>PB-10</t>
+          <t>PB-19</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
+          <t>Widok strony: ruch, TTFB, błędy 5xx, technologia i logi z węzła</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -8939,20 +8939,24 @@
         </is>
       </c>
       <c r="F105" s="10" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G105" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="H105" s="10" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="H105" s="10" t="inlineStr">
+        <is>
+          <t>Faza 3 — Wejście na rynek</t>
+        </is>
+      </c>
       <c r="I105" s="10" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="J105" s="10" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="K105" s="10" t="inlineStr">
@@ -8967,17 +8971,17 @@
       </c>
       <c r="M105" s="11" t="inlineStr">
         <is>
-          <t>PB-06 (kampania kieruje na landing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N105" s="11" t="inlineStr">
         <is>
-          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
+          <t>Na działającym węźle produkcyjnym: widok strony pokazuje ruch 7 dni, TTFB i 5xx z prawdziwych logów, wykrytą technologię i zakładkę „Logi”; brak danych = „—”, nie zero; testy parsera logów i detekcji technologii w CI; sprawdzone na D3 (serwer).</t>
         </is>
       </c>
       <c r="O105" s="11" t="inlineStr">
         <is>
-          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
+          <t>Braki makiety widoku strony (docs/design/wzorzec-panelu.html), których API nie ma, bo wymagają węzła: (1) odwiedziny, mediana TTFB i błędy 5xx per domena z logów serwera WWW przez agenta; (2) rozpoznanie technologii strony (WordPress, PrestaShop, Laravel, HTML, przekierowanie) skanem plików i narzędzia dopasowane do technologii; (3) zakładka „Logi” — log błędów i dostępu per domena. Dziś panel pokazuje tylko to, co realnie istnieje (docs/VERRIS.md, sekcja „Otwarte”). | 2026-09-25 KOD (D2): zadanie SITE_STATS + ops/scripts/node-site-stats.sh — technologia (WordPress/PrestaShop/Joomla/Drupal/Nextcloud/MediaWiki/Laravel/PHP/HTML/domyślna Verris, z wersją) sprawdzana jako klient; ruch 7 dni (żądania, odwiedzający = unikalne IP, 5xx) z logu DirectAdmina /var/log/httpd/domains/&lt;domena&gt;.log (combined), ścieżki bez parametrów; mediana TTFB z 5 żądań z samego serwera (127.0.0.1 + Host). Panel: widok strony → Przegląd → „Ruch i wydajność — 7 dni” (brak logu = „—”), nowa zakładka „Logi” (log dostępu i błędów tej domeny). Testy parsera i detekcji: site-stats.service.spec.ts. ZOSTAJE: D3 na węźle.</t>
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr">
@@ -8989,69 +8993,69 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>Z-18</t>
+          <t>PB-12</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
+          <t>Runbook startu i decyzja GO</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t>Z — Pass adwersaryjny</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>BLOKER STARTU</t>
+          <t>BLOKER BIZNESOWY</t>
         </is>
       </c>
       <c r="F106" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G106" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H106" s="10" t="inlineStr"/>
       <c r="I106" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J106" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K106" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L106" s="11" t="inlineStr">
         <is>
-          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M106" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-05 (decyzja GO po przejściu ścieżki na produkcji)</t>
         </is>
       </c>
       <c r="N106" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Każdy z 11 blokerów ma wpis: co zrobiono, gdzie jest dowód, kto potwierdził. Bez formuły „warunkowe GO”.</t>
         </is>
       </c>
       <c r="O106" s="11" t="inlineStr">
         <is>
-          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md | 2026-10-03: D3 na t1 — zerwane połączenie z DA przy zakładaniu (REJECT na :2222 do pierwszej odmowy): przed poprawką jedna odmowa spalała 3 próby w 15 s na otwartym bezpieczniku węzła → twarda porażka (przy portfelu zwrot+FAILED); po 80ef14a (opóźnienie ponowienia &gt; okno bezpiecznika) próba 1 RETRYING, próba 2 po ~2,5 min zakłada konto (z18b.d3.hvln.pl). Admin „Ponów” zeruje teraz licznik prób.</t>
+          <t>Domknięcie: przegląd wszystkich blokerów z dowodem zamknięcia, decyzja GO/NO-GO zapisana z datą.</t>
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr">
@@ -9063,69 +9067,69 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>NODE-02</t>
+          <t>PB-10</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>`main()` nie sprawdza kodów powrotu</t>
+          <t>Kampania gads-search-hosting-202607 — uruchomienie</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
         <is>
-          <t>audyt</t>
+          <t>poza audytem</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t>Q — Przewaga</t>
+          <t>Praca spoza audytu</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>ŚREDNI</t>
         </is>
       </c>
       <c r="F107" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G107" s="10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H107" s="10" t="inlineStr"/>
       <c r="I107" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J107" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2027-01-08</t>
         </is>
       </c>
       <c r="K107" s="10" t="inlineStr">
         <is>
-          <t>CZĘŚCIOWE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L107" s="11" t="inlineStr">
         <is>
-          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M107" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB-06 (kampania kieruje na landing)</t>
         </is>
       </c>
       <c r="N107" s="11" t="inlineStr">
         <is>
-          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
+          <t>Kampania utworzona wstrzymana, konwersje podpięte, budżet i stawki ustawione. Start dopiero po PB-05.</t>
         </is>
       </c>
       <c r="O107" s="11" t="inlineStr">
         <is>
-          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
+          <t>Konfiguracja kampanii wyszukiwarkowej, budżet 500–1000 zł/mies., oś przekazu: migracja bez przestoju.</t>
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr">
@@ -9137,12 +9141,12 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>Z-18</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>LiteSpeed / serwer o wysokiej wydajności</t>
+          <t>Prawdziwa przyczyna błędu provisioningu nie ginie po drodze (część)</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -9152,16 +9156,16 @@
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Z — Pass adwersaryjny</t>
         </is>
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>WYSOKA</t>
+          <t>BLOKER STARTU</t>
         </is>
       </c>
       <c r="F108" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G108" s="10" t="n">
         <v>21</v>
@@ -9169,12 +9173,12 @@
       <c r="H108" s="10" t="inlineStr"/>
       <c r="I108" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J108" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K108" s="10" t="inlineStr">
@@ -9184,7 +9188,7 @@
       </c>
       <c r="L108" s="11" t="inlineStr">
         <is>
-          <t>decyzja infrastrukturalna, poza kodem panelu; D3 t1 29.09 (panel klienta, d3.hvln.pl): LiteSpeed Enterprise (Server: LiteSpeed), CacheRoot z profilu [OK], strona główna WordPressa z x-litespeed-cache: hit</t>
+          <t>apps/api/src/subscriptions/provisioning-error.ts — BladEtapuProvisioningu (etap, przyczyna, message z doklejoną przyczyną); provisioning-queue.service.ts — kategoriaBledu(err), klasyfikacja obiektu zamiast napisu, pole przyczyna w audycie ponowienia i twardej porażki; provisioning.service.ts — trzy etapy DA (ensureUserPackage, createAccount, setAccountLimits) bez prania przyczyny; apps/api/src/test/blad-provisioningu-nie-klamie.spec.ts (18). BRAK: dowodu D3 — nie ma węzła obliczeniowego, więc ścieżki provisioningu nie da się dziś przejść na produkcji.</t>
         </is>
       </c>
       <c r="M108" s="11" t="inlineStr">
@@ -9199,7 +9203,7 @@
       </c>
       <c r="O108" s="11" t="inlineStr">
         <is>
-          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
+          <t>2026-09-24 PRZEGLĄD „CZEGO NIE OBEJMUJE” (Stripe, migracje, autoskalowanie + sąsiednie ścieżki pieniędzy): (1) twarda porażka provisioningu kończyła się zwykłym throw — BullMQ ponawiał i zakładał konto po zwrocie środków; teraz UnrecoverableError; (2) 503 z wyboru węzła (polski komunikat) był „trwały” → zwrot przy pierwszej próbie; teraz status HTTP przed prozą; (3) odnowienie portfelem: błąd bazy = PAST_DUE + mail „płatność nieudana”; teraz tylko ConflictException; (4) odnowienie VPS: catch {} + po karencji deleteServer — błąd bazy mógł skasować serwer klienta; (5) usunięcie konta DA (RODO): „Server not found”/„brak …” uznawane za „użytkownika nie ma”; (6) autoskalowanie: brak środków po typie. Stripe (webhooki z ewidencją i ponowieniami) bez zastrzeżeń. 18 testów zachowania. Pozycja nadal czeka na D3 na węźle #1. | Stan 2026-08-23: NAPRAWIONE W KODZIE (D2), POZYCJA OTWARTA — bloker startu do czasu dowodu D3 na węźle #1 (sprint 8). Krytyczność nadana decyzją właściciela produktu 2026-08-23. | JAK TO WYSZŁO: X-30 naprawiło alerting i w ciągu dziesięciu minut zapaliła się pierwsza reguła z PRAWDZIWEGO powodu — VerrisProvisioningQueueFailed. W kolejce leżały cztery martwe joby, a w panelu operatora stało przy nich „DirectAdmin package "starter" is missing on the node and could not be created automatically". W audycie stało co innego: ensureUserPackage / connect ECONNREFUSED 62.238.0.223:2222 (2026-07-07 i 07-10) oraz createAccount / „DirectAdmin API Error: Unable to Create User — A valid IP was not provided" (2026-05-30). Węzeł nie przyjmował połączeń; z pakietem nie było nic nie tak. Same joby są nieszkodliwe — konto testowe właściciela, domeny test.pl/testowa.pl/hvln.pl, sprzed trzech miesięcy, z czasów gdy węzeł testowy jeszcze istniał (dziś nie ma go wcale). Ale komunikat doprowadził mnie do hipotezy o złym mapowaniu planów na pakiety DA — całkowicie chybionej. Na tym polega koszt takiego błędu: nie na tym, że coś nie działa, tylko że wszyscy patrzą nie tam. | MECHANIZM: provisioning.service.ts łapał prawdziwy błąd, zapisywał go do audytu i rzucał dalej STAŁY NAPIS. Prawda zostawała w bazie, w górę szła zmyślona przyczyna. A wyżej: const errCategory = categorizeProvisioningError(msg) — klasyfikator dostawał ten wyprany napis. Jest napisany POPRAWNIE, ma econnrefused na liście błędów przejściowych; tylko nigdy nie widzi tego słowa. | DLACZEGO DOTYKA PIENIĘDZY: przy kliencie i chwilowym zerwaniu sieci — próba 1 → ECONNREFUSED przebrany za brak pakietu → permanent → ścieżka twardej porażki JUŻ PRZY PIERWSZEJ PRÓBIE: subskrypcja na FAILED, ZWROT ŚRODKÓW do portfela, status PENDING_PAYMENT; potem throw err i BullMQ i tak ponawia (attempts: 3, backoff wykładniczy); próba 2 przechodzi, konto powstaje, provisioning.service.ts:299 ustawia subskrypcję na ACTIVE. Klient ma działający hosting i odzyskane pieniądze, a zwrot jest idempotentny (sub-{id}-initial-refund), więc nic go nie cofnie. Wada uśpiona — nie ma dowodu, że się zdarzyła (te joby padły do końca, węzeł był wyłączony na dobre) — ale leży dokładnie na ścieżce pierwszego płacącego klienta. | RODZINA, NOWY WARIANT: to NIE jest „kontrola, która melduje zamiast zatrzymywać" (X-14, X-23, H-19, X-27), gdzie mechanizm istniał i niczego nie bramkował. To POPRAWNA KONTROLA, KTÓREJ SIĘ KŁAMIE: guard dobry, decyzja dobra, lista wyjątków kompletna — a wejście wyprane po drodze. Blisko też rodzinie „strażnik dopasowuje własną prozę" (dziesiąte wystąpienie): jeden z trzech komunikatów był ułożony tak, żeby TRAFIĆ w listę przejściowych — 'CloudLinux LVE limits could not be applied on this node.' kontra lower.includes('cloudlinux lve limits could not be applied'). Działało przypadkiem, dopóki ktoś nie poprawiłby zdania. | POPRAWKA: BladEtapuProvisioningu(etap, przyczyna, komunikatDlaCzlowieka) — klasa niosąca ORYGINALNĄ treść błędu; kategoriaBledu(err) pyta obiekt o przyczynę i dopiero na niej odpala istniejący klasyfikator, a napis zostaje ścieżką zapasową. Przyczyna jest DOKLEJONA także do message, bo panel pokazuje job.failedReason z BullMQ (czyli Error.message), a failedCategory liczy się z tego samego napisu — gdyby przyczyna została tylko we właściwości, panel dalej opowiadałby zmyśloną historię. Audyt dostał osobne pole przyczyna obok error. | Czerwieni się na starym kodzie: 4 z 18. Czternaście przechodziło, bo dotyczą zachowania kategoriaBledu, której przed poprawką nie było — redness siedzi w asercjach strukturalnych. Mówię o tym wprost, żeby „4 z 18" nie wyglądało słabiej, niż jest. | CZEGO NIE OBEJMUJE: innych miejsc, gdzie prawdziwy błąd może być prany (Stripe, migracje, autoskalowanie mają własne bloki catch i nie były przeglądane pod tym kątem — warte osobnego przejścia); sensowności samego zwrotu przy twardej porażce (zwrot jest właściwy, gdy błąd NAPRAWDĘ jest trwały — ta pozycja naprawia rozpoznanie, nie decyzję); czterech martwych jobów w kolejce (sprzątane po tej poprawce, decyzją właściciela produktu, żeby czyścić już na kodzie zapisującym prawdziwą przyczynę). | JAK ZAMKNĄĆ: na węźle #1 uruchomić provisioning, przerwać połączenie do DA w trakcie i pokazać w audycie PONOWIENIE zamiast zwrotu środków, a potem konto założone przy drugiej próbie. Dokumentacja: docs/archiwum/zadania/Z-18-blad-provisioningu-nie-klamie.md | 2026-10-03: D3 na t1 — zerwane połączenie z DA przy zakładaniu (REJECT na :2222 do pierwszej odmowy): przed poprawką jedna odmowa spalała 3 próby w 15 s na otwartym bezpieczniku węzła → twarda porażka (przy portfelu zwrot+FAILED); po 80ef14a (opóźnienie ponowienia &gt; okno bezpiecznika) próba 1 RETRYING, próba 2 po ~2,5 min zakłada konto (z18b.d3.hvln.pl). Admin „Ponów” zeruje teraz licznik prób.</t>
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr">
@@ -9211,12 +9215,12 @@
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>J-04</t>
+          <t>NODE-02</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>HTTP/3</t>
+          <t>`main()` nie sprawdza kodów powrotu</t>
         </is>
       </c>
       <c r="C109" s="10" t="inlineStr">
@@ -9226,12 +9230,12 @@
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t>J — Wydajność i cache</t>
+          <t>Q — Przewaga</t>
         </is>
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNIA</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F109" s="10" t="n">
@@ -9243,22 +9247,22 @@
       <c r="H109" s="10" t="inlineStr"/>
       <c r="I109" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J109" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K109" s="10" t="inlineStr">
         <is>
-          <t>DZIAŁA</t>
+          <t>CZĘŚCIOWE</t>
         </is>
       </c>
       <c r="L109" s="11" t="inlineStr">
         <is>
-          <t>poza kodem panelu; D3 t1 29.09 (panel klienta, d3.hvln.pl): brak alt-svc, połączenia po h2 — firewalld nie przepuszczał UDP 443; poprawka 68c7e95 (profil + hardening) czeka na push i profil; D3 t1 29.09 wieczór po profilu: curl -sI https://d3.hvln.pl → alt-svc: h3=":443", LiteSpeed nasłuchuje na UDP 443 (IPv4 i IPv6), firewalld przepuszcza 443/udp</t>
+          <t>ops/scripts/lib/przerwij-po-etapie.sh — przerwij_po_etapie zamienia zebrane [FAIL] w exit 1; node-onboard-live.sh main() — bramka po preflight_stack, run_security_hardening, ensure_da_ip; nieudana rejestracja IP w DA z log_warn na log_fail; node-live-readiness.sh main() — bramka po preflight (python3/curl); obie paczki wymagaja lib/przerwij-po-etapie.sh; test apps/api/src/test/instalator-wezla-zatrzymuje-sie.spec.ts</t>
         </is>
       </c>
       <c r="M109" s="11" t="inlineStr">
@@ -9268,12 +9272,12 @@
       </c>
       <c r="N109" s="11" t="inlineStr">
         <is>
-          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
+          <t>Ograniczenie opisane w uwagach macierzy zniknęło; test potwierdza zachowanie także w scenariuszu awaryjnym.</t>
         </is>
       </c>
       <c r="O109" s="11" t="inlineStr">
         <is>
-          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
+          <t>Przepisane do macierzy 2026-08-28 w ramach X-49 — pozycja powstala 2026-08-26 i do tego dnia istniala WYLACZNIE w dashboardzie, poza zasiegiem straznikow repozytorium. Obszar: instalator węzła. Krytycznosc i naklad zostaly puste SWIADOMIE: dashboard ich nie niosl, a wpisanie ich teraz byloby zgadywaniem. Do uzupelnienia przy najblizszym przegladzie tej pozycji. | TRESC ZE ZRODLA: `main()` nie sprawdza kodów powrotu. W `node-onboard-live.sh` i `node-live-readiness.sh` funkcje zwracają `1`, ale `main` leci dalej i dopiero na końcu drukuje `[FAIL]`. Instalacja kontynuuje po nieudanym preflighcie. Ta sama rodzina co SEC-01: kontrola wykrywa problem i nie zatrzymuje procesu. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Sprawdzanie kodow powrotu w main() obu skryptow. Male, ale instalacja kontynuuje po nieudanym preflighcie — dotyka PB-02 w W3. | 2026-09-22 KOREKTA OPISU: 'main() nie sprawdza kodow powrotu' bylo nieprecyzyjne — oba skrypty maja set -Eeuo pipefail, wiec funkcja z return 1 KONCZY skrypt (sprawdzone na bashu). Prawdziwa dziura: log_fail ustawia FAIL=1 bez return, a set -e tego nie widzi — preflight z brakujacym python3/curl przechodzil do instalacji agenta, a nieudany sync pakietow DA do readiness. Weryfikacja na koncu readiness swiadomie ZBIERA wszystkie usterki i odmawia raz (print_final_summary -&gt; return 1) — to zostaje, przerwanie po pierwszej kazaloby naprawiac je po jednej. POPRAWKA: bramka po kazdym etapie-bramce + IP w DA jako [FAIL] (bez IP kazde zakladanie konta konczy sie 'A valid IP was not provided' — poczatek Z-18). D2 2026-09-22: bramka lokalna zielona (886 testow, w tym 8 z instalator-wezla-zatrzymuje-sie.spec.ts); D3 przy onboardzie wezla #1 (PB-02).</t>
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr">
@@ -9285,12 +9289,12 @@
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji PHP dla całego konta</t>
+          <t>LiteSpeed / serwer o wysokiej wydajności</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
@@ -9300,12 +9304,12 @@
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t>B — Runtime WWW</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E110" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WYSOKA</t>
         </is>
       </c>
       <c r="F110" s="10" t="n">
@@ -9317,12 +9321,12 @@
       <c r="H110" s="10" t="inlineStr"/>
       <c r="I110" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J110" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K110" s="10" t="inlineStr">
@@ -9332,7 +9336,7 @@
       </c>
       <c r="L110" s="11" t="inlineStr">
         <is>
-          <t>services.controller.ts:125; D3 t1 28.09: FAIL — selektor bez alt-php (profil nie instalował els-php-release/alt-phpXX na CL10), panel pokazywał wersję mimo błędu → profil + PHP_APPLY cofa wersję (int: php-odrzucona-zmiana.int-spec.ts); retest po profilu; D3 t1 (d3.hvln.pl) 28.09 23:31: PHP 8.2 dla konta z panelu → strona zwraca 8.2.33 na LiteSpeed (PHP_APPLY zakończone); odrzucona zmiana cofa wersję (int)</t>
+          <t>decyzja infrastrukturalna, poza kodem panelu; D3 t1 29.09 (panel klienta, d3.hvln.pl): LiteSpeed Enterprise (Server: LiteSpeed), CacheRoot z profilu [OK], strona główna WordPressa z x-litespeed-cache: hit</t>
         </is>
       </c>
       <c r="M110" s="11" t="inlineStr">
@@ -9347,7 +9351,7 @@
       </c>
       <c r="O110" s="11" t="inlineStr">
         <is>
-          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
+          <t>koszt licencji — pozycja do unit economics | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — definicja ukonczenia dla b.d. to weryfikacja na produkcji z timestampem (D3), nie implementacja. Wykonalne na wezle #1. | 2026-09-25 (wg oficjalnej dokumentacji LiteSpeed dla DirectAdmin): profil węzła sprawdzał /usr/local/lsws/conf/httpd_config.conf — plik OpenLiteSpeed; na LSWS Enterprise (webserver=litespeed) go nie ma, więc konfiguracja cache nigdy się nie wykonywała. Teraz CacheRoot serwera w /etc/httpd/conf/extra/httpd-includes.conf i vhostów w templates/custom/cust_httpd.CUSTOM.2.pre, potem custombuild rewrite_confs — dokładnie jak w docs.litespeedtech.com/lsws/cp/directadmin/configuration/. D3 na węźle.</t>
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr">
@@ -9359,31 +9363,31 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>PB-02</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
+          <t>HTTP/3</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>J — Wydajność i cache</t>
         </is>
       </c>
       <c r="E111" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>ŚREDNIA</t>
         </is>
       </c>
       <c r="F111" s="10" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G111" s="10" t="n">
         <v>21</v>
@@ -9391,22 +9395,22 @@
       <c r="H111" s="10" t="inlineStr"/>
       <c r="I111" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J111" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K111" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L111" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>poza kodem panelu; D3 t1 29.09 (panel klienta, d3.hvln.pl): brak alt-svc, połączenia po h2 — firewalld nie przepuszczał UDP 443; poprawka 68c7e95 (profil + hardening) czeka na push i profil; D3 t1 29.09 wieczór po profilu: curl -sI https://d3.hvln.pl → alt-svc: h3=":443", LiteSpeed nasłuchuje na UDP 443 (IPv4 i IPv6), firewalld przepuszcza 443/udp</t>
         </is>
       </c>
       <c r="M111" s="11" t="inlineStr">
@@ -9416,12 +9420,12 @@
       </c>
       <c r="N111" s="11" t="inlineStr">
         <is>
-          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O111" s="11" t="inlineStr">
         <is>
-          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
+          <t>4 z 5 hostingów PL już ma | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Stan b.d. — jak J-01, weryfikacja na wezle #1.</t>
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr">
@@ -9433,31 +9437,31 @@
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>PB-29</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
-          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
+          <t>Zmiana wersji PHP dla całego konta</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>poza audytem</t>
+          <t>audyt</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t>Praca spoza audytu</t>
+          <t>B — Runtime WWW</t>
         </is>
       </c>
       <c r="E112" s="10" t="inlineStr">
         <is>
-          <t>KRYTYCZNY</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F112" s="10" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G112" s="10" t="n">
         <v>21</v>
@@ -9465,22 +9469,22 @@
       <c r="H112" s="10" t="inlineStr"/>
       <c r="I112" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J112" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K112" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DZIAŁA</t>
         </is>
       </c>
       <c r="L112" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>services.controller.ts:125; D3 t1 28.09: FAIL — selektor bez alt-php (profil nie instalował els-php-release/alt-phpXX na CL10), panel pokazywał wersję mimo błędu → profil + PHP_APPLY cofa wersję (int: php-odrzucona-zmiana.int-spec.ts); retest po profilu; D3 t1 (d3.hvln.pl) 28.09 23:31: PHP 8.2 dla konta z panelu → strona zwraca 8.2.33 na LiteSpeed (PHP_APPLY zakończone); odrzucona zmiana cofa wersję (int)</t>
         </is>
       </c>
       <c r="M112" s="11" t="inlineStr">
@@ -9490,12 +9494,12 @@
       </c>
       <c r="N112" s="11" t="inlineStr">
         <is>
-          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
+          <t>Funkcja dostępna z panelu klienta bez wychodzenia do DirectAdmina; test uruchamiany w CI.</t>
         </is>
       </c>
       <c r="O112" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
+          <t>KOREKTA: pozycja miała stan DZIAŁA na podstawie kodu i kolejki PHP_APPLY. Odkryte 2026-08-21 przy przeglądzie Dockerfile.api: loadery skryptów w API czytają plik z dysku i rzucają wyjątkiem, gdy go nie ma, a obraz produkcyjny kopiował tylko 7 z 10 potrzebnych skryptów. Endpoint /agent/tasks/php-apply/script zwracał 500, więc agent nie miał czego uruchomić — zadanie PHP_APPLY nie mogło się wykonać na produkcji ani razu. Naprawione (COPY + test apps/api/src/test/dockerfile-scripts.spec.ts), ale do czasu potwierdzenia na produkcji stan to CZĘŚCIOWE: kod i testy były zielone przez cały czas, więc D1 i D2 nic tu nie dowodzą — potrzebny D3. | 2026-08-21 21:57: przyczyna wdrożeniowa USUNIĘTA — node-php-apply.sh jest już w obrazie (potwierdzone na serwerze, X-12 D3). Pozycja zostaje CZĘŚCIOWE, bo jej własny dowód wymaga wykonania zadania PHP_APPLY na żywym węźle, a węzła jeszcze nie ma. Do przejścia z części B checklisty D3. | WYCENA 2026-09-19: krytycznosc i naklad uzupelnione przy wznowieniu. Pozycje przepisane 2026-08-28 w ramach X-49 zostaly bez wyceny, przez co nie liczyly sie do budzetu godzin i nie stały w zadnym sprincie. Podstawa wyceny: Zmiana wersji PHP dla calego konta — per domena juz dziala (B-02, S), to ten sam mechanizm o poziom wyzej. | 2026-09-22: przeniesione do sprintu 18 — kod i obraz sa gotowe, zostal wylacznie dowod D3 (PHP_APPLY na zywym wezle).</t>
         </is>
       </c>
       <c r="P112" s="10" t="inlineStr">
@@ -9507,12 +9511,12 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>PB-30</t>
+          <t>PB-02</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>Jeden plik wersji dla floty + test zgodności</t>
+          <t>Onboarding produkcyjnego węzła #1 (Hetzner AX102)</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
@@ -9531,7 +9535,7 @@
         </is>
       </c>
       <c r="F113" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G113" s="10" t="n">
         <v>21</v>
@@ -9539,12 +9543,12 @@
       <c r="H113" s="10" t="inlineStr"/>
       <c r="I113" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J113" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K113" s="10" t="inlineStr">
@@ -9564,12 +9568,12 @@
       </c>
       <c r="N113" s="11" t="inlineStr">
         <is>
-          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
+          <t>Węzeł przechodzi wszystkie 14 checków live-readiness. /etc/verris-backup.conf istnieje, pierwszy backup off-site wykonany i zaraportowany do control-plane.</t>
         </is>
       </c>
       <c r="O113" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
+          <t>Pełny przebieg node-onboard-live.sh na docelowym serwerze, z konfiguracją backupu off-site jako krokiem obowiązkowym.</t>
         </is>
       </c>
       <c r="P113" s="10" t="inlineStr">
@@ -9581,12 +9585,12 @@
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>PB-31</t>
+          <t>PB-29</t>
         </is>
       </c>
       <c r="B114" s="11" t="inlineStr">
         <is>
-          <t>Pełna automatyzacja kreatora węzła</t>
+          <t>Węzeł: blokery bezpieczeństwa i stabilności</t>
         </is>
       </c>
       <c r="C114" s="10" t="inlineStr">
@@ -9601,11 +9605,11 @@
       </c>
       <c r="E114" s="10" t="inlineStr">
         <is>
-          <t>WYSOKI</t>
+          <t>KRYTYCZNY</t>
         </is>
       </c>
       <c r="F114" s="10" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G114" s="10" t="n">
         <v>21</v>
@@ -9613,12 +9617,12 @@
       <c r="H114" s="10" t="inlineStr"/>
       <c r="I114" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J114" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K114" s="10" t="inlineStr">
@@ -9638,12 +9642,12 @@
       </c>
       <c r="N114" s="11" t="inlineStr">
         <is>
-          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
+          <t>Nowy węzeł nie dostaje kont przed zieloną weryfikacją; skrypty przechodzą test na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="O114" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z „da api-url”, kopie off-site floty raz w panelu (szyfrowane, node-backup-config.sh, rclone bez interakcji), auto-zlecenie onboardu po zatwierdzeniu/zapisie kopii, rekord A hosta w OVH, egress SSH/SFTP tylko dla roota + trwałe reguły nftables na AlmaLinux. Zostało ręcznie: OS, klucze licencji, stały klucz DA z ograniczeniem IP, zatwierdzenie. Test na D3.</t>
+          <t>Decyzja właściciela 2026-09-26. Węzeł przyjmuje klientów dopiero po pozytywnym onboardzie i weryfikacji (dziś ACTIVE już po zatwierdzeniu w kroku 3 — servers.service.ts:308); wykrywanie CloudLinux przez cldetect zamiast „lve” w nazwie jądra (dokumentacja CloudLinux: od CL9 jądro AlmaLinux); MariaDB 11.8 LTS zamiast 10.6 (EOL 6.07.2026 wg MariaDB.org); klucze licencji poza linkiem instalacyjnym i usuwane z dysku po instalacji; security-watch na każdym węźle; faza DA w API. | 2026-09-26 ZROBIONE W KODZIE: selektor tylko po zielonym raporcie onboardu (POST /agent/tasks/onboard-report) i bez hardened=false; MariaDB 11.4 (mariadb1104 — Governor nie dokumentuje 11.8; poprawione złe słowo kluczowe 11.x); cldetect + /proc/lve; klucze licencji przez POST /secrets (audyt, pamięć), token w nagłówku, sprzątanie po DONE; pakiet onboardu w układzie repo (security-watch na każdym węźle); faza DA. Zostało: przejście na węźle testowym (D3).</t>
         </is>
       </c>
       <c r="P114" s="10" t="inlineStr">
@@ -9655,12 +9659,12 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>PB-32</t>
+          <t>PB-30</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>Aktualizacje węzłów falami</t>
+          <t>Jeden plik wersji dla floty + test zgodności</t>
         </is>
       </c>
       <c r="C115" s="10" t="inlineStr">
@@ -9675,11 +9679,11 @@
       </c>
       <c r="E115" s="10" t="inlineStr">
         <is>
-          <t>ŚREDNI</t>
+          <t>WYSOKI</t>
         </is>
       </c>
       <c r="F115" s="10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G115" s="10" t="n">
         <v>21</v>
@@ -9687,12 +9691,12 @@
       <c r="H115" s="10" t="inlineStr"/>
       <c r="I115" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J115" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K115" s="10" t="inlineStr">
@@ -9712,12 +9716,12 @@
       </c>
       <c r="N115" s="11" t="inlineStr">
         <is>
-          <t>Fala zatrzymuje się na pierwszym błędzie; status w panelu zgodny z logiem.</t>
+          <t>Dwa węzły z tego samego manifestu dają identyczny raport wersji; różnica widoczna w panelu.</t>
         </is>
       </c>
       <c r="O115" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: najpierw węzeł kanarkowy, potem reszta po jednym; prawdziwy status (dziś skrypt zawsze zwraca ok); aktualizacje z panelu zamiast samodzielnego dnf-automatic. | 2026-09-26 ZROBIONE W KODZIE: fala — kanarek (najmniej kont), potem po jednym po sukcesie, błąd zatrzymuje, druga fala odmowa; skrypt aktualizacji zwraca błąd zamiast zawsze ok; dnf-automatic tylko pobiera. Test na PostgreSQL (fala-aktualizacji.int-spec.ts). Zostało: fala na dwóch węzłach.</t>
+          <t>Decyzja właściciela 2026-09-26: manifest z przypiętymi wersjami (kanał i commit DirectAdmin, LiteSpeed, PHP, MariaDB, reguły CRS), szablon options.conf, sumy kontrolne pobieranych skryptów; węzeł raportuje wersje (pola daVersion/clVersion/lsVersion istnieją, nikt ich nie zapisuje), panel pokazuje różnice między węzłami. | 2026-09-26 ZROBIONE W KODZIE: manifest stos-wezla.ts → /etc/verris-stack.env (bootstrap przed DA + agent co minutę), DA_CHANNEL/DA_COMMIT/php1_release/mariadb przed setup.sh, raport wersji z agenta, audyt „Zgodność z manifestem floty”. Sumy kontrolne: instalatory producentów (setup.sh, cldeploy) nie mają publikowanych sum — zapis zamiast blokady do decyzji po D3. Zostało: DA_COMMIT z testu D3.</t>
         </is>
       </c>
       <c r="P115" s="10" t="inlineStr">
@@ -9729,12 +9733,12 @@
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>PB-33</t>
+          <t>PB-31</t>
         </is>
       </c>
       <c r="B116" s="11" t="inlineStr">
         <is>
-          <t>Wersje stosu floty w panelu + wyrównanie falą</t>
+          <t>Pełna automatyzacja kreatora węzła</t>
         </is>
       </c>
       <c r="C116" s="10" t="inlineStr">
@@ -9753,7 +9757,7 @@
         </is>
       </c>
       <c r="F116" s="10" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="G116" s="10" t="n">
         <v>21</v>
@@ -9761,12 +9765,12 @@
       <c r="H116" s="10" t="inlineStr"/>
       <c r="I116" s="10" t="inlineStr">
         <is>
-          <t>2027-01-18</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="J116" s="10" t="inlineStr">
         <is>
-          <t>2027-01-22</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="K116" s="10" t="inlineStr">
@@ -9786,12 +9790,12 @@
       </c>
       <c r="N116" s="11" t="inlineStr">
         <is>
-          <t>Zmiana wersji w panelu → nowy węzeł instaluje ją, istniejące wyrównane falą; audyt zgodności zielony.</t>
+          <t>Węzeł testowy od czystego AlmaLinux do zielonego raportu bez SSH ręcznie.</t>
         </is>
       </c>
       <c r="O116" s="11" t="inlineStr">
         <is>
-          <t>Decyzja właściciela 2026-09-26: strona „Wersje stosu floty” w panelu admina (DB, PHP, LiteSpeed, DirectAdmin) z dozwolonymi wartościami z oficjalnych list; zmiana obowiązuje nowe węzły od razu, „Wyrównaj flotę” aktualizuje istniejące falą (PHP/LiteSpeed przez CustomBuild, MariaDB po jednej wersji z kopią bazy — wymóg CloudLinux Governor). | 2026-09-26 ZROBIONE W KODZIE: manifest w bazie (StosWezlaService), strona Admin → Wersje stosu floty (dozwolone wartości z oficjalnych list, tabela zgodności), „Wyrównaj flotę” = fala z php1_release + łańcuch DB_UPGRADE krok po kroku z kopią; bootstrap i agent biorą manifest z bazy. Testy na PostgreSQL. Zostało: wyrównanie na węzłach (D3).</t>
+          <t>Decyzja właściciela 2026-09-26: po jednej linijce reszta sama — onboard, profil, kopie off-site bez ręcznego rclone config, klucz logowania DA, IP w DA, TLS, test końcowy; właściciel wpisuje tylko klucze licencji i zatwierdza raport. Dziś ok. 12 ręcznych kroków (scp, SSH, eksport kluczy, rclone config, IP w DA…). | 2026-09-26 ZROBIONE W KODZIE: zadanie ONBOARD_LIVE (pakiet repo → /opt/verris, przycisk w kreatorze, stan i raport), klucz DA do onboardu z 